<commit_message>
Added more foods to diet
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FeedMgmt.xlsx
+++ b/data/prod_parameters/FeedMgmt.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1358" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="460">
   <si>
     <t>f_feed</t>
   </si>
@@ -1402,9 +1402,6 @@
   </si>
   <si>
     <t>include as crop??</t>
-  </si>
-  <si>
-    <t>until incl. as crop</t>
   </si>
 </sst>
 </file>
@@ -1863,7 +1860,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N106"/>
+  <dimension ref="A1:N99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="20.28515625" customWidth="1"/>
@@ -2510,128 +2507,176 @@
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G42" t="s">
-        <v>43</v>
-      </c>
-      <c r="I42" t="s">
-        <v>35</v>
-      </c>
-      <c r="J42" s="3">
-        <v>100</v>
-      </c>
-      <c r="K42" t="s">
-        <v>32</v>
-      </c>
-      <c r="L42" s="3" t="s">
-        <v>460</v>
-      </c>
+      <c r="J42" s="3"/>
+      <c r="L42" s="3"/>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G43" t="s">
-        <v>45</v>
-      </c>
-      <c r="I43" t="s">
-        <v>35</v>
-      </c>
-      <c r="J43" s="3">
-        <v>100</v>
-      </c>
-      <c r="K43" t="s">
-        <v>32</v>
-      </c>
-      <c r="L43" s="3" t="s">
-        <v>460</v>
-      </c>
+      <c r="A43" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
+      <c r="L43" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="M43" s="2"/>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G44" t="s">
-        <v>46</v>
-      </c>
-      <c r="I44" t="s">
-        <v>35</v>
-      </c>
-      <c r="J44" s="3">
-        <v>100</v>
-      </c>
-      <c r="K44" t="s">
-        <v>32</v>
-      </c>
-      <c r="L44" s="3" t="s">
-        <v>460</v>
-      </c>
+      <c r="A44" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B44" s="7"/>
+      <c r="C44" s="6"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6"/>
+      <c r="L44" s="6"/>
+      <c r="M44" s="6"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G45" t="s">
-        <v>39</v>
+      <c r="A45" t="s">
+        <v>28</v>
+      </c>
+      <c r="F45" t="s">
+        <v>19</v>
       </c>
       <c r="I45" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="J45" s="3">
-        <v>100</v>
+        <v>12.4</v>
       </c>
       <c r="K45" t="s">
-        <v>32</v>
-      </c>
-      <c r="L45" s="3" t="s">
-        <v>460</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="J46" s="3"/>
-      <c r="L46" s="3"/>
+      <c r="A46" t="s">
+        <v>28</v>
+      </c>
+      <c r="B46" t="s">
+        <v>22</v>
+      </c>
+      <c r="E46" t="s">
+        <v>23</v>
+      </c>
+      <c r="F46" t="s">
+        <v>2</v>
+      </c>
+      <c r="I46" t="s">
+        <v>20</v>
+      </c>
+      <c r="J46" s="3">
+        <v>12.5</v>
+      </c>
+      <c r="K46" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="J47" s="3"/>
-      <c r="L47" s="3"/>
+      <c r="A47" t="s">
+        <v>28</v>
+      </c>
+      <c r="F47" t="s">
+        <v>2</v>
+      </c>
+      <c r="I47" t="s">
+        <v>20</v>
+      </c>
+      <c r="J47" s="3">
+        <v>11</v>
+      </c>
+      <c r="K47" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="J48" s="3"/>
-      <c r="L48" s="3"/>
+      <c r="A48" t="s">
+        <v>28</v>
+      </c>
+      <c r="F48" t="s">
+        <v>13</v>
+      </c>
+      <c r="I48" t="s">
+        <v>20</v>
+      </c>
+      <c r="J48" s="3">
+        <v>13</v>
+      </c>
+      <c r="K48" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="J49" s="3"/>
-      <c r="L49" s="3"/>
+      <c r="A49" t="s">
+        <v>28</v>
+      </c>
+      <c r="F49" t="s">
+        <v>37</v>
+      </c>
+      <c r="I49" t="s">
+        <v>20</v>
+      </c>
+      <c r="J49" s="3">
+        <v>10</v>
+      </c>
+      <c r="K49" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B50" s="1"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="1"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
-      <c r="I50" s="2"/>
-      <c r="J50" s="2"/>
-      <c r="K50" s="2"/>
-      <c r="L50" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="M50" s="2"/>
+      <c r="A50" t="s">
+        <v>28</v>
+      </c>
+      <c r="F50" t="s">
+        <v>15</v>
+      </c>
+      <c r="I50" t="s">
+        <v>20</v>
+      </c>
+      <c r="J50" s="3">
+        <v>15</v>
+      </c>
+      <c r="K50" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A51" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B51" s="7"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
-      <c r="G51" s="6"/>
-      <c r="H51" s="6"/>
-      <c r="I51" s="6"/>
-      <c r="J51" s="6"/>
-      <c r="K51" s="6"/>
-      <c r="L51" s="6"/>
-      <c r="M51" s="6"/>
+      <c r="A51" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B51" s="8"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
+      <c r="I51" s="9"/>
+      <c r="J51" s="9"/>
+      <c r="K51" s="9"/>
+      <c r="L51" s="9"/>
+      <c r="M51" s="9"/>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="E52" t="s">
+        <v>454</v>
       </c>
       <c r="F52" t="s">
         <v>19</v>
@@ -2639,120 +2684,139 @@
       <c r="I52" t="s">
         <v>20</v>
       </c>
-      <c r="J52" s="3">
-        <v>12.4</v>
+      <c r="J52" s="23">
+        <f>'feed pars'!F6</f>
+        <v>12.3</v>
       </c>
       <c r="K52" t="s">
-        <v>21</v>
+        <v>455</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>28</v>
-      </c>
-      <c r="B53" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="E53" t="s">
-        <v>23</v>
+        <v>454</v>
       </c>
       <c r="F53" t="s">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="I53" t="s">
         <v>20</v>
       </c>
-      <c r="J53" s="3">
-        <v>12.5</v>
+      <c r="J53" s="23">
+        <f>'feed pars'!F7</f>
+        <v>11.2</v>
       </c>
       <c r="K53" t="s">
-        <v>21</v>
+        <v>455</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="E54" t="s">
+        <v>454</v>
       </c>
       <c r="F54" t="s">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="I54" t="s">
         <v>20</v>
       </c>
-      <c r="J54" s="3">
-        <v>11</v>
+      <c r="J54" s="23">
+        <f>'feed pars'!F8</f>
+        <v>9.4</v>
       </c>
       <c r="K54" t="s">
-        <v>21</v>
+        <v>455</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="E55" t="s">
+        <v>454</v>
       </c>
       <c r="F55" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="I55" t="s">
         <v>20</v>
       </c>
-      <c r="J55" s="3">
-        <v>13</v>
+      <c r="J55" s="23">
+        <f>'feed pars'!F9</f>
+        <v>12</v>
       </c>
       <c r="K55" t="s">
-        <v>21</v>
+        <v>455</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="E56" t="s">
+        <v>454</v>
       </c>
       <c r="F56" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="I56" t="s">
         <v>20</v>
       </c>
-      <c r="J56" s="3">
-        <v>10</v>
+      <c r="J56" s="23">
+        <f>'feed pars'!F10</f>
+        <v>13.2</v>
       </c>
       <c r="K56" t="s">
-        <v>21</v>
+        <v>455</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="E57" t="s">
+        <v>454</v>
       </c>
       <c r="F57" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="I57" t="s">
         <v>20</v>
       </c>
-      <c r="J57" s="3">
-        <v>15</v>
+      <c r="J57" s="23">
+        <f>'feed pars'!F11</f>
+        <v>11.5</v>
       </c>
       <c r="K57" t="s">
-        <v>21</v>
+        <v>455</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A58" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B58" s="8"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="9"/>
-      <c r="G58" s="9"/>
-      <c r="H58" s="9"/>
-      <c r="I58" s="9"/>
-      <c r="J58" s="9"/>
-      <c r="K58" s="9"/>
-      <c r="L58" s="9"/>
-      <c r="M58" s="9"/>
+      <c r="A58" t="s">
+        <v>29</v>
+      </c>
+      <c r="E58" t="s">
+        <v>454</v>
+      </c>
+      <c r="F58" t="s">
+        <v>46</v>
+      </c>
+      <c r="I58" t="s">
+        <v>20</v>
+      </c>
+      <c r="J58" s="23">
+        <f>'feed pars'!F12</f>
+        <v>10.9</v>
+      </c>
+      <c r="K58" t="s">
+        <v>455</v>
+      </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
@@ -2762,14 +2826,14 @@
         <v>454</v>
       </c>
       <c r="F59" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="I59" t="s">
         <v>20</v>
       </c>
       <c r="J59" s="23">
-        <f>'feed pars'!F6</f>
-        <v>12.3</v>
+        <f>'feed pars'!F13</f>
+        <v>18.5</v>
       </c>
       <c r="K59" t="s">
         <v>455</v>
@@ -2783,14 +2847,14 @@
         <v>454</v>
       </c>
       <c r="F60" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I60" t="s">
         <v>20</v>
       </c>
       <c r="J60" s="23">
-        <f>'feed pars'!F7</f>
-        <v>11.2</v>
+        <f>'feed pars'!F14</f>
+        <v>17.5</v>
       </c>
       <c r="K60" t="s">
         <v>455</v>
@@ -2804,14 +2868,14 @@
         <v>454</v>
       </c>
       <c r="F61" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="I61" t="s">
         <v>20</v>
       </c>
       <c r="J61" s="23">
-        <f>'feed pars'!F8</f>
-        <v>9.4</v>
+        <f>'feed pars'!F15</f>
+        <v>9.9</v>
       </c>
       <c r="K61" t="s">
         <v>455</v>
@@ -2825,14 +2889,14 @@
         <v>454</v>
       </c>
       <c r="F62" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I62" t="s">
         <v>20</v>
       </c>
       <c r="J62" s="23">
-        <f>'feed pars'!F9</f>
-        <v>12</v>
+        <f>'feed pars'!F16</f>
+        <v>10.3</v>
       </c>
       <c r="K62" t="s">
         <v>455</v>
@@ -2846,14 +2910,14 @@
         <v>454</v>
       </c>
       <c r="F63" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I63" t="s">
         <v>20</v>
       </c>
       <c r="J63" s="23">
-        <f>'feed pars'!F10</f>
-        <v>13.2</v>
+        <f>'feed pars'!F17</f>
+        <v>7.7</v>
       </c>
       <c r="K63" t="s">
         <v>455</v>
@@ -2867,14 +2931,14 @@
         <v>454</v>
       </c>
       <c r="F64" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="I64" t="s">
         <v>20</v>
       </c>
       <c r="J64" s="23">
-        <f>'feed pars'!F11</f>
-        <v>11.5</v>
+        <f>'feed pars'!F18</f>
+        <v>6.5</v>
       </c>
       <c r="K64" t="s">
         <v>455</v>
@@ -2888,14 +2952,14 @@
         <v>454</v>
       </c>
       <c r="F65" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="I65" t="s">
         <v>20</v>
       </c>
       <c r="J65" s="23">
-        <f>'feed pars'!F12</f>
-        <v>10.9</v>
+        <f>'feed pars'!F19</f>
+        <v>6.2</v>
       </c>
       <c r="K65" t="s">
         <v>455</v>
@@ -2909,14 +2973,14 @@
         <v>454</v>
       </c>
       <c r="F66" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="I66" t="s">
         <v>20</v>
       </c>
       <c r="J66" s="23">
-        <f>'feed pars'!F13</f>
-        <v>18.5</v>
+        <f>'feed pars'!F20</f>
+        <v>7.8</v>
       </c>
       <c r="K66" t="s">
         <v>455</v>
@@ -2930,14 +2994,14 @@
         <v>454</v>
       </c>
       <c r="F67" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="I67" t="s">
         <v>20</v>
       </c>
       <c r="J67" s="23">
-        <f>'feed pars'!F14</f>
-        <v>17.5</v>
+        <f>'feed pars'!F21</f>
+        <v>9.1999999999999993</v>
       </c>
       <c r="K67" t="s">
         <v>455</v>
@@ -2951,14 +3015,14 @@
         <v>454</v>
       </c>
       <c r="F68" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I68" t="s">
         <v>20</v>
       </c>
       <c r="J68" s="23">
-        <f>'feed pars'!F15</f>
-        <v>9.9</v>
+        <f>'feed pars'!F22</f>
+        <v>8.6999999999999993</v>
       </c>
       <c r="K68" t="s">
         <v>455</v>
@@ -2972,14 +3036,14 @@
         <v>454</v>
       </c>
       <c r="F69" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="I69" t="s">
         <v>20</v>
       </c>
       <c r="J69" s="23">
-        <f>'feed pars'!F16</f>
-        <v>10.3</v>
+        <f>'feed pars'!F23</f>
+        <v>8.9</v>
       </c>
       <c r="K69" t="s">
         <v>455</v>
@@ -2993,14 +3057,14 @@
         <v>454</v>
       </c>
       <c r="F70" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="I70" t="s">
         <v>20</v>
       </c>
       <c r="J70" s="23">
-        <f>'feed pars'!F17</f>
-        <v>7.7</v>
+        <f>'feed pars'!F24</f>
+        <v>9</v>
       </c>
       <c r="K70" t="s">
         <v>455</v>
@@ -3014,14 +3078,14 @@
         <v>454</v>
       </c>
       <c r="F71" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="I71" t="s">
         <v>20</v>
       </c>
       <c r="J71" s="23">
-        <f>'feed pars'!F18</f>
-        <v>6.5</v>
+        <f>'feed pars'!F25</f>
+        <v>8</v>
       </c>
       <c r="K71" t="s">
         <v>455</v>
@@ -3035,14 +3099,14 @@
         <v>454</v>
       </c>
       <c r="F72" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="I72" t="s">
         <v>20</v>
       </c>
       <c r="J72" s="23">
-        <f>'feed pars'!F19</f>
-        <v>6.2</v>
+        <f>'feed pars'!F26</f>
+        <v>12.2</v>
       </c>
       <c r="K72" t="s">
         <v>455</v>
@@ -3056,14 +3120,14 @@
         <v>454</v>
       </c>
       <c r="F73" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="I73" t="s">
         <v>20</v>
       </c>
       <c r="J73" s="23">
-        <f>'feed pars'!F20</f>
-        <v>7.8</v>
+        <f>'feed pars'!F27</f>
+        <v>12.2</v>
       </c>
       <c r="K73" t="s">
         <v>455</v>
@@ -3077,14 +3141,14 @@
         <v>454</v>
       </c>
       <c r="F74" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="I74" t="s">
         <v>20</v>
       </c>
       <c r="J74" s="23">
-        <f>'feed pars'!F21</f>
-        <v>9.1999999999999993</v>
+        <f>'feed pars'!F28</f>
+        <v>11.3</v>
       </c>
       <c r="K74" t="s">
         <v>455</v>
@@ -3098,14 +3162,14 @@
         <v>454</v>
       </c>
       <c r="F75" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="I75" t="s">
         <v>20</v>
       </c>
       <c r="J75" s="23">
-        <f>'feed pars'!F22</f>
-        <v>8.6999999999999993</v>
+        <f>'feed pars'!F29</f>
+        <v>10.8</v>
       </c>
       <c r="K75" t="s">
         <v>455</v>
@@ -3115,147 +3179,126 @@
       <c r="A76" t="s">
         <v>29</v>
       </c>
-      <c r="E76" t="s">
-        <v>454</v>
-      </c>
       <c r="F76" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="I76" t="s">
         <v>20</v>
       </c>
-      <c r="J76" s="23">
-        <f>'feed pars'!F23</f>
-        <v>8.9</v>
+      <c r="J76">
+        <f>'feed pars'!E6</f>
+        <v>12.1</v>
       </c>
       <c r="K76" t="s">
-        <v>455</v>
+        <v>26</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>29</v>
       </c>
-      <c r="E77" t="s">
-        <v>454</v>
-      </c>
       <c r="F77" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="I77" t="s">
         <v>20</v>
       </c>
-      <c r="J77" s="23">
-        <f>'feed pars'!F24</f>
-        <v>9</v>
+      <c r="J77">
+        <f>'feed pars'!E7</f>
+        <v>11</v>
       </c>
       <c r="K77" t="s">
-        <v>455</v>
+        <v>26</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>29</v>
       </c>
-      <c r="E78" t="s">
-        <v>454</v>
-      </c>
       <c r="F78" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="I78" t="s">
         <v>20</v>
       </c>
-      <c r="J78" s="23">
-        <f>'feed pars'!F25</f>
-        <v>8</v>
+      <c r="J78">
+        <f>'feed pars'!E8</f>
+        <v>9</v>
       </c>
       <c r="K78" t="s">
-        <v>455</v>
+        <v>26</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>29</v>
       </c>
-      <c r="E79" t="s">
-        <v>454</v>
-      </c>
       <c r="F79" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="I79" t="s">
         <v>20</v>
       </c>
-      <c r="J79" s="23">
-        <f>'feed pars'!F26</f>
-        <v>12.2</v>
+      <c r="J79">
+        <f>'feed pars'!E9</f>
+        <v>11.9</v>
       </c>
       <c r="K79" t="s">
-        <v>455</v>
+        <v>26</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>29</v>
       </c>
-      <c r="E80" t="s">
-        <v>454</v>
-      </c>
       <c r="F80" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="I80" t="s">
         <v>20</v>
       </c>
-      <c r="J80" s="23">
-        <f>'feed pars'!F27</f>
-        <v>12.2</v>
+      <c r="J80">
+        <f>'feed pars'!E10</f>
+        <v>12.8</v>
       </c>
       <c r="K80" t="s">
-        <v>455</v>
+        <v>26</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>29</v>
       </c>
-      <c r="E81" t="s">
-        <v>454</v>
-      </c>
       <c r="F81" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="I81" t="s">
         <v>20</v>
       </c>
-      <c r="J81" s="23">
-        <f>'feed pars'!F28</f>
-        <v>11.3</v>
+      <c r="J81">
+        <f>'feed pars'!E11</f>
+        <v>11.2</v>
       </c>
       <c r="K81" t="s">
-        <v>455</v>
+        <v>26</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>29</v>
       </c>
-      <c r="E82" t="s">
-        <v>454</v>
-      </c>
       <c r="F82" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="I82" t="s">
         <v>20</v>
       </c>
-      <c r="J82" s="23">
-        <f>'feed pars'!F29</f>
-        <v>10.8</v>
+      <c r="J82">
+        <f>'feed pars'!E12</f>
+        <v>10.7</v>
       </c>
       <c r="K82" t="s">
-        <v>455</v>
+        <v>26</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -3263,14 +3306,14 @@
         <v>29</v>
       </c>
       <c r="F83" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="I83" t="s">
         <v>20</v>
       </c>
       <c r="J83">
-        <f>'feed pars'!E6</f>
-        <v>12.1</v>
+        <f>'feed pars'!E13</f>
+        <v>18</v>
       </c>
       <c r="K83" t="s">
         <v>26</v>
@@ -3281,14 +3324,14 @@
         <v>29</v>
       </c>
       <c r="F84" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="I84" t="s">
         <v>20</v>
       </c>
       <c r="J84">
-        <f>'feed pars'!E7</f>
-        <v>11</v>
+        <f>'feed pars'!E14</f>
+        <v>17.3</v>
       </c>
       <c r="K84" t="s">
         <v>26</v>
@@ -3299,14 +3342,14 @@
         <v>29</v>
       </c>
       <c r="F85" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="I85" t="s">
         <v>20</v>
       </c>
       <c r="J85">
-        <f>'feed pars'!E8</f>
-        <v>9</v>
+        <f>'feed pars'!E15</f>
+        <v>9.3000000000000007</v>
       </c>
       <c r="K85" t="s">
         <v>26</v>
@@ -3317,14 +3360,14 @@
         <v>29</v>
       </c>
       <c r="F86" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I86" t="s">
         <v>20</v>
       </c>
       <c r="J86">
-        <f>'feed pars'!E9</f>
-        <v>11.9</v>
+        <f>'feed pars'!E16</f>
+        <v>9.6999999999999993</v>
       </c>
       <c r="K86" t="s">
         <v>26</v>
@@ -3335,14 +3378,14 @@
         <v>29</v>
       </c>
       <c r="F87" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I87" t="s">
         <v>20</v>
       </c>
       <c r="J87">
-        <f>'feed pars'!E10</f>
-        <v>12.8</v>
+        <f>'feed pars'!E17</f>
+        <v>7.1</v>
       </c>
       <c r="K87" t="s">
         <v>26</v>
@@ -3353,14 +3396,14 @@
         <v>29</v>
       </c>
       <c r="F88" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="I88" t="s">
         <v>20</v>
       </c>
       <c r="J88">
-        <f>'feed pars'!E11</f>
-        <v>11.2</v>
+        <f>'feed pars'!E18</f>
+        <v>5.9</v>
       </c>
       <c r="K88" t="s">
         <v>26</v>
@@ -3371,14 +3414,14 @@
         <v>29</v>
       </c>
       <c r="F89" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="I89" t="s">
         <v>20</v>
       </c>
       <c r="J89">
-        <f>'feed pars'!E12</f>
-        <v>10.7</v>
+        <f>'feed pars'!E19</f>
+        <v>5.4</v>
       </c>
       <c r="K89" t="s">
         <v>26</v>
@@ -3389,14 +3432,14 @@
         <v>29</v>
       </c>
       <c r="F90" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="I90" t="s">
         <v>20</v>
       </c>
       <c r="J90">
-        <f>'feed pars'!E13</f>
-        <v>18</v>
+        <f>'feed pars'!E20</f>
+        <v>7.2</v>
       </c>
       <c r="K90" t="s">
         <v>26</v>
@@ -3407,14 +3450,14 @@
         <v>29</v>
       </c>
       <c r="F91" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="I91" t="s">
         <v>20</v>
       </c>
       <c r="J91">
-        <f>'feed pars'!E14</f>
-        <v>17.3</v>
+        <f>'feed pars'!E21</f>
+        <v>8.6999999999999993</v>
       </c>
       <c r="K91" t="s">
         <v>26</v>
@@ -3425,14 +3468,14 @@
         <v>29</v>
       </c>
       <c r="F92" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I92" t="s">
         <v>20</v>
       </c>
       <c r="J92">
-        <f>'feed pars'!E15</f>
-        <v>9.3000000000000007</v>
+        <f>'feed pars'!E22</f>
+        <v>8.1</v>
       </c>
       <c r="K92" t="s">
         <v>26</v>
@@ -3443,14 +3486,14 @@
         <v>29</v>
       </c>
       <c r="F93" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="I93" t="s">
         <v>20</v>
       </c>
       <c r="J93">
-        <f>'feed pars'!E16</f>
-        <v>9.6999999999999993</v>
+        <f>'feed pars'!E23</f>
+        <v>8.1999999999999993</v>
       </c>
       <c r="K93" t="s">
         <v>26</v>
@@ -3461,14 +3504,14 @@
         <v>29</v>
       </c>
       <c r="F94" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="I94" t="s">
         <v>20</v>
       </c>
       <c r="J94">
-        <f>'feed pars'!E17</f>
-        <v>7.1</v>
+        <f>'feed pars'!E24</f>
+        <v>8.6999999999999993</v>
       </c>
       <c r="K94" t="s">
         <v>26</v>
@@ -3479,14 +3522,14 @@
         <v>29</v>
       </c>
       <c r="F95" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="I95" t="s">
         <v>20</v>
       </c>
       <c r="J95">
-        <f>'feed pars'!E18</f>
-        <v>5.9</v>
+        <f>'feed pars'!E25</f>
+        <v>6.9</v>
       </c>
       <c r="K95" t="s">
         <v>26</v>
@@ -3497,14 +3540,14 @@
         <v>29</v>
       </c>
       <c r="F96" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="I96" t="s">
         <v>20</v>
       </c>
       <c r="J96">
-        <f>'feed pars'!E19</f>
-        <v>5.4</v>
+        <f>'feed pars'!E26</f>
+        <v>12.4</v>
       </c>
       <c r="K96" t="s">
         <v>26</v>
@@ -3515,14 +3558,14 @@
         <v>29</v>
       </c>
       <c r="F97" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="I97" t="s">
         <v>20</v>
       </c>
       <c r="J97">
-        <f>'feed pars'!E20</f>
-        <v>7.2</v>
+        <f>'feed pars'!E27</f>
+        <v>12.4</v>
       </c>
       <c r="K97" t="s">
         <v>26</v>
@@ -3533,14 +3576,14 @@
         <v>29</v>
       </c>
       <c r="F98" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="I98" t="s">
         <v>20</v>
       </c>
       <c r="J98">
-        <f>'feed pars'!E21</f>
-        <v>8.6999999999999993</v>
+        <f>'feed pars'!E28</f>
+        <v>11.1</v>
       </c>
       <c r="K98" t="s">
         <v>26</v>
@@ -3551,142 +3594,16 @@
         <v>29</v>
       </c>
       <c r="F99" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="I99" t="s">
         <v>20</v>
       </c>
       <c r="J99">
-        <f>'feed pars'!E22</f>
-        <v>8.1</v>
-      </c>
-      <c r="K99" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>29</v>
-      </c>
-      <c r="F100" t="s">
-        <v>55</v>
-      </c>
-      <c r="I100" t="s">
-        <v>20</v>
-      </c>
-      <c r="J100">
-        <f>'feed pars'!E23</f>
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="K100" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>29</v>
-      </c>
-      <c r="F101" t="s">
-        <v>56</v>
-      </c>
-      <c r="I101" t="s">
-        <v>20</v>
-      </c>
-      <c r="J101">
-        <f>'feed pars'!E24</f>
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="K101" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>29</v>
-      </c>
-      <c r="F102" t="s">
-        <v>57</v>
-      </c>
-      <c r="I102" t="s">
-        <v>20</v>
-      </c>
-      <c r="J102">
-        <f>'feed pars'!E25</f>
-        <v>6.9</v>
-      </c>
-      <c r="K102" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>29</v>
-      </c>
-      <c r="F103" t="s">
-        <v>58</v>
-      </c>
-      <c r="I103" t="s">
-        <v>20</v>
-      </c>
-      <c r="J103">
-        <f>'feed pars'!E26</f>
-        <v>12.4</v>
-      </c>
-      <c r="K103" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>29</v>
-      </c>
-      <c r="F104" t="s">
-        <v>59</v>
-      </c>
-      <c r="I104" t="s">
-        <v>20</v>
-      </c>
-      <c r="J104">
-        <f>'feed pars'!E27</f>
-        <v>12.4</v>
-      </c>
-      <c r="K104" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>29</v>
-      </c>
-      <c r="F105" t="s">
-        <v>60</v>
-      </c>
-      <c r="I105" t="s">
-        <v>20</v>
-      </c>
-      <c r="J105">
-        <f>'feed pars'!E28</f>
-        <v>11.1</v>
-      </c>
-      <c r="K105" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>29</v>
-      </c>
-      <c r="F106" t="s">
-        <v>61</v>
-      </c>
-      <c r="I106" t="s">
-        <v>20</v>
-      </c>
-      <c r="J106">
         <f>'feed pars'!E29</f>
         <v>10.8</v>
       </c>
-      <c r="K106" t="s">
+      <c r="K99" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixes to deal with None attributes in AnimalHerds + implementation of attribute 'feed.max_supply_from_crop' to cater for constraint C5
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FeedMgmt.xlsx
+++ b/data/prod_parameters/FeedMgmt.xlsx
@@ -12,7 +12,7 @@
     <sheet name="pigs" sheetId="3" r:id="rId3"/>
     <sheet name="cattle" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913" iterate="1"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="337">
   <si>
     <t>f_feed</t>
   </si>
@@ -997,6 +997,54 @@
   </si>
   <si>
     <t>minerals</t>
+  </si>
+  <si>
+    <t>f_crop</t>
+  </si>
+  <si>
+    <t>dairy</t>
+  </si>
+  <si>
+    <t>cows</t>
+  </si>
+  <si>
+    <t>calves</t>
+  </si>
+  <si>
+    <t>bulls</t>
+  </si>
+  <si>
+    <t>heifers</t>
+  </si>
+  <si>
+    <t>steers</t>
+  </si>
+  <si>
+    <t>breeding bulls</t>
+  </si>
+  <si>
+    <t>beef</t>
+  </si>
+  <si>
+    <t>Semi-natural pastures</t>
+  </si>
+  <si>
+    <t>max_crop_in_crop_prod</t>
+  </si>
+  <si>
+    <r>
+      <t>Maximum contribution of crop to crop product demand for feed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Primarily used to limit semi-natural pastures in grazing)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1464,19 +1512,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N141"/>
+  <dimension ref="A1:O156"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="6" max="6" width="20.28515625" customWidth="1"/>
-    <col min="7" max="7" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.140625" customWidth="1"/>
-    <col min="9" max="9" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="38.140625" customWidth="1"/>
-    <col min="13" max="13" width="58" customWidth="1"/>
+    <col min="6" max="7" width="20.28515625" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.140625" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="38.140625" customWidth="1"/>
+    <col min="14" max="14" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>23</v>
       </c>
@@ -1496,28 +1544,31 @@
         <v>0</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -1528,589 +1579,592 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="2"/>
+      <c r="I2" s="1"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="2"/>
+      <c r="L2" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="L2" s="24" t="s">
+      <c r="M2" s="24" t="s">
         <v>309</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="5"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I3" s="10" t="s">
+      <c r="N2" s="2"/>
+      <c r="O2" s="5"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J3" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="21">
-        <v>0</v>
-      </c>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10" t="s">
+      <c r="K3" s="21">
+        <v>0</v>
+      </c>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F4" t="s">
         <v>310</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>10</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>32</v>
       </c>
-      <c r="J4" s="22">
+      <c r="K4" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F4,'feed pars'!B$6:B$42,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F5" t="s">
         <v>311</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>10</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>32</v>
       </c>
-      <c r="J5" s="22">
+      <c r="K5" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F5,'feed pars'!B$6:B$42,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F6" t="s">
         <v>312</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>10</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="22">
+      <c r="K6" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F6,'feed pars'!B$6:B$42,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F7" t="s">
         <v>2</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>10</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>32</v>
       </c>
-      <c r="J7" s="22">
+      <c r="K7" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F7,'feed pars'!B$6:B$42,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F8" t="s">
         <v>12</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>11</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>32</v>
       </c>
-      <c r="J8" s="22">
+      <c r="K8" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F8,'feed pars'!B$6:B$42,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F9" t="s">
         <v>33</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>33</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>32</v>
       </c>
-      <c r="J9" s="22">
+      <c r="K9" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F9,'feed pars'!B$6:B$42,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F10" t="s">
         <v>17</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>17</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>32</v>
       </c>
-      <c r="J10" s="22">
+      <c r="K10" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F10,'feed pars'!B$6:B$42,0))</f>
         <v>1.1494252873563218</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
         <v>37</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>37</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>32</v>
       </c>
-      <c r="J11" s="22">
+      <c r="K11" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F11,'feed pars'!B$6:B$42,0))</f>
         <v>1.1494252873563218</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
         <v>38</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>38</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>32</v>
       </c>
-      <c r="J12" s="22">
+      <c r="K12" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F12,'feed pars'!B$6:B$42,0))</f>
         <v>1.1627906976744187</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
         <v>39</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>39</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>32</v>
       </c>
-      <c r="J13" s="22">
+      <c r="K13" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F13,'feed pars'!B$6:B$42,0))</f>
         <v>1.1494252873563218</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
         <v>317</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>317</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>32</v>
       </c>
-      <c r="J14" s="22">
+      <c r="K14" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F14,'feed pars'!B$6:B$42,0))</f>
         <v>1.1494252873563218</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F15" t="s">
         <v>40</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>40</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>32</v>
       </c>
-      <c r="J15" s="22">
+      <c r="K15" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F15,'feed pars'!B$6:B$42,0))</f>
         <v>1.4814814814814814</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
         <v>41</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>41</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>32</v>
       </c>
-      <c r="J16" s="22">
+      <c r="K16" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F16,'feed pars'!B$6:B$42,0))</f>
         <v>1.1494252873563218</v>
       </c>
     </row>
-    <row r="17" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F17" t="s">
         <v>42</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>42</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>32</v>
       </c>
-      <c r="J17" s="22">
+      <c r="K17" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F17,'feed pars'!B$6:B$42,0))</f>
         <v>1.1520737327188941</v>
       </c>
     </row>
-    <row r="18" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F18" t="s">
         <v>35</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>35</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>32</v>
       </c>
-      <c r="J18" s="22">
+      <c r="K18" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F18,'feed pars'!B$6:B$42,0))</f>
         <v>1.0810810810810809</v>
       </c>
     </row>
-    <row r="19" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F19" t="s">
         <v>43</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>43</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>32</v>
       </c>
-      <c r="J19" s="22">
+      <c r="K19" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F19,'feed pars'!B$6:B$42,0))</f>
         <v>1.0869565217391304</v>
       </c>
     </row>
-    <row r="20" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F20" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="3"/>
+      <c r="H20" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3" t="s">
+      <c r="I20" s="3"/>
+      <c r="J20" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="J20" s="20">
+      <c r="K20" s="20">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F20,'feed pars'!B$6:B$42,0))*1/0.38</f>
         <v>2.6315789473684212</v>
       </c>
     </row>
-    <row r="21" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F21" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" s="3"/>
+      <c r="H21" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="I21" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="J21" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="J21" s="22"/>
-      <c r="L21" s="3" t="s">
+      <c r="K21" s="22"/>
+      <c r="M21" s="3" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="22" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F22" t="s">
         <v>305</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>305</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>32</v>
       </c>
-      <c r="J22" s="22">
+      <c r="K22" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F22,'feed pars'!B$6:B$42,0))</f>
         <v>1.1764705882352942</v>
       </c>
     </row>
-    <row r="23" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F23" t="s">
         <v>318</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>318</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>32</v>
       </c>
-      <c r="J23" s="22">
+      <c r="K23" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F23,'feed pars'!B$6:B$42,0))</f>
         <v>1.1494252873563218</v>
       </c>
     </row>
-    <row r="24" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F24" t="s">
         <v>44</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>44</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>32</v>
       </c>
-      <c r="J24" s="22">
+      <c r="K24" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F24,'feed pars'!B$6:B$42,0))</f>
         <v>1.1428571428571428</v>
       </c>
     </row>
-    <row r="25" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F25" t="s">
         <v>45</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>45</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>32</v>
       </c>
-      <c r="J25" s="22">
+      <c r="K25" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F25,'feed pars'!B$6:B$42,0))</f>
         <v>1.1494252873563218</v>
       </c>
     </row>
-    <row r="26" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F26" t="s">
         <v>36</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>36</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J26" t="s">
         <v>32</v>
       </c>
-      <c r="J26" s="22">
+      <c r="K26" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F26,'feed pars'!B$6:B$42,0))</f>
         <v>1.1173184357541899</v>
       </c>
     </row>
-    <row r="27" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F27" t="s">
         <v>46</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>46</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>32</v>
       </c>
-      <c r="J27" s="22">
+      <c r="K27" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F27,'feed pars'!B$6:B$42,0))</f>
         <v>1.0989010989010988</v>
       </c>
     </row>
-    <row r="28" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F28" t="s">
         <v>47</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>47</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" t="s">
         <v>32</v>
       </c>
-      <c r="J28" s="22">
+      <c r="K28" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F28,'feed pars'!B$6:B$42,0))</f>
         <v>1.0989010989010988</v>
       </c>
     </row>
-    <row r="29" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F29" t="s">
         <v>319</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>319</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>32</v>
       </c>
-      <c r="J29" s="22">
+      <c r="K29" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F29,'feed pars'!B$6:B$42,0))</f>
         <v>1.1111111111111112</v>
       </c>
     </row>
-    <row r="30" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F30" t="s">
         <v>48</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>48</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>32</v>
       </c>
-      <c r="J30" s="22">
+      <c r="K30" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F30,'feed pars'!B$6:B$42,0))</f>
         <v>1.1494252873563218</v>
       </c>
     </row>
-    <row r="31" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F31" t="s">
         <v>49</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>48</v>
       </c>
-      <c r="I31" t="s">
+      <c r="J31" t="s">
         <v>32</v>
       </c>
-      <c r="J31" s="22">
+      <c r="K31" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F31,'feed pars'!B$6:B$42,0))</f>
         <v>1.1363636363636365</v>
       </c>
     </row>
-    <row r="32" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F32" t="s">
         <v>50</v>
       </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
         <v>301</v>
       </c>
-      <c r="I32" t="s">
+      <c r="J32" t="s">
         <v>32</v>
       </c>
-      <c r="J32" s="20">
-        <f>J33</f>
+      <c r="K32" s="20">
+        <f>K33</f>
         <v>9.0909090909090917</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F33" t="s">
         <v>51</v>
       </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>301</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J33" t="s">
         <v>32</v>
       </c>
-      <c r="J33" s="22">
+      <c r="K33" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F33,'feed pars'!B$6:B$42,0))</f>
         <v>9.0909090909090917</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F34" t="s">
         <v>313</v>
       </c>
-      <c r="H34" t="s">
+      <c r="I34" t="s">
         <v>313</v>
       </c>
-      <c r="I34" t="s">
+      <c r="J34" t="s">
         <v>32</v>
       </c>
-      <c r="J34" s="20">
+      <c r="K34" s="20">
         <f>1/0.25</f>
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F35" t="s">
         <v>52</v>
       </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
         <v>52</v>
       </c>
-      <c r="I35" t="s">
+      <c r="J35" t="s">
         <v>32</v>
       </c>
-      <c r="J35" s="22">
+      <c r="K35" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F35,'feed pars'!B$6:B$42,0))</f>
         <v>1.3245033112582782</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F36" t="s">
         <v>53</v>
       </c>
-      <c r="H36" t="s">
+      <c r="I36" t="s">
         <v>53</v>
       </c>
-      <c r="I36" t="s">
+      <c r="J36" t="s">
         <v>32</v>
       </c>
-      <c r="J36" s="22">
+      <c r="K36" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F36,'feed pars'!B$6:B$42,0))</f>
         <v>1.1173184357541899</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F37" t="s">
         <v>54</v>
       </c>
-      <c r="H37" t="s">
+      <c r="I37" t="s">
         <v>54</v>
       </c>
-      <c r="I37" t="s">
+      <c r="J37" t="s">
         <v>32</v>
       </c>
-      <c r="J37" s="22">
+      <c r="K37" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F37,'feed pars'!B$6:B$42,0))</f>
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F38" t="s">
         <v>55</v>
       </c>
-      <c r="H38" t="s">
+      <c r="I38" t="s">
         <v>54</v>
       </c>
-      <c r="I38" t="s">
+      <c r="J38" t="s">
         <v>32</v>
       </c>
-      <c r="J38" s="20">
-        <f>J37</f>
+      <c r="K38" s="20">
+        <f>K37</f>
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F39" t="s">
         <v>56</v>
       </c>
-      <c r="H39" t="s">
+      <c r="I39" t="s">
         <v>56</v>
       </c>
-      <c r="I39" t="s">
+      <c r="J39" t="s">
         <v>32</v>
       </c>
-      <c r="J39" s="22">
+      <c r="K39" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F39,'feed pars'!B$6:B$42,0))</f>
         <v>1.0989010989010988</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F40" t="s">
         <v>57</v>
       </c>
-      <c r="H40" t="s">
+      <c r="I40" t="s">
         <v>57</v>
       </c>
-      <c r="I40" t="s">
+      <c r="J40" t="s">
         <v>32</v>
       </c>
-      <c r="J40" s="22">
+      <c r="K40" s="22">
         <f>1/INDEX('feed pars'!C$6:C$42/100,MATCH(F40,'feed pars'!B$6:B$42,0))</f>
         <v>1.0869565217391304</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>29</v>
       </c>
@@ -2126,62 +2180,63 @@
       <c r="K41" s="2"/>
       <c r="L41" s="2"/>
       <c r="M41" s="2"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="I42" s="10" t="s">
+      <c r="N41" s="2"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J42" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="J42" s="10">
-        <v>0</v>
-      </c>
-      <c r="K42" s="10"/>
-      <c r="L42" s="10" t="s">
+      <c r="K42" s="10">
+        <v>0</v>
+      </c>
+      <c r="L42" s="10"/>
+      <c r="M42" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G43" t="s">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H43" t="s">
         <v>10</v>
       </c>
-      <c r="I43" t="s">
+      <c r="J43" t="s">
         <v>27</v>
       </c>
-      <c r="J43" s="3">
+      <c r="K43" s="3">
         <v>95</v>
       </c>
-      <c r="K43" t="s">
+      <c r="L43" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G44" t="s">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H44" t="s">
         <v>11</v>
       </c>
-      <c r="I44" t="s">
+      <c r="J44" t="s">
         <v>27</v>
       </c>
-      <c r="J44" s="3">
+      <c r="K44" s="3">
         <v>95</v>
       </c>
-      <c r="K44" t="s">
+      <c r="L44" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G45" t="s">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H45" t="s">
         <v>33</v>
       </c>
-      <c r="I45" t="s">
+      <c r="J45" t="s">
         <v>27</v>
       </c>
-      <c r="J45" s="3">
+      <c r="K45" s="3">
         <v>95</v>
       </c>
-      <c r="K45" t="s">
+      <c r="L45" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>30</v>
       </c>
@@ -2197,928 +2252,967 @@
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="I47" s="10" t="s">
+      <c r="N46" s="2"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J47" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="J47" s="10">
-        <v>0</v>
-      </c>
-      <c r="K47" s="10"/>
-      <c r="L47" s="10" t="s">
+      <c r="K47" s="10">
+        <v>0</v>
+      </c>
+      <c r="L47" s="10"/>
+      <c r="M47" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H48" t="s">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I48" t="s">
         <v>318</v>
       </c>
-      <c r="I48" t="s">
+      <c r="J48" t="s">
         <v>31</v>
       </c>
-      <c r="J48" s="29">
+      <c r="K48" s="29">
         <v>100</v>
       </c>
-      <c r="K48" s="29" t="s">
+      <c r="L48" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="L48" s="10"/>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H49" t="s">
+      <c r="M48" s="10"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I49" t="s">
         <v>44</v>
       </c>
-      <c r="I49" t="s">
+      <c r="J49" t="s">
         <v>31</v>
       </c>
-      <c r="J49" s="29">
+      <c r="K49" s="29">
         <v>100</v>
       </c>
-      <c r="K49" s="29" t="s">
+      <c r="L49" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="L49" s="10"/>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="H50" t="s">
+      <c r="M49" s="10"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I50" t="s">
         <v>36</v>
       </c>
-      <c r="I50" t="s">
+      <c r="J50" t="s">
         <v>31</v>
       </c>
-      <c r="J50" s="29">
+      <c r="K50" s="29">
         <v>61</v>
       </c>
-      <c r="K50" t="s">
+      <c r="L50" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G51" t="s">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H51" t="s">
         <v>43</v>
       </c>
-      <c r="I51" t="s">
+      <c r="J51" t="s">
         <v>31</v>
       </c>
-      <c r="J51" s="3">
+      <c r="K51" s="3">
         <v>100</v>
       </c>
-      <c r="K51" t="s">
+      <c r="L51" t="s">
         <v>28</v>
       </c>
-      <c r="L51" s="3" t="s">
+      <c r="M51" s="3" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="J52" s="3"/>
-      <c r="L52" s="3"/>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
-      <c r="L53" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="M53" s="2"/>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A54" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B54" s="7"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6"/>
-      <c r="J54" s="6"/>
-      <c r="K54" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="L54" s="6"/>
-      <c r="M54" s="6"/>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
+      <c r="L52" s="2"/>
+      <c r="M52" s="2"/>
+      <c r="N52" s="2"/>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>24</v>
+      </c>
+      <c r="B53" t="s">
+        <v>326</v>
+      </c>
+      <c r="E53" t="s">
+        <v>327</v>
+      </c>
+      <c r="G53" t="s">
+        <v>334</v>
+      </c>
+      <c r="H53" t="s">
+        <v>33</v>
+      </c>
+      <c r="J53" t="s">
+        <v>335</v>
+      </c>
+      <c r="K53" s="3">
+        <v>5</v>
+      </c>
+      <c r="L53" t="s">
+        <v>28</v>
+      </c>
+      <c r="M53" s="3"/>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>24</v>
+      </c>
+      <c r="B54" t="s">
+        <v>326</v>
+      </c>
+      <c r="E54" t="s">
+        <v>328</v>
+      </c>
+      <c r="G54" t="s">
+        <v>334</v>
+      </c>
+      <c r="H54" t="s">
+        <v>33</v>
+      </c>
+      <c r="J54" t="s">
+        <v>335</v>
+      </c>
+      <c r="K54" s="3">
+        <v>5</v>
+      </c>
+      <c r="L54" t="s">
+        <v>28</v>
+      </c>
+      <c r="M54" s="3"/>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>24</v>
       </c>
-      <c r="F55" t="s">
-        <v>310</v>
-      </c>
-      <c r="I55" t="s">
-        <v>18</v>
-      </c>
-      <c r="J55" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F55,'feed pars'!B$6:B$42,0))</f>
-        <v>11.5</v>
-      </c>
-      <c r="L55" s="3"/>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>326</v>
+      </c>
+      <c r="E55" t="s">
+        <v>329</v>
+      </c>
+      <c r="G55" t="s">
+        <v>334</v>
+      </c>
+      <c r="H55" t="s">
+        <v>33</v>
+      </c>
+      <c r="J55" t="s">
+        <v>335</v>
+      </c>
+      <c r="K55" s="3">
+        <v>0</v>
+      </c>
+      <c r="L55" t="s">
+        <v>28</v>
+      </c>
+      <c r="M55" s="3"/>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>24</v>
       </c>
-      <c r="F56" t="s">
-        <v>311</v>
-      </c>
-      <c r="I56" t="s">
-        <v>18</v>
-      </c>
-      <c r="J56" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F56,'feed pars'!B$6:B$42,0))</f>
-        <v>10.4</v>
-      </c>
-      <c r="L56" s="3"/>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>326</v>
+      </c>
+      <c r="E56" t="s">
+        <v>330</v>
+      </c>
+      <c r="G56" t="s">
+        <v>334</v>
+      </c>
+      <c r="H56" t="s">
+        <v>33</v>
+      </c>
+      <c r="J56" t="s">
+        <v>335</v>
+      </c>
+      <c r="K56" s="3">
+        <v>90</v>
+      </c>
+      <c r="L56" t="s">
+        <v>28</v>
+      </c>
+      <c r="M56" s="3"/>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>24</v>
       </c>
-      <c r="F57" t="s">
-        <v>312</v>
-      </c>
-      <c r="I57" t="s">
-        <v>18</v>
-      </c>
-      <c r="J57" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F57,'feed pars'!B$6:B$42,0))</f>
-        <v>10</v>
-      </c>
-      <c r="L57" s="3"/>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>326</v>
+      </c>
+      <c r="E57" t="s">
+        <v>331</v>
+      </c>
+      <c r="G57" t="s">
+        <v>334</v>
+      </c>
+      <c r="H57" t="s">
+        <v>33</v>
+      </c>
+      <c r="J57" t="s">
+        <v>335</v>
+      </c>
+      <c r="K57" s="3">
+        <v>90</v>
+      </c>
+      <c r="L57" t="s">
+        <v>28</v>
+      </c>
+      <c r="M57" s="3"/>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>24</v>
       </c>
-      <c r="F58" t="s">
-        <v>12</v>
-      </c>
-      <c r="I58" t="s">
-        <v>18</v>
-      </c>
-      <c r="J58" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F58,'feed pars'!B$6:B$42,0))</f>
-        <v>11.3</v>
-      </c>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>326</v>
+      </c>
+      <c r="E58" t="s">
+        <v>332</v>
+      </c>
+      <c r="G58" t="s">
+        <v>334</v>
+      </c>
+      <c r="H58" t="s">
+        <v>33</v>
+      </c>
+      <c r="J58" t="s">
+        <v>335</v>
+      </c>
+      <c r="K58" s="3">
+        <v>0</v>
+      </c>
+      <c r="L58" t="s">
+        <v>28</v>
+      </c>
+      <c r="M58" s="3"/>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>24</v>
       </c>
-      <c r="F59" t="s">
+      <c r="B59" t="s">
+        <v>333</v>
+      </c>
+      <c r="E59" t="s">
+        <v>327</v>
+      </c>
+      <c r="G59" t="s">
+        <v>334</v>
+      </c>
+      <c r="H59" t="s">
         <v>33</v>
       </c>
-      <c r="I59" t="s">
-        <v>18</v>
-      </c>
-      <c r="J59" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F59,'feed pars'!B$6:B$42,0))</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="J60" s="3"/>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="J59" t="s">
+        <v>335</v>
+      </c>
+      <c r="K59" s="3">
+        <v>90</v>
+      </c>
+      <c r="L59" t="s">
+        <v>28</v>
+      </c>
+      <c r="M59" s="3"/>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>24</v>
+      </c>
+      <c r="B60" t="s">
+        <v>333</v>
+      </c>
+      <c r="E60" t="s">
+        <v>328</v>
+      </c>
+      <c r="G60" t="s">
+        <v>334</v>
+      </c>
+      <c r="H60" t="s">
+        <v>33</v>
+      </c>
+      <c r="J60" t="s">
+        <v>335</v>
+      </c>
+      <c r="K60" s="3">
+        <v>90</v>
+      </c>
+      <c r="L60" t="s">
+        <v>28</v>
+      </c>
+      <c r="M60" s="3"/>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>24</v>
       </c>
-      <c r="F61" t="s">
-        <v>17</v>
-      </c>
-      <c r="I61" t="s">
-        <v>18</v>
-      </c>
-      <c r="J61" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F61,'feed pars'!B$6:B$42,0))</f>
-        <v>14.1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>333</v>
+      </c>
+      <c r="E61" t="s">
+        <v>329</v>
+      </c>
+      <c r="G61" t="s">
+        <v>334</v>
+      </c>
+      <c r="H61" t="s">
+        <v>33</v>
+      </c>
+      <c r="J61" t="s">
+        <v>335</v>
+      </c>
+      <c r="K61" s="3">
+        <v>0</v>
+      </c>
+      <c r="L61" t="s">
+        <v>28</v>
+      </c>
+      <c r="M61" s="3"/>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>24</v>
       </c>
-      <c r="F62" t="s">
-        <v>37</v>
-      </c>
-      <c r="I62" t="s">
-        <v>18</v>
-      </c>
-      <c r="J62" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F62,'feed pars'!B$6:B$42,0))</f>
-        <v>13.2</v>
-      </c>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>333</v>
+      </c>
+      <c r="E62" t="s">
+        <v>330</v>
+      </c>
+      <c r="G62" t="s">
+        <v>334</v>
+      </c>
+      <c r="H62" t="s">
+        <v>33</v>
+      </c>
+      <c r="J62" t="s">
+        <v>335</v>
+      </c>
+      <c r="K62" s="3">
+        <v>90</v>
+      </c>
+      <c r="L62" t="s">
+        <v>28</v>
+      </c>
+      <c r="M62" s="3"/>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>24</v>
       </c>
-      <c r="F63" t="s">
-        <v>38</v>
-      </c>
-      <c r="I63" t="s">
-        <v>18</v>
-      </c>
-      <c r="J63" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F63,'feed pars'!B$6:B$42,0))</f>
-        <v>11.7</v>
-      </c>
-    </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>333</v>
+      </c>
+      <c r="E63" t="s">
+        <v>331</v>
+      </c>
+      <c r="G63" t="s">
+        <v>334</v>
+      </c>
+      <c r="H63" t="s">
+        <v>33</v>
+      </c>
+      <c r="J63" t="s">
+        <v>335</v>
+      </c>
+      <c r="K63" s="3">
+        <v>90</v>
+      </c>
+      <c r="L63" t="s">
+        <v>28</v>
+      </c>
+      <c r="M63" s="3"/>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>24</v>
       </c>
-      <c r="F64" t="s">
-        <v>39</v>
-      </c>
-      <c r="I64" t="s">
-        <v>18</v>
-      </c>
-      <c r="J64" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F64,'feed pars'!B$6:B$42,0))</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>24</v>
-      </c>
-      <c r="F65" t="s">
-        <v>317</v>
-      </c>
-      <c r="I65" t="s">
-        <v>18</v>
-      </c>
-      <c r="J65" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F65,'feed pars'!B$6:B$42,0))</f>
-        <v>13.9</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>24</v>
-      </c>
-      <c r="F66" t="s">
-        <v>40</v>
-      </c>
-      <c r="I66" t="s">
-        <v>18</v>
-      </c>
-      <c r="J66" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F66,'feed pars'!B$6:B$42,0))</f>
-        <v>12.8</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>24</v>
-      </c>
-      <c r="F67" t="s">
-        <v>41</v>
-      </c>
-      <c r="I67" t="s">
-        <v>18</v>
-      </c>
-      <c r="J67" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F67,'feed pars'!B$6:B$42,0))</f>
-        <v>13.8</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>24</v>
-      </c>
-      <c r="F68" t="s">
-        <v>42</v>
-      </c>
-      <c r="I68" t="s">
-        <v>18</v>
-      </c>
-      <c r="J68" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F68,'feed pars'!B$6:B$42,0))</f>
-        <v>13.3</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>24</v>
-      </c>
-      <c r="F69" t="s">
-        <v>35</v>
-      </c>
-      <c r="I69" t="s">
-        <v>18</v>
-      </c>
-      <c r="J69" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F69,'feed pars'!B$6:B$42,0))</f>
-        <v>22.1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>333</v>
+      </c>
+      <c r="E64" t="s">
+        <v>332</v>
+      </c>
+      <c r="G64" t="s">
+        <v>334</v>
+      </c>
+      <c r="H64" t="s">
+        <v>33</v>
+      </c>
+      <c r="J64" t="s">
+        <v>335</v>
+      </c>
+      <c r="K64" s="3">
+        <v>90</v>
+      </c>
+      <c r="L64" t="s">
+        <v>28</v>
+      </c>
+      <c r="M64" s="3"/>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K65" s="3"/>
+      <c r="M65" s="3"/>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K66" s="3"/>
+      <c r="M66" s="3"/>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K67" s="3"/>
+      <c r="M67" s="3"/>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B68" s="1"/>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="2"/>
+      <c r="F68" s="2"/>
+      <c r="G68" s="2"/>
+      <c r="H68" s="2"/>
+      <c r="I68" s="2"/>
+      <c r="J68" s="2"/>
+      <c r="K68" s="2"/>
+      <c r="L68" s="2"/>
+      <c r="M68" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="N68" s="2"/>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A69" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B69" s="7"/>
+      <c r="C69" s="6"/>
+      <c r="D69" s="6"/>
+      <c r="E69" s="6"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="6"/>
+      <c r="H69" s="6"/>
+      <c r="I69" s="6"/>
+      <c r="J69" s="6"/>
+      <c r="K69" s="6"/>
+      <c r="L69" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M69" s="6"/>
+      <c r="N69" s="6"/>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>24</v>
       </c>
       <c r="F70" t="s">
-        <v>43</v>
-      </c>
-      <c r="I70" t="s">
+        <v>310</v>
+      </c>
+      <c r="J70" t="s">
         <v>18</v>
       </c>
-      <c r="J70" s="26">
+      <c r="K70" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F70,'feed pars'!B$6:B$42,0))</f>
-        <v>20.100000000000001</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+        <v>11.5</v>
+      </c>
+      <c r="M70" s="3"/>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>24</v>
       </c>
       <c r="F71" t="s">
-        <v>305</v>
-      </c>
-      <c r="I71" t="s">
+        <v>311</v>
+      </c>
+      <c r="J71" t="s">
         <v>18</v>
       </c>
-      <c r="J71" s="26">
+      <c r="K71" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F71,'feed pars'!B$6:B$42,0))</f>
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+        <v>10.4</v>
+      </c>
+      <c r="M71" s="3"/>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>24</v>
       </c>
       <c r="F72" t="s">
-        <v>314</v>
-      </c>
-      <c r="I72" t="s">
+        <v>312</v>
+      </c>
+      <c r="J72" t="s">
         <v>18</v>
       </c>
-      <c r="J72" s="26">
+      <c r="K72" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F72,'feed pars'!B$6:B$42,0))</f>
-        <v>36.6</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="M72" s="3"/>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>24</v>
       </c>
       <c r="F73" t="s">
-        <v>318</v>
-      </c>
-      <c r="I73" t="s">
+        <v>12</v>
+      </c>
+      <c r="J73" t="s">
         <v>18</v>
       </c>
-      <c r="J73" s="26">
+      <c r="K73" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F73,'feed pars'!B$6:B$42,0))</f>
-        <v>16.399999999999999</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>24</v>
       </c>
       <c r="F74" t="s">
-        <v>44</v>
-      </c>
-      <c r="I74" t="s">
+        <v>33</v>
+      </c>
+      <c r="J74" t="s">
         <v>18</v>
       </c>
-      <c r="J74" s="26">
+      <c r="K74" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F74,'feed pars'!B$6:B$42,0))</f>
-        <v>14.6</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>24</v>
-      </c>
-      <c r="F75" t="s">
-        <v>36</v>
-      </c>
-      <c r="I75" t="s">
-        <v>18</v>
-      </c>
-      <c r="J75" s="26">
-        <f>INDEX('feed pars'!M$6:M$42,MATCH(F75,'feed pars'!B$6:B$42,0))</f>
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K75" s="3"/>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>24</v>
       </c>
       <c r="F76" t="s">
-        <v>46</v>
-      </c>
-      <c r="I76" t="s">
+        <v>17</v>
+      </c>
+      <c r="J76" t="s">
         <v>18</v>
       </c>
-      <c r="J76" s="26">
+      <c r="K76" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F76,'feed pars'!B$6:B$42,0))</f>
-        <v>11.4</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>24</v>
       </c>
       <c r="F77" t="s">
-        <v>47</v>
-      </c>
-      <c r="I77" t="s">
+        <v>37</v>
+      </c>
+      <c r="J77" t="s">
         <v>18</v>
       </c>
-      <c r="J77" s="26">
+      <c r="K77" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F77,'feed pars'!B$6:B$42,0))</f>
-        <v>13.4</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>24</v>
       </c>
       <c r="F78" t="s">
-        <v>319</v>
-      </c>
-      <c r="I78" t="s">
+        <v>38</v>
+      </c>
+      <c r="J78" t="s">
         <v>18</v>
       </c>
-      <c r="J78" s="26">
+      <c r="K78" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F78,'feed pars'!B$6:B$42,0))</f>
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>24</v>
       </c>
       <c r="F79" t="s">
-        <v>48</v>
-      </c>
-      <c r="I79" t="s">
+        <v>39</v>
+      </c>
+      <c r="J79" t="s">
         <v>18</v>
       </c>
-      <c r="J79" s="26">
+      <c r="K79" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F79,'feed pars'!B$6:B$42,0))</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>24</v>
       </c>
       <c r="F80" t="s">
-        <v>50</v>
-      </c>
-      <c r="I80" t="s">
+        <v>317</v>
+      </c>
+      <c r="J80" t="s">
         <v>18</v>
       </c>
-      <c r="J80" s="26">
+      <c r="K80" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F80,'feed pars'!B$6:B$42,0))</f>
-        <v>13.3</v>
-      </c>
-    </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>24</v>
       </c>
       <c r="F81" t="s">
-        <v>313</v>
-      </c>
-      <c r="I81" t="s">
+        <v>40</v>
+      </c>
+      <c r="J81" t="s">
         <v>18</v>
       </c>
-      <c r="J81" s="26">
+      <c r="K81" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F81,'feed pars'!B$6:B$42,0))</f>
-        <v>11.6</v>
-      </c>
-    </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>24</v>
       </c>
       <c r="F82" t="s">
-        <v>52</v>
-      </c>
-      <c r="I82" t="s">
+        <v>41</v>
+      </c>
+      <c r="J82" t="s">
         <v>18</v>
       </c>
-      <c r="J82" s="26">
+      <c r="K82" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F82,'feed pars'!B$6:B$42,0))</f>
-        <v>12.4</v>
-      </c>
-    </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>24</v>
       </c>
       <c r="F83" t="s">
-        <v>53</v>
-      </c>
-      <c r="I83" t="s">
+        <v>42</v>
+      </c>
+      <c r="J83" t="s">
         <v>18</v>
       </c>
-      <c r="J83" s="26">
+      <c r="K83" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F83,'feed pars'!B$6:B$42,0))</f>
-        <v>12.3</v>
-      </c>
-    </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>24</v>
       </c>
       <c r="F84" t="s">
-        <v>54</v>
-      </c>
-      <c r="I84" t="s">
+        <v>35</v>
+      </c>
+      <c r="J84" t="s">
         <v>18</v>
       </c>
-      <c r="J84" s="26">
+      <c r="K84" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F84,'feed pars'!B$6:B$42,0))</f>
-        <v>13.6</v>
-      </c>
-    </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>24</v>
       </c>
       <c r="F85" t="s">
-        <v>56</v>
-      </c>
-      <c r="I85" t="s">
+        <v>43</v>
+      </c>
+      <c r="J85" t="s">
         <v>18</v>
       </c>
-      <c r="J85" s="26">
+      <c r="K85" s="26">
         <f>INDEX('feed pars'!M$6:M$42,MATCH(F85,'feed pars'!B$6:B$42,0))</f>
-        <v>15.5</v>
-      </c>
-    </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+        <v>20.100000000000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>24</v>
       </c>
       <c r="F86" t="s">
+        <v>305</v>
+      </c>
+      <c r="J86" t="s">
+        <v>18</v>
+      </c>
+      <c r="K86" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F86,'feed pars'!B$6:B$42,0))</f>
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>24</v>
+      </c>
+      <c r="F87" t="s">
+        <v>314</v>
+      </c>
+      <c r="J87" t="s">
+        <v>18</v>
+      </c>
+      <c r="K87" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F87,'feed pars'!B$6:B$42,0))</f>
+        <v>36.6</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>24</v>
+      </c>
+      <c r="F88" t="s">
+        <v>318</v>
+      </c>
+      <c r="J88" t="s">
+        <v>18</v>
+      </c>
+      <c r="K88" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F88,'feed pars'!B$6:B$42,0))</f>
+        <v>16.399999999999999</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>24</v>
+      </c>
+      <c r="F89" t="s">
+        <v>44</v>
+      </c>
+      <c r="J89" t="s">
+        <v>18</v>
+      </c>
+      <c r="K89" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F89,'feed pars'!B$6:B$42,0))</f>
+        <v>14.6</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>24</v>
+      </c>
+      <c r="F90" t="s">
+        <v>36</v>
+      </c>
+      <c r="J90" t="s">
+        <v>18</v>
+      </c>
+      <c r="K90" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F90,'feed pars'!B$6:B$42,0))</f>
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>24</v>
+      </c>
+      <c r="F91" t="s">
+        <v>46</v>
+      </c>
+      <c r="J91" t="s">
+        <v>18</v>
+      </c>
+      <c r="K91" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F91,'feed pars'!B$6:B$42,0))</f>
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>24</v>
+      </c>
+      <c r="F92" t="s">
+        <v>47</v>
+      </c>
+      <c r="J92" t="s">
+        <v>18</v>
+      </c>
+      <c r="K92" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F92,'feed pars'!B$6:B$42,0))</f>
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>24</v>
+      </c>
+      <c r="F93" t="s">
+        <v>319</v>
+      </c>
+      <c r="J93" t="s">
+        <v>18</v>
+      </c>
+      <c r="K93" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F93,'feed pars'!B$6:B$42,0))</f>
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>24</v>
+      </c>
+      <c r="F94" t="s">
+        <v>48</v>
+      </c>
+      <c r="J94" t="s">
+        <v>18</v>
+      </c>
+      <c r="K94" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F94,'feed pars'!B$6:B$42,0))</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>24</v>
+      </c>
+      <c r="F95" t="s">
+        <v>50</v>
+      </c>
+      <c r="J95" t="s">
+        <v>18</v>
+      </c>
+      <c r="K95" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F95,'feed pars'!B$6:B$42,0))</f>
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>24</v>
+      </c>
+      <c r="F96" t="s">
+        <v>313</v>
+      </c>
+      <c r="J96" t="s">
+        <v>18</v>
+      </c>
+      <c r="K96" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F96,'feed pars'!B$6:B$42,0))</f>
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>24</v>
+      </c>
+      <c r="F97" t="s">
+        <v>52</v>
+      </c>
+      <c r="J97" t="s">
+        <v>18</v>
+      </c>
+      <c r="K97" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F97,'feed pars'!B$6:B$42,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>24</v>
+      </c>
+      <c r="F98" t="s">
+        <v>53</v>
+      </c>
+      <c r="J98" t="s">
+        <v>18</v>
+      </c>
+      <c r="K98" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F98,'feed pars'!B$6:B$42,0))</f>
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>24</v>
+      </c>
+      <c r="F99" t="s">
+        <v>54</v>
+      </c>
+      <c r="J99" t="s">
+        <v>18</v>
+      </c>
+      <c r="K99" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F99,'feed pars'!B$6:B$42,0))</f>
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>24</v>
+      </c>
+      <c r="F100" t="s">
+        <v>56</v>
+      </c>
+      <c r="J100" t="s">
+        <v>18</v>
+      </c>
+      <c r="K100" s="26">
+        <f>INDEX('feed pars'!M$6:M$42,MATCH(F100,'feed pars'!B$6:B$42,0))</f>
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>24</v>
+      </c>
+      <c r="F101" t="s">
         <v>324</v>
       </c>
-      <c r="I86" t="s">
+      <c r="J101" t="s">
         <v>18</v>
       </c>
-      <c r="J86" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="J87" s="3"/>
-    </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A88" s="8" t="s">
+      <c r="K101" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K102" s="3"/>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A103" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B88" s="8"/>
-      <c r="C88" s="9"/>
-      <c r="D88" s="9"/>
-      <c r="E88" s="9"/>
-      <c r="F88" s="9"/>
-      <c r="G88" s="9"/>
-      <c r="H88" s="9"/>
-      <c r="I88" s="9"/>
-      <c r="J88" s="9"/>
-      <c r="K88" s="9"/>
-      <c r="L88" s="9"/>
-      <c r="M88" s="9"/>
-    </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>25</v>
-      </c>
-      <c r="E89" t="s">
-        <v>299</v>
-      </c>
-      <c r="F89" t="s">
-        <v>17</v>
-      </c>
-      <c r="I89" t="s">
-        <v>18</v>
-      </c>
-      <c r="J89" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F89,'feed pars'!B$6:B$42,0))</f>
-        <v>12.3</v>
-      </c>
-      <c r="K89" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>25</v>
-      </c>
-      <c r="E90" t="s">
-        <v>299</v>
-      </c>
-      <c r="F90" t="s">
-        <v>37</v>
-      </c>
-      <c r="I90" t="s">
-        <v>18</v>
-      </c>
-      <c r="J90" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F90,'feed pars'!B$6:B$42,0))</f>
-        <v>11.2</v>
-      </c>
-      <c r="K90" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>25</v>
-      </c>
-      <c r="E91" t="s">
-        <v>299</v>
-      </c>
-      <c r="F91" t="s">
-        <v>38</v>
-      </c>
-      <c r="I91" t="s">
-        <v>18</v>
-      </c>
-      <c r="J91" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F91,'feed pars'!B$6:B$42,0))</f>
-        <v>9.4</v>
-      </c>
-      <c r="K91" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>25</v>
-      </c>
-      <c r="E92" t="s">
-        <v>299</v>
-      </c>
-      <c r="F92" t="s">
-        <v>39</v>
-      </c>
-      <c r="I92" t="s">
-        <v>18</v>
-      </c>
-      <c r="J92" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F92,'feed pars'!B$6:B$42,0))</f>
-        <v>12</v>
-      </c>
-      <c r="K92" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>25</v>
-      </c>
-      <c r="E93" t="s">
-        <v>299</v>
-      </c>
-      <c r="F93" t="s">
-        <v>40</v>
-      </c>
-      <c r="I93" t="s">
-        <v>18</v>
-      </c>
-      <c r="J93" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F93,'feed pars'!B$6:B$42,0))</f>
-        <v>13.2</v>
-      </c>
-      <c r="K93" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>25</v>
-      </c>
-      <c r="E94" t="s">
-        <v>299</v>
-      </c>
-      <c r="F94" t="s">
-        <v>41</v>
-      </c>
-      <c r="I94" t="s">
-        <v>18</v>
-      </c>
-      <c r="J94" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F94,'feed pars'!B$6:B$42,0))</f>
-        <v>11.5</v>
-      </c>
-      <c r="K94" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>25</v>
-      </c>
-      <c r="E95" t="s">
-        <v>299</v>
-      </c>
-      <c r="F95" t="s">
-        <v>42</v>
-      </c>
-      <c r="I95" t="s">
-        <v>18</v>
-      </c>
-      <c r="J95" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F95,'feed pars'!B$6:B$42,0))</f>
-        <v>10.9</v>
-      </c>
-      <c r="K95" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>25</v>
-      </c>
-      <c r="E96" t="s">
-        <v>299</v>
-      </c>
-      <c r="F96" t="s">
-        <v>35</v>
-      </c>
-      <c r="I96" t="s">
-        <v>18</v>
-      </c>
-      <c r="J96" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F96,'feed pars'!B$6:B$42,0))</f>
-        <v>18.5</v>
-      </c>
-      <c r="K96" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>25</v>
-      </c>
-      <c r="E97" t="s">
-        <v>299</v>
-      </c>
-      <c r="F97" t="s">
-        <v>43</v>
-      </c>
-      <c r="I97" t="s">
-        <v>18</v>
-      </c>
-      <c r="J97" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F97,'feed pars'!B$6:B$42,0))</f>
-        <v>17.5</v>
-      </c>
-      <c r="K97" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>25</v>
-      </c>
-      <c r="E98" t="s">
-        <v>299</v>
-      </c>
-      <c r="F98" t="s">
-        <v>314</v>
-      </c>
-      <c r="I98" t="s">
-        <v>18</v>
-      </c>
-      <c r="J98" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F98,'feed pars'!B$6:B$42,0))</f>
-        <v>29.8</v>
-      </c>
-      <c r="K98" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>25</v>
-      </c>
-      <c r="E99" t="s">
-        <v>299</v>
-      </c>
-      <c r="F99" t="s">
-        <v>44</v>
-      </c>
-      <c r="I99" t="s">
-        <v>18</v>
-      </c>
-      <c r="J99" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F99,'feed pars'!B$6:B$42,0))</f>
-        <v>9.9</v>
-      </c>
-      <c r="K99" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>25</v>
-      </c>
-      <c r="E100" t="s">
-        <v>299</v>
-      </c>
-      <c r="F100" t="s">
-        <v>45</v>
-      </c>
-      <c r="I100" t="s">
-        <v>18</v>
-      </c>
-      <c r="J100" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F100,'feed pars'!B$6:B$42,0))</f>
-        <v>10.3</v>
-      </c>
-      <c r="K100" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>25</v>
-      </c>
-      <c r="E101" t="s">
-        <v>299</v>
-      </c>
-      <c r="F101" t="s">
-        <v>36</v>
-      </c>
-      <c r="I101" t="s">
-        <v>18</v>
-      </c>
-      <c r="J101" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F101,'feed pars'!B$6:B$42,0))</f>
-        <v>7.7</v>
-      </c>
-      <c r="K101" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>25</v>
-      </c>
-      <c r="E102" t="s">
-        <v>299</v>
-      </c>
-      <c r="F102" t="s">
-        <v>46</v>
-      </c>
-      <c r="I102" t="s">
-        <v>18</v>
-      </c>
-      <c r="J102" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F102,'feed pars'!B$6:B$42,0))</f>
-        <v>6.5</v>
-      </c>
-      <c r="K102" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>25</v>
-      </c>
-      <c r="E103" t="s">
-        <v>299</v>
-      </c>
-      <c r="F103" t="s">
-        <v>47</v>
-      </c>
-      <c r="I103" t="s">
-        <v>18</v>
-      </c>
-      <c r="J103" s="26">
-        <f>INDEX('feed pars'!H$6:H$42,MATCH(F103,'feed pars'!B$6:B$42,0))</f>
-        <v>6.2</v>
-      </c>
-      <c r="K103" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B103" s="8"/>
+      <c r="C103" s="9"/>
+      <c r="D103" s="9"/>
+      <c r="E103" s="9"/>
+      <c r="F103" s="9"/>
+      <c r="G103" s="9"/>
+      <c r="H103" s="9"/>
+      <c r="I103" s="9"/>
+      <c r="J103" s="9"/>
+      <c r="K103" s="9"/>
+      <c r="L103" s="9"/>
+      <c r="M103" s="9"/>
+      <c r="N103" s="9"/>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>25</v>
       </c>
@@ -3126,20 +3220,20 @@
         <v>299</v>
       </c>
       <c r="F104" t="s">
-        <v>48</v>
-      </c>
-      <c r="I104" t="s">
+        <v>17</v>
+      </c>
+      <c r="J104" t="s">
         <v>18</v>
       </c>
-      <c r="J104" s="26">
+      <c r="K104" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F104,'feed pars'!B$6:B$42,0))</f>
-        <v>7.8</v>
-      </c>
-      <c r="K104" t="s">
+        <v>12.3</v>
+      </c>
+      <c r="L104" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>25</v>
       </c>
@@ -3147,20 +3241,20 @@
         <v>299</v>
       </c>
       <c r="F105" t="s">
-        <v>49</v>
-      </c>
-      <c r="I105" t="s">
+        <v>37</v>
+      </c>
+      <c r="J105" t="s">
         <v>18</v>
       </c>
-      <c r="J105" s="26">
+      <c r="K105" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F105,'feed pars'!B$6:B$42,0))</f>
-        <v>9.1999999999999993</v>
-      </c>
-      <c r="K105" t="s">
+        <v>11.2</v>
+      </c>
+      <c r="L105" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>25</v>
       </c>
@@ -3168,20 +3262,20 @@
         <v>299</v>
       </c>
       <c r="F106" t="s">
-        <v>50</v>
-      </c>
-      <c r="I106" t="s">
+        <v>38</v>
+      </c>
+      <c r="J106" t="s">
         <v>18</v>
       </c>
-      <c r="J106" s="26">
+      <c r="K106" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F106,'feed pars'!B$6:B$42,0))</f>
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="K106" t="s">
+        <v>9.4</v>
+      </c>
+      <c r="L106" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>25</v>
       </c>
@@ -3189,20 +3283,20 @@
         <v>299</v>
       </c>
       <c r="F107" t="s">
-        <v>51</v>
-      </c>
-      <c r="I107" t="s">
+        <v>39</v>
+      </c>
+      <c r="J107" t="s">
         <v>18</v>
       </c>
-      <c r="J107" s="26">
+      <c r="K107" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F107,'feed pars'!B$6:B$42,0))</f>
-        <v>8.9</v>
-      </c>
-      <c r="K107" t="s">
+        <v>12</v>
+      </c>
+      <c r="L107" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>25</v>
       </c>
@@ -3210,20 +3304,20 @@
         <v>299</v>
       </c>
       <c r="F108" t="s">
-        <v>313</v>
-      </c>
-      <c r="I108" t="s">
+        <v>40</v>
+      </c>
+      <c r="J108" t="s">
         <v>18</v>
       </c>
-      <c r="J108" s="26">
+      <c r="K108" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F108,'feed pars'!B$6:B$42,0))</f>
-        <v>7.0888888888888877</v>
-      </c>
-      <c r="K108" t="s">
+        <v>13.2</v>
+      </c>
+      <c r="L108" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>25</v>
       </c>
@@ -3231,20 +3325,20 @@
         <v>299</v>
       </c>
       <c r="F109" t="s">
-        <v>52</v>
-      </c>
-      <c r="I109" t="s">
+        <v>41</v>
+      </c>
+      <c r="J109" t="s">
         <v>18</v>
       </c>
-      <c r="J109" s="26">
+      <c r="K109" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F109,'feed pars'!B$6:B$42,0))</f>
-        <v>9</v>
-      </c>
-      <c r="K109" t="s">
+        <v>11.5</v>
+      </c>
+      <c r="L109" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>25</v>
       </c>
@@ -3252,20 +3346,20 @@
         <v>299</v>
       </c>
       <c r="F110" t="s">
-        <v>53</v>
-      </c>
-      <c r="I110" t="s">
+        <v>42</v>
+      </c>
+      <c r="J110" t="s">
         <v>18</v>
       </c>
-      <c r="J110" s="26">
+      <c r="K110" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F110,'feed pars'!B$6:B$42,0))</f>
-        <v>8</v>
-      </c>
-      <c r="K110" t="s">
+        <v>10.9</v>
+      </c>
+      <c r="L110" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>25</v>
       </c>
@@ -3273,20 +3367,20 @@
         <v>299</v>
       </c>
       <c r="F111" t="s">
-        <v>54</v>
-      </c>
-      <c r="I111" t="s">
+        <v>35</v>
+      </c>
+      <c r="J111" t="s">
         <v>18</v>
       </c>
-      <c r="J111" s="26">
+      <c r="K111" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F111,'feed pars'!B$6:B$42,0))</f>
-        <v>12.2</v>
-      </c>
-      <c r="K111" t="s">
+        <v>18.5</v>
+      </c>
+      <c r="L111" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>25</v>
       </c>
@@ -3294,20 +3388,20 @@
         <v>299</v>
       </c>
       <c r="F112" t="s">
-        <v>55</v>
-      </c>
-      <c r="I112" t="s">
+        <v>43</v>
+      </c>
+      <c r="J112" t="s">
         <v>18</v>
       </c>
-      <c r="J112" s="26">
+      <c r="K112" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F112,'feed pars'!B$6:B$42,0))</f>
-        <v>12.2</v>
-      </c>
-      <c r="K112" t="s">
+        <v>17.5</v>
+      </c>
+      <c r="L112" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>25</v>
       </c>
@@ -3315,20 +3409,20 @@
         <v>299</v>
       </c>
       <c r="F113" t="s">
-        <v>56</v>
-      </c>
-      <c r="I113" t="s">
+        <v>314</v>
+      </c>
+      <c r="J113" t="s">
         <v>18</v>
       </c>
-      <c r="J113" s="26">
+      <c r="K113" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F113,'feed pars'!B$6:B$42,0))</f>
-        <v>11.3</v>
-      </c>
-      <c r="K113" t="s">
+        <v>29.8</v>
+      </c>
+      <c r="L113" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>25</v>
       </c>
@@ -3336,487 +3430,802 @@
         <v>299</v>
       </c>
       <c r="F114" t="s">
-        <v>57</v>
-      </c>
-      <c r="I114" t="s">
+        <v>44</v>
+      </c>
+      <c r="J114" t="s">
         <v>18</v>
       </c>
-      <c r="J114" s="26">
+      <c r="K114" s="26">
         <f>INDEX('feed pars'!H$6:H$42,MATCH(F114,'feed pars'!B$6:B$42,0))</f>
-        <v>10.8</v>
-      </c>
-      <c r="K114" t="s">
+        <v>9.9</v>
+      </c>
+      <c r="L114" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="J115" s="26"/>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>25</v>
+      </c>
+      <c r="E115" t="s">
+        <v>299</v>
+      </c>
+      <c r="F115" t="s">
+        <v>45</v>
+      </c>
+      <c r="J115" t="s">
+        <v>18</v>
+      </c>
+      <c r="K115" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F115,'feed pars'!B$6:B$42,0))</f>
+        <v>10.3</v>
+      </c>
+      <c r="L115" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>25</v>
       </c>
+      <c r="E116" t="s">
+        <v>299</v>
+      </c>
       <c r="F116" t="s">
-        <v>17</v>
-      </c>
-      <c r="I116" t="s">
+        <v>36</v>
+      </c>
+      <c r="J116" t="s">
         <v>18</v>
       </c>
-      <c r="J116" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F116,'feed pars'!B$6:B$42,0))</f>
-        <v>12.1</v>
-      </c>
-      <c r="K116" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K116" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F116,'feed pars'!B$6:B$42,0))</f>
+        <v>7.7</v>
+      </c>
+      <c r="L116" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>25</v>
       </c>
+      <c r="E117" t="s">
+        <v>299</v>
+      </c>
       <c r="F117" t="s">
-        <v>37</v>
-      </c>
-      <c r="I117" t="s">
+        <v>46</v>
+      </c>
+      <c r="J117" t="s">
         <v>18</v>
       </c>
-      <c r="J117" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F117,'feed pars'!B$6:B$42,0))</f>
-        <v>11</v>
-      </c>
-      <c r="K117" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K117" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F117,'feed pars'!B$6:B$42,0))</f>
+        <v>6.5</v>
+      </c>
+      <c r="L117" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>25</v>
       </c>
+      <c r="E118" t="s">
+        <v>299</v>
+      </c>
       <c r="F118" t="s">
-        <v>38</v>
-      </c>
-      <c r="I118" t="s">
+        <v>47</v>
+      </c>
+      <c r="J118" t="s">
         <v>18</v>
       </c>
-      <c r="J118" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F118,'feed pars'!B$6:B$42,0))</f>
-        <v>9</v>
-      </c>
-      <c r="K118" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K118" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F118,'feed pars'!B$6:B$42,0))</f>
+        <v>6.2</v>
+      </c>
+      <c r="L118" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>25</v>
       </c>
+      <c r="E119" t="s">
+        <v>299</v>
+      </c>
       <c r="F119" t="s">
-        <v>39</v>
-      </c>
-      <c r="I119" t="s">
+        <v>48</v>
+      </c>
+      <c r="J119" t="s">
         <v>18</v>
       </c>
-      <c r="J119" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F119,'feed pars'!B$6:B$42,0))</f>
-        <v>11.9</v>
-      </c>
-      <c r="K119" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K119" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F119,'feed pars'!B$6:B$42,0))</f>
+        <v>7.8</v>
+      </c>
+      <c r="L119" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>25</v>
       </c>
+      <c r="E120" t="s">
+        <v>299</v>
+      </c>
       <c r="F120" t="s">
-        <v>40</v>
-      </c>
-      <c r="I120" t="s">
+        <v>49</v>
+      </c>
+      <c r="J120" t="s">
         <v>18</v>
       </c>
-      <c r="J120" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F120,'feed pars'!B$6:B$42,0))</f>
-        <v>12.8</v>
-      </c>
-      <c r="K120" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K120" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F120,'feed pars'!B$6:B$42,0))</f>
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="L120" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>25</v>
       </c>
+      <c r="E121" t="s">
+        <v>299</v>
+      </c>
       <c r="F121" t="s">
-        <v>41</v>
-      </c>
-      <c r="I121" t="s">
+        <v>50</v>
+      </c>
+      <c r="J121" t="s">
         <v>18</v>
       </c>
-      <c r="J121" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F121,'feed pars'!B$6:B$42,0))</f>
-        <v>11.2</v>
-      </c>
-      <c r="K121" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K121" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F121,'feed pars'!B$6:B$42,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="L121" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>25</v>
       </c>
+      <c r="E122" t="s">
+        <v>299</v>
+      </c>
       <c r="F122" t="s">
-        <v>42</v>
-      </c>
-      <c r="I122" t="s">
+        <v>51</v>
+      </c>
+      <c r="J122" t="s">
         <v>18</v>
       </c>
-      <c r="J122" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F122,'feed pars'!B$6:B$42,0))</f>
-        <v>10.7</v>
-      </c>
-      <c r="K122" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K122" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F122,'feed pars'!B$6:B$42,0))</f>
+        <v>8.9</v>
+      </c>
+      <c r="L122" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>25</v>
       </c>
+      <c r="E123" t="s">
+        <v>299</v>
+      </c>
       <c r="F123" t="s">
-        <v>35</v>
-      </c>
-      <c r="I123" t="s">
+        <v>313</v>
+      </c>
+      <c r="J123" t="s">
         <v>18</v>
       </c>
-      <c r="J123" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F123,'feed pars'!B$6:B$42,0))</f>
-        <v>18</v>
-      </c>
-      <c r="K123" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K123" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F123,'feed pars'!B$6:B$42,0))</f>
+        <v>7.0888888888888877</v>
+      </c>
+      <c r="L123" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>25</v>
       </c>
+      <c r="E124" t="s">
+        <v>299</v>
+      </c>
       <c r="F124" t="s">
-        <v>43</v>
-      </c>
-      <c r="I124" t="s">
+        <v>52</v>
+      </c>
+      <c r="J124" t="s">
         <v>18</v>
       </c>
-      <c r="J124" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F124,'feed pars'!B$6:B$42,0))</f>
-        <v>17.3</v>
-      </c>
-      <c r="K124" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K124" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F124,'feed pars'!B$6:B$42,0))</f>
+        <v>9</v>
+      </c>
+      <c r="L124" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>25</v>
       </c>
+      <c r="E125" t="s">
+        <v>299</v>
+      </c>
       <c r="F125" t="s">
-        <v>314</v>
-      </c>
-      <c r="I125" t="s">
+        <v>53</v>
+      </c>
+      <c r="J125" t="s">
         <v>18</v>
       </c>
-      <c r="J125" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F125,'feed pars'!B$6:B$42,0))</f>
-        <v>29.8</v>
-      </c>
-      <c r="K125" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K125" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F125,'feed pars'!B$6:B$42,0))</f>
+        <v>8</v>
+      </c>
+      <c r="L125" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>25</v>
       </c>
+      <c r="E126" t="s">
+        <v>299</v>
+      </c>
       <c r="F126" t="s">
-        <v>44</v>
-      </c>
-      <c r="I126" t="s">
+        <v>54</v>
+      </c>
+      <c r="J126" t="s">
         <v>18</v>
       </c>
-      <c r="J126" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F126,'feed pars'!B$6:B$42,0))</f>
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="K126" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K126" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F126,'feed pars'!B$6:B$42,0))</f>
+        <v>12.2</v>
+      </c>
+      <c r="L126" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>25</v>
       </c>
+      <c r="E127" t="s">
+        <v>299</v>
+      </c>
       <c r="F127" t="s">
-        <v>45</v>
-      </c>
-      <c r="I127" t="s">
+        <v>55</v>
+      </c>
+      <c r="J127" t="s">
         <v>18</v>
       </c>
-      <c r="J127" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F127,'feed pars'!B$6:B$42,0))</f>
-        <v>9.6999999999999993</v>
-      </c>
-      <c r="K127" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K127" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F127,'feed pars'!B$6:B$42,0))</f>
+        <v>12.2</v>
+      </c>
+      <c r="L127" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>25</v>
       </c>
+      <c r="E128" t="s">
+        <v>299</v>
+      </c>
       <c r="F128" t="s">
-        <v>36</v>
-      </c>
-      <c r="I128" t="s">
+        <v>56</v>
+      </c>
+      <c r="J128" t="s">
         <v>18</v>
       </c>
-      <c r="J128" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F128,'feed pars'!B$6:B$42,0))</f>
-        <v>7.1</v>
-      </c>
-      <c r="K128" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K128" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F128,'feed pars'!B$6:B$42,0))</f>
+        <v>11.3</v>
+      </c>
+      <c r="L128" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>25</v>
       </c>
+      <c r="E129" t="s">
+        <v>299</v>
+      </c>
       <c r="F129" t="s">
-        <v>46</v>
-      </c>
-      <c r="I129" t="s">
+        <v>57</v>
+      </c>
+      <c r="J129" t="s">
         <v>18</v>
       </c>
-      <c r="J129" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F129,'feed pars'!B$6:B$42,0))</f>
-        <v>5.9</v>
-      </c>
-      <c r="K129" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
-        <v>25</v>
-      </c>
-      <c r="F130" t="s">
-        <v>47</v>
-      </c>
-      <c r="I130" t="s">
-        <v>18</v>
-      </c>
-      <c r="J130" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F130,'feed pars'!B$6:B$42,0))</f>
-        <v>5.4</v>
-      </c>
-      <c r="K130" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K129" s="26">
+        <f>INDEX('feed pars'!H$6:H$42,MATCH(F129,'feed pars'!B$6:B$42,0))</f>
+        <v>10.8</v>
+      </c>
+      <c r="L129" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K130" s="26"/>
+    </row>
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>25</v>
       </c>
       <c r="F131" t="s">
-        <v>48</v>
-      </c>
-      <c r="I131" t="s">
+        <v>17</v>
+      </c>
+      <c r="J131" t="s">
         <v>18</v>
       </c>
-      <c r="J131" s="26">
+      <c r="K131" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F131,'feed pars'!B$6:B$42,0))</f>
-        <v>7.2</v>
-      </c>
-      <c r="K131" t="s">
+        <v>12.1</v>
+      </c>
+      <c r="L131" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>25</v>
       </c>
       <c r="F132" t="s">
-        <v>49</v>
-      </c>
-      <c r="I132" t="s">
+        <v>37</v>
+      </c>
+      <c r="J132" t="s">
         <v>18</v>
       </c>
-      <c r="J132" s="26">
+      <c r="K132" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F132,'feed pars'!B$6:B$42,0))</f>
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="K132" t="s">
+        <v>11</v>
+      </c>
+      <c r="L132" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>25</v>
       </c>
       <c r="F133" t="s">
-        <v>50</v>
-      </c>
-      <c r="I133" t="s">
+        <v>38</v>
+      </c>
+      <c r="J133" t="s">
         <v>18</v>
       </c>
-      <c r="J133" s="26">
+      <c r="K133" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F133,'feed pars'!B$6:B$42,0))</f>
-        <v>8.1</v>
-      </c>
-      <c r="K133" t="s">
+        <v>9</v>
+      </c>
+      <c r="L133" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>25</v>
       </c>
       <c r="F134" t="s">
-        <v>51</v>
-      </c>
-      <c r="I134" t="s">
+        <v>39</v>
+      </c>
+      <c r="J134" t="s">
         <v>18</v>
       </c>
-      <c r="J134" s="26">
+      <c r="K134" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F134,'feed pars'!B$6:B$42,0))</f>
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="K134" t="s">
+        <v>11.9</v>
+      </c>
+      <c r="L134" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>25</v>
       </c>
       <c r="F135" t="s">
-        <v>313</v>
-      </c>
-      <c r="I135" t="s">
+        <v>40</v>
+      </c>
+      <c r="J135" t="s">
         <v>18</v>
       </c>
-      <c r="J135" s="26">
+      <c r="K135" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F135,'feed pars'!B$6:B$42,0))</f>
-        <v>6.6</v>
-      </c>
-      <c r="K135" t="s">
+        <v>12.8</v>
+      </c>
+      <c r="L135" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>25</v>
       </c>
       <c r="F136" t="s">
-        <v>52</v>
-      </c>
-      <c r="I136" t="s">
+        <v>41</v>
+      </c>
+      <c r="J136" t="s">
         <v>18</v>
       </c>
-      <c r="J136" s="26">
+      <c r="K136" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F136,'feed pars'!B$6:B$42,0))</f>
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="K136" t="s">
+        <v>11.2</v>
+      </c>
+      <c r="L136" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>25</v>
       </c>
       <c r="F137" t="s">
-        <v>53</v>
-      </c>
-      <c r="I137" t="s">
+        <v>42</v>
+      </c>
+      <c r="J137" t="s">
         <v>18</v>
       </c>
-      <c r="J137" s="26">
+      <c r="K137" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F137,'feed pars'!B$6:B$42,0))</f>
-        <v>6.9</v>
-      </c>
-      <c r="K137" t="s">
+        <v>10.7</v>
+      </c>
+      <c r="L137" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>25</v>
       </c>
       <c r="F138" t="s">
-        <v>54</v>
-      </c>
-      <c r="I138" t="s">
+        <v>35</v>
+      </c>
+      <c r="J138" t="s">
         <v>18</v>
       </c>
-      <c r="J138" s="26">
+      <c r="K138" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F138,'feed pars'!B$6:B$42,0))</f>
-        <v>12.4</v>
-      </c>
-      <c r="K138" t="s">
+        <v>18</v>
+      </c>
+      <c r="L138" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>25</v>
       </c>
       <c r="F139" t="s">
-        <v>55</v>
-      </c>
-      <c r="I139" t="s">
+        <v>43</v>
+      </c>
+      <c r="J139" t="s">
         <v>18</v>
       </c>
-      <c r="J139" s="26">
+      <c r="K139" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F139,'feed pars'!B$6:B$42,0))</f>
-        <v>12.4</v>
-      </c>
-      <c r="K139" t="s">
+        <v>17.3</v>
+      </c>
+      <c r="L139" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>25</v>
       </c>
       <c r="F140" t="s">
-        <v>56</v>
-      </c>
-      <c r="I140" t="s">
+        <v>314</v>
+      </c>
+      <c r="J140" t="s">
         <v>18</v>
       </c>
-      <c r="J140" s="26">
+      <c r="K140" s="26">
         <f>INDEX('feed pars'!G$6:G$42,MATCH(F140,'feed pars'!B$6:B$42,0))</f>
-        <v>11.1</v>
-      </c>
-      <c r="K140" t="s">
+        <v>29.8</v>
+      </c>
+      <c r="L140" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>25</v>
       </c>
       <c r="F141" t="s">
+        <v>44</v>
+      </c>
+      <c r="J141" t="s">
+        <v>18</v>
+      </c>
+      <c r="K141" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F141,'feed pars'!B$6:B$42,0))</f>
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="L141" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>25</v>
+      </c>
+      <c r="F142" t="s">
+        <v>45</v>
+      </c>
+      <c r="J142" t="s">
+        <v>18</v>
+      </c>
+      <c r="K142" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F142,'feed pars'!B$6:B$42,0))</f>
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="L142" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>25</v>
+      </c>
+      <c r="F143" t="s">
+        <v>36</v>
+      </c>
+      <c r="J143" t="s">
+        <v>18</v>
+      </c>
+      <c r="K143" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F143,'feed pars'!B$6:B$42,0))</f>
+        <v>7.1</v>
+      </c>
+      <c r="L143" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>25</v>
+      </c>
+      <c r="F144" t="s">
+        <v>46</v>
+      </c>
+      <c r="J144" t="s">
+        <v>18</v>
+      </c>
+      <c r="K144" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F144,'feed pars'!B$6:B$42,0))</f>
+        <v>5.9</v>
+      </c>
+      <c r="L144" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="145" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>25</v>
+      </c>
+      <c r="F145" t="s">
+        <v>47</v>
+      </c>
+      <c r="J145" t="s">
+        <v>18</v>
+      </c>
+      <c r="K145" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F145,'feed pars'!B$6:B$42,0))</f>
+        <v>5.4</v>
+      </c>
+      <c r="L145" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>25</v>
+      </c>
+      <c r="F146" t="s">
+        <v>48</v>
+      </c>
+      <c r="J146" t="s">
+        <v>18</v>
+      </c>
+      <c r="K146" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F146,'feed pars'!B$6:B$42,0))</f>
+        <v>7.2</v>
+      </c>
+      <c r="L146" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>25</v>
+      </c>
+      <c r="F147" t="s">
+        <v>49</v>
+      </c>
+      <c r="J147" t="s">
+        <v>18</v>
+      </c>
+      <c r="K147" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F147,'feed pars'!B$6:B$42,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="L147" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>25</v>
+      </c>
+      <c r="F148" t="s">
+        <v>50</v>
+      </c>
+      <c r="J148" t="s">
+        <v>18</v>
+      </c>
+      <c r="K148" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F148,'feed pars'!B$6:B$42,0))</f>
+        <v>8.1</v>
+      </c>
+      <c r="L148" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>25</v>
+      </c>
+      <c r="F149" t="s">
+        <v>51</v>
+      </c>
+      <c r="J149" t="s">
+        <v>18</v>
+      </c>
+      <c r="K149" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F149,'feed pars'!B$6:B$42,0))</f>
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="L149" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>25</v>
+      </c>
+      <c r="F150" t="s">
+        <v>313</v>
+      </c>
+      <c r="J150" t="s">
+        <v>18</v>
+      </c>
+      <c r="K150" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F150,'feed pars'!B$6:B$42,0))</f>
+        <v>6.6</v>
+      </c>
+      <c r="L150" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>25</v>
+      </c>
+      <c r="F151" t="s">
+        <v>52</v>
+      </c>
+      <c r="J151" t="s">
+        <v>18</v>
+      </c>
+      <c r="K151" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F151,'feed pars'!B$6:B$42,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="L151" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>25</v>
+      </c>
+      <c r="F152" t="s">
+        <v>53</v>
+      </c>
+      <c r="J152" t="s">
+        <v>18</v>
+      </c>
+      <c r="K152" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F152,'feed pars'!B$6:B$42,0))</f>
+        <v>6.9</v>
+      </c>
+      <c r="L152" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>25</v>
+      </c>
+      <c r="F153" t="s">
+        <v>54</v>
+      </c>
+      <c r="J153" t="s">
+        <v>18</v>
+      </c>
+      <c r="K153" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F153,'feed pars'!B$6:B$42,0))</f>
+        <v>12.4</v>
+      </c>
+      <c r="L153" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>25</v>
+      </c>
+      <c r="F154" t="s">
+        <v>55</v>
+      </c>
+      <c r="J154" t="s">
+        <v>18</v>
+      </c>
+      <c r="K154" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F154,'feed pars'!B$6:B$42,0))</f>
+        <v>12.4</v>
+      </c>
+      <c r="L154" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>25</v>
+      </c>
+      <c r="F155" t="s">
+        <v>56</v>
+      </c>
+      <c r="J155" t="s">
+        <v>18</v>
+      </c>
+      <c r="K155" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F155,'feed pars'!B$6:B$42,0))</f>
+        <v>11.1</v>
+      </c>
+      <c r="L155" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>25</v>
+      </c>
+      <c r="F156" t="s">
         <v>57</v>
       </c>
-      <c r="I141" t="s">
+      <c r="J156" t="s">
         <v>18</v>
       </c>
-      <c r="J141" s="26">
-        <f>INDEX('feed pars'!G$6:G$42,MATCH(F141,'feed pars'!B$6:B$42,0))</f>
+      <c r="K156" s="26">
+        <f>INDEX('feed pars'!G$6:G$42,MATCH(F156,'feed pars'!B$6:B$42,0))</f>
         <v>10.8</v>
       </c>
-      <c r="K141" t="s">
+      <c r="L156" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
HorseHerd pretty much done. But, som bug in cream balance
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FeedMgmt.xlsx
+++ b/data/prod_parameters/FeedMgmt.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="397">
   <si>
     <t>f_feed</t>
   </si>
@@ -1220,6 +1220,12 @@
   </si>
   <si>
     <t>Borde denna vara 100%? Vad är den tröskade majsarealen?</t>
+  </si>
+  <si>
+    <t>horses</t>
+  </si>
+  <si>
+    <t>Horses</t>
   </si>
 </sst>
 </file>
@@ -1696,7 +1702,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O195"/>
+  <dimension ref="A1:O197"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -2871,7 +2877,24 @@
       <c r="M65" s="3"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K66" s="3"/>
+      <c r="A66" t="s">
+        <v>395</v>
+      </c>
+      <c r="G66" t="s">
+        <v>334</v>
+      </c>
+      <c r="H66" t="s">
+        <v>33</v>
+      </c>
+      <c r="J66" t="s">
+        <v>335</v>
+      </c>
+      <c r="K66" s="3">
+        <v>10</v>
+      </c>
+      <c r="L66" t="s">
+        <v>28</v>
+      </c>
       <c r="M66" s="3"/>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
@@ -3987,81 +4010,90 @@
       </c>
     </row>
     <row r="140" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K140" s="3"/>
+      <c r="A140" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="B140" s="7"/>
+      <c r="C140" s="6"/>
+      <c r="D140" s="6"/>
+      <c r="E140" s="6"/>
+      <c r="F140" s="6"/>
+      <c r="G140" s="6"/>
+      <c r="H140" s="6"/>
+      <c r="I140" s="6"/>
+      <c r="J140" s="6"/>
+      <c r="K140" s="6"/>
+      <c r="L140" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M140" s="6"/>
+      <c r="N140" s="6"/>
     </row>
     <row r="141" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A141" s="8" t="s">
+      <c r="A141" t="s">
+        <v>395</v>
+      </c>
+      <c r="F141" t="s">
+        <v>2</v>
+      </c>
+      <c r="J141" t="s">
+        <v>18</v>
+      </c>
+      <c r="K141" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="142" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>395</v>
+      </c>
+      <c r="F142" t="s">
+        <v>33</v>
+      </c>
+      <c r="J142" t="s">
+        <v>18</v>
+      </c>
+      <c r="K142" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A143" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B141" s="8"/>
-      <c r="C141" s="9"/>
-      <c r="D141" s="9"/>
-      <c r="E141" s="9"/>
-      <c r="F141" s="9"/>
-      <c r="G141" s="9"/>
-      <c r="H141" s="9"/>
-      <c r="I141" s="9"/>
-      <c r="J141" s="9"/>
-      <c r="K141" s="9"/>
-      <c r="L141" s="9"/>
-      <c r="M141" s="9"/>
-      <c r="N141" s="9"/>
-    </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A142" s="30" t="s">
+      <c r="B143" s="8"/>
+      <c r="C143" s="9"/>
+      <c r="D143" s="9"/>
+      <c r="E143" s="9"/>
+      <c r="F143" s="9"/>
+      <c r="G143" s="9"/>
+      <c r="H143" s="9"/>
+      <c r="I143" s="9"/>
+      <c r="J143" s="9"/>
+      <c r="K143" s="9"/>
+      <c r="L143" s="9"/>
+      <c r="M143" s="9"/>
+      <c r="N143" s="9"/>
+    </row>
+    <row r="144" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A144" s="30" t="s">
         <v>391</v>
       </c>
-      <c r="B142" s="31"/>
-      <c r="C142" s="32"/>
-      <c r="D142" s="32"/>
-      <c r="E142" s="32"/>
-      <c r="F142" s="32"/>
-      <c r="G142" s="32"/>
-      <c r="H142" s="32"/>
-      <c r="I142" s="32"/>
-      <c r="J142" s="32"/>
-      <c r="K142" s="32"/>
-      <c r="L142" s="32" t="s">
+      <c r="B144" s="31"/>
+      <c r="C144" s="32"/>
+      <c r="D144" s="32"/>
+      <c r="E144" s="32"/>
+      <c r="F144" s="32"/>
+      <c r="G144" s="32"/>
+      <c r="H144" s="32"/>
+      <c r="I144" s="32"/>
+      <c r="J144" s="32"/>
+      <c r="K144" s="32"/>
+      <c r="L144" s="32" t="s">
         <v>300</v>
       </c>
-      <c r="M142" s="32"/>
-      <c r="N142" s="32"/>
-    </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
-        <v>25</v>
-      </c>
-      <c r="E143" t="s">
-        <v>299</v>
-      </c>
-      <c r="F143" t="s">
-        <v>17</v>
-      </c>
-      <c r="J143" t="s">
-        <v>18</v>
-      </c>
-      <c r="K143" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F143,'feed pars'!B$6:B$43,0))</f>
-        <v>12.3</v>
-      </c>
-    </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A144" t="s">
-        <v>25</v>
-      </c>
-      <c r="E144" t="s">
-        <v>299</v>
-      </c>
-      <c r="F144" t="s">
-        <v>37</v>
-      </c>
-      <c r="J144" t="s">
-        <v>18</v>
-      </c>
-      <c r="K144" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F144,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
-      </c>
+      <c r="M144" s="32"/>
+      <c r="N144" s="32"/>
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
@@ -4071,14 +4103,14 @@
         <v>299</v>
       </c>
       <c r="F145" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="J145" t="s">
         <v>18</v>
       </c>
       <c r="K145" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F145,'feed pars'!B$6:B$43,0))</f>
-        <v>9.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.25">
@@ -4089,14 +4121,14 @@
         <v>299</v>
       </c>
       <c r="F146" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J146" t="s">
         <v>18</v>
       </c>
       <c r="K146" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F146,'feed pars'!B$6:B$43,0))</f>
-        <v>12</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="147" spans="1:11" x14ac:dyDescent="0.25">
@@ -4107,14 +4139,14 @@
         <v>299</v>
       </c>
       <c r="F147" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J147" t="s">
         <v>18</v>
       </c>
       <c r="K147" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F147,'feed pars'!B$6:B$43,0))</f>
-        <v>13.2</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="148" spans="1:11" x14ac:dyDescent="0.25">
@@ -4125,14 +4157,14 @@
         <v>299</v>
       </c>
       <c r="F148" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="J148" t="s">
         <v>18</v>
       </c>
       <c r="K148" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F148,'feed pars'!B$6:B$43,0))</f>
-        <v>11.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.25">
@@ -4143,14 +4175,14 @@
         <v>299</v>
       </c>
       <c r="F149" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J149" t="s">
         <v>18</v>
       </c>
       <c r="K149" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F149,'feed pars'!B$6:B$43,0))</f>
-        <v>10.9</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.25">
@@ -4161,14 +4193,14 @@
         <v>299</v>
       </c>
       <c r="F150" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="J150" t="s">
         <v>18</v>
       </c>
       <c r="K150" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F150,'feed pars'!B$6:B$43,0))</f>
-        <v>18.5</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.25">
@@ -4179,14 +4211,14 @@
         <v>299</v>
       </c>
       <c r="F151" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J151" t="s">
         <v>18</v>
       </c>
       <c r="K151" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F151,'feed pars'!B$6:B$43,0))</f>
-        <v>17.5</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.25">
@@ -4197,14 +4229,14 @@
         <v>299</v>
       </c>
       <c r="F152" t="s">
-        <v>314</v>
+        <v>35</v>
       </c>
       <c r="J152" t="s">
         <v>18</v>
       </c>
       <c r="K152" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F152,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.25">
@@ -4215,14 +4247,14 @@
         <v>299</v>
       </c>
       <c r="F153" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J153" t="s">
         <v>18</v>
       </c>
       <c r="K153" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F153,'feed pars'!B$6:B$43,0))</f>
-        <v>9.9</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.25">
@@ -4233,14 +4265,14 @@
         <v>299</v>
       </c>
       <c r="F154" t="s">
-        <v>45</v>
+        <v>314</v>
       </c>
       <c r="J154" t="s">
         <v>18</v>
       </c>
       <c r="K154" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F154,'feed pars'!B$6:B$43,0))</f>
-        <v>10.3</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.25">
@@ -4251,14 +4283,14 @@
         <v>299</v>
       </c>
       <c r="F155" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="J155" t="s">
         <v>18</v>
       </c>
       <c r="K155" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F155,'feed pars'!B$6:B$43,0))</f>
-        <v>7.7</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.25">
@@ -4269,14 +4301,14 @@
         <v>299</v>
       </c>
       <c r="F156" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J156" t="s">
         <v>18</v>
       </c>
       <c r="K156" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F156,'feed pars'!B$6:B$43,0))</f>
-        <v>6.5</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.25">
@@ -4287,14 +4319,14 @@
         <v>299</v>
       </c>
       <c r="F157" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="J157" t="s">
         <v>18</v>
       </c>
       <c r="K157" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F157,'feed pars'!B$6:B$43,0))</f>
-        <v>6.2</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.25">
@@ -4305,14 +4337,14 @@
         <v>299</v>
       </c>
       <c r="F158" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J158" t="s">
         <v>18</v>
       </c>
       <c r="K158" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F158,'feed pars'!B$6:B$43,0))</f>
-        <v>7.8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.25">
@@ -4323,14 +4355,14 @@
         <v>299</v>
       </c>
       <c r="F159" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J159" t="s">
         <v>18</v>
       </c>
       <c r="K159" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F159,'feed pars'!B$6:B$43,0))</f>
-        <v>9.1999999999999993</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.25">
@@ -4341,14 +4373,14 @@
         <v>299</v>
       </c>
       <c r="F160" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J160" t="s">
         <v>18</v>
       </c>
       <c r="K160" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F160,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="161" spans="1:14" x14ac:dyDescent="0.25">
@@ -4359,14 +4391,14 @@
         <v>299</v>
       </c>
       <c r="F161" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J161" t="s">
         <v>18</v>
       </c>
       <c r="K161" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F161,'feed pars'!B$6:B$43,0))</f>
-        <v>8.9</v>
+        <v>9.1999999999999993</v>
       </c>
     </row>
     <row r="162" spans="1:14" x14ac:dyDescent="0.25">
@@ -4377,14 +4409,14 @@
         <v>299</v>
       </c>
       <c r="F162" t="s">
-        <v>313</v>
+        <v>50</v>
       </c>
       <c r="J162" t="s">
         <v>18</v>
       </c>
       <c r="K162" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F162,'feed pars'!B$6:B$43,0))</f>
-        <v>7.0888888888888877</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="163" spans="1:14" x14ac:dyDescent="0.25">
@@ -4395,14 +4427,14 @@
         <v>299</v>
       </c>
       <c r="F163" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J163" t="s">
         <v>18</v>
       </c>
       <c r="K163" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F163,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="164" spans="1:14" x14ac:dyDescent="0.25">
@@ -4413,14 +4445,14 @@
         <v>299</v>
       </c>
       <c r="F164" t="s">
-        <v>53</v>
+        <v>313</v>
       </c>
       <c r="J164" t="s">
         <v>18</v>
       </c>
       <c r="K164" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F164,'feed pars'!B$6:B$43,0))</f>
-        <v>8</v>
+        <v>7.0888888888888877</v>
       </c>
     </row>
     <row r="165" spans="1:14" x14ac:dyDescent="0.25">
@@ -4431,14 +4463,14 @@
         <v>299</v>
       </c>
       <c r="F165" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J165" t="s">
         <v>18</v>
       </c>
       <c r="K165" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F165,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="166" spans="1:14" x14ac:dyDescent="0.25">
@@ -4449,14 +4481,14 @@
         <v>299</v>
       </c>
       <c r="F166" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J166" t="s">
         <v>18</v>
       </c>
       <c r="K166" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F166,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="167" spans="1:14" x14ac:dyDescent="0.25">
@@ -4467,14 +4499,14 @@
         <v>299</v>
       </c>
       <c r="F167" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J167" t="s">
         <v>18</v>
       </c>
       <c r="K167" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F167,'feed pars'!B$6:B$43,0))</f>
-        <v>11.3</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="168" spans="1:14" x14ac:dyDescent="0.25">
@@ -4485,79 +4517,85 @@
         <v>299</v>
       </c>
       <c r="F168" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J168" t="s">
         <v>18</v>
       </c>
       <c r="K168" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F168,'feed pars'!B$6:B$43,0))</f>
-        <v>10.8</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="169" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A169" s="30" t="s">
-        <v>392</v>
-      </c>
-      <c r="B169" s="31"/>
-      <c r="C169" s="32"/>
-      <c r="D169" s="32"/>
-      <c r="E169" s="32"/>
-      <c r="F169" s="32"/>
-      <c r="G169" s="32"/>
-      <c r="H169" s="32"/>
-      <c r="I169" s="32"/>
-      <c r="J169" s="32"/>
-      <c r="K169" s="32"/>
-      <c r="L169" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="M169" s="32"/>
-      <c r="N169" s="32"/>
+      <c r="A169" t="s">
+        <v>25</v>
+      </c>
+      <c r="E169" t="s">
+        <v>299</v>
+      </c>
+      <c r="F169" t="s">
+        <v>56</v>
+      </c>
+      <c r="J169" t="s">
+        <v>18</v>
+      </c>
+      <c r="K169" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F169,'feed pars'!B$6:B$43,0))</f>
+        <v>11.3</v>
+      </c>
     </row>
     <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>25</v>
       </c>
+      <c r="E170" t="s">
+        <v>299</v>
+      </c>
       <c r="F170" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="J170" t="s">
         <v>18</v>
       </c>
       <c r="K170" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F170,'feed pars'!B$6:B$43,0))</f>
-        <v>12.1</v>
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F170,'feed pars'!B$6:B$43,0))</f>
+        <v>10.8</v>
       </c>
     </row>
     <row r="171" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A171" t="s">
-        <v>25</v>
-      </c>
-      <c r="F171" t="s">
-        <v>37</v>
-      </c>
-      <c r="J171" t="s">
-        <v>18</v>
-      </c>
-      <c r="K171" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F171,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
-      </c>
+      <c r="A171" s="30" t="s">
+        <v>392</v>
+      </c>
+      <c r="B171" s="31"/>
+      <c r="C171" s="32"/>
+      <c r="D171" s="32"/>
+      <c r="E171" s="32"/>
+      <c r="F171" s="32"/>
+      <c r="G171" s="32"/>
+      <c r="H171" s="32"/>
+      <c r="I171" s="32"/>
+      <c r="J171" s="32"/>
+      <c r="K171" s="32"/>
+      <c r="L171" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="M171" s="32"/>
+      <c r="N171" s="32"/>
     </row>
     <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>25</v>
       </c>
       <c r="F172" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="J172" t="s">
         <v>18</v>
       </c>
       <c r="K172" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F172,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="173" spans="1:14" x14ac:dyDescent="0.25">
@@ -4565,14 +4603,14 @@
         <v>25</v>
       </c>
       <c r="F173" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J173" t="s">
         <v>18</v>
       </c>
       <c r="K173" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F173,'feed pars'!B$6:B$43,0))</f>
-        <v>11.9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="174" spans="1:14" x14ac:dyDescent="0.25">
@@ -4580,14 +4618,14 @@
         <v>25</v>
       </c>
       <c r="F174" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J174" t="s">
         <v>18</v>
       </c>
       <c r="K174" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F174,'feed pars'!B$6:B$43,0))</f>
-        <v>12.8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="175" spans="1:14" x14ac:dyDescent="0.25">
@@ -4595,14 +4633,14 @@
         <v>25</v>
       </c>
       <c r="F175" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="J175" t="s">
         <v>18</v>
       </c>
       <c r="K175" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F175,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="176" spans="1:14" x14ac:dyDescent="0.25">
@@ -4610,14 +4648,14 @@
         <v>25</v>
       </c>
       <c r="F176" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J176" t="s">
         <v>18</v>
       </c>
       <c r="K176" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F176,'feed pars'!B$6:B$43,0))</f>
-        <v>10.7</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.25">
@@ -4625,14 +4663,14 @@
         <v>25</v>
       </c>
       <c r="F177" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="J177" t="s">
         <v>18</v>
       </c>
       <c r="K177" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F177,'feed pars'!B$6:B$43,0))</f>
-        <v>18</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.25">
@@ -4640,14 +4678,14 @@
         <v>25</v>
       </c>
       <c r="F178" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J178" t="s">
         <v>18</v>
       </c>
       <c r="K178" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F178,'feed pars'!B$6:B$43,0))</f>
-        <v>17.3</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.25">
@@ -4655,14 +4693,14 @@
         <v>25</v>
       </c>
       <c r="F179" t="s">
-        <v>314</v>
+        <v>35</v>
       </c>
       <c r="J179" t="s">
         <v>18</v>
       </c>
       <c r="K179" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F179,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="180" spans="1:11" x14ac:dyDescent="0.25">
@@ -4670,14 +4708,14 @@
         <v>25</v>
       </c>
       <c r="F180" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J180" t="s">
         <v>18</v>
       </c>
       <c r="K180" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F180,'feed pars'!B$6:B$43,0))</f>
-        <v>9.3000000000000007</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="181" spans="1:11" x14ac:dyDescent="0.25">
@@ -4685,14 +4723,14 @@
         <v>25</v>
       </c>
       <c r="F181" t="s">
-        <v>45</v>
+        <v>314</v>
       </c>
       <c r="J181" t="s">
         <v>18</v>
       </c>
       <c r="K181" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F181,'feed pars'!B$6:B$43,0))</f>
-        <v>9.6999999999999993</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="182" spans="1:11" x14ac:dyDescent="0.25">
@@ -4700,14 +4738,14 @@
         <v>25</v>
       </c>
       <c r="F182" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="J182" t="s">
         <v>18</v>
       </c>
       <c r="K182" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F182,'feed pars'!B$6:B$43,0))</f>
-        <v>7.1</v>
+        <v>9.3000000000000007</v>
       </c>
     </row>
     <row r="183" spans="1:11" x14ac:dyDescent="0.25">
@@ -4715,14 +4753,14 @@
         <v>25</v>
       </c>
       <c r="F183" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J183" t="s">
         <v>18</v>
       </c>
       <c r="K183" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F183,'feed pars'!B$6:B$43,0))</f>
-        <v>5.9</v>
+        <v>9.6999999999999993</v>
       </c>
     </row>
     <row r="184" spans="1:11" x14ac:dyDescent="0.25">
@@ -4730,14 +4768,14 @@
         <v>25</v>
       </c>
       <c r="F184" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="J184" t="s">
         <v>18</v>
       </c>
       <c r="K184" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F184,'feed pars'!B$6:B$43,0))</f>
-        <v>5.4</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="185" spans="1:11" x14ac:dyDescent="0.25">
@@ -4745,14 +4783,14 @@
         <v>25</v>
       </c>
       <c r="F185" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J185" t="s">
         <v>18</v>
       </c>
       <c r="K185" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F185,'feed pars'!B$6:B$43,0))</f>
-        <v>7.2</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="186" spans="1:11" x14ac:dyDescent="0.25">
@@ -4760,14 +4798,14 @@
         <v>25</v>
       </c>
       <c r="F186" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J186" t="s">
         <v>18</v>
       </c>
       <c r="K186" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F186,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="187" spans="1:11" x14ac:dyDescent="0.25">
@@ -4775,14 +4813,14 @@
         <v>25</v>
       </c>
       <c r="F187" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J187" t="s">
         <v>18</v>
       </c>
       <c r="K187" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F187,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.25">
@@ -4790,14 +4828,14 @@
         <v>25</v>
       </c>
       <c r="F188" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J188" t="s">
         <v>18</v>
       </c>
       <c r="K188" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F188,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1999999999999993</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="189" spans="1:11" x14ac:dyDescent="0.25">
@@ -4805,14 +4843,14 @@
         <v>25</v>
       </c>
       <c r="F189" t="s">
-        <v>313</v>
+        <v>50</v>
       </c>
       <c r="J189" t="s">
         <v>18</v>
       </c>
       <c r="K189" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F189,'feed pars'!B$6:B$43,0))</f>
-        <v>6.6</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="190" spans="1:11" x14ac:dyDescent="0.25">
@@ -4820,14 +4858,14 @@
         <v>25</v>
       </c>
       <c r="F190" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J190" t="s">
         <v>18</v>
       </c>
       <c r="K190" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F190,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
+        <v>8.1999999999999993</v>
       </c>
     </row>
     <row r="191" spans="1:11" x14ac:dyDescent="0.25">
@@ -4835,14 +4873,14 @@
         <v>25</v>
       </c>
       <c r="F191" t="s">
-        <v>53</v>
+        <v>313</v>
       </c>
       <c r="J191" t="s">
         <v>18</v>
       </c>
       <c r="K191" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F191,'feed pars'!B$6:B$43,0))</f>
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="192" spans="1:11" x14ac:dyDescent="0.25">
@@ -4850,14 +4888,14 @@
         <v>25</v>
       </c>
       <c r="F192" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J192" t="s">
         <v>18</v>
       </c>
       <c r="K192" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F192,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="193" spans="1:11" x14ac:dyDescent="0.25">
@@ -4865,14 +4903,14 @@
         <v>25</v>
       </c>
       <c r="F193" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J193" t="s">
         <v>18</v>
       </c>
       <c r="K193" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F193,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="194" spans="1:11" x14ac:dyDescent="0.25">
@@ -4880,14 +4918,14 @@
         <v>25</v>
       </c>
       <c r="F194" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J194" t="s">
         <v>18</v>
       </c>
       <c r="K194" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F194,'feed pars'!B$6:B$43,0))</f>
-        <v>11.1</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="195" spans="1:11" x14ac:dyDescent="0.25">
@@ -4895,13 +4933,43 @@
         <v>25</v>
       </c>
       <c r="F195" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J195" t="s">
         <v>18</v>
       </c>
       <c r="K195" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F195,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>25</v>
+      </c>
+      <c r="F196" t="s">
+        <v>56</v>
+      </c>
+      <c r="J196" t="s">
+        <v>18</v>
+      </c>
+      <c r="K196" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F196,'feed pars'!B$6:B$43,0))</f>
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>25</v>
+      </c>
+      <c r="F197" t="s">
+        <v>57</v>
+      </c>
+      <c r="J197" t="s">
+        <v>18</v>
+      </c>
+      <c r="K197" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F197,'feed pars'!B$6:B$43,0))</f>
         <v>10.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implemented feed storage and feeding losses and parametrised for roughages
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FeedMgmt.xlsx
+++ b/data/prod_parameters/FeedMgmt.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="410">
   <si>
     <t>f_feed</t>
   </si>
@@ -1227,6 +1227,45 @@
   <si>
     <t>Horses</t>
   </si>
+  <si>
+    <t>storage_losses</t>
+  </si>
+  <si>
+    <t>feeding_losses</t>
+  </si>
+  <si>
+    <t>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</t>
+  </si>
+  <si>
+    <t>Storage and feeding losses</t>
+  </si>
+  <si>
+    <t>100% - pasture utilisation</t>
+  </si>
+  <si>
+    <t>sheep</t>
+  </si>
+  <si>
+    <t>80% in silo</t>
+  </si>
+  <si>
+    <t>60% in silo</t>
+  </si>
+  <si>
+    <t>0% in silo</t>
+  </si>
+  <si>
+    <t>No feeding on pasture</t>
+  </si>
+  <si>
+    <t>10% feeding on pasture</t>
+  </si>
+  <si>
+    <t>Need to add losses for grains and concentrates</t>
+  </si>
+  <si>
+    <t>No storage</t>
+  </si>
 </sst>
 </file>
 
@@ -1235,7 +1274,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1297,6 +1336,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.499984740745262"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1371,7 +1417,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1421,6 +1467,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1702,7 +1749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O197"/>
+  <dimension ref="A1:O242"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -2902,2074 +2949,3208 @@
       <c r="M67" s="3"/>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K68" s="3"/>
-      <c r="M68" s="3"/>
+      <c r="A68" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="B68" s="1"/>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="2"/>
+      <c r="F68" s="2"/>
+      <c r="G68" s="2"/>
+      <c r="H68" s="2"/>
+      <c r="I68" s="2"/>
+      <c r="J68" s="2"/>
+      <c r="K68" s="2"/>
+      <c r="L68" s="2"/>
+      <c r="M68" s="2"/>
+      <c r="N68" s="2"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B69" s="1"/>
-      <c r="C69" s="1"/>
-      <c r="D69" s="1"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="2"/>
-      <c r="G69" s="2"/>
-      <c r="H69" s="2"/>
-      <c r="I69" s="2"/>
-      <c r="J69" s="2"/>
-      <c r="K69" s="2"/>
-      <c r="L69" s="2"/>
-      <c r="M69" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="N69" s="2"/>
+      <c r="J69" s="10" t="s">
+        <v>397</v>
+      </c>
+      <c r="K69" s="10">
+        <v>0</v>
+      </c>
+      <c r="L69" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="M69" s="10" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F70" t="s">
+      <c r="J70" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="K70" s="10">
+        <v>0</v>
+      </c>
+      <c r="L70" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="M70" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>24</v>
+      </c>
+      <c r="B71" t="s">
+        <v>326</v>
+      </c>
+      <c r="E71" t="s">
+        <v>327</v>
+      </c>
+      <c r="F71" t="s">
         <v>310</v>
       </c>
-      <c r="J70" t="s">
-        <v>390</v>
-      </c>
-      <c r="K70" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F70,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L70" t="s">
+      <c r="J71" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K71" s="29">
+        <f>(0.8*20+0.2*2)</f>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="L71" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="M70" s="29" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F71" t="s">
+      <c r="M71" s="29" t="s">
+        <v>403</v>
+      </c>
+      <c r="N71" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>24</v>
+      </c>
+      <c r="F72" t="s">
+        <v>310</v>
+      </c>
+      <c r="J72" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K72" s="29">
+        <f>(0.6*20+0.4*2)</f>
+        <v>12.8</v>
+      </c>
+      <c r="L72" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M72" s="29" t="s">
+        <v>404</v>
+      </c>
+      <c r="N72" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>402</v>
+      </c>
+      <c r="F73" t="s">
+        <v>310</v>
+      </c>
+      <c r="J73" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K73" s="29">
+        <v>2</v>
+      </c>
+      <c r="L73" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M73" s="29" t="s">
+        <v>405</v>
+      </c>
+      <c r="N73" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>395</v>
+      </c>
+      <c r="F74" t="s">
+        <v>310</v>
+      </c>
+      <c r="J74" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K74" s="29">
+        <v>2</v>
+      </c>
+      <c r="L74" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M74" s="29" t="s">
+        <v>405</v>
+      </c>
+      <c r="N74" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>24</v>
+      </c>
+      <c r="B75" t="s">
+        <v>326</v>
+      </c>
+      <c r="E75" t="s">
+        <v>327</v>
+      </c>
+      <c r="F75" t="s">
+        <v>310</v>
+      </c>
+      <c r="J75" s="29" t="s">
+        <v>398</v>
+      </c>
+      <c r="K75" s="29">
+        <v>5</v>
+      </c>
+      <c r="L75" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M75" s="29" t="s">
+        <v>406</v>
+      </c>
+      <c r="N75" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>24</v>
+      </c>
+      <c r="E76" t="s">
+        <v>329</v>
+      </c>
+      <c r="F76" t="s">
+        <v>310</v>
+      </c>
+      <c r="J76" s="29" t="s">
+        <v>398</v>
+      </c>
+      <c r="K76" s="29">
+        <v>5</v>
+      </c>
+      <c r="L76" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M76" s="29" t="s">
+        <v>406</v>
+      </c>
+      <c r="N76" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>24</v>
+      </c>
+      <c r="F77" t="s">
+        <v>310</v>
+      </c>
+      <c r="J77" s="29" t="s">
+        <v>398</v>
+      </c>
+      <c r="K77" s="29">
+        <f>0.9*5+0.1*15</f>
+        <v>6</v>
+      </c>
+      <c r="L77" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M77" s="29" t="s">
+        <v>407</v>
+      </c>
+      <c r="N77" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>402</v>
+      </c>
+      <c r="F78" t="s">
+        <v>310</v>
+      </c>
+      <c r="J78" s="29" t="s">
+        <v>398</v>
+      </c>
+      <c r="K78" s="29">
+        <v>15</v>
+      </c>
+      <c r="L78" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M78" s="29"/>
+      <c r="N78" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>395</v>
+      </c>
+      <c r="F79" t="s">
+        <v>310</v>
+      </c>
+      <c r="J79" s="29" t="s">
+        <v>398</v>
+      </c>
+      <c r="K79" s="29">
+        <v>15</v>
+      </c>
+      <c r="L79" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M79" s="29"/>
+      <c r="N79" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A80" s="33" t="str">
+        <f>A71</f>
+        <v>cattle</v>
+      </c>
+      <c r="B80" s="33" t="str">
+        <f>B71</f>
+        <v>dairy</v>
+      </c>
+      <c r="E80" s="33" t="str">
+        <f>E71</f>
+        <v>cows</v>
+      </c>
+      <c r="F80" t="s">
         <v>311</v>
       </c>
-      <c r="J71" t="s">
-        <v>390</v>
-      </c>
-      <c r="K71" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F71,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L71" t="s">
+      <c r="J80" s="33" t="str">
+        <f>J71</f>
+        <v>storage_losses</v>
+      </c>
+      <c r="K80" s="33">
+        <f>K71</f>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="L80" s="33" t="str">
+        <f>L71</f>
+        <v>%</v>
+      </c>
+      <c r="M80" s="33" t="str">
+        <f>M71</f>
+        <v>80% in silo</v>
+      </c>
+      <c r="N80" s="33" t="str">
+        <f>N71</f>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A81" s="33" t="str">
+        <f t="shared" ref="A81:A88" si="0">A72</f>
+        <v>cattle</v>
+      </c>
+      <c r="F81" t="s">
+        <v>311</v>
+      </c>
+      <c r="J81" s="33" t="str">
+        <f t="shared" ref="J81:N88" si="1">J72</f>
+        <v>storage_losses</v>
+      </c>
+      <c r="K81" s="33">
+        <f t="shared" si="1"/>
+        <v>12.8</v>
+      </c>
+      <c r="L81" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M81" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>60% in silo</v>
+      </c>
+      <c r="N81" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A82" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>sheep</v>
+      </c>
+      <c r="F82" t="s">
+        <v>311</v>
+      </c>
+      <c r="J82" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>storage_losses</v>
+      </c>
+      <c r="K82" s="33">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="L82" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M82" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>0% in silo</v>
+      </c>
+      <c r="N82" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A83" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>horses</v>
+      </c>
+      <c r="F83" t="s">
+        <v>311</v>
+      </c>
+      <c r="J83" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>storage_losses</v>
+      </c>
+      <c r="K83" s="33">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="L83" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M83" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>0% in silo</v>
+      </c>
+      <c r="N83" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A84" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>cattle</v>
+      </c>
+      <c r="B84" s="33" t="str">
+        <f>B75</f>
+        <v>dairy</v>
+      </c>
+      <c r="E84" s="33" t="str">
+        <f>E75</f>
+        <v>cows</v>
+      </c>
+      <c r="F84" t="s">
+        <v>311</v>
+      </c>
+      <c r="J84" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K84" s="33">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L84" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M84" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="N84" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A85" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>cattle</v>
+      </c>
+      <c r="E85" s="33" t="str">
+        <f>E76</f>
+        <v>bulls</v>
+      </c>
+      <c r="F85" t="s">
+        <v>311</v>
+      </c>
+      <c r="J85" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K85" s="33">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L85" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M85" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="N85" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A86" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>cattle</v>
+      </c>
+      <c r="F86" t="s">
+        <v>311</v>
+      </c>
+      <c r="J86" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K86" s="33">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="L86" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M86" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="N86" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A87" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>sheep</v>
+      </c>
+      <c r="F87" t="s">
+        <v>311</v>
+      </c>
+      <c r="J87" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K87" s="33">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L87" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M87" s="33"/>
+      <c r="N87" s="33" t="str">
+        <f t="shared" ref="N87:N88" si="2">N78</f>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A88" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>horses</v>
+      </c>
+      <c r="F88" t="s">
+        <v>311</v>
+      </c>
+      <c r="J88" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K88" s="33">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L88" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M88" s="33"/>
+      <c r="N88" s="33" t="str">
+        <f t="shared" si="2"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A89" s="33"/>
+      <c r="B89" s="33"/>
+      <c r="E89" s="33"/>
+      <c r="F89" t="s">
+        <v>312</v>
+      </c>
+      <c r="J89" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K89" s="29">
+        <v>5</v>
+      </c>
+      <c r="L89" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="M71" s="3"/>
-    </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F72" t="s">
+      <c r="M89" s="29"/>
+      <c r="N89" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A90" s="33" t="str">
+        <f>A75</f>
+        <v>cattle</v>
+      </c>
+      <c r="B90" s="33" t="str">
+        <f>B75</f>
+        <v>dairy</v>
+      </c>
+      <c r="E90" s="33" t="str">
+        <f t="shared" ref="E90:E91" si="3">E75</f>
+        <v>cows</v>
+      </c>
+      <c r="F90" t="s">
         <v>312</v>
       </c>
-      <c r="J72" t="s">
-        <v>390</v>
-      </c>
-      <c r="K72" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F72,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L72" t="s">
+      <c r="J90" s="33" t="str">
+        <f t="shared" ref="J90:N94" si="4">J75</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K90" s="33">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="L90" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="M90" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="N90" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A91" s="33" t="str">
+        <f t="shared" ref="A91:A94" si="5">A76</f>
+        <v>cattle</v>
+      </c>
+      <c r="E91" s="33" t="str">
+        <f t="shared" si="3"/>
+        <v>bulls</v>
+      </c>
+      <c r="F91" t="s">
+        <v>312</v>
+      </c>
+      <c r="J91" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K91" s="33">
+        <f t="shared" si="4"/>
+        <v>5</v>
+      </c>
+      <c r="L91" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="M91" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="N91" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A92" s="33" t="str">
+        <f t="shared" si="5"/>
+        <v>cattle</v>
+      </c>
+      <c r="F92" t="s">
+        <v>312</v>
+      </c>
+      <c r="J92" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K92" s="33">
+        <f t="shared" si="4"/>
+        <v>6</v>
+      </c>
+      <c r="L92" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="M92" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="N92" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A93" s="33" t="str">
+        <f t="shared" si="5"/>
+        <v>sheep</v>
+      </c>
+      <c r="F93" t="s">
+        <v>312</v>
+      </c>
+      <c r="J93" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K93" s="33">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="L93" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="M93" s="33"/>
+      <c r="N93" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A94" s="33" t="str">
+        <f t="shared" si="5"/>
+        <v>horses</v>
+      </c>
+      <c r="F94" t="s">
+        <v>312</v>
+      </c>
+      <c r="J94" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K94" s="33">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="L94" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="M94" s="33"/>
+      <c r="N94" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F95" t="s">
+        <v>2</v>
+      </c>
+      <c r="J95" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K95" s="29">
+        <v>5</v>
+      </c>
+      <c r="L95" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="M72" s="3"/>
-    </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F73" t="s">
+      <c r="M95" s="29"/>
+      <c r="N95" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A96" s="33" t="str">
+        <f>A75</f>
+        <v>cattle</v>
+      </c>
+      <c r="B96" s="33" t="str">
+        <f>B75</f>
+        <v>dairy</v>
+      </c>
+      <c r="E96" s="33" t="str">
+        <f t="shared" ref="E96:E97" si="6">E75</f>
+        <v>cows</v>
+      </c>
+      <c r="F96" t="s">
         <v>2</v>
       </c>
-      <c r="J73" t="s">
-        <v>390</v>
-      </c>
-      <c r="K73" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F73,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L73" t="s">
-        <v>28</v>
-      </c>
-      <c r="M73" s="3"/>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F74" t="s">
-        <v>12</v>
-      </c>
-      <c r="J74" t="s">
-        <v>390</v>
-      </c>
-      <c r="K74" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F74,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L74" t="s">
-        <v>28</v>
-      </c>
-      <c r="M74" s="3"/>
-    </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F75" t="s">
-        <v>33</v>
-      </c>
-      <c r="J75" t="s">
-        <v>390</v>
-      </c>
-      <c r="K75" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F75,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L75" t="s">
-        <v>28</v>
-      </c>
-      <c r="M75" s="3"/>
-    </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F76" t="s">
-        <v>17</v>
-      </c>
-      <c r="J76" t="s">
-        <v>390</v>
-      </c>
-      <c r="K76" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F76,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="L76" t="s">
-        <v>28</v>
-      </c>
-      <c r="M76" s="3"/>
-    </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F77" t="s">
-        <v>37</v>
-      </c>
-      <c r="J77" t="s">
-        <v>390</v>
-      </c>
-      <c r="K77" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F77,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="L77" t="s">
-        <v>28</v>
-      </c>
-      <c r="M77" s="3"/>
-    </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F78" t="s">
-        <v>38</v>
-      </c>
-      <c r="J78" t="s">
-        <v>390</v>
-      </c>
-      <c r="K78" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F78,'feed pars'!B$6:B$43,0))</f>
-        <v>86</v>
-      </c>
-      <c r="L78" t="s">
-        <v>28</v>
-      </c>
-      <c r="M78" s="3"/>
-    </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F79" t="s">
-        <v>39</v>
-      </c>
-      <c r="J79" t="s">
-        <v>390</v>
-      </c>
-      <c r="K79" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F79,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="L79" t="s">
-        <v>28</v>
-      </c>
-      <c r="M79" s="3"/>
-    </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F80" t="s">
-        <v>317</v>
-      </c>
-      <c r="J80" t="s">
-        <v>390</v>
-      </c>
-      <c r="K80" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F80,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="L80" t="s">
-        <v>28</v>
-      </c>
-      <c r="M80" s="3"/>
-    </row>
-    <row r="81" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F81" t="s">
-        <v>40</v>
-      </c>
-      <c r="J81" t="s">
-        <v>390</v>
-      </c>
-      <c r="K81" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F81,'feed pars'!B$6:B$43,0))</f>
-        <v>67.5</v>
-      </c>
-      <c r="L81" t="s">
-        <v>28</v>
-      </c>
-      <c r="M81" s="3"/>
-    </row>
-    <row r="82" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F82" t="s">
-        <v>41</v>
-      </c>
-      <c r="J82" t="s">
-        <v>390</v>
-      </c>
-      <c r="K82" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F82,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="L82" t="s">
-        <v>28</v>
-      </c>
-      <c r="M82" s="3"/>
-    </row>
-    <row r="83" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F83" t="s">
-        <v>42</v>
-      </c>
-      <c r="J83" t="s">
-        <v>390</v>
-      </c>
-      <c r="K83" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F83,'feed pars'!B$6:B$43,0))</f>
-        <v>86.8</v>
-      </c>
-      <c r="L83" t="s">
-        <v>28</v>
-      </c>
-      <c r="M83" s="3"/>
-    </row>
-    <row r="84" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F84" t="s">
-        <v>35</v>
-      </c>
-      <c r="J84" t="s">
-        <v>390</v>
-      </c>
-      <c r="K84" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F84,'feed pars'!B$6:B$43,0))</f>
-        <v>92.5</v>
-      </c>
-      <c r="L84" t="s">
-        <v>28</v>
-      </c>
-      <c r="M84" s="3"/>
-    </row>
-    <row r="85" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F85" t="s">
-        <v>43</v>
-      </c>
-      <c r="J85" t="s">
-        <v>390</v>
-      </c>
-      <c r="K85" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F85,'feed pars'!B$6:B$43,0))</f>
-        <v>92</v>
-      </c>
-      <c r="L85" t="s">
-        <v>28</v>
-      </c>
-      <c r="M85" s="3"/>
-    </row>
-    <row r="86" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F86" t="s">
-        <v>314</v>
-      </c>
-      <c r="J86" t="s">
-        <v>390</v>
-      </c>
-      <c r="K86" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F86,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L86" t="s">
-        <v>28</v>
-      </c>
-      <c r="M86" s="3"/>
-    </row>
-    <row r="87" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F87" t="s">
-        <v>305</v>
-      </c>
-      <c r="J87" t="s">
-        <v>390</v>
-      </c>
-      <c r="K87" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F87,'feed pars'!B$6:B$43,0))</f>
-        <v>85</v>
-      </c>
-      <c r="L87" t="s">
-        <v>28</v>
-      </c>
-      <c r="M87" s="3"/>
-    </row>
-    <row r="88" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F88" t="s">
-        <v>318</v>
-      </c>
-      <c r="J88" t="s">
-        <v>390</v>
-      </c>
-      <c r="K88" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F88,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="L88" t="s">
-        <v>28</v>
-      </c>
-      <c r="M88" s="3"/>
-    </row>
-    <row r="89" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F89" t="s">
-        <v>44</v>
-      </c>
-      <c r="J89" t="s">
-        <v>390</v>
-      </c>
-      <c r="K89" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F89,'feed pars'!B$6:B$43,0))</f>
-        <v>87.5</v>
-      </c>
-      <c r="L89" t="s">
-        <v>28</v>
-      </c>
-      <c r="M89" s="3"/>
-    </row>
-    <row r="90" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F90" t="s">
-        <v>45</v>
-      </c>
-      <c r="J90" t="s">
-        <v>390</v>
-      </c>
-      <c r="K90" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F90,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="L90" t="s">
-        <v>28</v>
-      </c>
-      <c r="M90" s="3"/>
-    </row>
-    <row r="91" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F91" t="s">
-        <v>36</v>
-      </c>
-      <c r="J91" t="s">
-        <v>390</v>
-      </c>
-      <c r="K91" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F91,'feed pars'!B$6:B$43,0))</f>
-        <v>89.5</v>
-      </c>
-      <c r="L91" t="s">
-        <v>28</v>
-      </c>
-      <c r="M91" s="3"/>
-    </row>
-    <row r="92" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F92" t="s">
-        <v>46</v>
-      </c>
-      <c r="J92" t="s">
-        <v>390</v>
-      </c>
-      <c r="K92" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F92,'feed pars'!B$6:B$43,0))</f>
-        <v>91</v>
-      </c>
-      <c r="L92" t="s">
-        <v>28</v>
-      </c>
-      <c r="M92" s="3"/>
-    </row>
-    <row r="93" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F93" t="s">
-        <v>47</v>
-      </c>
-      <c r="J93" t="s">
-        <v>390</v>
-      </c>
-      <c r="K93" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F93,'feed pars'!B$6:B$43,0))</f>
-        <v>91</v>
-      </c>
-      <c r="L93" t="s">
-        <v>28</v>
-      </c>
-      <c r="M93" s="3"/>
-    </row>
-    <row r="94" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F94" t="s">
-        <v>319</v>
-      </c>
-      <c r="J94" t="s">
-        <v>390</v>
-      </c>
-      <c r="K94" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F94,'feed pars'!B$6:B$43,0))</f>
-        <v>90</v>
-      </c>
-      <c r="L94" t="s">
-        <v>28</v>
-      </c>
-      <c r="M94" s="3"/>
-    </row>
-    <row r="95" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F95" t="s">
-        <v>48</v>
-      </c>
-      <c r="J95" t="s">
-        <v>390</v>
-      </c>
-      <c r="K95" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F95,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="L95" t="s">
-        <v>28</v>
-      </c>
-      <c r="M95" s="3"/>
-    </row>
-    <row r="96" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F96" t="s">
-        <v>49</v>
-      </c>
-      <c r="J96" t="s">
-        <v>390</v>
-      </c>
-      <c r="K96" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F96,'feed pars'!B$6:B$43,0))</f>
-        <v>88</v>
-      </c>
-      <c r="L96" t="s">
-        <v>28</v>
-      </c>
-      <c r="M96" s="3"/>
+      <c r="J96" s="33" t="str">
+        <f t="shared" ref="J96:N100" si="7">J75</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K96" s="33">
+        <f t="shared" si="7"/>
+        <v>5</v>
+      </c>
+      <c r="L96" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>%</v>
+      </c>
+      <c r="M96" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="N96" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A97" s="33" t="str">
+        <f t="shared" ref="A97:A100" si="8">A76</f>
+        <v>cattle</v>
+      </c>
+      <c r="E97" s="33" t="str">
+        <f t="shared" si="6"/>
+        <v>bulls</v>
+      </c>
       <c r="F97" t="s">
-        <v>50</v>
-      </c>
-      <c r="J97" t="s">
-        <v>390</v>
-      </c>
-      <c r="K97" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F97,'feed pars'!B$6:B$43,0))</f>
-        <v>90</v>
-      </c>
-      <c r="L97" t="s">
-        <v>28</v>
-      </c>
-      <c r="M97" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="J97" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K97" s="33">
+        <f t="shared" si="7"/>
+        <v>5</v>
+      </c>
+      <c r="L97" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>%</v>
+      </c>
+      <c r="M97" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="N97" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A98" s="33" t="str">
+        <f t="shared" si="8"/>
+        <v>cattle</v>
+      </c>
       <c r="F98" t="s">
-        <v>51</v>
-      </c>
-      <c r="J98" t="s">
-        <v>390</v>
-      </c>
-      <c r="K98" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F98,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
-      </c>
-      <c r="L98" t="s">
-        <v>28</v>
-      </c>
-      <c r="M98" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="J98" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K98" s="33">
+        <f t="shared" si="7"/>
+        <v>6</v>
+      </c>
+      <c r="L98" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>%</v>
+      </c>
+      <c r="M98" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="N98" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A99" s="33" t="str">
+        <f t="shared" si="8"/>
+        <v>sheep</v>
+      </c>
       <c r="F99" t="s">
-        <v>313</v>
-      </c>
-      <c r="J99" t="s">
-        <v>390</v>
-      </c>
-      <c r="K99" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F99,'feed pars'!B$6:B$43,0))</f>
-        <v>90</v>
-      </c>
-      <c r="L99" t="s">
-        <v>28</v>
-      </c>
-      <c r="M99" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="J99" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K99" s="33">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="L99" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>%</v>
+      </c>
+      <c r="M99" s="29"/>
+      <c r="N99" s="33" t="str">
+        <f t="shared" ref="N99:N100" si="9">N78</f>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A100" s="33" t="str">
+        <f t="shared" si="8"/>
+        <v>horses</v>
+      </c>
       <c r="F100" t="s">
-        <v>388</v>
-      </c>
-      <c r="J100" t="s">
-        <v>390</v>
-      </c>
-      <c r="K100" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F100,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="L100" t="s">
-        <v>28</v>
-      </c>
-      <c r="M100" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="J100" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K100" s="33">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="L100" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>%</v>
+      </c>
+      <c r="M100" s="29"/>
+      <c r="N100" s="33" t="str">
+        <f t="shared" si="9"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F101" t="s">
-        <v>52</v>
-      </c>
-      <c r="J101" t="s">
-        <v>390</v>
-      </c>
-      <c r="K101" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F101,'feed pars'!B$6:B$43,0))</f>
-        <v>75.5</v>
-      </c>
-      <c r="L101" t="s">
+        <v>12</v>
+      </c>
+      <c r="J101" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K101" s="29">
+        <v>5</v>
+      </c>
+      <c r="L101" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="M101" s="3"/>
+      <c r="M101" s="29"/>
+      <c r="N101" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A102" s="33" t="str">
+        <f>A75</f>
+        <v>cattle</v>
+      </c>
+      <c r="B102" s="33" t="str">
+        <f>B75</f>
+        <v>dairy</v>
+      </c>
+      <c r="E102" s="33" t="str">
+        <f t="shared" ref="E102:E103" si="10">E75</f>
+        <v>cows</v>
+      </c>
       <c r="F102" t="s">
-        <v>53</v>
-      </c>
-      <c r="J102" t="s">
-        <v>390</v>
-      </c>
-      <c r="K102" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F102,'feed pars'!B$6:B$43,0))</f>
-        <v>89.5</v>
-      </c>
-      <c r="L102" t="s">
+        <v>12</v>
+      </c>
+      <c r="J102" s="33" t="str">
+        <f t="shared" ref="J102:N106" si="11">J75</f>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K102" s="33">
+        <f t="shared" si="11"/>
+        <v>5</v>
+      </c>
+      <c r="L102" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>%</v>
+      </c>
+      <c r="M102" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="N102" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A103" s="33" t="str">
+        <f t="shared" ref="A103:A106" si="12">A76</f>
+        <v>cattle</v>
+      </c>
+      <c r="E103" s="33" t="str">
+        <f t="shared" si="10"/>
+        <v>bulls</v>
+      </c>
+      <c r="F103" t="s">
+        <v>12</v>
+      </c>
+      <c r="J103" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K103" s="33">
+        <f t="shared" si="11"/>
+        <v>5</v>
+      </c>
+      <c r="L103" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>%</v>
+      </c>
+      <c r="M103" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>No feeding on pasture</v>
+      </c>
+      <c r="N103" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A104" s="33" t="str">
+        <f t="shared" si="12"/>
+        <v>cattle</v>
+      </c>
+      <c r="F104" t="s">
+        <v>12</v>
+      </c>
+      <c r="J104" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K104" s="33">
+        <f t="shared" si="11"/>
+        <v>6</v>
+      </c>
+      <c r="L104" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>%</v>
+      </c>
+      <c r="M104" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>10% feeding on pasture</v>
+      </c>
+      <c r="N104" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A105" s="33" t="str">
+        <f t="shared" si="12"/>
+        <v>sheep</v>
+      </c>
+      <c r="F105" t="s">
+        <v>12</v>
+      </c>
+      <c r="J105" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K105" s="33">
+        <f t="shared" si="11"/>
+        <v>15</v>
+      </c>
+      <c r="L105" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>%</v>
+      </c>
+      <c r="M105" s="29"/>
+      <c r="N105" s="33" t="str">
+        <f t="shared" ref="N105:N106" si="13">N78</f>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A106" s="33" t="str">
+        <f t="shared" si="12"/>
+        <v>horses</v>
+      </c>
+      <c r="F106" t="s">
+        <v>12</v>
+      </c>
+      <c r="J106" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K106" s="33">
+        <f t="shared" si="11"/>
+        <v>15</v>
+      </c>
+      <c r="L106" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>%</v>
+      </c>
+      <c r="M106" s="29"/>
+      <c r="N106" s="33" t="str">
+        <f t="shared" si="13"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A107" s="33"/>
+      <c r="F107" t="s">
+        <v>33</v>
+      </c>
+      <c r="J107" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K107" s="29">
+        <v>0</v>
+      </c>
+      <c r="L107" t="s">
         <v>28</v>
       </c>
-      <c r="M102" s="3"/>
-    </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F103" t="s">
-        <v>54</v>
-      </c>
-      <c r="J103" t="s">
-        <v>390</v>
-      </c>
-      <c r="K103" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F103,'feed pars'!B$6:B$43,0))</f>
-        <v>6.25</v>
-      </c>
-      <c r="L103" t="s">
-        <v>28</v>
-      </c>
-      <c r="M103" s="3"/>
-    </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F104" t="s">
-        <v>55</v>
-      </c>
-      <c r="J104" t="s">
-        <v>390</v>
-      </c>
-      <c r="K104" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F104,'feed pars'!B$6:B$43,0))</f>
-        <v>97</v>
-      </c>
-      <c r="L104" t="s">
-        <v>28</v>
-      </c>
-      <c r="M104" s="3"/>
-    </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F105" t="s">
-        <v>56</v>
-      </c>
-      <c r="J105" t="s">
-        <v>390</v>
-      </c>
-      <c r="K105" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F105,'feed pars'!B$6:B$43,0))</f>
-        <v>91</v>
-      </c>
-      <c r="L105" t="s">
-        <v>28</v>
-      </c>
-      <c r="M105" s="3"/>
-    </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F106" t="s">
-        <v>57</v>
-      </c>
-      <c r="J106" t="s">
-        <v>390</v>
-      </c>
-      <c r="K106" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F106,'feed pars'!B$6:B$43,0))</f>
-        <v>92</v>
-      </c>
-      <c r="L106" t="s">
-        <v>28</v>
-      </c>
-      <c r="M106" s="3"/>
-    </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A107" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B107" s="7"/>
-      <c r="C107" s="6"/>
-      <c r="D107" s="6"/>
-      <c r="E107" s="6"/>
-      <c r="F107" s="6"/>
-      <c r="G107" s="6"/>
-      <c r="H107" s="6"/>
-      <c r="I107" s="6"/>
-      <c r="J107" s="6"/>
-      <c r="K107" s="6"/>
-      <c r="L107" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="M107" s="6"/>
-      <c r="N107" s="6"/>
+      <c r="M107" s="29" t="s">
+        <v>409</v>
+      </c>
+      <c r="N107" s="33"/>
     </row>
     <row r="108" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>24</v>
       </c>
       <c r="F108" t="s">
-        <v>310</v>
+        <v>33</v>
       </c>
       <c r="J108" t="s">
-        <v>18</v>
-      </c>
-      <c r="K108" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F108,'feed pars'!B$6:B$43,0))</f>
-        <v>11.5</v>
-      </c>
-      <c r="M108" s="3"/>
+        <v>398</v>
+      </c>
+      <c r="K108" s="29">
+        <f>100-55</f>
+        <v>45</v>
+      </c>
+      <c r="L108" t="s">
+        <v>28</v>
+      </c>
+      <c r="M108" s="29" t="s">
+        <v>401</v>
+      </c>
+      <c r="N108" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>395</v>
+      </c>
+      <c r="F109" t="s">
+        <v>33</v>
+      </c>
+      <c r="J109" t="s">
+        <v>398</v>
+      </c>
+      <c r="K109" s="29">
+        <f>100-50</f>
+        <v>50</v>
+      </c>
+      <c r="L109" t="s">
+        <v>28</v>
+      </c>
+      <c r="M109" s="29" t="s">
+        <v>401</v>
+      </c>
+      <c r="N109" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K110" s="3"/>
+      <c r="M110" s="29"/>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A111" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="K111" s="3"/>
+      <c r="M111" s="29"/>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K112" s="3"/>
+      <c r="M112" s="29"/>
+    </row>
+    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K113" s="3"/>
+      <c r="M113" s="3"/>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A114" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B114" s="1"/>
+      <c r="C114" s="1"/>
+      <c r="D114" s="1"/>
+      <c r="E114" s="2"/>
+      <c r="F114" s="2"/>
+      <c r="G114" s="2"/>
+      <c r="H114" s="2"/>
+      <c r="I114" s="2"/>
+      <c r="J114" s="2"/>
+      <c r="K114" s="2"/>
+      <c r="L114" s="2"/>
+      <c r="M114" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="N114" s="2"/>
+    </row>
+    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F115" t="s">
+        <v>310</v>
+      </c>
+      <c r="J115" t="s">
+        <v>390</v>
+      </c>
+      <c r="K115" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F115,'feed pars'!B$6:B$43,0))</f>
+        <v>100</v>
+      </c>
+      <c r="L115" t="s">
+        <v>28</v>
+      </c>
+      <c r="M115" s="29" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F116" t="s">
+        <v>311</v>
+      </c>
+      <c r="J116" t="s">
+        <v>390</v>
+      </c>
+      <c r="K116" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F116,'feed pars'!B$6:B$43,0))</f>
+        <v>100</v>
+      </c>
+      <c r="L116" t="s">
+        <v>28</v>
+      </c>
+      <c r="M116" s="3"/>
+    </row>
+    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F117" t="s">
+        <v>312</v>
+      </c>
+      <c r="J117" t="s">
+        <v>390</v>
+      </c>
+      <c r="K117" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F117,'feed pars'!B$6:B$43,0))</f>
+        <v>100</v>
+      </c>
+      <c r="L117" t="s">
+        <v>28</v>
+      </c>
+      <c r="M117" s="3"/>
+    </row>
+    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F118" t="s">
+        <v>2</v>
+      </c>
+      <c r="J118" t="s">
+        <v>390</v>
+      </c>
+      <c r="K118" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F118,'feed pars'!B$6:B$43,0))</f>
+        <v>100</v>
+      </c>
+      <c r="L118" t="s">
+        <v>28</v>
+      </c>
+      <c r="M118" s="3"/>
+    </row>
+    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F119" t="s">
+        <v>12</v>
+      </c>
+      <c r="J119" t="s">
+        <v>390</v>
+      </c>
+      <c r="K119" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F119,'feed pars'!B$6:B$43,0))</f>
+        <v>100</v>
+      </c>
+      <c r="L119" t="s">
+        <v>28</v>
+      </c>
+      <c r="M119" s="3"/>
+    </row>
+    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F120" t="s">
+        <v>33</v>
+      </c>
+      <c r="J120" t="s">
+        <v>390</v>
+      </c>
+      <c r="K120" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F120,'feed pars'!B$6:B$43,0))</f>
+        <v>100</v>
+      </c>
+      <c r="L120" t="s">
+        <v>28</v>
+      </c>
+      <c r="M120" s="3"/>
+    </row>
+    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F121" t="s">
+        <v>17</v>
+      </c>
+      <c r="J121" t="s">
+        <v>390</v>
+      </c>
+      <c r="K121" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F121,'feed pars'!B$6:B$43,0))</f>
+        <v>87</v>
+      </c>
+      <c r="L121" t="s">
+        <v>28</v>
+      </c>
+      <c r="M121" s="3"/>
+    </row>
+    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F122" t="s">
+        <v>37</v>
+      </c>
+      <c r="J122" t="s">
+        <v>390</v>
+      </c>
+      <c r="K122" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F122,'feed pars'!B$6:B$43,0))</f>
+        <v>87</v>
+      </c>
+      <c r="L122" t="s">
+        <v>28</v>
+      </c>
+      <c r="M122" s="3"/>
+    </row>
+    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F123" t="s">
+        <v>38</v>
+      </c>
+      <c r="J123" t="s">
+        <v>390</v>
+      </c>
+      <c r="K123" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F123,'feed pars'!B$6:B$43,0))</f>
+        <v>86</v>
+      </c>
+      <c r="L123" t="s">
+        <v>28</v>
+      </c>
+      <c r="M123" s="3"/>
+    </row>
+    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F124" t="s">
+        <v>39</v>
+      </c>
+      <c r="J124" t="s">
+        <v>390</v>
+      </c>
+      <c r="K124" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F124,'feed pars'!B$6:B$43,0))</f>
+        <v>87</v>
+      </c>
+      <c r="L124" t="s">
+        <v>28</v>
+      </c>
+      <c r="M124" s="3"/>
+    </row>
+    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F125" t="s">
+        <v>317</v>
+      </c>
+      <c r="J125" t="s">
+        <v>390</v>
+      </c>
+      <c r="K125" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F125,'feed pars'!B$6:B$43,0))</f>
+        <v>87</v>
+      </c>
+      <c r="L125" t="s">
+        <v>28</v>
+      </c>
+      <c r="M125" s="3"/>
+    </row>
+    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F126" t="s">
+        <v>40</v>
+      </c>
+      <c r="J126" t="s">
+        <v>390</v>
+      </c>
+      <c r="K126" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F126,'feed pars'!B$6:B$43,0))</f>
+        <v>67.5</v>
+      </c>
+      <c r="L126" t="s">
+        <v>28</v>
+      </c>
+      <c r="M126" s="3"/>
+    </row>
+    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F127" t="s">
+        <v>41</v>
+      </c>
+      <c r="J127" t="s">
+        <v>390</v>
+      </c>
+      <c r="K127" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F127,'feed pars'!B$6:B$43,0))</f>
+        <v>87</v>
+      </c>
+      <c r="L127" t="s">
+        <v>28</v>
+      </c>
+      <c r="M127" s="3"/>
+    </row>
+    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F128" t="s">
+        <v>42</v>
+      </c>
+      <c r="J128" t="s">
+        <v>390</v>
+      </c>
+      <c r="K128" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F128,'feed pars'!B$6:B$43,0))</f>
+        <v>86.8</v>
+      </c>
+      <c r="L128" t="s">
+        <v>28</v>
+      </c>
+      <c r="M128" s="3"/>
+    </row>
+    <row r="129" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F129" t="s">
+        <v>35</v>
+      </c>
+      <c r="J129" t="s">
+        <v>390</v>
+      </c>
+      <c r="K129" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F129,'feed pars'!B$6:B$43,0))</f>
+        <v>92.5</v>
+      </c>
+      <c r="L129" t="s">
+        <v>28</v>
+      </c>
+      <c r="M129" s="3"/>
+    </row>
+    <row r="130" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F130" t="s">
+        <v>43</v>
+      </c>
+      <c r="J130" t="s">
+        <v>390</v>
+      </c>
+      <c r="K130" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F130,'feed pars'!B$6:B$43,0))</f>
+        <v>92</v>
+      </c>
+      <c r="L130" t="s">
+        <v>28</v>
+      </c>
+      <c r="M130" s="3"/>
+    </row>
+    <row r="131" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F131" t="s">
+        <v>314</v>
+      </c>
+      <c r="J131" t="s">
+        <v>390</v>
+      </c>
+      <c r="K131" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F131,'feed pars'!B$6:B$43,0))</f>
+        <v>100</v>
+      </c>
+      <c r="L131" t="s">
+        <v>28</v>
+      </c>
+      <c r="M131" s="3"/>
+    </row>
+    <row r="132" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F132" t="s">
+        <v>305</v>
+      </c>
+      <c r="J132" t="s">
+        <v>390</v>
+      </c>
+      <c r="K132" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F132,'feed pars'!B$6:B$43,0))</f>
+        <v>85</v>
+      </c>
+      <c r="L132" t="s">
+        <v>28</v>
+      </c>
+      <c r="M132" s="3"/>
+    </row>
+    <row r="133" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F133" t="s">
+        <v>318</v>
+      </c>
+      <c r="J133" t="s">
+        <v>390</v>
+      </c>
+      <c r="K133" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F133,'feed pars'!B$6:B$43,0))</f>
+        <v>87</v>
+      </c>
+      <c r="L133" t="s">
+        <v>28</v>
+      </c>
+      <c r="M133" s="3"/>
+    </row>
+    <row r="134" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F134" t="s">
+        <v>44</v>
+      </c>
+      <c r="J134" t="s">
+        <v>390</v>
+      </c>
+      <c r="K134" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F134,'feed pars'!B$6:B$43,0))</f>
+        <v>87.5</v>
+      </c>
+      <c r="L134" t="s">
+        <v>28</v>
+      </c>
+      <c r="M134" s="3"/>
+    </row>
+    <row r="135" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F135" t="s">
+        <v>45</v>
+      </c>
+      <c r="J135" t="s">
+        <v>390</v>
+      </c>
+      <c r="K135" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F135,'feed pars'!B$6:B$43,0))</f>
+        <v>87</v>
+      </c>
+      <c r="L135" t="s">
+        <v>28</v>
+      </c>
+      <c r="M135" s="3"/>
+    </row>
+    <row r="136" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F136" t="s">
+        <v>36</v>
+      </c>
+      <c r="J136" t="s">
+        <v>390</v>
+      </c>
+      <c r="K136" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F136,'feed pars'!B$6:B$43,0))</f>
+        <v>89.5</v>
+      </c>
+      <c r="L136" t="s">
+        <v>28</v>
+      </c>
+      <c r="M136" s="3"/>
+    </row>
+    <row r="137" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F137" t="s">
+        <v>46</v>
+      </c>
+      <c r="J137" t="s">
+        <v>390</v>
+      </c>
+      <c r="K137" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F137,'feed pars'!B$6:B$43,0))</f>
+        <v>91</v>
+      </c>
+      <c r="L137" t="s">
+        <v>28</v>
+      </c>
+      <c r="M137" s="3"/>
+    </row>
+    <row r="138" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F138" t="s">
+        <v>47</v>
+      </c>
+      <c r="J138" t="s">
+        <v>390</v>
+      </c>
+      <c r="K138" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F138,'feed pars'!B$6:B$43,0))</f>
+        <v>91</v>
+      </c>
+      <c r="L138" t="s">
+        <v>28</v>
+      </c>
+      <c r="M138" s="3"/>
+    </row>
+    <row r="139" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F139" t="s">
+        <v>319</v>
+      </c>
+      <c r="J139" t="s">
+        <v>390</v>
+      </c>
+      <c r="K139" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F139,'feed pars'!B$6:B$43,0))</f>
+        <v>90</v>
+      </c>
+      <c r="L139" t="s">
+        <v>28</v>
+      </c>
+      <c r="M139" s="3"/>
+    </row>
+    <row r="140" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F140" t="s">
+        <v>48</v>
+      </c>
+      <c r="J140" t="s">
+        <v>390</v>
+      </c>
+      <c r="K140" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F140,'feed pars'!B$6:B$43,0))</f>
+        <v>87</v>
+      </c>
+      <c r="L140" t="s">
+        <v>28</v>
+      </c>
+      <c r="M140" s="3"/>
+    </row>
+    <row r="141" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F141" t="s">
+        <v>49</v>
+      </c>
+      <c r="J141" t="s">
+        <v>390</v>
+      </c>
+      <c r="K141" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F141,'feed pars'!B$6:B$43,0))</f>
+        <v>88</v>
+      </c>
+      <c r="L141" t="s">
+        <v>28</v>
+      </c>
+      <c r="M141" s="3"/>
+    </row>
+    <row r="142" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F142" t="s">
+        <v>50</v>
+      </c>
+      <c r="J142" t="s">
+        <v>390</v>
+      </c>
+      <c r="K142" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F142,'feed pars'!B$6:B$43,0))</f>
+        <v>90</v>
+      </c>
+      <c r="L142" t="s">
+        <v>28</v>
+      </c>
+      <c r="M142" s="3"/>
+    </row>
+    <row r="143" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F143" t="s">
+        <v>51</v>
+      </c>
+      <c r="J143" t="s">
+        <v>390</v>
+      </c>
+      <c r="K143" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F143,'feed pars'!B$6:B$43,0))</f>
+        <v>11</v>
+      </c>
+      <c r="L143" t="s">
+        <v>28</v>
+      </c>
+      <c r="M143" s="3"/>
+    </row>
+    <row r="144" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F144" t="s">
+        <v>313</v>
+      </c>
+      <c r="J144" t="s">
+        <v>390</v>
+      </c>
+      <c r="K144" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F144,'feed pars'!B$6:B$43,0))</f>
+        <v>90</v>
+      </c>
+      <c r="L144" t="s">
+        <v>28</v>
+      </c>
+      <c r="M144" s="3"/>
+    </row>
+    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F145" t="s">
+        <v>388</v>
+      </c>
+      <c r="J145" t="s">
+        <v>390</v>
+      </c>
+      <c r="K145" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F145,'feed pars'!B$6:B$43,0))</f>
+        <v>87</v>
+      </c>
+      <c r="L145" t="s">
+        <v>28</v>
+      </c>
+      <c r="M145" s="3"/>
+    </row>
+    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F146" t="s">
+        <v>52</v>
+      </c>
+      <c r="J146" t="s">
+        <v>390</v>
+      </c>
+      <c r="K146" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F146,'feed pars'!B$6:B$43,0))</f>
+        <v>75.5</v>
+      </c>
+      <c r="L146" t="s">
+        <v>28</v>
+      </c>
+      <c r="M146" s="3"/>
+    </row>
+    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F147" t="s">
+        <v>53</v>
+      </c>
+      <c r="J147" t="s">
+        <v>390</v>
+      </c>
+      <c r="K147" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F147,'feed pars'!B$6:B$43,0))</f>
+        <v>89.5</v>
+      </c>
+      <c r="L147" t="s">
+        <v>28</v>
+      </c>
+      <c r="M147" s="3"/>
+    </row>
+    <row r="148" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F148" t="s">
+        <v>54</v>
+      </c>
+      <c r="J148" t="s">
+        <v>390</v>
+      </c>
+      <c r="K148" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F148,'feed pars'!B$6:B$43,0))</f>
+        <v>6.25</v>
+      </c>
+      <c r="L148" t="s">
+        <v>28</v>
+      </c>
+      <c r="M148" s="3"/>
+    </row>
+    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F149" t="s">
+        <v>55</v>
+      </c>
+      <c r="J149" t="s">
+        <v>390</v>
+      </c>
+      <c r="K149" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F149,'feed pars'!B$6:B$43,0))</f>
+        <v>97</v>
+      </c>
+      <c r="L149" t="s">
+        <v>28</v>
+      </c>
+      <c r="M149" s="3"/>
+    </row>
+    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F150" t="s">
+        <v>56</v>
+      </c>
+      <c r="J150" t="s">
+        <v>390</v>
+      </c>
+      <c r="K150" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F150,'feed pars'!B$6:B$43,0))</f>
+        <v>91</v>
+      </c>
+      <c r="L150" t="s">
+        <v>28</v>
+      </c>
+      <c r="M150" s="3"/>
+    </row>
+    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F151" t="s">
+        <v>57</v>
+      </c>
+      <c r="J151" t="s">
+        <v>390</v>
+      </c>
+      <c r="K151" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F151,'feed pars'!B$6:B$43,0))</f>
+        <v>92</v>
+      </c>
+      <c r="L151" t="s">
+        <v>28</v>
+      </c>
+      <c r="M151" s="3"/>
+    </row>
+    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A152" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B152" s="7"/>
+      <c r="C152" s="6"/>
+      <c r="D152" s="6"/>
+      <c r="E152" s="6"/>
+      <c r="F152" s="6"/>
+      <c r="G152" s="6"/>
+      <c r="H152" s="6"/>
+      <c r="I152" s="6"/>
+      <c r="J152" s="6"/>
+      <c r="K152" s="6"/>
+      <c r="L152" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M152" s="6"/>
+      <c r="N152" s="6"/>
+    </row>
+    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
         <v>24</v>
       </c>
-      <c r="F109" t="s">
-        <v>311</v>
-      </c>
-      <c r="J109" t="s">
-        <v>18</v>
-      </c>
-      <c r="K109" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F109,'feed pars'!B$6:B$43,0))</f>
-        <v>10.4</v>
-      </c>
-      <c r="M109" s="3"/>
-    </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>24</v>
-      </c>
-      <c r="F110" t="s">
-        <v>312</v>
-      </c>
-      <c r="J110" t="s">
-        <v>18</v>
-      </c>
-      <c r="K110" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F110,'feed pars'!B$6:B$43,0))</f>
-        <v>10</v>
-      </c>
-      <c r="M110" s="3"/>
-    </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>24</v>
-      </c>
-      <c r="F111" t="s">
-        <v>12</v>
-      </c>
-      <c r="J111" t="s">
-        <v>18</v>
-      </c>
-      <c r="K111" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F111,'feed pars'!B$6:B$43,0))</f>
-        <v>11.3</v>
-      </c>
-    </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>24</v>
-      </c>
-      <c r="F112" t="s">
-        <v>33</v>
-      </c>
-      <c r="J112" t="s">
-        <v>18</v>
-      </c>
-      <c r="K112" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F112,'feed pars'!B$6:B$43,0))</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="K113" s="3"/>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>24</v>
-      </c>
-      <c r="F114" t="s">
-        <v>17</v>
-      </c>
-      <c r="J114" t="s">
-        <v>18</v>
-      </c>
-      <c r="K114" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F114,'feed pars'!B$6:B$43,0))</f>
-        <v>14.1</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>24</v>
-      </c>
-      <c r="F115" t="s">
-        <v>37</v>
-      </c>
-      <c r="J115" t="s">
-        <v>18</v>
-      </c>
-      <c r="K115" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F115,'feed pars'!B$6:B$43,0))</f>
-        <v>13.2</v>
-      </c>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>24</v>
-      </c>
-      <c r="F116" t="s">
-        <v>38</v>
-      </c>
-      <c r="J116" t="s">
-        <v>18</v>
-      </c>
-      <c r="K116" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F116,'feed pars'!B$6:B$43,0))</f>
-        <v>11.7</v>
-      </c>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>24</v>
-      </c>
-      <c r="F117" t="s">
-        <v>39</v>
-      </c>
-      <c r="J117" t="s">
-        <v>18</v>
-      </c>
-      <c r="K117" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F117,'feed pars'!B$6:B$43,0))</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>24</v>
-      </c>
-      <c r="F118" t="s">
-        <v>317</v>
-      </c>
-      <c r="J118" t="s">
-        <v>18</v>
-      </c>
-      <c r="K118" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F118,'feed pars'!B$6:B$43,0))</f>
-        <v>13.9</v>
-      </c>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>24</v>
-      </c>
-      <c r="F119" t="s">
-        <v>40</v>
-      </c>
-      <c r="J119" t="s">
-        <v>18</v>
-      </c>
-      <c r="K119" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F119,'feed pars'!B$6:B$43,0))</f>
-        <v>12.8</v>
-      </c>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>24</v>
-      </c>
-      <c r="F120" t="s">
-        <v>41</v>
-      </c>
-      <c r="J120" t="s">
-        <v>18</v>
-      </c>
-      <c r="K120" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F120,'feed pars'!B$6:B$43,0))</f>
-        <v>13.8</v>
-      </c>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>24</v>
-      </c>
-      <c r="F121" t="s">
-        <v>42</v>
-      </c>
-      <c r="J121" t="s">
-        <v>18</v>
-      </c>
-      <c r="K121" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F121,'feed pars'!B$6:B$43,0))</f>
-        <v>13.3</v>
-      </c>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>24</v>
-      </c>
-      <c r="F122" t="s">
-        <v>35</v>
-      </c>
-      <c r="J122" t="s">
-        <v>18</v>
-      </c>
-      <c r="K122" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F122,'feed pars'!B$6:B$43,0))</f>
-        <v>22.1</v>
-      </c>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>24</v>
-      </c>
-      <c r="F123" t="s">
-        <v>43</v>
-      </c>
-      <c r="J123" t="s">
-        <v>18</v>
-      </c>
-      <c r="K123" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F123,'feed pars'!B$6:B$43,0))</f>
-        <v>20.100000000000001</v>
-      </c>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>24</v>
-      </c>
-      <c r="F124" t="s">
-        <v>305</v>
-      </c>
-      <c r="J124" t="s">
-        <v>18</v>
-      </c>
-      <c r="K124" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F124,'feed pars'!B$6:B$43,0))</f>
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>24</v>
-      </c>
-      <c r="F125" t="s">
-        <v>314</v>
-      </c>
-      <c r="J125" t="s">
-        <v>18</v>
-      </c>
-      <c r="K125" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F125,'feed pars'!B$6:B$43,0))</f>
-        <v>36.6</v>
-      </c>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>24</v>
-      </c>
-      <c r="F126" t="s">
-        <v>318</v>
-      </c>
-      <c r="J126" t="s">
-        <v>18</v>
-      </c>
-      <c r="K126" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F126,'feed pars'!B$6:B$43,0))</f>
-        <v>16.399999999999999</v>
-      </c>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>24</v>
-      </c>
-      <c r="F127" t="s">
-        <v>44</v>
-      </c>
-      <c r="J127" t="s">
-        <v>18</v>
-      </c>
-      <c r="K127" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F127,'feed pars'!B$6:B$43,0))</f>
-        <v>14.6</v>
-      </c>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>24</v>
-      </c>
-      <c r="F128" t="s">
-        <v>36</v>
-      </c>
-      <c r="J128" t="s">
-        <v>18</v>
-      </c>
-      <c r="K128" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F128,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
-        <v>24</v>
-      </c>
-      <c r="F129" t="s">
-        <v>46</v>
-      </c>
-      <c r="J129" t="s">
-        <v>18</v>
-      </c>
-      <c r="K129" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F129,'feed pars'!B$6:B$43,0))</f>
-        <v>11.4</v>
-      </c>
-    </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
-        <v>24</v>
-      </c>
-      <c r="F130" t="s">
-        <v>47</v>
-      </c>
-      <c r="J130" t="s">
-        <v>18</v>
-      </c>
-      <c r="K130" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F130,'feed pars'!B$6:B$43,0))</f>
-        <v>13.4</v>
-      </c>
-    </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
-        <v>24</v>
-      </c>
-      <c r="F131" t="s">
-        <v>319</v>
-      </c>
-      <c r="J131" t="s">
-        <v>18</v>
-      </c>
-      <c r="K131" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F131,'feed pars'!B$6:B$43,0))</f>
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
-        <v>24</v>
-      </c>
-      <c r="F132" t="s">
-        <v>48</v>
-      </c>
-      <c r="J132" t="s">
-        <v>18</v>
-      </c>
-      <c r="K132" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F132,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
-        <v>24</v>
-      </c>
-      <c r="F133" t="s">
-        <v>50</v>
-      </c>
-      <c r="J133" t="s">
-        <v>18</v>
-      </c>
-      <c r="K133" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F133,'feed pars'!B$6:B$43,0))</f>
-        <v>13.3</v>
-      </c>
-    </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>24</v>
-      </c>
-      <c r="F134" t="s">
-        <v>313</v>
-      </c>
-      <c r="J134" t="s">
-        <v>18</v>
-      </c>
-      <c r="K134" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F134,'feed pars'!B$6:B$43,0))</f>
-        <v>11.6</v>
-      </c>
-    </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
-        <v>24</v>
-      </c>
-      <c r="F135" t="s">
-        <v>52</v>
-      </c>
-      <c r="J135" t="s">
-        <v>18</v>
-      </c>
-      <c r="K135" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F135,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
-      </c>
-    </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>24</v>
-      </c>
-      <c r="F136" t="s">
-        <v>53</v>
-      </c>
-      <c r="J136" t="s">
-        <v>18</v>
-      </c>
-      <c r="K136" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F136,'feed pars'!B$6:B$43,0))</f>
-        <v>12.3</v>
-      </c>
-    </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>24</v>
-      </c>
-      <c r="F137" t="s">
-        <v>54</v>
-      </c>
-      <c r="J137" t="s">
-        <v>18</v>
-      </c>
-      <c r="K137" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F137,'feed pars'!B$6:B$43,0))</f>
-        <v>13.6</v>
-      </c>
-    </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>24</v>
-      </c>
-      <c r="F138" t="s">
-        <v>56</v>
-      </c>
-      <c r="J138" t="s">
-        <v>18</v>
-      </c>
-      <c r="K138" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F138,'feed pars'!B$6:B$43,0))</f>
-        <v>15.5</v>
-      </c>
-    </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>24</v>
-      </c>
-      <c r="F139" t="s">
-        <v>324</v>
-      </c>
-      <c r="J139" t="s">
-        <v>18</v>
-      </c>
-      <c r="K139" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A140" s="7" t="s">
-        <v>396</v>
-      </c>
-      <c r="B140" s="7"/>
-      <c r="C140" s="6"/>
-      <c r="D140" s="6"/>
-      <c r="E140" s="6"/>
-      <c r="F140" s="6"/>
-      <c r="G140" s="6"/>
-      <c r="H140" s="6"/>
-      <c r="I140" s="6"/>
-      <c r="J140" s="6"/>
-      <c r="K140" s="6"/>
-      <c r="L140" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="M140" s="6"/>
-      <c r="N140" s="6"/>
-    </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>395</v>
-      </c>
-      <c r="F141" t="s">
-        <v>2</v>
-      </c>
-      <c r="J141" t="s">
-        <v>18</v>
-      </c>
-      <c r="K141" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
-        <v>395</v>
-      </c>
-      <c r="F142" t="s">
-        <v>33</v>
-      </c>
-      <c r="J142" t="s">
-        <v>18</v>
-      </c>
-      <c r="K142" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A143" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B143" s="8"/>
-      <c r="C143" s="9"/>
-      <c r="D143" s="9"/>
-      <c r="E143" s="9"/>
-      <c r="F143" s="9"/>
-      <c r="G143" s="9"/>
-      <c r="H143" s="9"/>
-      <c r="I143" s="9"/>
-      <c r="J143" s="9"/>
-      <c r="K143" s="9"/>
-      <c r="L143" s="9"/>
-      <c r="M143" s="9"/>
-      <c r="N143" s="9"/>
-    </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A144" s="30" t="s">
-        <v>391</v>
-      </c>
-      <c r="B144" s="31"/>
-      <c r="C144" s="32"/>
-      <c r="D144" s="32"/>
-      <c r="E144" s="32"/>
-      <c r="F144" s="32"/>
-      <c r="G144" s="32"/>
-      <c r="H144" s="32"/>
-      <c r="I144" s="32"/>
-      <c r="J144" s="32"/>
-      <c r="K144" s="32"/>
-      <c r="L144" s="32" t="s">
-        <v>300</v>
-      </c>
-      <c r="M144" s="32"/>
-      <c r="N144" s="32"/>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
-        <v>25</v>
-      </c>
-      <c r="E145" t="s">
-        <v>299</v>
-      </c>
-      <c r="F145" t="s">
-        <v>17</v>
-      </c>
-      <c r="J145" t="s">
-        <v>18</v>
-      </c>
-      <c r="K145" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F145,'feed pars'!B$6:B$43,0))</f>
-        <v>12.3</v>
-      </c>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A146" t="s">
-        <v>25</v>
-      </c>
-      <c r="E146" t="s">
-        <v>299</v>
-      </c>
-      <c r="F146" t="s">
-        <v>37</v>
-      </c>
-      <c r="J146" t="s">
-        <v>18</v>
-      </c>
-      <c r="K146" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F146,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
-      </c>
-    </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A147" t="s">
-        <v>25</v>
-      </c>
-      <c r="E147" t="s">
-        <v>299</v>
-      </c>
-      <c r="F147" t="s">
-        <v>38</v>
-      </c>
-      <c r="J147" t="s">
-        <v>18</v>
-      </c>
-      <c r="K147" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F147,'feed pars'!B$6:B$43,0))</f>
-        <v>9.4</v>
-      </c>
-    </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
-        <v>25</v>
-      </c>
-      <c r="E148" t="s">
-        <v>299</v>
-      </c>
-      <c r="F148" t="s">
-        <v>39</v>
-      </c>
-      <c r="J148" t="s">
-        <v>18</v>
-      </c>
-      <c r="K148" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F148,'feed pars'!B$6:B$43,0))</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
-        <v>25</v>
-      </c>
-      <c r="E149" t="s">
-        <v>299</v>
-      </c>
-      <c r="F149" t="s">
-        <v>40</v>
-      </c>
-      <c r="J149" t="s">
-        <v>18</v>
-      </c>
-      <c r="K149" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F149,'feed pars'!B$6:B$43,0))</f>
-        <v>13.2</v>
-      </c>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
-        <v>25</v>
-      </c>
-      <c r="E150" t="s">
-        <v>299</v>
-      </c>
-      <c r="F150" t="s">
-        <v>41</v>
-      </c>
-      <c r="J150" t="s">
-        <v>18</v>
-      </c>
-      <c r="K150" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F150,'feed pars'!B$6:B$43,0))</f>
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
-        <v>25</v>
-      </c>
-      <c r="E151" t="s">
-        <v>299</v>
-      </c>
-      <c r="F151" t="s">
-        <v>42</v>
-      </c>
-      <c r="J151" t="s">
-        <v>18</v>
-      </c>
-      <c r="K151" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F151,'feed pars'!B$6:B$43,0))</f>
-        <v>10.9</v>
-      </c>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
-        <v>25</v>
-      </c>
-      <c r="E152" t="s">
-        <v>299</v>
-      </c>
-      <c r="F152" t="s">
-        <v>35</v>
-      </c>
-      <c r="J152" t="s">
-        <v>18</v>
-      </c>
-      <c r="K152" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F152,'feed pars'!B$6:B$43,0))</f>
-        <v>18.5</v>
-      </c>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
-        <v>25</v>
-      </c>
-      <c r="E153" t="s">
-        <v>299</v>
-      </c>
       <c r="F153" t="s">
-        <v>43</v>
+        <v>310</v>
       </c>
       <c r="J153" t="s">
         <v>18</v>
       </c>
       <c r="K153" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F153,'feed pars'!B$6:B$43,0))</f>
-        <v>17.5</v>
-      </c>
-    </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F153,'feed pars'!B$6:B$43,0))</f>
+        <v>11.5</v>
+      </c>
+      <c r="M153" s="3"/>
+    </row>
+    <row r="154" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>25</v>
-      </c>
-      <c r="E154" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F154" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="J154" t="s">
         <v>18</v>
       </c>
       <c r="K154" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F154,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
-      </c>
-    </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F154,'feed pars'!B$6:B$43,0))</f>
+        <v>10.4</v>
+      </c>
+      <c r="M154" s="3"/>
+    </row>
+    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>25</v>
-      </c>
-      <c r="E155" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F155" t="s">
-        <v>44</v>
+        <v>312</v>
       </c>
       <c r="J155" t="s">
         <v>18</v>
       </c>
       <c r="K155" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F155,'feed pars'!B$6:B$43,0))</f>
-        <v>9.9</v>
-      </c>
-    </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F155,'feed pars'!B$6:B$43,0))</f>
+        <v>10</v>
+      </c>
+      <c r="M155" s="3"/>
+    </row>
+    <row r="156" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>25</v>
-      </c>
-      <c r="E156" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F156" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="J156" t="s">
         <v>18</v>
       </c>
       <c r="K156" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F156,'feed pars'!B$6:B$43,0))</f>
-        <v>10.3</v>
-      </c>
-    </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F156,'feed pars'!B$6:B$43,0))</f>
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>25</v>
-      </c>
-      <c r="E157" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F157" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="J157" t="s">
         <v>18</v>
       </c>
       <c r="K157" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F157,'feed pars'!B$6:B$43,0))</f>
-        <v>7.7</v>
-      </c>
-    </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A158" t="s">
-        <v>25</v>
-      </c>
-      <c r="E158" t="s">
-        <v>299</v>
-      </c>
-      <c r="F158" t="s">
-        <v>46</v>
-      </c>
-      <c r="J158" t="s">
-        <v>18</v>
-      </c>
-      <c r="K158" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F158,'feed pars'!B$6:B$43,0))</f>
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F157,'feed pars'!B$6:B$43,0))</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K158" s="3"/>
+    </row>
+    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>25</v>
-      </c>
-      <c r="E159" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F159" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="J159" t="s">
         <v>18</v>
       </c>
       <c r="K159" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F159,'feed pars'!B$6:B$43,0))</f>
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F159,'feed pars'!B$6:B$43,0))</f>
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="160" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>25</v>
-      </c>
-      <c r="E160" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F160" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="J160" t="s">
         <v>18</v>
       </c>
       <c r="K160" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F160,'feed pars'!B$6:B$43,0))</f>
-        <v>7.8</v>
-      </c>
-    </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F160,'feed pars'!B$6:B$43,0))</f>
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>25</v>
-      </c>
-      <c r="E161" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F161" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="J161" t="s">
         <v>18</v>
       </c>
       <c r="K161" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F161,'feed pars'!B$6:B$43,0))</f>
-        <v>9.1999999999999993</v>
-      </c>
-    </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F161,'feed pars'!B$6:B$43,0))</f>
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>25</v>
-      </c>
-      <c r="E162" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F162" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="J162" t="s">
         <v>18</v>
       </c>
       <c r="K162" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F162,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
-      </c>
-    </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F162,'feed pars'!B$6:B$43,0))</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>25</v>
-      </c>
-      <c r="E163" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F163" t="s">
-        <v>51</v>
+        <v>317</v>
       </c>
       <c r="J163" t="s">
         <v>18</v>
       </c>
       <c r="K163" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F163,'feed pars'!B$6:B$43,0))</f>
-        <v>8.9</v>
-      </c>
-    </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F163,'feed pars'!B$6:B$43,0))</f>
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>25</v>
-      </c>
-      <c r="E164" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F164" t="s">
-        <v>313</v>
+        <v>40</v>
       </c>
       <c r="J164" t="s">
         <v>18</v>
       </c>
       <c r="K164" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F164,'feed pars'!B$6:B$43,0))</f>
-        <v>7.0888888888888877</v>
-      </c>
-    </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F164,'feed pars'!B$6:B$43,0))</f>
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>25</v>
-      </c>
-      <c r="E165" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F165" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="J165" t="s">
         <v>18</v>
       </c>
       <c r="K165" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F165,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F165,'feed pars'!B$6:B$43,0))</f>
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>25</v>
-      </c>
-      <c r="E166" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F166" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="J166" t="s">
         <v>18</v>
       </c>
       <c r="K166" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F166,'feed pars'!B$6:B$43,0))</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F166,'feed pars'!B$6:B$43,0))</f>
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>25</v>
-      </c>
-      <c r="E167" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F167" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="J167" t="s">
         <v>18</v>
       </c>
       <c r="K167" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F167,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F167,'feed pars'!B$6:B$43,0))</f>
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>25</v>
-      </c>
-      <c r="E168" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F168" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="J168" t="s">
         <v>18</v>
       </c>
       <c r="K168" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F168,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F168,'feed pars'!B$6:B$43,0))</f>
+        <v>20.100000000000001</v>
+      </c>
+    </row>
+    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>25</v>
-      </c>
-      <c r="E169" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F169" t="s">
-        <v>56</v>
+        <v>305</v>
       </c>
       <c r="J169" t="s">
         <v>18</v>
       </c>
       <c r="K169" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F169,'feed pars'!B$6:B$43,0))</f>
-        <v>11.3</v>
-      </c>
-    </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F169,'feed pars'!B$6:B$43,0))</f>
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>25</v>
-      </c>
-      <c r="E170" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="F170" t="s">
-        <v>57</v>
+        <v>314</v>
       </c>
       <c r="J170" t="s">
         <v>18</v>
       </c>
       <c r="K170" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F170,'feed pars'!B$6:B$43,0))</f>
-        <v>10.8</v>
-      </c>
-    </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A171" s="30" t="s">
-        <v>392</v>
-      </c>
-      <c r="B171" s="31"/>
-      <c r="C171" s="32"/>
-      <c r="D171" s="32"/>
-      <c r="E171" s="32"/>
-      <c r="F171" s="32"/>
-      <c r="G171" s="32"/>
-      <c r="H171" s="32"/>
-      <c r="I171" s="32"/>
-      <c r="J171" s="32"/>
-      <c r="K171" s="32"/>
-      <c r="L171" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="M171" s="32"/>
-      <c r="N171" s="32"/>
-    </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F170,'feed pars'!B$6:B$43,0))</f>
+        <v>36.6</v>
+      </c>
+    </row>
+    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>24</v>
+      </c>
+      <c r="F171" t="s">
+        <v>318</v>
+      </c>
+      <c r="J171" t="s">
+        <v>18</v>
+      </c>
+      <c r="K171" s="26">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F171,'feed pars'!B$6:B$43,0))</f>
+        <v>16.399999999999999</v>
+      </c>
+    </row>
+    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F172" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="J172" t="s">
         <v>18</v>
       </c>
       <c r="K172" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F172,'feed pars'!B$6:B$43,0))</f>
-        <v>12.1</v>
-      </c>
-    </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F172,'feed pars'!B$6:B$43,0))</f>
+        <v>14.6</v>
+      </c>
+    </row>
+    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F173" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J173" t="s">
         <v>18</v>
       </c>
       <c r="K173" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F173,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F173,'feed pars'!B$6:B$43,0))</f>
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F174" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="J174" t="s">
         <v>18</v>
       </c>
       <c r="K174" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F174,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F174,'feed pars'!B$6:B$43,0))</f>
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F175" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="J175" t="s">
         <v>18</v>
       </c>
       <c r="K175" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F175,'feed pars'!B$6:B$43,0))</f>
-        <v>11.9</v>
-      </c>
-    </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F175,'feed pars'!B$6:B$43,0))</f>
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F176" t="s">
-        <v>40</v>
+        <v>319</v>
       </c>
       <c r="J176" t="s">
         <v>18</v>
       </c>
       <c r="K176" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F176,'feed pars'!B$6:B$43,0))</f>
-        <v>12.8</v>
-      </c>
-    </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F176,'feed pars'!B$6:B$43,0))</f>
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="177" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F177" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="J177" t="s">
         <v>18</v>
       </c>
       <c r="K177" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F177,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
-      </c>
-    </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F177,'feed pars'!B$6:B$43,0))</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="178" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F178" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="J178" t="s">
         <v>18</v>
       </c>
       <c r="K178" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F178,'feed pars'!B$6:B$43,0))</f>
-        <v>10.7</v>
-      </c>
-    </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F178,'feed pars'!B$6:B$43,0))</f>
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="179" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F179" t="s">
-        <v>35</v>
+        <v>313</v>
       </c>
       <c r="J179" t="s">
         <v>18</v>
       </c>
       <c r="K179" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F179,'feed pars'!B$6:B$43,0))</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F179,'feed pars'!B$6:B$43,0))</f>
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="180" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F180" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="J180" t="s">
         <v>18</v>
       </c>
       <c r="K180" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F180,'feed pars'!B$6:B$43,0))</f>
-        <v>17.3</v>
-      </c>
-    </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F180,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="181" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F181" t="s">
-        <v>314</v>
+        <v>53</v>
       </c>
       <c r="J181" t="s">
         <v>18</v>
       </c>
       <c r="K181" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F181,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
-      </c>
-    </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F181,'feed pars'!B$6:B$43,0))</f>
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="182" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F182" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="J182" t="s">
         <v>18</v>
       </c>
       <c r="K182" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F182,'feed pars'!B$6:B$43,0))</f>
-        <v>9.3000000000000007</v>
-      </c>
-    </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F182,'feed pars'!B$6:B$43,0))</f>
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="183" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F183" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="J183" t="s">
         <v>18</v>
       </c>
       <c r="K183" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F183,'feed pars'!B$6:B$43,0))</f>
-        <v>9.6999999999999993</v>
-      </c>
-    </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F183,'feed pars'!B$6:B$43,0))</f>
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="184" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F184" t="s">
-        <v>36</v>
+        <v>324</v>
       </c>
       <c r="J184" t="s">
         <v>18</v>
       </c>
-      <c r="K184" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F184,'feed pars'!B$6:B$43,0))</f>
-        <v>7.1</v>
-      </c>
-    </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A185" t="s">
-        <v>25</v>
-      </c>
-      <c r="F185" t="s">
-        <v>46</v>
-      </c>
-      <c r="J185" t="s">
-        <v>18</v>
-      </c>
-      <c r="K185" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F185,'feed pars'!B$6:B$43,0))</f>
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K184" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A185" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="B185" s="7"/>
+      <c r="C185" s="6"/>
+      <c r="D185" s="6"/>
+      <c r="E185" s="6"/>
+      <c r="F185" s="6"/>
+      <c r="G185" s="6"/>
+      <c r="H185" s="6"/>
+      <c r="I185" s="6"/>
+      <c r="J185" s="6"/>
+      <c r="K185" s="6"/>
+      <c r="L185" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M185" s="6"/>
+      <c r="N185" s="6"/>
+    </row>
+    <row r="186" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>25</v>
+        <v>395</v>
       </c>
       <c r="F186" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="J186" t="s">
         <v>18</v>
       </c>
-      <c r="K186" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F186,'feed pars'!B$6:B$43,0))</f>
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K186" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="187" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>25</v>
+        <v>395</v>
       </c>
       <c r="F187" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="J187" t="s">
         <v>18</v>
       </c>
-      <c r="K187" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F187,'feed pars'!B$6:B$43,0))</f>
-        <v>7.2</v>
-      </c>
-    </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A188" t="s">
-        <v>25</v>
-      </c>
-      <c r="F188" t="s">
-        <v>49</v>
-      </c>
-      <c r="J188" t="s">
-        <v>18</v>
-      </c>
-      <c r="K188" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F188,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
-      </c>
-    </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A189" t="s">
-        <v>25</v>
-      </c>
-      <c r="F189" t="s">
-        <v>50</v>
-      </c>
-      <c r="J189" t="s">
-        <v>18</v>
-      </c>
-      <c r="K189" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F189,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1</v>
-      </c>
-    </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K187" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="188" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A188" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B188" s="8"/>
+      <c r="C188" s="9"/>
+      <c r="D188" s="9"/>
+      <c r="E188" s="9"/>
+      <c r="F188" s="9"/>
+      <c r="G188" s="9"/>
+      <c r="H188" s="9"/>
+      <c r="I188" s="9"/>
+      <c r="J188" s="9"/>
+      <c r="K188" s="9"/>
+      <c r="L188" s="9"/>
+      <c r="M188" s="9"/>
+      <c r="N188" s="9"/>
+    </row>
+    <row r="189" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A189" s="30" t="s">
+        <v>391</v>
+      </c>
+      <c r="B189" s="31"/>
+      <c r="C189" s="32"/>
+      <c r="D189" s="32"/>
+      <c r="E189" s="32"/>
+      <c r="F189" s="32"/>
+      <c r="G189" s="32"/>
+      <c r="H189" s="32"/>
+      <c r="I189" s="32"/>
+      <c r="J189" s="32"/>
+      <c r="K189" s="32"/>
+      <c r="L189" s="32" t="s">
+        <v>300</v>
+      </c>
+      <c r="M189" s="32"/>
+      <c r="N189" s="32"/>
+    </row>
+    <row r="190" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>25</v>
       </c>
+      <c r="E190" t="s">
+        <v>299</v>
+      </c>
       <c r="F190" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="J190" t="s">
         <v>18</v>
       </c>
       <c r="K190" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F190,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1999999999999993</v>
-      </c>
-    </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F190,'feed pars'!B$6:B$43,0))</f>
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="191" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>25</v>
       </c>
+      <c r="E191" t="s">
+        <v>299</v>
+      </c>
       <c r="F191" t="s">
-        <v>313</v>
+        <v>37</v>
       </c>
       <c r="J191" t="s">
         <v>18</v>
       </c>
       <c r="K191" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F191,'feed pars'!B$6:B$43,0))</f>
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F191,'feed pars'!B$6:B$43,0))</f>
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="192" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>25</v>
       </c>
+      <c r="E192" t="s">
+        <v>299</v>
+      </c>
       <c r="F192" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="J192" t="s">
         <v>18</v>
       </c>
       <c r="K192" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F192,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F192,'feed pars'!B$6:B$43,0))</f>
+        <v>9.4</v>
       </c>
     </row>
     <row r="193" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>25</v>
       </c>
+      <c r="E193" t="s">
+        <v>299</v>
+      </c>
       <c r="F193" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="J193" t="s">
         <v>18</v>
       </c>
       <c r="K193" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F193,'feed pars'!B$6:B$43,0))</f>
-        <v>6.9</v>
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F193,'feed pars'!B$6:B$43,0))</f>
+        <v>12</v>
       </c>
     </row>
     <row r="194" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>25</v>
       </c>
+      <c r="E194" t="s">
+        <v>299</v>
+      </c>
       <c r="F194" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="J194" t="s">
         <v>18</v>
       </c>
       <c r="K194" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F194,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F194,'feed pars'!B$6:B$43,0))</f>
+        <v>13.2</v>
       </c>
     </row>
     <row r="195" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>25</v>
       </c>
+      <c r="E195" t="s">
+        <v>299</v>
+      </c>
       <c r="F195" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="J195" t="s">
         <v>18</v>
       </c>
       <c r="K195" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F195,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F195,'feed pars'!B$6:B$43,0))</f>
+        <v>11.5</v>
       </c>
     </row>
     <row r="196" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>25</v>
       </c>
+      <c r="E196" t="s">
+        <v>299</v>
+      </c>
       <c r="F196" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="J196" t="s">
         <v>18</v>
       </c>
       <c r="K196" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F196,'feed pars'!B$6:B$43,0))</f>
-        <v>11.1</v>
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F196,'feed pars'!B$6:B$43,0))</f>
+        <v>10.9</v>
       </c>
     </row>
     <row r="197" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>25</v>
       </c>
+      <c r="E197" t="s">
+        <v>299</v>
+      </c>
       <c r="F197" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="J197" t="s">
         <v>18</v>
       </c>
       <c r="K197" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F197,'feed pars'!B$6:B$43,0))</f>
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F197,'feed pars'!B$6:B$43,0))</f>
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>25</v>
+      </c>
+      <c r="E198" t="s">
+        <v>299</v>
+      </c>
+      <c r="F198" t="s">
+        <v>43</v>
+      </c>
+      <c r="J198" t="s">
+        <v>18</v>
+      </c>
+      <c r="K198" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F198,'feed pars'!B$6:B$43,0))</f>
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>25</v>
+      </c>
+      <c r="E199" t="s">
+        <v>299</v>
+      </c>
+      <c r="F199" t="s">
+        <v>314</v>
+      </c>
+      <c r="J199" t="s">
+        <v>18</v>
+      </c>
+      <c r="K199" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F199,'feed pars'!B$6:B$43,0))</f>
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>25</v>
+      </c>
+      <c r="E200" t="s">
+        <v>299</v>
+      </c>
+      <c r="F200" t="s">
+        <v>44</v>
+      </c>
+      <c r="J200" t="s">
+        <v>18</v>
+      </c>
+      <c r="K200" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F200,'feed pars'!B$6:B$43,0))</f>
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>25</v>
+      </c>
+      <c r="E201" t="s">
+        <v>299</v>
+      </c>
+      <c r="F201" t="s">
+        <v>45</v>
+      </c>
+      <c r="J201" t="s">
+        <v>18</v>
+      </c>
+      <c r="K201" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F201,'feed pars'!B$6:B$43,0))</f>
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>25</v>
+      </c>
+      <c r="E202" t="s">
+        <v>299</v>
+      </c>
+      <c r="F202" t="s">
+        <v>36</v>
+      </c>
+      <c r="J202" t="s">
+        <v>18</v>
+      </c>
+      <c r="K202" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F202,'feed pars'!B$6:B$43,0))</f>
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>25</v>
+      </c>
+      <c r="E203" t="s">
+        <v>299</v>
+      </c>
+      <c r="F203" t="s">
+        <v>46</v>
+      </c>
+      <c r="J203" t="s">
+        <v>18</v>
+      </c>
+      <c r="K203" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F203,'feed pars'!B$6:B$43,0))</f>
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>25</v>
+      </c>
+      <c r="E204" t="s">
+        <v>299</v>
+      </c>
+      <c r="F204" t="s">
+        <v>47</v>
+      </c>
+      <c r="J204" t="s">
+        <v>18</v>
+      </c>
+      <c r="K204" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F204,'feed pars'!B$6:B$43,0))</f>
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>25</v>
+      </c>
+      <c r="E205" t="s">
+        <v>299</v>
+      </c>
+      <c r="F205" t="s">
+        <v>48</v>
+      </c>
+      <c r="J205" t="s">
+        <v>18</v>
+      </c>
+      <c r="K205" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F205,'feed pars'!B$6:B$43,0))</f>
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>25</v>
+      </c>
+      <c r="E206" t="s">
+        <v>299</v>
+      </c>
+      <c r="F206" t="s">
+        <v>49</v>
+      </c>
+      <c r="J206" t="s">
+        <v>18</v>
+      </c>
+      <c r="K206" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F206,'feed pars'!B$6:B$43,0))</f>
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>25</v>
+      </c>
+      <c r="E207" t="s">
+        <v>299</v>
+      </c>
+      <c r="F207" t="s">
+        <v>50</v>
+      </c>
+      <c r="J207" t="s">
+        <v>18</v>
+      </c>
+      <c r="K207" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F207,'feed pars'!B$6:B$43,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>25</v>
+      </c>
+      <c r="E208" t="s">
+        <v>299</v>
+      </c>
+      <c r="F208" t="s">
+        <v>51</v>
+      </c>
+      <c r="J208" t="s">
+        <v>18</v>
+      </c>
+      <c r="K208" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F208,'feed pars'!B$6:B$43,0))</f>
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="209" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>25</v>
+      </c>
+      <c r="E209" t="s">
+        <v>299</v>
+      </c>
+      <c r="F209" t="s">
+        <v>313</v>
+      </c>
+      <c r="J209" t="s">
+        <v>18</v>
+      </c>
+      <c r="K209" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F209,'feed pars'!B$6:B$43,0))</f>
+        <v>7.0888888888888877</v>
+      </c>
+    </row>
+    <row r="210" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>25</v>
+      </c>
+      <c r="E210" t="s">
+        <v>299</v>
+      </c>
+      <c r="F210" t="s">
+        <v>52</v>
+      </c>
+      <c r="J210" t="s">
+        <v>18</v>
+      </c>
+      <c r="K210" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F210,'feed pars'!B$6:B$43,0))</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="211" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>25</v>
+      </c>
+      <c r="E211" t="s">
+        <v>299</v>
+      </c>
+      <c r="F211" t="s">
+        <v>53</v>
+      </c>
+      <c r="J211" t="s">
+        <v>18</v>
+      </c>
+      <c r="K211" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F211,'feed pars'!B$6:B$43,0))</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="212" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>25</v>
+      </c>
+      <c r="E212" t="s">
+        <v>299</v>
+      </c>
+      <c r="F212" t="s">
+        <v>54</v>
+      </c>
+      <c r="J212" t="s">
+        <v>18</v>
+      </c>
+      <c r="K212" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F212,'feed pars'!B$6:B$43,0))</f>
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="213" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>25</v>
+      </c>
+      <c r="E213" t="s">
+        <v>299</v>
+      </c>
+      <c r="F213" t="s">
+        <v>55</v>
+      </c>
+      <c r="J213" t="s">
+        <v>18</v>
+      </c>
+      <c r="K213" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F213,'feed pars'!B$6:B$43,0))</f>
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="214" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>25</v>
+      </c>
+      <c r="E214" t="s">
+        <v>299</v>
+      </c>
+      <c r="F214" t="s">
+        <v>56</v>
+      </c>
+      <c r="J214" t="s">
+        <v>18</v>
+      </c>
+      <c r="K214" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F214,'feed pars'!B$6:B$43,0))</f>
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="215" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>25</v>
+      </c>
+      <c r="E215" t="s">
+        <v>299</v>
+      </c>
+      <c r="F215" t="s">
+        <v>57</v>
+      </c>
+      <c r="J215" t="s">
+        <v>18</v>
+      </c>
+      <c r="K215" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F215,'feed pars'!B$6:B$43,0))</f>
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="216" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A216" s="30" t="s">
+        <v>392</v>
+      </c>
+      <c r="B216" s="31"/>
+      <c r="C216" s="32"/>
+      <c r="D216" s="32"/>
+      <c r="E216" s="32"/>
+      <c r="F216" s="32"/>
+      <c r="G216" s="32"/>
+      <c r="H216" s="32"/>
+      <c r="I216" s="32"/>
+      <c r="J216" s="32"/>
+      <c r="K216" s="32"/>
+      <c r="L216" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="M216" s="32"/>
+      <c r="N216" s="32"/>
+    </row>
+    <row r="217" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>25</v>
+      </c>
+      <c r="F217" t="s">
+        <v>17</v>
+      </c>
+      <c r="J217" t="s">
+        <v>18</v>
+      </c>
+      <c r="K217" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F217,'feed pars'!B$6:B$43,0))</f>
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="218" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>25</v>
+      </c>
+      <c r="F218" t="s">
+        <v>37</v>
+      </c>
+      <c r="J218" t="s">
+        <v>18</v>
+      </c>
+      <c r="K218" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F218,'feed pars'!B$6:B$43,0))</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="219" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>25</v>
+      </c>
+      <c r="F219" t="s">
+        <v>38</v>
+      </c>
+      <c r="J219" t="s">
+        <v>18</v>
+      </c>
+      <c r="K219" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F219,'feed pars'!B$6:B$43,0))</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="220" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>25</v>
+      </c>
+      <c r="F220" t="s">
+        <v>39</v>
+      </c>
+      <c r="J220" t="s">
+        <v>18</v>
+      </c>
+      <c r="K220" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F220,'feed pars'!B$6:B$43,0))</f>
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="221" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>25</v>
+      </c>
+      <c r="F221" t="s">
+        <v>40</v>
+      </c>
+      <c r="J221" t="s">
+        <v>18</v>
+      </c>
+      <c r="K221" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F221,'feed pars'!B$6:B$43,0))</f>
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="222" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>25</v>
+      </c>
+      <c r="F222" t="s">
+        <v>41</v>
+      </c>
+      <c r="J222" t="s">
+        <v>18</v>
+      </c>
+      <c r="K222" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F222,'feed pars'!B$6:B$43,0))</f>
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="223" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>25</v>
+      </c>
+      <c r="F223" t="s">
+        <v>42</v>
+      </c>
+      <c r="J223" t="s">
+        <v>18</v>
+      </c>
+      <c r="K223" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F223,'feed pars'!B$6:B$43,0))</f>
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="224" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>25</v>
+      </c>
+      <c r="F224" t="s">
+        <v>35</v>
+      </c>
+      <c r="J224" t="s">
+        <v>18</v>
+      </c>
+      <c r="K224" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F224,'feed pars'!B$6:B$43,0))</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="225" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>25</v>
+      </c>
+      <c r="F225" t="s">
+        <v>43</v>
+      </c>
+      <c r="J225" t="s">
+        <v>18</v>
+      </c>
+      <c r="K225" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F225,'feed pars'!B$6:B$43,0))</f>
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="226" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>25</v>
+      </c>
+      <c r="F226" t="s">
+        <v>314</v>
+      </c>
+      <c r="J226" t="s">
+        <v>18</v>
+      </c>
+      <c r="K226" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F226,'feed pars'!B$6:B$43,0))</f>
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="227" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>25</v>
+      </c>
+      <c r="F227" t="s">
+        <v>44</v>
+      </c>
+      <c r="J227" t="s">
+        <v>18</v>
+      </c>
+      <c r="K227" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F227,'feed pars'!B$6:B$43,0))</f>
+        <v>9.3000000000000007</v>
+      </c>
+    </row>
+    <row r="228" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>25</v>
+      </c>
+      <c r="F228" t="s">
+        <v>45</v>
+      </c>
+      <c r="J228" t="s">
+        <v>18</v>
+      </c>
+      <c r="K228" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F228,'feed pars'!B$6:B$43,0))</f>
+        <v>9.6999999999999993</v>
+      </c>
+    </row>
+    <row r="229" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>25</v>
+      </c>
+      <c r="F229" t="s">
+        <v>36</v>
+      </c>
+      <c r="J229" t="s">
+        <v>18</v>
+      </c>
+      <c r="K229" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F229,'feed pars'!B$6:B$43,0))</f>
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="230" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>25</v>
+      </c>
+      <c r="F230" t="s">
+        <v>46</v>
+      </c>
+      <c r="J230" t="s">
+        <v>18</v>
+      </c>
+      <c r="K230" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F230,'feed pars'!B$6:B$43,0))</f>
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="231" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>25</v>
+      </c>
+      <c r="F231" t="s">
+        <v>47</v>
+      </c>
+      <c r="J231" t="s">
+        <v>18</v>
+      </c>
+      <c r="K231" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F231,'feed pars'!B$6:B$43,0))</f>
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="232" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>25</v>
+      </c>
+      <c r="F232" t="s">
+        <v>48</v>
+      </c>
+      <c r="J232" t="s">
+        <v>18</v>
+      </c>
+      <c r="K232" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F232,'feed pars'!B$6:B$43,0))</f>
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="233" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>25</v>
+      </c>
+      <c r="F233" t="s">
+        <v>49</v>
+      </c>
+      <c r="J233" t="s">
+        <v>18</v>
+      </c>
+      <c r="K233" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F233,'feed pars'!B$6:B$43,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="234" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
+        <v>25</v>
+      </c>
+      <c r="F234" t="s">
+        <v>50</v>
+      </c>
+      <c r="J234" t="s">
+        <v>18</v>
+      </c>
+      <c r="K234" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F234,'feed pars'!B$6:B$43,0))</f>
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="235" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>25</v>
+      </c>
+      <c r="F235" t="s">
+        <v>51</v>
+      </c>
+      <c r="J235" t="s">
+        <v>18</v>
+      </c>
+      <c r="K235" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F235,'feed pars'!B$6:B$43,0))</f>
+        <v>8.1999999999999993</v>
+      </c>
+    </row>
+    <row r="236" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>25</v>
+      </c>
+      <c r="F236" t="s">
+        <v>313</v>
+      </c>
+      <c r="J236" t="s">
+        <v>18</v>
+      </c>
+      <c r="K236" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F236,'feed pars'!B$6:B$43,0))</f>
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="237" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>25</v>
+      </c>
+      <c r="F237" t="s">
+        <v>52</v>
+      </c>
+      <c r="J237" t="s">
+        <v>18</v>
+      </c>
+      <c r="K237" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F237,'feed pars'!B$6:B$43,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="238" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
+        <v>25</v>
+      </c>
+      <c r="F238" t="s">
+        <v>53</v>
+      </c>
+      <c r="J238" t="s">
+        <v>18</v>
+      </c>
+      <c r="K238" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F238,'feed pars'!B$6:B$43,0))</f>
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="239" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>25</v>
+      </c>
+      <c r="F239" t="s">
+        <v>54</v>
+      </c>
+      <c r="J239" t="s">
+        <v>18</v>
+      </c>
+      <c r="K239" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F239,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="240" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>25</v>
+      </c>
+      <c r="F240" t="s">
+        <v>55</v>
+      </c>
+      <c r="J240" t="s">
+        <v>18</v>
+      </c>
+      <c r="K240" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F240,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="241" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>25</v>
+      </c>
+      <c r="F241" t="s">
+        <v>56</v>
+      </c>
+      <c r="J241" t="s">
+        <v>18</v>
+      </c>
+      <c r="K241" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F241,'feed pars'!B$6:B$43,0))</f>
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="242" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>25</v>
+      </c>
+      <c r="F242" t="s">
+        <v>57</v>
+      </c>
+      <c r="J242" t="s">
+        <v>18</v>
+      </c>
+      <c r="K242" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F242,'feed pars'!B$6:B$43,0))</f>
         <v>10.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added concentrates to horse rations
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FeedMgmt.xlsx
+++ b/data/prod_parameters/FeedMgmt.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1243" uniqueCount="411">
   <si>
     <t>f_feed</t>
   </si>
@@ -1225,9 +1225,6 @@
     <t>horses</t>
   </si>
   <si>
-    <t>Horses</t>
-  </si>
-  <si>
     <t>storage_losses</t>
   </si>
   <si>
@@ -1265,6 +1262,25 @@
   </si>
   <si>
     <t>No storage</t>
+  </si>
+  <si>
+    <r>
+      <t>Horses</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Assume same as cattle for now)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://glw-feeds.co.uk/index.php/wheat-feed-2/</t>
   </si>
 </sst>
 </file>
@@ -1274,7 +1290,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1343,6 +1359,14 @@
     <font>
       <sz val="11"/>
       <color theme="2" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1417,7 +1441,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1468,6 +1492,7 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1749,7 +1774,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O242"/>
+  <dimension ref="A1:O254"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -2263,7 +2288,7 @@
       </c>
       <c r="K31" s="22">
         <f>1/INDEX('feed pars'!C$6:C$43/100,MATCH(F31,'feed pars'!B$6:B$43,0))</f>
-        <v>1.1363636363636365</v>
+        <v>1.1299435028248588</v>
       </c>
     </row>
     <row r="32" spans="6:13" x14ac:dyDescent="0.25">
@@ -2950,7 +2975,7 @@
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -2968,7 +2993,7 @@
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J69" s="10" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K69" s="10">
         <v>0</v>
@@ -2982,7 +3007,7 @@
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J70" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K70" s="10">
         <v>0</v>
@@ -3008,7 +3033,7 @@
         <v>310</v>
       </c>
       <c r="J71" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K71" s="29">
         <f>(0.8*20+0.2*2)</f>
@@ -3018,10 +3043,10 @@
         <v>28</v>
       </c>
       <c r="M71" s="29" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="N71" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
@@ -3032,7 +3057,7 @@
         <v>310</v>
       </c>
       <c r="J72" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K72" s="29">
         <f>(0.6*20+0.4*2)</f>
@@ -3042,21 +3067,21 @@
         <v>28</v>
       </c>
       <c r="M72" s="29" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="N72" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F73" t="s">
         <v>310</v>
       </c>
       <c r="J73" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K73" s="29">
         <v>2</v>
@@ -3065,10 +3090,10 @@
         <v>28</v>
       </c>
       <c r="M73" s="29" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="N73" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">
@@ -3079,7 +3104,7 @@
         <v>310</v>
       </c>
       <c r="J74" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K74" s="29">
         <v>2</v>
@@ -3088,10 +3113,10 @@
         <v>28</v>
       </c>
       <c r="M74" s="29" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="N74" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
@@ -3108,7 +3133,7 @@
         <v>310</v>
       </c>
       <c r="J75" s="29" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K75" s="29">
         <v>5</v>
@@ -3117,10 +3142,10 @@
         <v>28</v>
       </c>
       <c r="M75" s="29" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="N75" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
@@ -3134,7 +3159,7 @@
         <v>310</v>
       </c>
       <c r="J76" s="29" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K76" s="29">
         <v>5</v>
@@ -3143,10 +3168,10 @@
         <v>28</v>
       </c>
       <c r="M76" s="29" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="N76" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.25">
@@ -3157,7 +3182,7 @@
         <v>310</v>
       </c>
       <c r="J77" s="29" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K77" s="29">
         <f>0.9*5+0.1*15</f>
@@ -3167,21 +3192,21 @@
         <v>28</v>
       </c>
       <c r="M77" s="29" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="N77" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F78" t="s">
         <v>310</v>
       </c>
       <c r="J78" s="29" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K78" s="29">
         <v>15</v>
@@ -3191,7 +3216,7 @@
       </c>
       <c r="M78" s="29"/>
       <c r="N78" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.25">
@@ -3202,7 +3227,7 @@
         <v>310</v>
       </c>
       <c r="J79" s="29" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K79" s="29">
         <v>15</v>
@@ -3212,7 +3237,7 @@
       </c>
       <c r="M79" s="29"/>
       <c r="N79" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.25">
@@ -3498,7 +3523,7 @@
         <v>312</v>
       </c>
       <c r="J89" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K89" s="29">
         <v>5</v>
@@ -3508,7 +3533,7 @@
       </c>
       <c r="M89" s="29"/>
       <c r="N89" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
@@ -3667,7 +3692,7 @@
         <v>2</v>
       </c>
       <c r="J95" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K95" s="29">
         <v>5</v>
@@ -3677,7 +3702,7 @@
       </c>
       <c r="M95" s="29"/>
       <c r="N95" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.25">
@@ -3836,7 +3861,7 @@
         <v>12</v>
       </c>
       <c r="J101" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K101" s="29">
         <v>5</v>
@@ -3846,7 +3871,7 @@
       </c>
       <c r="M101" s="29"/>
       <c r="N101" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.25">
@@ -4006,7 +4031,7 @@
         <v>33</v>
       </c>
       <c r="J107" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K107" s="29">
         <v>0</v>
@@ -4015,7 +4040,7 @@
         <v>28</v>
       </c>
       <c r="M107" s="29" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="N107" s="33"/>
     </row>
@@ -4027,7 +4052,7 @@
         <v>33</v>
       </c>
       <c r="J108" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K108" s="29">
         <f>100-55</f>
@@ -4037,10 +4062,10 @@
         <v>28</v>
       </c>
       <c r="M108" s="29" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="N108" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.25">
@@ -4051,7 +4076,7 @@
         <v>33</v>
       </c>
       <c r="J109" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K109" s="29">
         <f>100-50</f>
@@ -4061,10 +4086,10 @@
         <v>28</v>
       </c>
       <c r="M109" s="29" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="N109" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="110" spans="1:14" x14ac:dyDescent="0.25">
@@ -4073,7 +4098,7 @@
     </row>
     <row r="111" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="K111" s="3"/>
       <c r="M111" s="29"/>
@@ -4533,7 +4558,7 @@
       </c>
       <c r="K141" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F141,'feed pars'!B$6:B$43,0))</f>
-        <v>88</v>
+        <v>88.5</v>
       </c>
       <c r="L141" t="s">
         <v>28</v>
@@ -5192,7 +5217,7 @@
     </row>
     <row r="185" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A185" s="7" t="s">
-        <v>396</v>
+        <v>409</v>
       </c>
       <c r="B185" s="7"/>
       <c r="C185" s="6"/>
@@ -5220,8 +5245,9 @@
       <c r="J186" t="s">
         <v>18</v>
       </c>
-      <c r="K186" s="3">
-        <v>10</v>
+      <c r="K186" s="26">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F186,'feed pars'!B$6:B$43,0))</f>
+        <v>9.1</v>
       </c>
     </row>
     <row r="187" spans="1:14" x14ac:dyDescent="0.25">
@@ -5234,265 +5260,206 @@
       <c r="J187" t="s">
         <v>18</v>
       </c>
-      <c r="K187" s="3">
+      <c r="K187" s="34">
+        <f>K157</f>
         <v>10</v>
       </c>
     </row>
     <row r="188" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A188" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B188" s="8"/>
-      <c r="C188" s="9"/>
-      <c r="D188" s="9"/>
-      <c r="E188" s="9"/>
-      <c r="F188" s="9"/>
-      <c r="G188" s="9"/>
-      <c r="H188" s="9"/>
-      <c r="I188" s="9"/>
-      <c r="J188" s="9"/>
-      <c r="K188" s="9"/>
-      <c r="L188" s="9"/>
-      <c r="M188" s="9"/>
-      <c r="N188" s="9"/>
+      <c r="K188" s="34"/>
     </row>
     <row r="189" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A189" s="30" t="s">
-        <v>391</v>
-      </c>
-      <c r="B189" s="31"/>
-      <c r="C189" s="32"/>
-      <c r="D189" s="32"/>
-      <c r="E189" s="32"/>
-      <c r="F189" s="32"/>
-      <c r="G189" s="32"/>
-      <c r="H189" s="32"/>
-      <c r="I189" s="32"/>
-      <c r="J189" s="32"/>
-      <c r="K189" s="32"/>
-      <c r="L189" s="32" t="s">
-        <v>300</v>
-      </c>
-      <c r="M189" s="32"/>
-      <c r="N189" s="32"/>
+      <c r="A189" t="s">
+        <v>395</v>
+      </c>
+      <c r="F189" t="s">
+        <v>38</v>
+      </c>
+      <c r="J189" t="s">
+        <v>18</v>
+      </c>
+      <c r="K189" s="34">
+        <f>K161</f>
+        <v>11.7</v>
+      </c>
     </row>
     <row r="190" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>25</v>
-      </c>
-      <c r="E190" t="s">
-        <v>299</v>
+        <v>395</v>
       </c>
       <c r="F190" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="J190" t="s">
         <v>18</v>
       </c>
-      <c r="K190" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F190,'feed pars'!B$6:B$43,0))</f>
-        <v>12.3</v>
+      <c r="K190" s="34">
+        <f>K160</f>
+        <v>13.2</v>
       </c>
     </row>
     <row r="191" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>25</v>
-      </c>
-      <c r="E191" t="s">
-        <v>299</v>
+        <v>395</v>
       </c>
       <c r="F191" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="J191" t="s">
         <v>18</v>
       </c>
-      <c r="K191" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F191,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
+      <c r="K191" s="34">
+        <f>K159</f>
+        <v>14.1</v>
       </c>
     </row>
     <row r="192" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>25</v>
-      </c>
-      <c r="E192" t="s">
-        <v>299</v>
+        <v>395</v>
       </c>
       <c r="F192" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="J192" t="s">
         <v>18</v>
       </c>
-      <c r="K192" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F192,'feed pars'!B$6:B$43,0))</f>
-        <v>9.4</v>
-      </c>
-    </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K192" s="34">
+        <f t="shared" ref="K192:K198" si="14">K160</f>
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="193" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>25</v>
-      </c>
-      <c r="E193" t="s">
-        <v>299</v>
+        <v>395</v>
       </c>
       <c r="F193" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="J193" t="s">
         <v>18</v>
       </c>
-      <c r="K193" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F193,'feed pars'!B$6:B$43,0))</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K193" s="34">
+        <f t="shared" si="14"/>
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="194" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>25</v>
-      </c>
-      <c r="E194" t="s">
-        <v>299</v>
+        <v>395</v>
       </c>
       <c r="F194" t="s">
-        <v>40</v>
+        <v>314</v>
       </c>
       <c r="J194" t="s">
         <v>18</v>
       </c>
-      <c r="K194" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F194,'feed pars'!B$6:B$43,0))</f>
-        <v>13.2</v>
-      </c>
-    </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K194" s="34">
+        <f t="shared" si="14"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="195" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>25</v>
-      </c>
-      <c r="E195" t="s">
-        <v>299</v>
+        <v>395</v>
       </c>
       <c r="F195" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="J195" t="s">
         <v>18</v>
       </c>
-      <c r="K195" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F195,'feed pars'!B$6:B$43,0))</f>
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K195" s="34">
+        <f t="shared" si="14"/>
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="196" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>25</v>
-      </c>
-      <c r="E196" t="s">
-        <v>299</v>
+        <v>395</v>
       </c>
       <c r="F196" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="J196" t="s">
         <v>18</v>
       </c>
-      <c r="K196" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F196,'feed pars'!B$6:B$43,0))</f>
-        <v>10.9</v>
-      </c>
-    </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K196" s="34">
+        <f t="shared" si="14"/>
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="197" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>25</v>
-      </c>
-      <c r="E197" t="s">
-        <v>299</v>
+        <v>395</v>
       </c>
       <c r="F197" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="J197" t="s">
         <v>18</v>
       </c>
-      <c r="K197" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F197,'feed pars'!B$6:B$43,0))</f>
-        <v>18.5</v>
-      </c>
-    </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K197" s="34">
+        <f t="shared" si="14"/>
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="198" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>25</v>
-      </c>
-      <c r="E198" t="s">
-        <v>299</v>
+        <v>395</v>
       </c>
       <c r="F198" t="s">
-        <v>43</v>
+        <v>319</v>
       </c>
       <c r="J198" t="s">
         <v>18</v>
       </c>
-      <c r="K198" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F198,'feed pars'!B$6:B$43,0))</f>
-        <v>17.5</v>
-      </c>
-    </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A199" t="s">
-        <v>25</v>
-      </c>
-      <c r="E199" t="s">
-        <v>299</v>
-      </c>
-      <c r="F199" t="s">
-        <v>314</v>
-      </c>
-      <c r="J199" t="s">
-        <v>18</v>
-      </c>
-      <c r="K199" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F199,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
-      </c>
-    </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A200" t="s">
-        <v>25</v>
-      </c>
-      <c r="E200" t="s">
-        <v>299</v>
-      </c>
-      <c r="F200" t="s">
-        <v>44</v>
-      </c>
-      <c r="J200" t="s">
-        <v>18</v>
-      </c>
-      <c r="K200" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F200,'feed pars'!B$6:B$43,0))</f>
-        <v>9.9</v>
-      </c>
-    </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A201" t="s">
-        <v>25</v>
-      </c>
-      <c r="E201" t="s">
-        <v>299</v>
-      </c>
-      <c r="F201" t="s">
-        <v>45</v>
-      </c>
-      <c r="J201" t="s">
-        <v>18</v>
-      </c>
-      <c r="K201" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F201,'feed pars'!B$6:B$43,0))</f>
-        <v>10.3</v>
-      </c>
-    </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K198" s="34">
+        <f t="shared" si="14"/>
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="199" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K199" s="3"/>
+    </row>
+    <row r="200" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A200" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B200" s="8"/>
+      <c r="C200" s="9"/>
+      <c r="D200" s="9"/>
+      <c r="E200" s="9"/>
+      <c r="F200" s="9"/>
+      <c r="G200" s="9"/>
+      <c r="H200" s="9"/>
+      <c r="I200" s="9"/>
+      <c r="J200" s="9"/>
+      <c r="K200" s="9"/>
+      <c r="L200" s="9"/>
+      <c r="M200" s="9"/>
+      <c r="N200" s="9"/>
+    </row>
+    <row r="201" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A201" s="30" t="s">
+        <v>391</v>
+      </c>
+      <c r="B201" s="31"/>
+      <c r="C201" s="32"/>
+      <c r="D201" s="32"/>
+      <c r="E201" s="32"/>
+      <c r="F201" s="32"/>
+      <c r="G201" s="32"/>
+      <c r="H201" s="32"/>
+      <c r="I201" s="32"/>
+      <c r="J201" s="32"/>
+      <c r="K201" s="32"/>
+      <c r="L201" s="32" t="s">
+        <v>300</v>
+      </c>
+      <c r="M201" s="32"/>
+      <c r="N201" s="32"/>
+    </row>
+    <row r="202" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>25</v>
       </c>
@@ -5500,17 +5467,17 @@
         <v>299</v>
       </c>
       <c r="F202" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="J202" t="s">
         <v>18</v>
       </c>
       <c r="K202" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F202,'feed pars'!B$6:B$43,0))</f>
-        <v>7.7</v>
-      </c>
-    </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="203" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>25</v>
       </c>
@@ -5518,17 +5485,17 @@
         <v>299</v>
       </c>
       <c r="F203" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="J203" t="s">
         <v>18</v>
       </c>
       <c r="K203" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F203,'feed pars'!B$6:B$43,0))</f>
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="204" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>25</v>
       </c>
@@ -5536,17 +5503,17 @@
         <v>299</v>
       </c>
       <c r="F204" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="J204" t="s">
         <v>18</v>
       </c>
       <c r="K204" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F204,'feed pars'!B$6:B$43,0))</f>
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="205" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>25</v>
       </c>
@@ -5554,17 +5521,17 @@
         <v>299</v>
       </c>
       <c r="F205" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="J205" t="s">
         <v>18</v>
       </c>
       <c r="K205" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F205,'feed pars'!B$6:B$43,0))</f>
-        <v>7.8</v>
-      </c>
-    </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="206" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>25</v>
       </c>
@@ -5572,17 +5539,17 @@
         <v>299</v>
       </c>
       <c r="F206" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="J206" t="s">
         <v>18</v>
       </c>
       <c r="K206" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F206,'feed pars'!B$6:B$43,0))</f>
-        <v>9.1999999999999993</v>
-      </c>
-    </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="207" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>25</v>
       </c>
@@ -5590,17 +5557,17 @@
         <v>299</v>
       </c>
       <c r="F207" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="J207" t="s">
         <v>18</v>
       </c>
       <c r="K207" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F207,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
-      </c>
-    </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="208" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>25</v>
       </c>
@@ -5608,17 +5575,17 @@
         <v>299</v>
       </c>
       <c r="F208" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="J208" t="s">
         <v>18</v>
       </c>
       <c r="K208" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F208,'feed pars'!B$6:B$43,0))</f>
-        <v>8.9</v>
-      </c>
-    </row>
-    <row r="209" spans="1:14" x14ac:dyDescent="0.25">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="209" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>25</v>
       </c>
@@ -5626,17 +5593,17 @@
         <v>299</v>
       </c>
       <c r="F209" t="s">
-        <v>313</v>
+        <v>35</v>
       </c>
       <c r="J209" t="s">
         <v>18</v>
       </c>
       <c r="K209" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F209,'feed pars'!B$6:B$43,0))</f>
-        <v>7.0888888888888877</v>
-      </c>
-    </row>
-    <row r="210" spans="1:14" x14ac:dyDescent="0.25">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="210" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>25</v>
       </c>
@@ -5644,17 +5611,17 @@
         <v>299</v>
       </c>
       <c r="F210" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="J210" t="s">
         <v>18</v>
       </c>
       <c r="K210" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F210,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="211" spans="1:14" x14ac:dyDescent="0.25">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="211" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>25</v>
       </c>
@@ -5662,17 +5629,17 @@
         <v>299</v>
       </c>
       <c r="F211" t="s">
-        <v>53</v>
+        <v>314</v>
       </c>
       <c r="J211" t="s">
         <v>18</v>
       </c>
       <c r="K211" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F211,'feed pars'!B$6:B$43,0))</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="212" spans="1:14" x14ac:dyDescent="0.25">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="212" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>25</v>
       </c>
@@ -5680,17 +5647,17 @@
         <v>299</v>
       </c>
       <c r="F212" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="J212" t="s">
         <v>18</v>
       </c>
       <c r="K212" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F212,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="213" spans="1:14" x14ac:dyDescent="0.25">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="213" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>25</v>
       </c>
@@ -5698,17 +5665,17 @@
         <v>299</v>
       </c>
       <c r="F213" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="J213" t="s">
         <v>18</v>
       </c>
       <c r="K213" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F213,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="214" spans="1:14" x14ac:dyDescent="0.25">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="214" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>25</v>
       </c>
@@ -5716,17 +5683,17 @@
         <v>299</v>
       </c>
       <c r="F214" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="J214" t="s">
         <v>18</v>
       </c>
       <c r="K214" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F214,'feed pars'!B$6:B$43,0))</f>
-        <v>11.3</v>
-      </c>
-    </row>
-    <row r="215" spans="1:14" x14ac:dyDescent="0.25">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="215" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>25</v>
       </c>
@@ -5734,394 +5701,430 @@
         <v>299</v>
       </c>
       <c r="F215" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="J215" t="s">
         <v>18</v>
       </c>
       <c r="K215" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F215,'feed pars'!B$6:B$43,0))</f>
-        <v>10.8</v>
-      </c>
-    </row>
-    <row r="216" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A216" s="30" t="s">
-        <v>392</v>
-      </c>
-      <c r="B216" s="31"/>
-      <c r="C216" s="32"/>
-      <c r="D216" s="32"/>
-      <c r="E216" s="32"/>
-      <c r="F216" s="32"/>
-      <c r="G216" s="32"/>
-      <c r="H216" s="32"/>
-      <c r="I216" s="32"/>
-      <c r="J216" s="32"/>
-      <c r="K216" s="32"/>
-      <c r="L216" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="M216" s="32"/>
-      <c r="N216" s="32"/>
-    </row>
-    <row r="217" spans="1:14" x14ac:dyDescent="0.25">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="216" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>25</v>
+      </c>
+      <c r="E216" t="s">
+        <v>299</v>
+      </c>
+      <c r="F216" t="s">
+        <v>47</v>
+      </c>
+      <c r="J216" t="s">
+        <v>18</v>
+      </c>
+      <c r="K216" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F216,'feed pars'!B$6:B$43,0))</f>
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="217" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>25</v>
       </c>
+      <c r="E217" t="s">
+        <v>299</v>
+      </c>
       <c r="F217" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="J217" t="s">
         <v>18</v>
       </c>
       <c r="K217" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F217,'feed pars'!B$6:B$43,0))</f>
-        <v>12.1</v>
-      </c>
-    </row>
-    <row r="218" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F217,'feed pars'!B$6:B$43,0))</f>
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="218" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>25</v>
       </c>
+      <c r="E218" t="s">
+        <v>299</v>
+      </c>
       <c r="F218" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="J218" t="s">
         <v>18</v>
       </c>
       <c r="K218" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F218,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="219" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F218,'feed pars'!B$6:B$43,0))</f>
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="219" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>25</v>
       </c>
+      <c r="E219" t="s">
+        <v>299</v>
+      </c>
       <c r="F219" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="J219" t="s">
         <v>18</v>
       </c>
       <c r="K219" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F219,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="220" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F219,'feed pars'!B$6:B$43,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="220" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>25</v>
       </c>
+      <c r="E220" t="s">
+        <v>299</v>
+      </c>
       <c r="F220" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="J220" t="s">
         <v>18</v>
       </c>
       <c r="K220" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F220,'feed pars'!B$6:B$43,0))</f>
-        <v>11.9</v>
-      </c>
-    </row>
-    <row r="221" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F220,'feed pars'!B$6:B$43,0))</f>
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="221" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>25</v>
       </c>
+      <c r="E221" t="s">
+        <v>299</v>
+      </c>
       <c r="F221" t="s">
-        <v>40</v>
+        <v>313</v>
       </c>
       <c r="J221" t="s">
         <v>18</v>
       </c>
       <c r="K221" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F221,'feed pars'!B$6:B$43,0))</f>
-        <v>12.8</v>
-      </c>
-    </row>
-    <row r="222" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F221,'feed pars'!B$6:B$43,0))</f>
+        <v>7.0888888888888877</v>
+      </c>
+    </row>
+    <row r="222" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>25</v>
       </c>
+      <c r="E222" t="s">
+        <v>299</v>
+      </c>
       <c r="F222" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="J222" t="s">
         <v>18</v>
       </c>
       <c r="K222" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F222,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
-      </c>
-    </row>
-    <row r="223" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F222,'feed pars'!B$6:B$43,0))</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="223" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>25</v>
       </c>
+      <c r="E223" t="s">
+        <v>299</v>
+      </c>
       <c r="F223" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="J223" t="s">
         <v>18</v>
       </c>
       <c r="K223" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F223,'feed pars'!B$6:B$43,0))</f>
-        <v>10.7</v>
-      </c>
-    </row>
-    <row r="224" spans="1:14" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F223,'feed pars'!B$6:B$43,0))</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="224" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>25</v>
       </c>
+      <c r="E224" t="s">
+        <v>299</v>
+      </c>
       <c r="F224" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="J224" t="s">
         <v>18</v>
       </c>
       <c r="K224" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F224,'feed pars'!B$6:B$43,0))</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="225" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F224,'feed pars'!B$6:B$43,0))</f>
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="225" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>25</v>
       </c>
+      <c r="E225" t="s">
+        <v>299</v>
+      </c>
       <c r="F225" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="J225" t="s">
         <v>18</v>
       </c>
       <c r="K225" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F225,'feed pars'!B$6:B$43,0))</f>
-        <v>17.3</v>
-      </c>
-    </row>
-    <row r="226" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F225,'feed pars'!B$6:B$43,0))</f>
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="226" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>25</v>
       </c>
+      <c r="E226" t="s">
+        <v>299</v>
+      </c>
       <c r="F226" t="s">
-        <v>314</v>
+        <v>56</v>
       </c>
       <c r="J226" t="s">
         <v>18</v>
       </c>
       <c r="K226" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F226,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
-      </c>
-    </row>
-    <row r="227" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F226,'feed pars'!B$6:B$43,0))</f>
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="227" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>25</v>
       </c>
+      <c r="E227" t="s">
+        <v>299</v>
+      </c>
       <c r="F227" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="J227" t="s">
         <v>18</v>
       </c>
       <c r="K227" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F227,'feed pars'!B$6:B$43,0))</f>
-        <v>9.3000000000000007</v>
-      </c>
-    </row>
-    <row r="228" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A228" t="s">
-        <v>25</v>
-      </c>
-      <c r="F228" t="s">
-        <v>45</v>
-      </c>
-      <c r="J228" t="s">
-        <v>18</v>
-      </c>
-      <c r="K228" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F228,'feed pars'!B$6:B$43,0))</f>
-        <v>9.6999999999999993</v>
-      </c>
-    </row>
-    <row r="229" spans="1:11" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F227,'feed pars'!B$6:B$43,0))</f>
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="228" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A228" s="30" t="s">
+        <v>392</v>
+      </c>
+      <c r="B228" s="31"/>
+      <c r="C228" s="32"/>
+      <c r="D228" s="32"/>
+      <c r="E228" s="32"/>
+      <c r="F228" s="32"/>
+      <c r="G228" s="32"/>
+      <c r="H228" s="32"/>
+      <c r="I228" s="32"/>
+      <c r="J228" s="32"/>
+      <c r="K228" s="32"/>
+      <c r="L228" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="M228" s="32"/>
+      <c r="N228" s="32"/>
+    </row>
+    <row r="229" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>25</v>
       </c>
       <c r="F229" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="J229" t="s">
         <v>18</v>
       </c>
       <c r="K229" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F229,'feed pars'!B$6:B$43,0))</f>
-        <v>7.1</v>
-      </c>
-    </row>
-    <row r="230" spans="1:11" x14ac:dyDescent="0.25">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="230" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>25</v>
       </c>
       <c r="F230" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="J230" t="s">
         <v>18</v>
       </c>
       <c r="K230" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F230,'feed pars'!B$6:B$43,0))</f>
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="231" spans="1:11" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="231" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>25</v>
       </c>
       <c r="F231" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="J231" t="s">
         <v>18</v>
       </c>
       <c r="K231" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F231,'feed pars'!B$6:B$43,0))</f>
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="232" spans="1:11" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="232" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>25</v>
       </c>
       <c r="F232" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="J232" t="s">
         <v>18</v>
       </c>
       <c r="K232" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F232,'feed pars'!B$6:B$43,0))</f>
-        <v>7.2</v>
-      </c>
-    </row>
-    <row r="233" spans="1:11" x14ac:dyDescent="0.25">
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="233" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>25</v>
       </c>
       <c r="F233" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="J233" t="s">
         <v>18</v>
       </c>
       <c r="K233" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F233,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
-      </c>
-    </row>
-    <row r="234" spans="1:11" x14ac:dyDescent="0.25">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="234" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>25</v>
       </c>
       <c r="F234" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="J234" t="s">
         <v>18</v>
       </c>
       <c r="K234" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F234,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1</v>
-      </c>
-    </row>
-    <row r="235" spans="1:11" x14ac:dyDescent="0.25">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="235" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>25</v>
       </c>
       <c r="F235" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="J235" t="s">
         <v>18</v>
       </c>
       <c r="K235" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F235,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1999999999999993</v>
-      </c>
-    </row>
-    <row r="236" spans="1:11" x14ac:dyDescent="0.25">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="236" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>25</v>
       </c>
       <c r="F236" t="s">
-        <v>313</v>
+        <v>35</v>
       </c>
       <c r="J236" t="s">
         <v>18</v>
       </c>
       <c r="K236" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F236,'feed pars'!B$6:B$43,0))</f>
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="237" spans="1:11" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="237" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>25</v>
       </c>
       <c r="F237" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="J237" t="s">
         <v>18</v>
       </c>
       <c r="K237" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F237,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
-      </c>
-    </row>
-    <row r="238" spans="1:11" x14ac:dyDescent="0.25">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="238" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>25</v>
       </c>
       <c r="F238" t="s">
-        <v>53</v>
+        <v>314</v>
       </c>
       <c r="J238" t="s">
         <v>18</v>
       </c>
       <c r="K238" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F238,'feed pars'!B$6:B$43,0))</f>
-        <v>6.9</v>
-      </c>
-    </row>
-    <row r="239" spans="1:11" x14ac:dyDescent="0.25">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="239" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>25</v>
       </c>
       <c r="F239" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="J239" t="s">
         <v>18</v>
       </c>
       <c r="K239" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F239,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
-      </c>
-    </row>
-    <row r="240" spans="1:11" x14ac:dyDescent="0.25">
+        <v>9.3000000000000007</v>
+      </c>
+    </row>
+    <row r="240" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>25</v>
       </c>
       <c r="F240" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="J240" t="s">
         <v>18</v>
       </c>
       <c r="K240" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F240,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <v>9.6999999999999993</v>
       </c>
     </row>
     <row r="241" spans="1:11" x14ac:dyDescent="0.25">
@@ -6129,14 +6132,14 @@
         <v>25</v>
       </c>
       <c r="F241" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="J241" t="s">
         <v>18</v>
       </c>
       <c r="K241" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F241,'feed pars'!B$6:B$43,0))</f>
-        <v>11.1</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="242" spans="1:11" x14ac:dyDescent="0.25">
@@ -6144,13 +6147,193 @@
         <v>25</v>
       </c>
       <c r="F242" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="J242" t="s">
         <v>18</v>
       </c>
       <c r="K242" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F242,'feed pars'!B$6:B$43,0))</f>
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="243" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>25</v>
+      </c>
+      <c r="F243" t="s">
+        <v>47</v>
+      </c>
+      <c r="J243" t="s">
+        <v>18</v>
+      </c>
+      <c r="K243" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F243,'feed pars'!B$6:B$43,0))</f>
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="244" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>25</v>
+      </c>
+      <c r="F244" t="s">
+        <v>48</v>
+      </c>
+      <c r="J244" t="s">
+        <v>18</v>
+      </c>
+      <c r="K244" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F244,'feed pars'!B$6:B$43,0))</f>
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="245" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>25</v>
+      </c>
+      <c r="F245" t="s">
+        <v>49</v>
+      </c>
+      <c r="J245" t="s">
+        <v>18</v>
+      </c>
+      <c r="K245" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F245,'feed pars'!B$6:B$43,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="246" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
+        <v>25</v>
+      </c>
+      <c r="F246" t="s">
+        <v>50</v>
+      </c>
+      <c r="J246" t="s">
+        <v>18</v>
+      </c>
+      <c r="K246" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F246,'feed pars'!B$6:B$43,0))</f>
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="247" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>25</v>
+      </c>
+      <c r="F247" t="s">
+        <v>51</v>
+      </c>
+      <c r="J247" t="s">
+        <v>18</v>
+      </c>
+      <c r="K247" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F247,'feed pars'!B$6:B$43,0))</f>
+        <v>8.1999999999999993</v>
+      </c>
+    </row>
+    <row r="248" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
+        <v>25</v>
+      </c>
+      <c r="F248" t="s">
+        <v>313</v>
+      </c>
+      <c r="J248" t="s">
+        <v>18</v>
+      </c>
+      <c r="K248" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F248,'feed pars'!B$6:B$43,0))</f>
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="249" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>25</v>
+      </c>
+      <c r="F249" t="s">
+        <v>52</v>
+      </c>
+      <c r="J249" t="s">
+        <v>18</v>
+      </c>
+      <c r="K249" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F249,'feed pars'!B$6:B$43,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="250" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
+        <v>25</v>
+      </c>
+      <c r="F250" t="s">
+        <v>53</v>
+      </c>
+      <c r="J250" t="s">
+        <v>18</v>
+      </c>
+      <c r="K250" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F250,'feed pars'!B$6:B$43,0))</f>
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="251" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
+        <v>25</v>
+      </c>
+      <c r="F251" t="s">
+        <v>54</v>
+      </c>
+      <c r="J251" t="s">
+        <v>18</v>
+      </c>
+      <c r="K251" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F251,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="252" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
+        <v>25</v>
+      </c>
+      <c r="F252" t="s">
+        <v>55</v>
+      </c>
+      <c r="J252" t="s">
+        <v>18</v>
+      </c>
+      <c r="K252" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F252,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="253" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
+        <v>25</v>
+      </c>
+      <c r="F253" t="s">
+        <v>56</v>
+      </c>
+      <c r="J253" t="s">
+        <v>18</v>
+      </c>
+      <c r="K253" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F253,'feed pars'!B$6:B$43,0))</f>
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="254" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>25</v>
+      </c>
+      <c r="F254" t="s">
+        <v>57</v>
+      </c>
+      <c r="J254" t="s">
+        <v>18</v>
+      </c>
+      <c r="K254" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F254,'feed pars'!B$6:B$43,0))</f>
         <v>10.8</v>
       </c>
     </row>
@@ -7130,7 +7313,7 @@
       </c>
       <c r="C33" s="23">
         <f t="shared" si="0"/>
-        <v>88</v>
+        <v>88.5</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4">
@@ -7150,7 +7333,15 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="J33" s="4"/>
-      <c r="L33" s="27"/>
+      <c r="K33">
+        <v>89</v>
+      </c>
+      <c r="L33" s="27">
+        <v>11.5</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>410</v>
+      </c>
       <c r="N33" s="4">
         <f>MATCH($B33,poultry!$A$3:$A$41,0)</f>
         <v>36</v>
@@ -7521,9 +7712,10 @@
     <hyperlink ref="C1" r:id="rId1"/>
     <hyperlink ref="I36" r:id="rId2"/>
     <hyperlink ref="M31" r:id="rId3"/>
+    <hyperlink ref="M33" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Reintroduced regional share for cereals for pig and poultry
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FeedMgmt.xlsx
+++ b/data/prod_parameters/FeedMgmt.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1271" uniqueCount="415">
   <si>
     <t>f_feed</t>
   </si>
@@ -1283,13 +1283,16 @@
     <t>https://glw-feeds.co.uk/index.php/wheat-feed-2/</t>
   </si>
   <si>
-    <t>no solution if these are used…</t>
-  </si>
-  <si>
-    <t>probably some problem with animals</t>
-  </si>
-  <si>
-    <t>needing to be exactly 0 in some regions</t>
+    <t>Slow solving and inaccurate solution warning</t>
+  </si>
+  <si>
+    <t>if these are used. Potential solution: remove</t>
+  </si>
+  <si>
+    <t>crops and animals that cant be pressent in</t>
+  </si>
+  <si>
+    <t>a region from variables instead of using constraints.</t>
   </si>
 </sst>
 </file>
@@ -1783,7 +1786,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O258"/>
+  <dimension ref="A1:O260"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -2514,8 +2517,11 @@
       <c r="H46" t="s">
         <v>37</v>
       </c>
+      <c r="J46" t="s">
+        <v>27</v>
+      </c>
       <c r="K46" s="3">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="L46" t="s">
         <v>28</v>
@@ -2531,8 +2537,11 @@
       <c r="H47" t="s">
         <v>37</v>
       </c>
+      <c r="J47" t="s">
+        <v>27</v>
+      </c>
       <c r="K47" s="3">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="L47" t="s">
         <v>28</v>
@@ -2548,8 +2557,11 @@
       <c r="H48" t="s">
         <v>17</v>
       </c>
+      <c r="J48" t="s">
+        <v>27</v>
+      </c>
       <c r="K48" s="3">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="L48" t="s">
         <v>28</v>
@@ -2565,192 +2577,180 @@
       <c r="H49" t="s">
         <v>17</v>
       </c>
+      <c r="J49" t="s">
+        <v>27</v>
+      </c>
       <c r="K49" s="3">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="L49" t="s">
         <v>28</v>
       </c>
+      <c r="M49" s="3" t="s">
+        <v>414</v>
+      </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
+      <c r="A50" t="s">
+        <v>25</v>
+      </c>
+      <c r="H50" t="s">
+        <v>38</v>
+      </c>
+      <c r="J50" t="s">
+        <v>27</v>
+      </c>
+      <c r="K50" s="3">
+        <v>40</v>
+      </c>
+      <c r="L50" t="s">
+        <v>28</v>
+      </c>
+      <c r="M50" s="3"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>389</v>
+      </c>
+      <c r="H51" t="s">
+        <v>38</v>
+      </c>
+      <c r="J51" t="s">
+        <v>27</v>
+      </c>
+      <c r="K51" s="3">
+        <v>40</v>
+      </c>
+      <c r="L51" t="s">
+        <v>28</v>
+      </c>
+      <c r="M51" s="3"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B50" s="1"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="1"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
-      <c r="I50" s="2"/>
-      <c r="J50" s="2"/>
-      <c r="K50" s="2"/>
-      <c r="L50" s="2"/>
-      <c r="M50" s="2"/>
-      <c r="N50" s="2"/>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J51" s="10" t="s">
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
+      <c r="L52" s="2"/>
+      <c r="M52" s="2"/>
+      <c r="N52" s="2"/>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J53" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="K51" s="10">
-        <v>0</v>
-      </c>
-      <c r="L51" s="10"/>
-      <c r="M51" s="10" t="s">
+      <c r="K53" s="10">
+        <v>0</v>
+      </c>
+      <c r="L53" s="10"/>
+      <c r="M53" s="10" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I52" t="s">
-        <v>318</v>
-      </c>
-      <c r="J52" t="s">
-        <v>31</v>
-      </c>
-      <c r="K52" s="29">
-        <v>100</v>
-      </c>
-      <c r="L52" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="M52" s="10"/>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I53" t="s">
-        <v>44</v>
-      </c>
-      <c r="J53" t="s">
-        <v>31</v>
-      </c>
-      <c r="K53" s="29">
-        <v>100</v>
-      </c>
-      <c r="L53" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="M53" s="10"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="I54" t="s">
-        <v>36</v>
+        <v>318</v>
       </c>
       <c r="J54" t="s">
         <v>31</v>
       </c>
       <c r="K54" s="29">
-        <v>61</v>
-      </c>
-      <c r="L54" t="s">
+        <v>100</v>
+      </c>
+      <c r="L54" s="29" t="s">
         <v>28</v>
       </c>
+      <c r="M54" s="10"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H55" t="s">
-        <v>43</v>
+      <c r="I55" t="s">
+        <v>44</v>
       </c>
       <c r="J55" t="s">
         <v>31</v>
       </c>
-      <c r="K55" s="3">
+      <c r="K55" s="29">
         <v>100</v>
       </c>
-      <c r="L55" t="s">
+      <c r="L55" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="M55" s="3" t="s">
-        <v>304</v>
-      </c>
+      <c r="M55" s="10"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H56" t="s">
-        <v>40</v>
+      <c r="I56" t="s">
+        <v>36</v>
       </c>
       <c r="J56" t="s">
         <v>31</v>
       </c>
-      <c r="K56" s="3">
-        <v>50</v>
+      <c r="K56" s="29">
+        <v>61</v>
       </c>
       <c r="L56" t="s">
         <v>28</v>
       </c>
-      <c r="M56" s="3" t="s">
-        <v>394</v>
-      </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>336</v>
-      </c>
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="1"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
-      <c r="I57" s="2"/>
-      <c r="J57" s="2"/>
-      <c r="K57" s="2"/>
-      <c r="L57" s="2"/>
-      <c r="M57" s="2"/>
-      <c r="N57" s="2"/>
+      <c r="H57" t="s">
+        <v>43</v>
+      </c>
+      <c r="J57" t="s">
+        <v>31</v>
+      </c>
+      <c r="K57" s="3">
+        <v>100</v>
+      </c>
+      <c r="L57" t="s">
+        <v>28</v>
+      </c>
+      <c r="M57" s="3" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>24</v>
-      </c>
-      <c r="B58" t="s">
-        <v>326</v>
-      </c>
-      <c r="E58" t="s">
-        <v>327</v>
-      </c>
-      <c r="G58" t="s">
-        <v>334</v>
-      </c>
       <c r="H58" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="J58" t="s">
-        <v>335</v>
+        <v>31</v>
       </c>
       <c r="K58" s="3">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="L58" t="s">
         <v>28</v>
       </c>
-      <c r="M58" s="3"/>
+      <c r="M58" s="3" t="s">
+        <v>394</v>
+      </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>24</v>
-      </c>
-      <c r="B59" t="s">
-        <v>326</v>
-      </c>
-      <c r="E59" t="s">
-        <v>328</v>
-      </c>
-      <c r="G59" t="s">
-        <v>334</v>
-      </c>
-      <c r="H59" t="s">
-        <v>33</v>
-      </c>
-      <c r="J59" t="s">
-        <v>335</v>
-      </c>
-      <c r="K59" s="3">
-        <v>5</v>
-      </c>
-      <c r="L59" t="s">
-        <v>28</v>
-      </c>
-      <c r="M59" s="3"/>
+      <c r="A59" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
+      <c r="L59" s="2"/>
+      <c r="M59" s="2"/>
+      <c r="N59" s="2"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
@@ -2760,7 +2760,7 @@
         <v>326</v>
       </c>
       <c r="E60" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="G60" t="s">
         <v>334</v>
@@ -2772,7 +2772,7 @@
         <v>335</v>
       </c>
       <c r="K60" s="3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L60" t="s">
         <v>28</v>
@@ -2787,7 +2787,7 @@
         <v>326</v>
       </c>
       <c r="E61" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="G61" t="s">
         <v>334</v>
@@ -2799,7 +2799,7 @@
         <v>335</v>
       </c>
       <c r="K61" s="3">
-        <v>90</v>
+        <v>5</v>
       </c>
       <c r="L61" t="s">
         <v>28</v>
@@ -2814,7 +2814,7 @@
         <v>326</v>
       </c>
       <c r="E62" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="G62" t="s">
         <v>334</v>
@@ -2826,7 +2826,7 @@
         <v>335</v>
       </c>
       <c r="K62" s="3">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L62" t="s">
         <v>28</v>
@@ -2841,7 +2841,7 @@
         <v>326</v>
       </c>
       <c r="E63" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="G63" t="s">
         <v>334</v>
@@ -2853,7 +2853,7 @@
         <v>335</v>
       </c>
       <c r="K63" s="3">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L63" t="s">
         <v>28</v>
@@ -2865,10 +2865,10 @@
         <v>24</v>
       </c>
       <c r="B64" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="E64" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="G64" t="s">
         <v>334</v>
@@ -2892,10 +2892,10 @@
         <v>24</v>
       </c>
       <c r="B65" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="E65" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="G65" t="s">
         <v>334</v>
@@ -2907,7 +2907,7 @@
         <v>335</v>
       </c>
       <c r="K65" s="3">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L65" t="s">
         <v>28</v>
@@ -2922,7 +2922,7 @@
         <v>333</v>
       </c>
       <c r="E66" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="G66" t="s">
         <v>334</v>
@@ -2934,7 +2934,7 @@
         <v>335</v>
       </c>
       <c r="K66" s="3">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L66" t="s">
         <v>28</v>
@@ -2949,7 +2949,7 @@
         <v>333</v>
       </c>
       <c r="E67" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="G67" t="s">
         <v>334</v>
@@ -2976,7 +2976,7 @@
         <v>333</v>
       </c>
       <c r="E68" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="G68" t="s">
         <v>334</v>
@@ -2988,7 +2988,7 @@
         <v>335</v>
       </c>
       <c r="K68" s="3">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L68" t="s">
         <v>28</v>
@@ -3003,7 +3003,7 @@
         <v>333</v>
       </c>
       <c r="E69" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="G69" t="s">
         <v>334</v>
@@ -3024,7 +3024,13 @@
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>395</v>
+        <v>24</v>
+      </c>
+      <c r="B70" t="s">
+        <v>333</v>
+      </c>
+      <c r="E70" t="s">
+        <v>331</v>
       </c>
       <c r="G70" t="s">
         <v>334</v>
@@ -3036,7 +3042,7 @@
         <v>335</v>
       </c>
       <c r="K70" s="3">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="L70" t="s">
         <v>28</v>
@@ -3044,150 +3050,152 @@
       <c r="M70" s="3"/>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K71" s="3"/>
+      <c r="A71" t="s">
+        <v>24</v>
+      </c>
+      <c r="B71" t="s">
+        <v>333</v>
+      </c>
+      <c r="E71" t="s">
+        <v>332</v>
+      </c>
+      <c r="G71" t="s">
+        <v>334</v>
+      </c>
+      <c r="H71" t="s">
+        <v>33</v>
+      </c>
+      <c r="J71" t="s">
+        <v>335</v>
+      </c>
+      <c r="K71" s="3">
+        <v>90</v>
+      </c>
+      <c r="L71" t="s">
+        <v>28</v>
+      </c>
       <c r="M71" s="3"/>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
+      <c r="A72" t="s">
+        <v>395</v>
+      </c>
+      <c r="G72" t="s">
+        <v>334</v>
+      </c>
+      <c r="H72" t="s">
+        <v>33</v>
+      </c>
+      <c r="J72" t="s">
+        <v>335</v>
+      </c>
+      <c r="K72" s="3">
+        <v>10</v>
+      </c>
+      <c r="L72" t="s">
+        <v>28</v>
+      </c>
+      <c r="M72" s="3"/>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K73" s="3"/>
+      <c r="M73" s="3"/>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="B72" s="1"/>
-      <c r="C72" s="1"/>
-      <c r="D72" s="1"/>
-      <c r="E72" s="2"/>
-      <c r="F72" s="2"/>
-      <c r="G72" s="2"/>
-      <c r="H72" s="2"/>
-      <c r="I72" s="2"/>
-      <c r="J72" s="2"/>
-      <c r="K72" s="2"/>
-      <c r="L72" s="2"/>
-      <c r="M72" s="2"/>
-      <c r="N72" s="2"/>
-    </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J73" s="10" t="s">
+      <c r="B74" s="1"/>
+      <c r="C74" s="1"/>
+      <c r="D74" s="1"/>
+      <c r="E74" s="2"/>
+      <c r="F74" s="2"/>
+      <c r="G74" s="2"/>
+      <c r="H74" s="2"/>
+      <c r="I74" s="2"/>
+      <c r="J74" s="2"/>
+      <c r="K74" s="2"/>
+      <c r="L74" s="2"/>
+      <c r="M74" s="2"/>
+      <c r="N74" s="2"/>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J75" s="10" t="s">
         <v>396</v>
       </c>
-      <c r="K73" s="10">
-        <v>0</v>
-      </c>
-      <c r="L73" s="10" t="s">
+      <c r="K75" s="10">
+        <v>0</v>
+      </c>
+      <c r="L75" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M73" s="10" t="s">
+      <c r="M75" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J74" s="10" t="s">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J76" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="K74" s="10">
-        <v>0</v>
-      </c>
-      <c r="L74" s="10" t="s">
+      <c r="K76" s="10">
+        <v>0</v>
+      </c>
+      <c r="L76" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M74" s="10" t="s">
+      <c r="M76" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>24</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B77" t="s">
         <v>326</v>
       </c>
-      <c r="E75" t="s">
+      <c r="E77" t="s">
         <v>327</v>
       </c>
-      <c r="F75" t="s">
+      <c r="F77" t="s">
         <v>310</v>
       </c>
-      <c r="J75" s="29" t="s">
+      <c r="J77" s="29" t="s">
         <v>396</v>
       </c>
-      <c r="K75" s="29">
+      <c r="K77" s="29">
         <f>(0.8*20+0.2*2)</f>
         <v>16.399999999999999</v>
       </c>
-      <c r="L75" s="29" t="s">
+      <c r="L77" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="M75" s="29" t="s">
+      <c r="M77" s="29" t="s">
         <v>402</v>
       </c>
-      <c r="N75" t="s">
+      <c r="N77" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>24</v>
       </c>
-      <c r="F76" t="s">
+      <c r="F78" t="s">
         <v>310</v>
       </c>
-      <c r="J76" s="29" t="s">
+      <c r="J78" s="29" t="s">
         <v>396</v>
       </c>
-      <c r="K76" s="29">
+      <c r="K78" s="29">
         <f>(0.6*20+0.4*2)</f>
         <v>12.8</v>
       </c>
-      <c r="L76" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="M76" s="29" t="s">
-        <v>403</v>
-      </c>
-      <c r="N76" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>401</v>
-      </c>
-      <c r="F77" t="s">
-        <v>310</v>
-      </c>
-      <c r="J77" s="29" t="s">
-        <v>396</v>
-      </c>
-      <c r="K77" s="29">
-        <v>2</v>
-      </c>
-      <c r="L77" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="M77" s="29" t="s">
-        <v>404</v>
-      </c>
-      <c r="N77" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>395</v>
-      </c>
-      <c r="F78" t="s">
-        <v>310</v>
-      </c>
-      <c r="J78" s="29" t="s">
-        <v>396</v>
-      </c>
-      <c r="K78" s="29">
-        <v>2</v>
-      </c>
       <c r="L78" s="29" t="s">
         <v>28</v>
       </c>
       <c r="M78" s="29" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="N78" t="s">
         <v>398</v>
@@ -3195,28 +3203,22 @@
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>24</v>
-      </c>
-      <c r="B79" t="s">
-        <v>326</v>
-      </c>
-      <c r="E79" t="s">
-        <v>327</v>
+        <v>401</v>
       </c>
       <c r="F79" t="s">
         <v>310</v>
       </c>
       <c r="J79" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K79" s="29">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L79" s="29" t="s">
         <v>28</v>
       </c>
       <c r="M79" s="29" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="N79" t="s">
         <v>398</v>
@@ -3224,25 +3226,22 @@
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>24</v>
-      </c>
-      <c r="E80" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="F80" t="s">
         <v>310</v>
       </c>
       <c r="J80" s="29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="K80" s="29">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L80" s="29" t="s">
         <v>28</v>
       </c>
       <c r="M80" s="29" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="N80" t="s">
         <v>398</v>
@@ -3252,6 +3251,12 @@
       <c r="A81" t="s">
         <v>24</v>
       </c>
+      <c r="B81" t="s">
+        <v>326</v>
+      </c>
+      <c r="E81" t="s">
+        <v>327</v>
+      </c>
       <c r="F81" t="s">
         <v>310</v>
       </c>
@@ -3259,171 +3264,162 @@
         <v>397</v>
       </c>
       <c r="K81" s="29">
+        <v>5</v>
+      </c>
+      <c r="L81" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M81" s="29" t="s">
+        <v>405</v>
+      </c>
+      <c r="N81" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>24</v>
+      </c>
+      <c r="E82" t="s">
+        <v>329</v>
+      </c>
+      <c r="F82" t="s">
+        <v>310</v>
+      </c>
+      <c r="J82" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K82" s="29">
+        <v>5</v>
+      </c>
+      <c r="L82" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M82" s="29" t="s">
+        <v>405</v>
+      </c>
+      <c r="N82" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>24</v>
+      </c>
+      <c r="F83" t="s">
+        <v>310</v>
+      </c>
+      <c r="J83" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K83" s="29">
         <f>0.9*5+0.1*15</f>
         <v>6</v>
       </c>
-      <c r="L81" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="M81" s="29" t="s">
-        <v>406</v>
-      </c>
-      <c r="N81" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>401</v>
-      </c>
-      <c r="F82" t="s">
-        <v>310</v>
-      </c>
-      <c r="J82" s="29" t="s">
-        <v>397</v>
-      </c>
-      <c r="K82" s="29">
-        <v>15</v>
-      </c>
-      <c r="L82" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="M82" s="29"/>
-      <c r="N82" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>395</v>
-      </c>
-      <c r="F83" t="s">
-        <v>310</v>
-      </c>
-      <c r="J83" s="29" t="s">
-        <v>397</v>
-      </c>
-      <c r="K83" s="29">
-        <v>15</v>
-      </c>
       <c r="L83" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="M83" s="29"/>
+      <c r="M83" s="29" t="s">
+        <v>406</v>
+      </c>
       <c r="N83" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A84" s="33" t="str">
-        <f>A75</f>
+      <c r="A84" t="s">
+        <v>401</v>
+      </c>
+      <c r="F84" t="s">
+        <v>310</v>
+      </c>
+      <c r="J84" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K84" s="29">
+        <v>15</v>
+      </c>
+      <c r="L84" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M84" s="29"/>
+      <c r="N84" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>395</v>
+      </c>
+      <c r="F85" t="s">
+        <v>310</v>
+      </c>
+      <c r="J85" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="K85" s="29">
+        <v>15</v>
+      </c>
+      <c r="L85" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M85" s="29"/>
+      <c r="N85" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A86" s="33" t="str">
+        <f>A77</f>
         <v>cattle</v>
       </c>
-      <c r="B84" s="33" t="str">
-        <f>B75</f>
+      <c r="B86" s="33" t="str">
+        <f>B77</f>
         <v>dairy</v>
       </c>
-      <c r="E84" s="33" t="str">
-        <f>E75</f>
+      <c r="E86" s="33" t="str">
+        <f>E77</f>
         <v>cows</v>
       </c>
-      <c r="F84" t="s">
+      <c r="F86" t="s">
         <v>311</v>
       </c>
-      <c r="J84" s="33" t="str">
-        <f>J75</f>
+      <c r="J86" s="33" t="str">
+        <f>J77</f>
         <v>storage_losses</v>
       </c>
-      <c r="K84" s="33">
-        <f>K75</f>
+      <c r="K86" s="33">
+        <f>K77</f>
         <v>16.399999999999999</v>
       </c>
-      <c r="L84" s="33" t="str">
-        <f>L75</f>
+      <c r="L86" s="33" t="str">
+        <f>L77</f>
         <v>%</v>
       </c>
-      <c r="M84" s="33" t="str">
-        <f>M75</f>
+      <c r="M86" s="33" t="str">
+        <f>M77</f>
         <v>80% in silo</v>
       </c>
-      <c r="N84" s="33" t="str">
-        <f>N75</f>
+      <c r="N86" s="33" t="str">
+        <f>N77</f>
         <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A85" s="33" t="str">
-        <f t="shared" ref="A85:A92" si="0">A76</f>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A87" s="33" t="str">
+        <f t="shared" ref="A87:A94" si="0">A78</f>
         <v>cattle</v>
       </c>
-      <c r="F85" t="s">
+      <c r="F87" t="s">
         <v>311</v>
       </c>
-      <c r="J85" s="33" t="str">
-        <f t="shared" ref="J85:N92" si="1">J76</f>
+      <c r="J87" s="33" t="str">
+        <f t="shared" ref="J87:N94" si="1">J78</f>
         <v>storage_losses</v>
       </c>
-      <c r="K85" s="33">
+      <c r="K87" s="33">
         <f t="shared" si="1"/>
         <v>12.8</v>
-      </c>
-      <c r="L85" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="M85" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>60% in silo</v>
-      </c>
-      <c r="N85" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
-      </c>
-    </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A86" s="33" t="str">
-        <f t="shared" si="0"/>
-        <v>sheep</v>
-      </c>
-      <c r="F86" t="s">
-        <v>311</v>
-      </c>
-      <c r="J86" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>storage_losses</v>
-      </c>
-      <c r="K86" s="33">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="L86" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>%</v>
-      </c>
-      <c r="M86" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>0% in silo</v>
-      </c>
-      <c r="N86" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
-      </c>
-    </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A87" s="33" t="str">
-        <f t="shared" si="0"/>
-        <v>horses</v>
-      </c>
-      <c r="F87" t="s">
-        <v>311</v>
-      </c>
-      <c r="J87" s="33" t="str">
-        <f t="shared" si="1"/>
-        <v>storage_losses</v>
-      </c>
-      <c r="K87" s="33">
-        <f t="shared" si="1"/>
-        <v>2</v>
       </c>
       <c r="L87" s="33" t="str">
         <f t="shared" si="1"/>
@@ -3431,7 +3427,7 @@
       </c>
       <c r="M87" s="33" t="str">
         <f t="shared" si="1"/>
-        <v>0% in silo</v>
+        <v>60% in silo</v>
       </c>
       <c r="N87" s="33" t="str">
         <f t="shared" si="1"/>
@@ -3441,26 +3437,18 @@
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="33" t="str">
         <f t="shared" si="0"/>
-        <v>cattle</v>
-      </c>
-      <c r="B88" s="33" t="str">
-        <f>B79</f>
-        <v>dairy</v>
-      </c>
-      <c r="E88" s="33" t="str">
-        <f>E79</f>
-        <v>cows</v>
+        <v>sheep</v>
       </c>
       <c r="F88" t="s">
         <v>311</v>
       </c>
       <c r="J88" s="33" t="str">
         <f t="shared" si="1"/>
-        <v>feeding_losses</v>
+        <v>storage_losses</v>
       </c>
       <c r="K88" s="33">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L88" s="33" t="str">
         <f t="shared" si="1"/>
@@ -3468,7 +3456,7 @@
       </c>
       <c r="M88" s="33" t="str">
         <f t="shared" si="1"/>
-        <v>No feeding on pasture</v>
+        <v>0% in silo</v>
       </c>
       <c r="N88" s="33" t="str">
         <f t="shared" si="1"/>
@@ -3478,22 +3466,18 @@
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="33" t="str">
         <f t="shared" si="0"/>
-        <v>cattle</v>
-      </c>
-      <c r="E89" s="33" t="str">
-        <f>E80</f>
-        <v>bulls</v>
+        <v>horses</v>
       </c>
       <c r="F89" t="s">
         <v>311</v>
       </c>
       <c r="J89" s="33" t="str">
         <f t="shared" si="1"/>
-        <v>feeding_losses</v>
+        <v>storage_losses</v>
       </c>
       <c r="K89" s="33">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L89" s="33" t="str">
         <f t="shared" si="1"/>
@@ -3501,7 +3485,7 @@
       </c>
       <c r="M89" s="33" t="str">
         <f t="shared" si="1"/>
-        <v>No feeding on pasture</v>
+        <v>0% in silo</v>
       </c>
       <c r="N89" s="33" t="str">
         <f t="shared" si="1"/>
@@ -3513,6 +3497,14 @@
         <f t="shared" si="0"/>
         <v>cattle</v>
       </c>
+      <c r="B90" s="33" t="str">
+        <f>B81</f>
+        <v>dairy</v>
+      </c>
+      <c r="E90" s="33" t="str">
+        <f>E81</f>
+        <v>cows</v>
+      </c>
       <c r="F90" t="s">
         <v>311</v>
       </c>
@@ -3522,7 +3514,7 @@
       </c>
       <c r="K90" s="33">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L90" s="33" t="str">
         <f t="shared" si="1"/>
@@ -3530,7 +3522,7 @@
       </c>
       <c r="M90" s="33" t="str">
         <f t="shared" si="1"/>
-        <v>10% feeding on pasture</v>
+        <v>No feeding on pasture</v>
       </c>
       <c r="N90" s="33" t="str">
         <f t="shared" si="1"/>
@@ -3540,7 +3532,11 @@
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91" s="33" t="str">
         <f t="shared" si="0"/>
-        <v>sheep</v>
+        <v>cattle</v>
+      </c>
+      <c r="E91" s="33" t="str">
+        <f>E82</f>
+        <v>bulls</v>
       </c>
       <c r="F91" t="s">
         <v>311</v>
@@ -3551,22 +3547,25 @@
       </c>
       <c r="K91" s="33">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="L91" s="33" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="M91" s="33"/>
+      <c r="M91" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="N91" s="33" t="str">
-        <f t="shared" ref="N91:N92" si="2">N82</f>
+        <f t="shared" si="1"/>
         <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
       </c>
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92" s="33" t="str">
         <f t="shared" si="0"/>
-        <v>horses</v>
+        <v>cattle</v>
       </c>
       <c r="F92" t="s">
         <v>311</v>
@@ -3577,124 +3576,117 @@
       </c>
       <c r="K92" s="33">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="L92" s="33" t="str">
         <f t="shared" si="1"/>
         <v>%</v>
       </c>
-      <c r="M92" s="33"/>
+      <c r="M92" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>10% feeding on pasture</v>
+      </c>
       <c r="N92" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A93" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>sheep</v>
+      </c>
+      <c r="F93" t="s">
+        <v>311</v>
+      </c>
+      <c r="J93" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K93" s="33">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L93" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M93" s="33"/>
+      <c r="N93" s="33" t="str">
+        <f t="shared" ref="N93:N94" si="2">N84</f>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A94" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>horses</v>
+      </c>
+      <c r="F94" t="s">
+        <v>311</v>
+      </c>
+      <c r="J94" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K94" s="33">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L94" s="33" t="str">
+        <f t="shared" si="1"/>
+        <v>%</v>
+      </c>
+      <c r="M94" s="33"/>
+      <c r="N94" s="33" t="str">
         <f t="shared" si="2"/>
         <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A93" s="33"/>
-      <c r="B93" s="33"/>
-      <c r="E93" s="33"/>
-      <c r="F93" t="s">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A95" s="33"/>
+      <c r="B95" s="33"/>
+      <c r="E95" s="33"/>
+      <c r="F95" t="s">
         <v>312</v>
       </c>
-      <c r="J93" s="29" t="s">
+      <c r="J95" s="29" t="s">
         <v>396</v>
       </c>
-      <c r="K93" s="29">
+      <c r="K95" s="29">
         <v>5</v>
       </c>
-      <c r="L93" s="29" t="s">
+      <c r="L95" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="M93" s="29"/>
-      <c r="N93" t="s">
+      <c r="M95" s="29"/>
+      <c r="N95" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A94" s="33" t="str">
-        <f>A79</f>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A96" s="33" t="str">
+        <f>A81</f>
         <v>cattle</v>
       </c>
-      <c r="B94" s="33" t="str">
-        <f>B79</f>
+      <c r="B96" s="33" t="str">
+        <f>B81</f>
         <v>dairy</v>
       </c>
-      <c r="E94" s="33" t="str">
-        <f t="shared" ref="E94:E95" si="3">E79</f>
+      <c r="E96" s="33" t="str">
+        <f t="shared" ref="E96:E97" si="3">E81</f>
         <v>cows</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F96" t="s">
         <v>312</v>
       </c>
-      <c r="J94" s="33" t="str">
-        <f t="shared" ref="J94:N98" si="4">J79</f>
+      <c r="J96" s="33" t="str">
+        <f t="shared" ref="J96:N100" si="4">J81</f>
         <v>feeding_losses</v>
       </c>
-      <c r="K94" s="33">
+      <c r="K96" s="33">
         <f t="shared" si="4"/>
         <v>5</v>
-      </c>
-      <c r="L94" s="33" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="M94" s="33" t="str">
-        <f t="shared" si="4"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="N94" s="33" t="str">
-        <f t="shared" si="4"/>
-        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
-      </c>
-    </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A95" s="33" t="str">
-        <f t="shared" ref="A95:A98" si="5">A80</f>
-        <v>cattle</v>
-      </c>
-      <c r="E95" s="33" t="str">
-        <f t="shared" si="3"/>
-        <v>bulls</v>
-      </c>
-      <c r="F95" t="s">
-        <v>312</v>
-      </c>
-      <c r="J95" s="33" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="K95" s="33">
-        <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="L95" s="33" t="str">
-        <f t="shared" si="4"/>
-        <v>%</v>
-      </c>
-      <c r="M95" s="33" t="str">
-        <f t="shared" si="4"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="N95" s="33" t="str">
-        <f t="shared" si="4"/>
-        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
-      </c>
-    </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A96" s="33" t="str">
-        <f t="shared" si="5"/>
-        <v>cattle</v>
-      </c>
-      <c r="F96" t="s">
-        <v>312</v>
-      </c>
-      <c r="J96" s="33" t="str">
-        <f t="shared" si="4"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="K96" s="33">
-        <f t="shared" si="4"/>
-        <v>6</v>
       </c>
       <c r="L96" s="33" t="str">
         <f t="shared" si="4"/>
@@ -3702,7 +3694,7 @@
       </c>
       <c r="M96" s="33" t="str">
         <f t="shared" si="4"/>
-        <v>10% feeding on pasture</v>
+        <v>No feeding on pasture</v>
       </c>
       <c r="N96" s="33" t="str">
         <f t="shared" si="4"/>
@@ -3711,8 +3703,12 @@
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" s="33" t="str">
-        <f t="shared" si="5"/>
-        <v>sheep</v>
+        <f t="shared" ref="A97:A100" si="5">A82</f>
+        <v>cattle</v>
+      </c>
+      <c r="E97" s="33" t="str">
+        <f t="shared" si="3"/>
+        <v>bulls</v>
       </c>
       <c r="F97" t="s">
         <v>312</v>
@@ -3723,13 +3719,16 @@
       </c>
       <c r="K97" s="33">
         <f t="shared" si="4"/>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="L97" s="33" t="str">
         <f t="shared" si="4"/>
         <v>%</v>
       </c>
-      <c r="M97" s="33"/>
+      <c r="M97" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="N97" s="33" t="str">
         <f t="shared" si="4"/>
         <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
@@ -3738,7 +3737,7 @@
     <row r="98" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" s="33" t="str">
         <f t="shared" si="5"/>
-        <v>horses</v>
+        <v>cattle</v>
       </c>
       <c r="F98" t="s">
         <v>312</v>
@@ -3749,121 +3748,114 @@
       </c>
       <c r="K98" s="33">
         <f t="shared" si="4"/>
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="L98" s="33" t="str">
         <f t="shared" si="4"/>
         <v>%</v>
       </c>
-      <c r="M98" s="33"/>
+      <c r="M98" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>10% feeding on pasture</v>
+      </c>
       <c r="N98" s="33" t="str">
         <f t="shared" si="4"/>
         <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
       </c>
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A99" s="33" t="str">
+        <f t="shared" si="5"/>
+        <v>sheep</v>
+      </c>
       <c r="F99" t="s">
-        <v>2</v>
-      </c>
-      <c r="J99" s="29" t="s">
-        <v>396</v>
-      </c>
-      <c r="K99" s="29">
-        <v>5</v>
-      </c>
-      <c r="L99" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="M99" s="29"/>
-      <c r="N99" t="s">
-        <v>398</v>
+        <v>312</v>
+      </c>
+      <c r="J99" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K99" s="33">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="L99" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="M99" s="33"/>
+      <c r="N99" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
       </c>
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" s="33" t="str">
-        <f>A79</f>
+        <f t="shared" si="5"/>
+        <v>horses</v>
+      </c>
+      <c r="F100" t="s">
+        <v>312</v>
+      </c>
+      <c r="J100" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K100" s="33">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="L100" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>%</v>
+      </c>
+      <c r="M100" s="33"/>
+      <c r="N100" s="33" t="str">
+        <f t="shared" si="4"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F101" t="s">
+        <v>2</v>
+      </c>
+      <c r="J101" s="29" t="s">
+        <v>396</v>
+      </c>
+      <c r="K101" s="29">
+        <v>5</v>
+      </c>
+      <c r="L101" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M101" s="29"/>
+      <c r="N101" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A102" s="33" t="str">
+        <f>A81</f>
         <v>cattle</v>
       </c>
-      <c r="B100" s="33" t="str">
-        <f>B79</f>
+      <c r="B102" s="33" t="str">
+        <f>B81</f>
         <v>dairy</v>
       </c>
-      <c r="E100" s="33" t="str">
-        <f t="shared" ref="E100:E101" si="6">E79</f>
+      <c r="E102" s="33" t="str">
+        <f t="shared" ref="E102:E103" si="6">E81</f>
         <v>cows</v>
       </c>
-      <c r="F100" t="s">
+      <c r="F102" t="s">
         <v>2</v>
       </c>
-      <c r="J100" s="33" t="str">
-        <f t="shared" ref="J100:N104" si="7">J79</f>
+      <c r="J102" s="33" t="str">
+        <f t="shared" ref="J102:N106" si="7">J81</f>
         <v>feeding_losses</v>
       </c>
-      <c r="K100" s="33">
+      <c r="K102" s="33">
         <f t="shared" si="7"/>
         <v>5</v>
-      </c>
-      <c r="L100" s="33" t="str">
-        <f t="shared" si="7"/>
-        <v>%</v>
-      </c>
-      <c r="M100" s="33" t="str">
-        <f t="shared" si="7"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="N100" s="33" t="str">
-        <f t="shared" si="7"/>
-        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
-      </c>
-    </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A101" s="33" t="str">
-        <f t="shared" ref="A101:A104" si="8">A80</f>
-        <v>cattle</v>
-      </c>
-      <c r="E101" s="33" t="str">
-        <f t="shared" si="6"/>
-        <v>bulls</v>
-      </c>
-      <c r="F101" t="s">
-        <v>2</v>
-      </c>
-      <c r="J101" s="33" t="str">
-        <f t="shared" si="7"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="K101" s="33">
-        <f t="shared" si="7"/>
-        <v>5</v>
-      </c>
-      <c r="L101" s="33" t="str">
-        <f t="shared" si="7"/>
-        <v>%</v>
-      </c>
-      <c r="M101" s="33" t="str">
-        <f t="shared" si="7"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="N101" s="33" t="str">
-        <f t="shared" si="7"/>
-        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
-      </c>
-    </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A102" s="33" t="str">
-        <f t="shared" si="8"/>
-        <v>cattle</v>
-      </c>
-      <c r="F102" t="s">
-        <v>2</v>
-      </c>
-      <c r="J102" s="33" t="str">
-        <f t="shared" si="7"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="K102" s="33">
-        <f t="shared" si="7"/>
-        <v>6</v>
       </c>
       <c r="L102" s="33" t="str">
         <f t="shared" si="7"/>
@@ -3871,7 +3863,7 @@
       </c>
       <c r="M102" s="33" t="str">
         <f t="shared" si="7"/>
-        <v>10% feeding on pasture</v>
+        <v>No feeding on pasture</v>
       </c>
       <c r="N102" s="33" t="str">
         <f t="shared" si="7"/>
@@ -3880,8 +3872,12 @@
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A103" s="33" t="str">
-        <f t="shared" si="8"/>
-        <v>sheep</v>
+        <f t="shared" ref="A103:A106" si="8">A82</f>
+        <v>cattle</v>
+      </c>
+      <c r="E103" s="33" t="str">
+        <f t="shared" si="6"/>
+        <v>bulls</v>
       </c>
       <c r="F103" t="s">
         <v>2</v>
@@ -3892,22 +3888,25 @@
       </c>
       <c r="K103" s="33">
         <f t="shared" si="7"/>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="L103" s="33" t="str">
         <f t="shared" si="7"/>
         <v>%</v>
       </c>
-      <c r="M103" s="29"/>
+      <c r="M103" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="N103" s="33" t="str">
-        <f t="shared" ref="N103:N104" si="9">N82</f>
+        <f t="shared" si="7"/>
         <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
       </c>
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A104" s="33" t="str">
         <f t="shared" si="8"/>
-        <v>horses</v>
+        <v>cattle</v>
       </c>
       <c r="F104" t="s">
         <v>2</v>
@@ -3918,121 +3917,114 @@
       </c>
       <c r="K104" s="33">
         <f t="shared" si="7"/>
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="L104" s="33" t="str">
         <f t="shared" si="7"/>
         <v>%</v>
       </c>
-      <c r="M104" s="29"/>
+      <c r="M104" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>10% feeding on pasture</v>
+      </c>
       <c r="N104" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A105" s="33" t="str">
+        <f t="shared" si="8"/>
+        <v>sheep</v>
+      </c>
+      <c r="F105" t="s">
+        <v>2</v>
+      </c>
+      <c r="J105" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K105" s="33">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="L105" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>%</v>
+      </c>
+      <c r="M105" s="29"/>
+      <c r="N105" s="33" t="str">
+        <f t="shared" ref="N105:N106" si="9">N84</f>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A106" s="33" t="str">
+        <f t="shared" si="8"/>
+        <v>horses</v>
+      </c>
+      <c r="F106" t="s">
+        <v>2</v>
+      </c>
+      <c r="J106" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K106" s="33">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="L106" s="33" t="str">
+        <f t="shared" si="7"/>
+        <v>%</v>
+      </c>
+      <c r="M106" s="29"/>
+      <c r="N106" s="33" t="str">
         <f t="shared" si="9"/>
         <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
       </c>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F105" t="s">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F107" t="s">
         <v>12</v>
       </c>
-      <c r="J105" s="29" t="s">
+      <c r="J107" s="29" t="s">
         <v>396</v>
       </c>
-      <c r="K105" s="29">
+      <c r="K107" s="29">
         <v>5</v>
       </c>
-      <c r="L105" s="29" t="s">
+      <c r="L107" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="M105" s="29"/>
-      <c r="N105" t="s">
+      <c r="M107" s="29"/>
+      <c r="N107" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A106" s="33" t="str">
-        <f>A79</f>
+    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A108" s="33" t="str">
+        <f>A81</f>
         <v>cattle</v>
       </c>
-      <c r="B106" s="33" t="str">
-        <f>B79</f>
+      <c r="B108" s="33" t="str">
+        <f>B81</f>
         <v>dairy</v>
       </c>
-      <c r="E106" s="33" t="str">
-        <f t="shared" ref="E106:E107" si="10">E79</f>
+      <c r="E108" s="33" t="str">
+        <f t="shared" ref="E108:E109" si="10">E81</f>
         <v>cows</v>
       </c>
-      <c r="F106" t="s">
+      <c r="F108" t="s">
         <v>12</v>
       </c>
-      <c r="J106" s="33" t="str">
-        <f t="shared" ref="J106:N110" si="11">J79</f>
+      <c r="J108" s="33" t="str">
+        <f t="shared" ref="J108:N112" si="11">J81</f>
         <v>feeding_losses</v>
       </c>
-      <c r="K106" s="33">
+      <c r="K108" s="33">
         <f t="shared" si="11"/>
         <v>5</v>
-      </c>
-      <c r="L106" s="33" t="str">
-        <f t="shared" si="11"/>
-        <v>%</v>
-      </c>
-      <c r="M106" s="33" t="str">
-        <f t="shared" si="11"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="N106" s="33" t="str">
-        <f t="shared" si="11"/>
-        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
-      </c>
-    </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A107" s="33" t="str">
-        <f t="shared" ref="A107:A110" si="12">A80</f>
-        <v>cattle</v>
-      </c>
-      <c r="E107" s="33" t="str">
-        <f t="shared" si="10"/>
-        <v>bulls</v>
-      </c>
-      <c r="F107" t="s">
-        <v>12</v>
-      </c>
-      <c r="J107" s="33" t="str">
-        <f t="shared" si="11"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="K107" s="33">
-        <f t="shared" si="11"/>
-        <v>5</v>
-      </c>
-      <c r="L107" s="33" t="str">
-        <f t="shared" si="11"/>
-        <v>%</v>
-      </c>
-      <c r="M107" s="33" t="str">
-        <f t="shared" si="11"/>
-        <v>No feeding on pasture</v>
-      </c>
-      <c r="N107" s="33" t="str">
-        <f t="shared" si="11"/>
-        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
-      </c>
-    </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A108" s="33" t="str">
-        <f t="shared" si="12"/>
-        <v>cattle</v>
-      </c>
-      <c r="F108" t="s">
-        <v>12</v>
-      </c>
-      <c r="J108" s="33" t="str">
-        <f t="shared" si="11"/>
-        <v>feeding_losses</v>
-      </c>
-      <c r="K108" s="33">
-        <f t="shared" si="11"/>
-        <v>6</v>
       </c>
       <c r="L108" s="33" t="str">
         <f t="shared" si="11"/>
@@ -4040,7 +4032,7 @@
       </c>
       <c r="M108" s="33" t="str">
         <f t="shared" si="11"/>
-        <v>10% feeding on pasture</v>
+        <v>No feeding on pasture</v>
       </c>
       <c r="N108" s="33" t="str">
         <f t="shared" si="11"/>
@@ -4049,8 +4041,12 @@
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" s="33" t="str">
-        <f t="shared" si="12"/>
-        <v>sheep</v>
+        <f t="shared" ref="A109:A112" si="12">A82</f>
+        <v>cattle</v>
+      </c>
+      <c r="E109" s="33" t="str">
+        <f t="shared" si="10"/>
+        <v>bulls</v>
       </c>
       <c r="F109" t="s">
         <v>12</v>
@@ -4061,22 +4057,25 @@
       </c>
       <c r="K109" s="33">
         <f t="shared" si="11"/>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="L109" s="33" t="str">
         <f t="shared" si="11"/>
         <v>%</v>
       </c>
-      <c r="M109" s="29"/>
+      <c r="M109" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>No feeding on pasture</v>
+      </c>
       <c r="N109" s="33" t="str">
-        <f t="shared" ref="N109:N110" si="13">N82</f>
+        <f t="shared" si="11"/>
         <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
       </c>
     </row>
     <row r="110" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A110" s="33" t="str">
         <f t="shared" si="12"/>
-        <v>horses</v>
+        <v>cattle</v>
       </c>
       <c r="F110" t="s">
         <v>12</v>
@@ -4087,161 +4086,182 @@
       </c>
       <c r="K110" s="33">
         <f t="shared" si="11"/>
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="L110" s="33" t="str">
         <f t="shared" si="11"/>
         <v>%</v>
       </c>
-      <c r="M110" s="29"/>
+      <c r="M110" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>10% feeding on pasture</v>
+      </c>
       <c r="N110" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A111" s="33" t="str">
+        <f t="shared" si="12"/>
+        <v>sheep</v>
+      </c>
+      <c r="F111" t="s">
+        <v>12</v>
+      </c>
+      <c r="J111" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K111" s="33">
+        <f t="shared" si="11"/>
+        <v>15</v>
+      </c>
+      <c r="L111" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>%</v>
+      </c>
+      <c r="M111" s="29"/>
+      <c r="N111" s="33" t="str">
+        <f t="shared" ref="N111:N112" si="13">N84</f>
+        <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A112" s="33" t="str">
+        <f t="shared" si="12"/>
+        <v>horses</v>
+      </c>
+      <c r="F112" t="s">
+        <v>12</v>
+      </c>
+      <c r="J112" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>feeding_losses</v>
+      </c>
+      <c r="K112" s="33">
+        <f t="shared" si="11"/>
+        <v>15</v>
+      </c>
+      <c r="L112" s="33" t="str">
+        <f t="shared" si="11"/>
+        <v>%</v>
+      </c>
+      <c r="M112" s="29"/>
+      <c r="N112" s="33" t="str">
         <f t="shared" si="13"/>
         <v>Cederberg &amp; Henriksson. 2020. Gräsmarkernas användning i jordbruket</v>
       </c>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A111" s="33"/>
-      <c r="F111" t="s">
+    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A113" s="33"/>
+      <c r="F113" t="s">
         <v>33</v>
       </c>
-      <c r="J111" s="29" t="s">
+      <c r="J113" s="29" t="s">
         <v>396</v>
       </c>
-      <c r="K111" s="29">
-        <v>0</v>
-      </c>
-      <c r="L111" t="s">
+      <c r="K113" s="29">
+        <v>0</v>
+      </c>
+      <c r="L113" t="s">
         <v>28</v>
       </c>
-      <c r="M111" s="29" t="s">
+      <c r="M113" s="29" t="s">
         <v>408</v>
       </c>
-      <c r="N111" s="33"/>
-    </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
+      <c r="N113" s="33"/>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
         <v>24</v>
       </c>
-      <c r="F112" t="s">
+      <c r="F114" t="s">
         <v>33</v>
       </c>
-      <c r="J112" t="s">
+      <c r="J114" t="s">
         <v>397</v>
       </c>
-      <c r="K112" s="29">
+      <c r="K114" s="29">
         <f>100-55</f>
         <v>45</v>
       </c>
-      <c r="L112" t="s">
+      <c r="L114" t="s">
         <v>28</v>
       </c>
-      <c r="M112" s="29" t="s">
+      <c r="M114" s="29" t="s">
         <v>400</v>
       </c>
-      <c r="N112" t="s">
+      <c r="N114" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
+    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
         <v>395</v>
       </c>
-      <c r="F113" t="s">
+      <c r="F115" t="s">
         <v>33</v>
       </c>
-      <c r="J113" t="s">
+      <c r="J115" t="s">
         <v>397</v>
       </c>
-      <c r="K113" s="29">
+      <c r="K115" s="29">
         <f>100-50</f>
         <v>50</v>
       </c>
-      <c r="L113" t="s">
+      <c r="L115" t="s">
         <v>28</v>
       </c>
-      <c r="M113" s="29" t="s">
+      <c r="M115" s="29" t="s">
         <v>400</v>
       </c>
-      <c r="N113" t="s">
+      <c r="N115" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K114" s="3"/>
-      <c r="M114" s="29"/>
-    </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A115" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="K115" s="3"/>
-      <c r="M115" s="29"/>
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.25">
       <c r="K116" s="3"/>
       <c r="M116" s="29"/>
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A117" s="3" t="s">
+        <v>407</v>
+      </c>
       <c r="K117" s="3"/>
-      <c r="M117" s="3"/>
+      <c r="M117" s="29"/>
     </row>
     <row r="118" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A118" s="1" t="s">
+      <c r="K118" s="3"/>
+      <c r="M118" s="29"/>
+    </row>
+    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K119" s="3"/>
+      <c r="M119" s="3"/>
+    </row>
+    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A120" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B118" s="1"/>
-      <c r="C118" s="1"/>
-      <c r="D118" s="1"/>
-      <c r="E118" s="2"/>
-      <c r="F118" s="2"/>
-      <c r="G118" s="2"/>
-      <c r="H118" s="2"/>
-      <c r="I118" s="2"/>
-      <c r="J118" s="2"/>
-      <c r="K118" s="2"/>
-      <c r="L118" s="2"/>
-      <c r="M118" s="2" t="s">
+      <c r="B120" s="1"/>
+      <c r="C120" s="1"/>
+      <c r="D120" s="1"/>
+      <c r="E120" s="2"/>
+      <c r="F120" s="2"/>
+      <c r="G120" s="2"/>
+      <c r="H120" s="2"/>
+      <c r="I120" s="2"/>
+      <c r="J120" s="2"/>
+      <c r="K120" s="2"/>
+      <c r="L120" s="2"/>
+      <c r="M120" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="N118" s="2"/>
-    </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F119" t="s">
-        <v>310</v>
-      </c>
-      <c r="J119" t="s">
-        <v>390</v>
-      </c>
-      <c r="K119" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F119,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L119" t="s">
-        <v>28</v>
-      </c>
-      <c r="M119" s="29" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F120" t="s">
-        <v>311</v>
-      </c>
-      <c r="J120" t="s">
-        <v>390</v>
-      </c>
-      <c r="K120" s="26">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F120,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L120" t="s">
-        <v>28</v>
-      </c>
-      <c r="M120" s="3"/>
+      <c r="N120" s="2"/>
     </row>
     <row r="121" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F121" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J121" t="s">
         <v>390</v>
@@ -4253,11 +4273,13 @@
       <c r="L121" t="s">
         <v>28</v>
       </c>
-      <c r="M121" s="3"/>
+      <c r="M121" s="29" t="s">
+        <v>393</v>
+      </c>
     </row>
     <row r="122" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F122" t="s">
-        <v>2</v>
+        <v>311</v>
       </c>
       <c r="J122" t="s">
         <v>390</v>
@@ -4273,7 +4295,7 @@
     </row>
     <row r="123" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F123" t="s">
-        <v>12</v>
+        <v>312</v>
       </c>
       <c r="J123" t="s">
         <v>390</v>
@@ -4289,7 +4311,7 @@
     </row>
     <row r="124" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F124" t="s">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="J124" t="s">
         <v>390</v>
@@ -4305,14 +4327,14 @@
     </row>
     <row r="125" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F125" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="J125" t="s">
         <v>390</v>
       </c>
       <c r="K125" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F125,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="L125" t="s">
         <v>28</v>
@@ -4321,14 +4343,14 @@
     </row>
     <row r="126" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F126" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J126" t="s">
         <v>390</v>
       </c>
       <c r="K126" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F126,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="L126" t="s">
         <v>28</v>
@@ -4337,14 +4359,14 @@
     </row>
     <row r="127" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F127" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="J127" t="s">
         <v>390</v>
       </c>
       <c r="K127" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F127,'feed pars'!B$6:B$43,0))</f>
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L127" t="s">
         <v>28</v>
@@ -4353,7 +4375,7 @@
     </row>
     <row r="128" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F128" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J128" t="s">
         <v>390</v>
@@ -4369,14 +4391,14 @@
     </row>
     <row r="129" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F129" t="s">
-        <v>317</v>
+        <v>38</v>
       </c>
       <c r="J129" t="s">
         <v>390</v>
       </c>
       <c r="K129" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F129,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L129" t="s">
         <v>28</v>
@@ -4385,14 +4407,14 @@
     </row>
     <row r="130" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F130" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J130" t="s">
         <v>390</v>
       </c>
       <c r="K130" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F130,'feed pars'!B$6:B$43,0))</f>
-        <v>67.5</v>
+        <v>87</v>
       </c>
       <c r="L130" t="s">
         <v>28</v>
@@ -4401,7 +4423,7 @@
     </row>
     <row r="131" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F131" t="s">
-        <v>41</v>
+        <v>317</v>
       </c>
       <c r="J131" t="s">
         <v>390</v>
@@ -4417,14 +4439,14 @@
     </row>
     <row r="132" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F132" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J132" t="s">
         <v>390</v>
       </c>
       <c r="K132" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F132,'feed pars'!B$6:B$43,0))</f>
-        <v>86.8</v>
+        <v>67.5</v>
       </c>
       <c r="L132" t="s">
         <v>28</v>
@@ -4433,14 +4455,14 @@
     </row>
     <row r="133" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F133" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="J133" t="s">
         <v>390</v>
       </c>
       <c r="K133" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F133,'feed pars'!B$6:B$43,0))</f>
-        <v>92.5</v>
+        <v>87</v>
       </c>
       <c r="L133" t="s">
         <v>28</v>
@@ -4449,14 +4471,14 @@
     </row>
     <row r="134" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F134" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J134" t="s">
         <v>390</v>
       </c>
       <c r="K134" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F134,'feed pars'!B$6:B$43,0))</f>
-        <v>92</v>
+        <v>86.8</v>
       </c>
       <c r="L134" t="s">
         <v>28</v>
@@ -4465,14 +4487,14 @@
     </row>
     <row r="135" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F135" t="s">
-        <v>314</v>
+        <v>35</v>
       </c>
       <c r="J135" t="s">
         <v>390</v>
       </c>
       <c r="K135" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F135,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
+        <v>92.5</v>
       </c>
       <c r="L135" t="s">
         <v>28</v>
@@ -4481,14 +4503,14 @@
     </row>
     <row r="136" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F136" t="s">
-        <v>305</v>
+        <v>43</v>
       </c>
       <c r="J136" t="s">
         <v>390</v>
       </c>
       <c r="K136" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F136,'feed pars'!B$6:B$43,0))</f>
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="L136" t="s">
         <v>28</v>
@@ -4497,14 +4519,14 @@
     </row>
     <row r="137" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F137" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="J137" t="s">
         <v>390</v>
       </c>
       <c r="K137" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F137,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="L137" t="s">
         <v>28</v>
@@ -4513,14 +4535,14 @@
     </row>
     <row r="138" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F138" t="s">
-        <v>44</v>
+        <v>305</v>
       </c>
       <c r="J138" t="s">
         <v>390</v>
       </c>
       <c r="K138" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F138,'feed pars'!B$6:B$43,0))</f>
-        <v>87.5</v>
+        <v>85</v>
       </c>
       <c r="L138" t="s">
         <v>28</v>
@@ -4529,7 +4551,7 @@
     </row>
     <row r="139" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F139" t="s">
-        <v>45</v>
+        <v>318</v>
       </c>
       <c r="J139" t="s">
         <v>390</v>
@@ -4545,14 +4567,14 @@
     </row>
     <row r="140" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F140" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="J140" t="s">
         <v>390</v>
       </c>
       <c r="K140" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F140,'feed pars'!B$6:B$43,0))</f>
-        <v>89.5</v>
+        <v>87.5</v>
       </c>
       <c r="L140" t="s">
         <v>28</v>
@@ -4561,14 +4583,14 @@
     </row>
     <row r="141" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F141" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J141" t="s">
         <v>390</v>
       </c>
       <c r="K141" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F141,'feed pars'!B$6:B$43,0))</f>
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="L141" t="s">
         <v>28</v>
@@ -4577,14 +4599,14 @@
     </row>
     <row r="142" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F142" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="J142" t="s">
         <v>390</v>
       </c>
       <c r="K142" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F142,'feed pars'!B$6:B$43,0))</f>
-        <v>91</v>
+        <v>89.5</v>
       </c>
       <c r="L142" t="s">
         <v>28</v>
@@ -4593,14 +4615,14 @@
     </row>
     <row r="143" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F143" t="s">
-        <v>319</v>
+        <v>46</v>
       </c>
       <c r="J143" t="s">
         <v>390</v>
       </c>
       <c r="K143" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F143,'feed pars'!B$6:B$43,0))</f>
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L143" t="s">
         <v>28</v>
@@ -4609,14 +4631,14 @@
     </row>
     <row r="144" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F144" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J144" t="s">
         <v>390</v>
       </c>
       <c r="K144" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F144,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="L144" t="s">
         <v>28</v>
@@ -4625,14 +4647,14 @@
     </row>
     <row r="145" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F145" t="s">
-        <v>49</v>
+        <v>319</v>
       </c>
       <c r="J145" t="s">
         <v>390</v>
       </c>
       <c r="K145" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F145,'feed pars'!B$6:B$43,0))</f>
-        <v>88.5</v>
+        <v>90</v>
       </c>
       <c r="L145" t="s">
         <v>28</v>
@@ -4641,14 +4663,14 @@
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F146" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J146" t="s">
         <v>390</v>
       </c>
       <c r="K146" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F146,'feed pars'!B$6:B$43,0))</f>
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="L146" t="s">
         <v>28</v>
@@ -4657,14 +4679,14 @@
     </row>
     <row r="147" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F147" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J147" t="s">
         <v>390</v>
       </c>
       <c r="K147" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F147,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
+        <v>88.5</v>
       </c>
       <c r="L147" t="s">
         <v>28</v>
@@ -4673,7 +4695,7 @@
     </row>
     <row r="148" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F148" t="s">
-        <v>313</v>
+        <v>50</v>
       </c>
       <c r="J148" t="s">
         <v>390</v>
@@ -4689,14 +4711,14 @@
     </row>
     <row r="149" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F149" t="s">
-        <v>388</v>
+        <v>51</v>
       </c>
       <c r="J149" t="s">
         <v>390</v>
       </c>
       <c r="K149" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F149,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="L149" t="s">
         <v>28</v>
@@ -4705,14 +4727,14 @@
     </row>
     <row r="150" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F150" t="s">
-        <v>52</v>
+        <v>313</v>
       </c>
       <c r="J150" t="s">
         <v>390</v>
       </c>
       <c r="K150" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F150,'feed pars'!B$6:B$43,0))</f>
-        <v>75.5</v>
+        <v>90</v>
       </c>
       <c r="L150" t="s">
         <v>28</v>
@@ -4721,14 +4743,14 @@
     </row>
     <row r="151" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F151" t="s">
-        <v>53</v>
+        <v>388</v>
       </c>
       <c r="J151" t="s">
         <v>390</v>
       </c>
       <c r="K151" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F151,'feed pars'!B$6:B$43,0))</f>
-        <v>89.5</v>
+        <v>87</v>
       </c>
       <c r="L151" t="s">
         <v>28</v>
@@ -4737,14 +4759,14 @@
     </row>
     <row r="152" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F152" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J152" t="s">
         <v>390</v>
       </c>
       <c r="K152" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F152,'feed pars'!B$6:B$43,0))</f>
-        <v>6.25</v>
+        <v>75.5</v>
       </c>
       <c r="L152" t="s">
         <v>28</v>
@@ -4753,14 +4775,14 @@
     </row>
     <row r="153" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F153" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J153" t="s">
         <v>390</v>
       </c>
       <c r="K153" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F153,'feed pars'!B$6:B$43,0))</f>
-        <v>97</v>
+        <v>89.5</v>
       </c>
       <c r="L153" t="s">
         <v>28</v>
@@ -4769,14 +4791,14 @@
     </row>
     <row r="154" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F154" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J154" t="s">
         <v>390</v>
       </c>
       <c r="K154" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F154,'feed pars'!B$6:B$43,0))</f>
-        <v>91</v>
+        <v>6.25</v>
       </c>
       <c r="L154" t="s">
         <v>28</v>
@@ -4785,14 +4807,14 @@
     </row>
     <row r="155" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F155" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J155" t="s">
         <v>390</v>
       </c>
       <c r="K155" s="26">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F155,'feed pars'!B$6:B$43,0))</f>
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="L155" t="s">
         <v>28</v>
@@ -4800,70 +4822,70 @@
       <c r="M155" s="3"/>
     </row>
     <row r="156" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A156" s="7" t="s">
+      <c r="F156" t="s">
+        <v>56</v>
+      </c>
+      <c r="J156" t="s">
+        <v>390</v>
+      </c>
+      <c r="K156" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F156,'feed pars'!B$6:B$43,0))</f>
+        <v>91</v>
+      </c>
+      <c r="L156" t="s">
+        <v>28</v>
+      </c>
+      <c r="M156" s="3"/>
+    </row>
+    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F157" t="s">
+        <v>57</v>
+      </c>
+      <c r="J157" t="s">
+        <v>390</v>
+      </c>
+      <c r="K157" s="26">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F157,'feed pars'!B$6:B$43,0))</f>
+        <v>92</v>
+      </c>
+      <c r="L157" t="s">
+        <v>28</v>
+      </c>
+      <c r="M157" s="3"/>
+    </row>
+    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A158" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B156" s="7"/>
-      <c r="C156" s="6"/>
-      <c r="D156" s="6"/>
-      <c r="E156" s="6"/>
-      <c r="F156" s="6"/>
-      <c r="G156" s="6"/>
-      <c r="H156" s="6"/>
-      <c r="I156" s="6"/>
-      <c r="J156" s="6"/>
-      <c r="K156" s="6"/>
-      <c r="L156" s="6" t="s">
+      <c r="B158" s="7"/>
+      <c r="C158" s="6"/>
+      <c r="D158" s="6"/>
+      <c r="E158" s="6"/>
+      <c r="F158" s="6"/>
+      <c r="G158" s="6"/>
+      <c r="H158" s="6"/>
+      <c r="I158" s="6"/>
+      <c r="J158" s="6"/>
+      <c r="K158" s="6"/>
+      <c r="L158" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="M156" s="6"/>
-      <c r="N156" s="6"/>
-    </row>
-    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A157" t="s">
-        <v>24</v>
-      </c>
-      <c r="F157" t="s">
-        <v>310</v>
-      </c>
-      <c r="J157" t="s">
-        <v>18</v>
-      </c>
-      <c r="K157" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F157,'feed pars'!B$6:B$43,0))</f>
-        <v>11.5</v>
-      </c>
-      <c r="M157" s="3"/>
-    </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A158" t="s">
-        <v>24</v>
-      </c>
-      <c r="F158" t="s">
-        <v>311</v>
-      </c>
-      <c r="J158" t="s">
-        <v>18</v>
-      </c>
-      <c r="K158" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F158,'feed pars'!B$6:B$43,0))</f>
-        <v>10.4</v>
-      </c>
-      <c r="M158" s="3"/>
+      <c r="M158" s="6"/>
+      <c r="N158" s="6"/>
     </row>
     <row r="159" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>24</v>
       </c>
       <c r="F159" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J159" t="s">
         <v>18</v>
       </c>
       <c r="K159" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F159,'feed pars'!B$6:B$43,0))</f>
-        <v>10</v>
+        <v>11.5</v>
       </c>
       <c r="M159" s="3"/>
     </row>
@@ -4872,22 +4894,23 @@
         <v>24</v>
       </c>
       <c r="F160" t="s">
-        <v>12</v>
+        <v>311</v>
       </c>
       <c r="J160" t="s">
         <v>18</v>
       </c>
       <c r="K160" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F160,'feed pars'!B$6:B$43,0))</f>
-        <v>11.3</v>
-      </c>
-    </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+        <v>10.4</v>
+      </c>
+      <c r="M160" s="3"/>
+    </row>
+    <row r="161" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>24</v>
       </c>
       <c r="F161" t="s">
-        <v>33</v>
+        <v>312</v>
       </c>
       <c r="J161" t="s">
         <v>18</v>
@@ -4896,218 +4919,219 @@
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F161,'feed pars'!B$6:B$43,0))</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="K162" s="3"/>
-    </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M161" s="3"/>
+    </row>
+    <row r="162" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>24</v>
+      </c>
+      <c r="F162" t="s">
+        <v>12</v>
+      </c>
+      <c r="J162" t="s">
+        <v>18</v>
+      </c>
+      <c r="K162" s="26">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F162,'feed pars'!B$6:B$43,0))</f>
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="163" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>24</v>
       </c>
       <c r="F163" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="J163" t="s">
         <v>18</v>
       </c>
       <c r="K163" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F163,'feed pars'!B$6:B$43,0))</f>
-        <v>14.1</v>
-      </c>
-    </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A164" t="s">
-        <v>24</v>
-      </c>
-      <c r="F164" t="s">
-        <v>37</v>
-      </c>
-      <c r="J164" t="s">
-        <v>18</v>
-      </c>
-      <c r="K164" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F164,'feed pars'!B$6:B$43,0))</f>
-        <v>13.2</v>
-      </c>
-    </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="164" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K164" s="3"/>
+    </row>
+    <row r="165" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>24</v>
       </c>
       <c r="F165" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="J165" t="s">
         <v>18</v>
       </c>
       <c r="K165" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F165,'feed pars'!B$6:B$43,0))</f>
-        <v>11.7</v>
-      </c>
-    </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="166" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>24</v>
       </c>
       <c r="F166" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J166" t="s">
         <v>18</v>
       </c>
       <c r="K166" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F166,'feed pars'!B$6:B$43,0))</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="167" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>24</v>
       </c>
       <c r="F167" t="s">
-        <v>317</v>
+        <v>38</v>
       </c>
       <c r="J167" t="s">
         <v>18</v>
       </c>
       <c r="K167" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F167,'feed pars'!B$6:B$43,0))</f>
-        <v>13.9</v>
-      </c>
-    </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="168" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>24</v>
       </c>
       <c r="F168" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J168" t="s">
         <v>18</v>
       </c>
       <c r="K168" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F168,'feed pars'!B$6:B$43,0))</f>
-        <v>12.8</v>
-      </c>
-    </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="169" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>24</v>
       </c>
       <c r="F169" t="s">
-        <v>41</v>
+        <v>317</v>
       </c>
       <c r="J169" t="s">
         <v>18</v>
       </c>
       <c r="K169" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F169,'feed pars'!B$6:B$43,0))</f>
-        <v>13.8</v>
-      </c>
-    </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="170" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>24</v>
       </c>
       <c r="F170" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J170" t="s">
         <v>18</v>
       </c>
       <c r="K170" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F170,'feed pars'!B$6:B$43,0))</f>
-        <v>13.3</v>
-      </c>
-    </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="171" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>24</v>
       </c>
       <c r="F171" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="J171" t="s">
         <v>18</v>
       </c>
       <c r="K171" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F171,'feed pars'!B$6:B$43,0))</f>
-        <v>22.1</v>
-      </c>
-    </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="172" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>24</v>
       </c>
       <c r="F172" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J172" t="s">
         <v>18</v>
       </c>
       <c r="K172" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F172,'feed pars'!B$6:B$43,0))</f>
-        <v>20.100000000000001</v>
-      </c>
-    </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="173" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>24</v>
       </c>
       <c r="F173" t="s">
-        <v>305</v>
+        <v>35</v>
       </c>
       <c r="J173" t="s">
         <v>18</v>
       </c>
       <c r="K173" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F173,'feed pars'!B$6:B$43,0))</f>
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>24</v>
       </c>
       <c r="F174" t="s">
-        <v>314</v>
+        <v>43</v>
       </c>
       <c r="J174" t="s">
         <v>18</v>
       </c>
       <c r="K174" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F174,'feed pars'!B$6:B$43,0))</f>
-        <v>36.6</v>
-      </c>
-    </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+        <v>20.100000000000001</v>
+      </c>
+    </row>
+    <row r="175" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>24</v>
       </c>
       <c r="F175" t="s">
-        <v>318</v>
+        <v>305</v>
       </c>
       <c r="J175" t="s">
         <v>18</v>
       </c>
       <c r="K175" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F175,'feed pars'!B$6:B$43,0))</f>
-        <v>16.399999999999999</v>
-      </c>
-    </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="176" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>24</v>
       </c>
       <c r="F176" t="s">
-        <v>44</v>
+        <v>314</v>
       </c>
       <c r="J176" t="s">
         <v>18</v>
       </c>
       <c r="K176" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F176,'feed pars'!B$6:B$43,0))</f>
-        <v>14.6</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="177" spans="1:14" x14ac:dyDescent="0.25">
@@ -5115,14 +5139,14 @@
         <v>24</v>
       </c>
       <c r="F177" t="s">
-        <v>36</v>
+        <v>318</v>
       </c>
       <c r="J177" t="s">
         <v>18</v>
       </c>
       <c r="K177" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F177,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
+        <v>16.399999999999999</v>
       </c>
     </row>
     <row r="178" spans="1:14" x14ac:dyDescent="0.25">
@@ -5130,14 +5154,14 @@
         <v>24</v>
       </c>
       <c r="F178" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J178" t="s">
         <v>18</v>
       </c>
       <c r="K178" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F178,'feed pars'!B$6:B$43,0))</f>
-        <v>11.4</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="179" spans="1:14" x14ac:dyDescent="0.25">
@@ -5145,14 +5169,14 @@
         <v>24</v>
       </c>
       <c r="F179" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="J179" t="s">
         <v>18</v>
       </c>
       <c r="K179" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F179,'feed pars'!B$6:B$43,0))</f>
-        <v>13.4</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="180" spans="1:14" x14ac:dyDescent="0.25">
@@ -5160,14 +5184,14 @@
         <v>24</v>
       </c>
       <c r="F180" t="s">
-        <v>319</v>
+        <v>46</v>
       </c>
       <c r="J180" t="s">
         <v>18</v>
       </c>
       <c r="K180" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F180,'feed pars'!B$6:B$43,0))</f>
-        <v>8.5</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="181" spans="1:14" x14ac:dyDescent="0.25">
@@ -5175,14 +5199,14 @@
         <v>24</v>
       </c>
       <c r="F181" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J181" t="s">
         <v>18</v>
       </c>
       <c r="K181" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F181,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="182" spans="1:14" x14ac:dyDescent="0.25">
@@ -5190,14 +5214,14 @@
         <v>24</v>
       </c>
       <c r="F182" t="s">
-        <v>50</v>
+        <v>319</v>
       </c>
       <c r="J182" t="s">
         <v>18</v>
       </c>
       <c r="K182" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F182,'feed pars'!B$6:B$43,0))</f>
-        <v>13.3</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="183" spans="1:14" x14ac:dyDescent="0.25">
@@ -5205,14 +5229,14 @@
         <v>24</v>
       </c>
       <c r="F183" t="s">
-        <v>313</v>
+        <v>48</v>
       </c>
       <c r="J183" t="s">
         <v>18</v>
       </c>
       <c r="K183" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F183,'feed pars'!B$6:B$43,0))</f>
-        <v>11.6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="184" spans="1:14" x14ac:dyDescent="0.25">
@@ -5220,14 +5244,14 @@
         <v>24</v>
       </c>
       <c r="F184" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J184" t="s">
         <v>18</v>
       </c>
       <c r="K184" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F184,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="185" spans="1:14" x14ac:dyDescent="0.25">
@@ -5235,14 +5259,14 @@
         <v>24</v>
       </c>
       <c r="F185" t="s">
-        <v>53</v>
+        <v>313</v>
       </c>
       <c r="J185" t="s">
         <v>18</v>
       </c>
       <c r="K185" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F185,'feed pars'!B$6:B$43,0))</f>
-        <v>12.3</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="186" spans="1:14" x14ac:dyDescent="0.25">
@@ -5250,14 +5274,14 @@
         <v>24</v>
       </c>
       <c r="F186" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J186" t="s">
         <v>18</v>
       </c>
       <c r="K186" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F186,'feed pars'!B$6:B$43,0))</f>
-        <v>13.6</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="187" spans="1:14" x14ac:dyDescent="0.25">
@@ -5265,14 +5289,14 @@
         <v>24</v>
       </c>
       <c r="F187" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J187" t="s">
         <v>18</v>
       </c>
       <c r="K187" s="26">
         <f>INDEX('feed pars'!L$6:L$43,MATCH(F187,'feed pars'!B$6:B$43,0))</f>
-        <v>15.5</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="188" spans="1:14" x14ac:dyDescent="0.25">
@@ -5280,111 +5304,111 @@
         <v>24</v>
       </c>
       <c r="F188" t="s">
-        <v>324</v>
+        <v>54</v>
       </c>
       <c r="J188" t="s">
         <v>18</v>
       </c>
-      <c r="K188" s="3">
-        <v>0</v>
+      <c r="K188" s="26">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F188,'feed pars'!B$6:B$43,0))</f>
+        <v>13.6</v>
       </c>
     </row>
     <row r="189" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A189" s="7" t="s">
-        <v>409</v>
-      </c>
-      <c r="B189" s="7"/>
-      <c r="C189" s="6"/>
-      <c r="D189" s="6"/>
-      <c r="E189" s="6"/>
-      <c r="F189" s="6"/>
-      <c r="G189" s="6"/>
-      <c r="H189" s="6"/>
-      <c r="I189" s="6"/>
-      <c r="J189" s="6"/>
-      <c r="K189" s="6"/>
-      <c r="L189" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="M189" s="6"/>
-      <c r="N189" s="6"/>
+      <c r="A189" t="s">
+        <v>24</v>
+      </c>
+      <c r="F189" t="s">
+        <v>56</v>
+      </c>
+      <c r="J189" t="s">
+        <v>18</v>
+      </c>
+      <c r="K189" s="26">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F189,'feed pars'!B$6:B$43,0))</f>
+        <v>15.5</v>
+      </c>
     </row>
     <row r="190" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>395</v>
+        <v>24</v>
       </c>
       <c r="F190" t="s">
-        <v>2</v>
+        <v>324</v>
       </c>
       <c r="J190" t="s">
         <v>18</v>
       </c>
-      <c r="K190" s="26">
-        <f>INDEX('feed pars'!L$6:L$43,MATCH(F190,'feed pars'!B$6:B$43,0))</f>
+      <c r="K190" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A191" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="B191" s="7"/>
+      <c r="C191" s="6"/>
+      <c r="D191" s="6"/>
+      <c r="E191" s="6"/>
+      <c r="F191" s="6"/>
+      <c r="G191" s="6"/>
+      <c r="H191" s="6"/>
+      <c r="I191" s="6"/>
+      <c r="J191" s="6"/>
+      <c r="K191" s="6"/>
+      <c r="L191" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M191" s="6"/>
+      <c r="N191" s="6"/>
+    </row>
+    <row r="192" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>395</v>
+      </c>
+      <c r="F192" t="s">
+        <v>2</v>
+      </c>
+      <c r="J192" t="s">
+        <v>18</v>
+      </c>
+      <c r="K192" s="26">
+        <f>INDEX('feed pars'!L$6:L$43,MATCH(F192,'feed pars'!B$6:B$43,0))</f>
         <v>9.1</v>
       </c>
-    </row>
-    <row r="191" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A191" t="s">
-        <v>395</v>
-      </c>
-      <c r="F191" t="s">
-        <v>33</v>
-      </c>
-      <c r="J191" t="s">
-        <v>18</v>
-      </c>
-      <c r="K191" s="34">
-        <f>K161</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="192" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K192" s="34"/>
     </row>
     <row r="193" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>395</v>
       </c>
       <c r="F193" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="J193" t="s">
         <v>18</v>
       </c>
       <c r="K193" s="34">
-        <f>K165</f>
-        <v>11.7</v>
+        <f>K163</f>
+        <v>10</v>
       </c>
     </row>
     <row r="194" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A194" t="s">
-        <v>395</v>
-      </c>
-      <c r="F194" t="s">
-        <v>37</v>
-      </c>
-      <c r="J194" t="s">
-        <v>18</v>
-      </c>
-      <c r="K194" s="34">
-        <f>K164</f>
-        <v>13.2</v>
-      </c>
+      <c r="K194" s="34"/>
     </row>
     <row r="195" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>395</v>
       </c>
       <c r="F195" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J195" t="s">
         <v>18</v>
       </c>
       <c r="K195" s="34">
-        <f>K163</f>
-        <v>14.1</v>
+        <f>K167</f>
+        <v>11.7</v>
       </c>
     </row>
     <row r="196" spans="1:14" x14ac:dyDescent="0.25">
@@ -5392,13 +5416,13 @@
         <v>395</v>
       </c>
       <c r="F196" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="J196" t="s">
         <v>18</v>
       </c>
       <c r="K196" s="34">
-        <f t="shared" ref="K196:K202" si="14">K164</f>
+        <f>K166</f>
         <v>13.2</v>
       </c>
     </row>
@@ -5407,14 +5431,14 @@
         <v>395</v>
       </c>
       <c r="F197" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="J197" t="s">
         <v>18</v>
       </c>
       <c r="K197" s="34">
-        <f t="shared" si="14"/>
-        <v>11.7</v>
+        <f>K165</f>
+        <v>14.1</v>
       </c>
     </row>
     <row r="198" spans="1:14" x14ac:dyDescent="0.25">
@@ -5422,14 +5446,14 @@
         <v>395</v>
       </c>
       <c r="F198" t="s">
-        <v>314</v>
+        <v>49</v>
       </c>
       <c r="J198" t="s">
         <v>18</v>
       </c>
       <c r="K198" s="34">
-        <f t="shared" si="14"/>
-        <v>14</v>
+        <f t="shared" ref="K198:K204" si="14">K166</f>
+        <v>13.2</v>
       </c>
     </row>
     <row r="199" spans="1:14" x14ac:dyDescent="0.25">
@@ -5437,14 +5461,14 @@
         <v>395</v>
       </c>
       <c r="F199" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="J199" t="s">
         <v>18</v>
       </c>
       <c r="K199" s="34">
         <f t="shared" si="14"/>
-        <v>13.9</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="200" spans="1:14" x14ac:dyDescent="0.25">
@@ -5452,14 +5476,14 @@
         <v>395</v>
       </c>
       <c r="F200" t="s">
-        <v>52</v>
+        <v>314</v>
       </c>
       <c r="J200" t="s">
         <v>18</v>
       </c>
       <c r="K200" s="34">
         <f t="shared" si="14"/>
-        <v>12.8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="201" spans="1:14" x14ac:dyDescent="0.25">
@@ -5467,14 +5491,14 @@
         <v>395</v>
       </c>
       <c r="F201" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="J201" t="s">
         <v>18</v>
       </c>
       <c r="K201" s="34">
         <f t="shared" si="14"/>
-        <v>13.8</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="202" spans="1:14" x14ac:dyDescent="0.25">
@@ -5482,92 +5506,86 @@
         <v>395</v>
       </c>
       <c r="F202" t="s">
-        <v>319</v>
+        <v>52</v>
       </c>
       <c r="J202" t="s">
         <v>18</v>
       </c>
       <c r="K202" s="34">
         <f t="shared" si="14"/>
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="203" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>395</v>
+      </c>
+      <c r="F203" t="s">
+        <v>56</v>
+      </c>
+      <c r="J203" t="s">
+        <v>18</v>
+      </c>
+      <c r="K203" s="34">
+        <f t="shared" si="14"/>
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="204" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>395</v>
+      </c>
+      <c r="F204" t="s">
+        <v>319</v>
+      </c>
+      <c r="J204" t="s">
+        <v>18</v>
+      </c>
+      <c r="K204" s="34">
+        <f t="shared" si="14"/>
         <v>13.3</v>
       </c>
     </row>
-    <row r="203" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K203" s="3"/>
-    </row>
-    <row r="204" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A204" s="8" t="s">
+    <row r="205" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K205" s="3"/>
+    </row>
+    <row r="206" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A206" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B204" s="8"/>
-      <c r="C204" s="9"/>
-      <c r="D204" s="9"/>
-      <c r="E204" s="9"/>
-      <c r="F204" s="9"/>
-      <c r="G204" s="9"/>
-      <c r="H204" s="9"/>
-      <c r="I204" s="9"/>
-      <c r="J204" s="9"/>
-      <c r="K204" s="9"/>
-      <c r="L204" s="9"/>
-      <c r="M204" s="9"/>
-      <c r="N204" s="9"/>
-    </row>
-    <row r="205" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A205" s="30" t="s">
+      <c r="B206" s="8"/>
+      <c r="C206" s="9"/>
+      <c r="D206" s="9"/>
+      <c r="E206" s="9"/>
+      <c r="F206" s="9"/>
+      <c r="G206" s="9"/>
+      <c r="H206" s="9"/>
+      <c r="I206" s="9"/>
+      <c r="J206" s="9"/>
+      <c r="K206" s="9"/>
+      <c r="L206" s="9"/>
+      <c r="M206" s="9"/>
+      <c r="N206" s="9"/>
+    </row>
+    <row r="207" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A207" s="30" t="s">
         <v>391</v>
       </c>
-      <c r="B205" s="31"/>
-      <c r="C205" s="32"/>
-      <c r="D205" s="32"/>
-      <c r="E205" s="32"/>
-      <c r="F205" s="32"/>
-      <c r="G205" s="32"/>
-      <c r="H205" s="32"/>
-      <c r="I205" s="32"/>
-      <c r="J205" s="32"/>
-      <c r="K205" s="32"/>
-      <c r="L205" s="32" t="s">
+      <c r="B207" s="31"/>
+      <c r="C207" s="32"/>
+      <c r="D207" s="32"/>
+      <c r="E207" s="32"/>
+      <c r="F207" s="32"/>
+      <c r="G207" s="32"/>
+      <c r="H207" s="32"/>
+      <c r="I207" s="32"/>
+      <c r="J207" s="32"/>
+      <c r="K207" s="32"/>
+      <c r="L207" s="32" t="s">
         <v>300</v>
       </c>
-      <c r="M205" s="32"/>
-      <c r="N205" s="32"/>
-    </row>
-    <row r="206" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A206" t="s">
-        <v>25</v>
-      </c>
-      <c r="E206" t="s">
-        <v>299</v>
-      </c>
-      <c r="F206" t="s">
-        <v>17</v>
-      </c>
-      <c r="J206" t="s">
-        <v>18</v>
-      </c>
-      <c r="K206" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F206,'feed pars'!B$6:B$43,0))</f>
-        <v>12.3</v>
-      </c>
-    </row>
-    <row r="207" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A207" t="s">
-        <v>25</v>
-      </c>
-      <c r="E207" t="s">
-        <v>299</v>
-      </c>
-      <c r="F207" t="s">
-        <v>37</v>
-      </c>
-      <c r="J207" t="s">
-        <v>18</v>
-      </c>
-      <c r="K207" s="26">
-        <f>INDEX('feed pars'!H$6:H$43,MATCH(F207,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
-      </c>
+      <c r="M207" s="32"/>
+      <c r="N207" s="32"/>
     </row>
     <row r="208" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
@@ -5577,14 +5595,14 @@
         <v>299</v>
       </c>
       <c r="F208" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="J208" t="s">
         <v>18</v>
       </c>
       <c r="K208" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F208,'feed pars'!B$6:B$43,0))</f>
-        <v>9.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="209" spans="1:11" x14ac:dyDescent="0.25">
@@ -5595,14 +5613,14 @@
         <v>299</v>
       </c>
       <c r="F209" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J209" t="s">
         <v>18</v>
       </c>
       <c r="K209" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F209,'feed pars'!B$6:B$43,0))</f>
-        <v>12</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="210" spans="1:11" x14ac:dyDescent="0.25">
@@ -5613,14 +5631,14 @@
         <v>299</v>
       </c>
       <c r="F210" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J210" t="s">
         <v>18</v>
       </c>
       <c r="K210" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F210,'feed pars'!B$6:B$43,0))</f>
-        <v>13.2</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="211" spans="1:11" x14ac:dyDescent="0.25">
@@ -5631,14 +5649,14 @@
         <v>299</v>
       </c>
       <c r="F211" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="J211" t="s">
         <v>18</v>
       </c>
       <c r="K211" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F211,'feed pars'!B$6:B$43,0))</f>
-        <v>11.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="212" spans="1:11" x14ac:dyDescent="0.25">
@@ -5649,14 +5667,14 @@
         <v>299</v>
       </c>
       <c r="F212" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J212" t="s">
         <v>18</v>
       </c>
       <c r="K212" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F212,'feed pars'!B$6:B$43,0))</f>
-        <v>10.9</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="213" spans="1:11" x14ac:dyDescent="0.25">
@@ -5667,14 +5685,14 @@
         <v>299</v>
       </c>
       <c r="F213" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="J213" t="s">
         <v>18</v>
       </c>
       <c r="K213" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F213,'feed pars'!B$6:B$43,0))</f>
-        <v>18.5</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="214" spans="1:11" x14ac:dyDescent="0.25">
@@ -5685,14 +5703,14 @@
         <v>299</v>
       </c>
       <c r="F214" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J214" t="s">
         <v>18</v>
       </c>
       <c r="K214" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F214,'feed pars'!B$6:B$43,0))</f>
-        <v>17.5</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="215" spans="1:11" x14ac:dyDescent="0.25">
@@ -5703,14 +5721,14 @@
         <v>299</v>
       </c>
       <c r="F215" t="s">
-        <v>314</v>
+        <v>35</v>
       </c>
       <c r="J215" t="s">
         <v>18</v>
       </c>
       <c r="K215" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F215,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="216" spans="1:11" x14ac:dyDescent="0.25">
@@ -5721,14 +5739,14 @@
         <v>299</v>
       </c>
       <c r="F216" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J216" t="s">
         <v>18</v>
       </c>
       <c r="K216" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F216,'feed pars'!B$6:B$43,0))</f>
-        <v>9.9</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="217" spans="1:11" x14ac:dyDescent="0.25">
@@ -5739,14 +5757,14 @@
         <v>299</v>
       </c>
       <c r="F217" t="s">
-        <v>45</v>
+        <v>314</v>
       </c>
       <c r="J217" t="s">
         <v>18</v>
       </c>
       <c r="K217" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F217,'feed pars'!B$6:B$43,0))</f>
-        <v>10.3</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="218" spans="1:11" x14ac:dyDescent="0.25">
@@ -5757,14 +5775,14 @@
         <v>299</v>
       </c>
       <c r="F218" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="J218" t="s">
         <v>18</v>
       </c>
       <c r="K218" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F218,'feed pars'!B$6:B$43,0))</f>
-        <v>7.7</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="219" spans="1:11" x14ac:dyDescent="0.25">
@@ -5775,14 +5793,14 @@
         <v>299</v>
       </c>
       <c r="F219" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J219" t="s">
         <v>18</v>
       </c>
       <c r="K219" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F219,'feed pars'!B$6:B$43,0))</f>
-        <v>6.5</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="220" spans="1:11" x14ac:dyDescent="0.25">
@@ -5793,14 +5811,14 @@
         <v>299</v>
       </c>
       <c r="F220" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="J220" t="s">
         <v>18</v>
       </c>
       <c r="K220" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F220,'feed pars'!B$6:B$43,0))</f>
-        <v>6.2</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="221" spans="1:11" x14ac:dyDescent="0.25">
@@ -5811,14 +5829,14 @@
         <v>299</v>
       </c>
       <c r="F221" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J221" t="s">
         <v>18</v>
       </c>
       <c r="K221" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F221,'feed pars'!B$6:B$43,0))</f>
-        <v>7.8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="222" spans="1:11" x14ac:dyDescent="0.25">
@@ -5829,14 +5847,14 @@
         <v>299</v>
       </c>
       <c r="F222" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J222" t="s">
         <v>18</v>
       </c>
       <c r="K222" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F222,'feed pars'!B$6:B$43,0))</f>
-        <v>9.1999999999999993</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="223" spans="1:11" x14ac:dyDescent="0.25">
@@ -5847,14 +5865,14 @@
         <v>299</v>
       </c>
       <c r="F223" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J223" t="s">
         <v>18</v>
       </c>
       <c r="K223" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F223,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="224" spans="1:11" x14ac:dyDescent="0.25">
@@ -5865,14 +5883,14 @@
         <v>299</v>
       </c>
       <c r="F224" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J224" t="s">
         <v>18</v>
       </c>
       <c r="K224" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F224,'feed pars'!B$6:B$43,0))</f>
-        <v>8.9</v>
+        <v>9.1999999999999993</v>
       </c>
     </row>
     <row r="225" spans="1:14" x14ac:dyDescent="0.25">
@@ -5883,14 +5901,14 @@
         <v>299</v>
       </c>
       <c r="F225" t="s">
-        <v>313</v>
+        <v>50</v>
       </c>
       <c r="J225" t="s">
         <v>18</v>
       </c>
       <c r="K225" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F225,'feed pars'!B$6:B$43,0))</f>
-        <v>7.0888888888888877</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="226" spans="1:14" x14ac:dyDescent="0.25">
@@ -5901,14 +5919,14 @@
         <v>299</v>
       </c>
       <c r="F226" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J226" t="s">
         <v>18</v>
       </c>
       <c r="K226" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F226,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="227" spans="1:14" x14ac:dyDescent="0.25">
@@ -5919,14 +5937,14 @@
         <v>299</v>
       </c>
       <c r="F227" t="s">
-        <v>53</v>
+        <v>313</v>
       </c>
       <c r="J227" t="s">
         <v>18</v>
       </c>
       <c r="K227" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F227,'feed pars'!B$6:B$43,0))</f>
-        <v>8</v>
+        <v>7.0888888888888877</v>
       </c>
     </row>
     <row r="228" spans="1:14" x14ac:dyDescent="0.25">
@@ -5937,14 +5955,14 @@
         <v>299</v>
       </c>
       <c r="F228" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J228" t="s">
         <v>18</v>
       </c>
       <c r="K228" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F228,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="229" spans="1:14" x14ac:dyDescent="0.25">
@@ -5955,14 +5973,14 @@
         <v>299</v>
       </c>
       <c r="F229" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J229" t="s">
         <v>18</v>
       </c>
       <c r="K229" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F229,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="230" spans="1:14" x14ac:dyDescent="0.25">
@@ -5973,14 +5991,14 @@
         <v>299</v>
       </c>
       <c r="F230" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J230" t="s">
         <v>18</v>
       </c>
       <c r="K230" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F230,'feed pars'!B$6:B$43,0))</f>
-        <v>11.3</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="231" spans="1:14" x14ac:dyDescent="0.25">
@@ -5991,79 +6009,85 @@
         <v>299</v>
       </c>
       <c r="F231" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J231" t="s">
         <v>18</v>
       </c>
       <c r="K231" s="26">
         <f>INDEX('feed pars'!H$6:H$43,MATCH(F231,'feed pars'!B$6:B$43,0))</f>
-        <v>10.8</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="232" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A232" s="30" t="s">
-        <v>392</v>
-      </c>
-      <c r="B232" s="31"/>
-      <c r="C232" s="32"/>
-      <c r="D232" s="32"/>
-      <c r="E232" s="32"/>
-      <c r="F232" s="32"/>
-      <c r="G232" s="32"/>
-      <c r="H232" s="32"/>
-      <c r="I232" s="32"/>
-      <c r="J232" s="32"/>
-      <c r="K232" s="32"/>
-      <c r="L232" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="M232" s="32"/>
-      <c r="N232" s="32"/>
+      <c r="A232" t="s">
+        <v>25</v>
+      </c>
+      <c r="E232" t="s">
+        <v>299</v>
+      </c>
+      <c r="F232" t="s">
+        <v>56</v>
+      </c>
+      <c r="J232" t="s">
+        <v>18</v>
+      </c>
+      <c r="K232" s="26">
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F232,'feed pars'!B$6:B$43,0))</f>
+        <v>11.3</v>
+      </c>
     </row>
     <row r="233" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>25</v>
       </c>
+      <c r="E233" t="s">
+        <v>299</v>
+      </c>
       <c r="F233" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="J233" t="s">
         <v>18</v>
       </c>
       <c r="K233" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F233,'feed pars'!B$6:B$43,0))</f>
-        <v>12.1</v>
+        <f>INDEX('feed pars'!H$6:H$43,MATCH(F233,'feed pars'!B$6:B$43,0))</f>
+        <v>10.8</v>
       </c>
     </row>
     <row r="234" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A234" t="s">
-        <v>25</v>
-      </c>
-      <c r="F234" t="s">
-        <v>37</v>
-      </c>
-      <c r="J234" t="s">
-        <v>18</v>
-      </c>
-      <c r="K234" s="26">
-        <f>INDEX('feed pars'!G$6:G$43,MATCH(F234,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
-      </c>
+      <c r="A234" s="30" t="s">
+        <v>392</v>
+      </c>
+      <c r="B234" s="31"/>
+      <c r="C234" s="32"/>
+      <c r="D234" s="32"/>
+      <c r="E234" s="32"/>
+      <c r="F234" s="32"/>
+      <c r="G234" s="32"/>
+      <c r="H234" s="32"/>
+      <c r="I234" s="32"/>
+      <c r="J234" s="32"/>
+      <c r="K234" s="32"/>
+      <c r="L234" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="M234" s="32"/>
+      <c r="N234" s="32"/>
     </row>
     <row r="235" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>25</v>
       </c>
       <c r="F235" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="J235" t="s">
         <v>18</v>
       </c>
       <c r="K235" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F235,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="236" spans="1:14" x14ac:dyDescent="0.25">
@@ -6071,14 +6095,14 @@
         <v>25</v>
       </c>
       <c r="F236" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J236" t="s">
         <v>18</v>
       </c>
       <c r="K236" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F236,'feed pars'!B$6:B$43,0))</f>
-        <v>11.9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="237" spans="1:14" x14ac:dyDescent="0.25">
@@ -6086,14 +6110,14 @@
         <v>25</v>
       </c>
       <c r="F237" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J237" t="s">
         <v>18</v>
       </c>
       <c r="K237" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F237,'feed pars'!B$6:B$43,0))</f>
-        <v>12.8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="238" spans="1:14" x14ac:dyDescent="0.25">
@@ -6101,14 +6125,14 @@
         <v>25</v>
       </c>
       <c r="F238" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="J238" t="s">
         <v>18</v>
       </c>
       <c r="K238" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F238,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="239" spans="1:14" x14ac:dyDescent="0.25">
@@ -6116,14 +6140,14 @@
         <v>25</v>
       </c>
       <c r="F239" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J239" t="s">
         <v>18</v>
       </c>
       <c r="K239" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F239,'feed pars'!B$6:B$43,0))</f>
-        <v>10.7</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="240" spans="1:14" x14ac:dyDescent="0.25">
@@ -6131,14 +6155,14 @@
         <v>25</v>
       </c>
       <c r="F240" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="J240" t="s">
         <v>18</v>
       </c>
       <c r="K240" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F240,'feed pars'!B$6:B$43,0))</f>
-        <v>18</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="241" spans="1:11" x14ac:dyDescent="0.25">
@@ -6146,14 +6170,14 @@
         <v>25</v>
       </c>
       <c r="F241" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J241" t="s">
         <v>18</v>
       </c>
       <c r="K241" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F241,'feed pars'!B$6:B$43,0))</f>
-        <v>17.3</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="242" spans="1:11" x14ac:dyDescent="0.25">
@@ -6161,14 +6185,14 @@
         <v>25</v>
       </c>
       <c r="F242" t="s">
-        <v>314</v>
+        <v>35</v>
       </c>
       <c r="J242" t="s">
         <v>18</v>
       </c>
       <c r="K242" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F242,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="243" spans="1:11" x14ac:dyDescent="0.25">
@@ -6176,14 +6200,14 @@
         <v>25</v>
       </c>
       <c r="F243" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J243" t="s">
         <v>18</v>
       </c>
       <c r="K243" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F243,'feed pars'!B$6:B$43,0))</f>
-        <v>9.3000000000000007</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="244" spans="1:11" x14ac:dyDescent="0.25">
@@ -6191,14 +6215,14 @@
         <v>25</v>
       </c>
       <c r="F244" t="s">
-        <v>45</v>
+        <v>314</v>
       </c>
       <c r="J244" t="s">
         <v>18</v>
       </c>
       <c r="K244" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F244,'feed pars'!B$6:B$43,0))</f>
-        <v>9.6999999999999993</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="245" spans="1:11" x14ac:dyDescent="0.25">
@@ -6206,14 +6230,14 @@
         <v>25</v>
       </c>
       <c r="F245" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="J245" t="s">
         <v>18</v>
       </c>
       <c r="K245" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F245,'feed pars'!B$6:B$43,0))</f>
-        <v>7.1</v>
+        <v>9.3000000000000007</v>
       </c>
     </row>
     <row r="246" spans="1:11" x14ac:dyDescent="0.25">
@@ -6221,14 +6245,14 @@
         <v>25</v>
       </c>
       <c r="F246" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J246" t="s">
         <v>18</v>
       </c>
       <c r="K246" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F246,'feed pars'!B$6:B$43,0))</f>
-        <v>5.9</v>
+        <v>9.6999999999999993</v>
       </c>
     </row>
     <row r="247" spans="1:11" x14ac:dyDescent="0.25">
@@ -6236,14 +6260,14 @@
         <v>25</v>
       </c>
       <c r="F247" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="J247" t="s">
         <v>18</v>
       </c>
       <c r="K247" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F247,'feed pars'!B$6:B$43,0))</f>
-        <v>5.4</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="248" spans="1:11" x14ac:dyDescent="0.25">
@@ -6251,14 +6275,14 @@
         <v>25</v>
       </c>
       <c r="F248" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J248" t="s">
         <v>18</v>
       </c>
       <c r="K248" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F248,'feed pars'!B$6:B$43,0))</f>
-        <v>7.2</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="249" spans="1:11" x14ac:dyDescent="0.25">
@@ -6266,14 +6290,14 @@
         <v>25</v>
       </c>
       <c r="F249" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J249" t="s">
         <v>18</v>
       </c>
       <c r="K249" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F249,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="250" spans="1:11" x14ac:dyDescent="0.25">
@@ -6281,14 +6305,14 @@
         <v>25</v>
       </c>
       <c r="F250" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J250" t="s">
         <v>18</v>
       </c>
       <c r="K250" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F250,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="251" spans="1:11" x14ac:dyDescent="0.25">
@@ -6296,14 +6320,14 @@
         <v>25</v>
       </c>
       <c r="F251" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J251" t="s">
         <v>18</v>
       </c>
       <c r="K251" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F251,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1999999999999993</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="252" spans="1:11" x14ac:dyDescent="0.25">
@@ -6311,14 +6335,14 @@
         <v>25</v>
       </c>
       <c r="F252" t="s">
-        <v>313</v>
+        <v>50</v>
       </c>
       <c r="J252" t="s">
         <v>18</v>
       </c>
       <c r="K252" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F252,'feed pars'!B$6:B$43,0))</f>
-        <v>6.6</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="253" spans="1:11" x14ac:dyDescent="0.25">
@@ -6326,14 +6350,14 @@
         <v>25</v>
       </c>
       <c r="F253" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J253" t="s">
         <v>18</v>
       </c>
       <c r="K253" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F253,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
+        <v>8.1999999999999993</v>
       </c>
     </row>
     <row r="254" spans="1:11" x14ac:dyDescent="0.25">
@@ -6341,14 +6365,14 @@
         <v>25</v>
       </c>
       <c r="F254" t="s">
-        <v>53</v>
+        <v>313</v>
       </c>
       <c r="J254" t="s">
         <v>18</v>
       </c>
       <c r="K254" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F254,'feed pars'!B$6:B$43,0))</f>
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="255" spans="1:11" x14ac:dyDescent="0.25">
@@ -6356,14 +6380,14 @@
         <v>25</v>
       </c>
       <c r="F255" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J255" t="s">
         <v>18</v>
       </c>
       <c r="K255" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F255,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="256" spans="1:11" x14ac:dyDescent="0.25">
@@ -6371,14 +6395,14 @@
         <v>25</v>
       </c>
       <c r="F256" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J256" t="s">
         <v>18</v>
       </c>
       <c r="K256" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F256,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="257" spans="1:11" x14ac:dyDescent="0.25">
@@ -6386,14 +6410,14 @@
         <v>25</v>
       </c>
       <c r="F257" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J257" t="s">
         <v>18</v>
       </c>
       <c r="K257" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F257,'feed pars'!B$6:B$43,0))</f>
-        <v>11.1</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="258" spans="1:11" x14ac:dyDescent="0.25">
@@ -6401,13 +6425,43 @@
         <v>25</v>
       </c>
       <c r="F258" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J258" t="s">
         <v>18</v>
       </c>
       <c r="K258" s="26">
         <f>INDEX('feed pars'!G$6:G$43,MATCH(F258,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="259" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A259" t="s">
+        <v>25</v>
+      </c>
+      <c r="F259" t="s">
+        <v>56</v>
+      </c>
+      <c r="J259" t="s">
+        <v>18</v>
+      </c>
+      <c r="K259" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F259,'feed pars'!B$6:B$43,0))</f>
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="260" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A260" t="s">
+        <v>25</v>
+      </c>
+      <c r="F260" t="s">
+        <v>57</v>
+      </c>
+      <c r="J260" t="s">
+        <v>18</v>
+      </c>
+      <c r="K260" s="26">
+        <f>INDEX('feed pars'!G$6:G$43,MATCH(F260,'feed pars'!B$6:B$43,0))</f>
         <v>10.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implemented CH4 EFs for non-cattle as parameters
</commit_message>
<xml_diff>
--- a/data/prod_parameters/FeedMgmt.xlsx
+++ b/data/prod_parameters/FeedMgmt.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1523" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1544" uniqueCount="513">
   <si>
     <t>f_feed</t>
   </si>
@@ -1567,6 +1567,39 @@
   </si>
   <si>
     <t>Total fat</t>
+  </si>
+  <si>
+    <r>
+      <t>Enteric fermentation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (for cattle Ym is calculated from feed ration)</t>
+    </r>
+  </si>
+  <si>
+    <t>EF_enteric</t>
+  </si>
+  <si>
+    <t>Ym_enteric</t>
+  </si>
+  <si>
+    <t>NIR 2021</t>
+  </si>
+  <si>
+    <t>lambs</t>
+  </si>
+  <si>
+    <t>% of GE</t>
+  </si>
+  <si>
+    <t>kg CH4/head/year</t>
   </si>
 </sst>
 </file>
@@ -2300,7 +2333,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O330"/>
+  <dimension ref="A1:O336"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="20.28515625" customWidth="1"/>
@@ -4742,211 +4775,255 @@
       <c r="M118" s="26"/>
     </row>
     <row r="119" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K119" s="3"/>
-      <c r="M119" s="3"/>
+      <c r="A119" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="B119" s="1"/>
+      <c r="C119" s="1"/>
+      <c r="D119" s="1"/>
+      <c r="E119" s="2"/>
+      <c r="F119" s="2"/>
+      <c r="G119" s="2"/>
+      <c r="H119" s="2"/>
+      <c r="I119" s="2"/>
+      <c r="J119" s="2"/>
+      <c r="K119" s="2"/>
+      <c r="L119" s="2"/>
+      <c r="M119" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="N119" s="2"/>
     </row>
     <row r="120" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A120" s="1" t="s">
+      <c r="A120" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="B120" s="3"/>
+      <c r="C120" s="3"/>
+      <c r="D120" s="3"/>
+      <c r="E120" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="F120" s="3"/>
+      <c r="G120" s="3"/>
+      <c r="H120" s="3"/>
+      <c r="I120" s="3"/>
+      <c r="J120" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="K120" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="L120" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="M120" s="3"/>
+    </row>
+    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A121" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="B121" s="3"/>
+      <c r="C121" s="3"/>
+      <c r="D121" s="3"/>
+      <c r="E121" s="3"/>
+      <c r="F121" s="3"/>
+      <c r="G121" s="3"/>
+      <c r="H121" s="3"/>
+      <c r="I121" s="3"/>
+      <c r="J121" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="K121" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="L121" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="M121" s="3"/>
+    </row>
+    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>391</v>
+      </c>
+      <c r="J122" t="s">
+        <v>507</v>
+      </c>
+      <c r="K122" s="26">
+        <v>18</v>
+      </c>
+      <c r="L122" t="s">
+        <v>512</v>
+      </c>
+      <c r="M122" s="3"/>
+      <c r="N122" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>25</v>
+      </c>
+      <c r="J123" t="s">
+        <v>507</v>
+      </c>
+      <c r="K123" s="26">
+        <v>1.5</v>
+      </c>
+      <c r="L123" t="s">
+        <v>512</v>
+      </c>
+      <c r="M123" s="3"/>
+      <c r="N123" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>385</v>
+      </c>
+      <c r="J124" t="s">
+        <v>507</v>
+      </c>
+      <c r="K124" s="26">
+        <v>0</v>
+      </c>
+      <c r="L124" t="s">
+        <v>512</v>
+      </c>
+      <c r="M124" s="3"/>
+      <c r="N124" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K125" s="3"/>
+      <c r="M125" s="3"/>
+    </row>
+    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A126" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B120" s="1"/>
-      <c r="C120" s="1"/>
-      <c r="D120" s="1"/>
-      <c r="E120" s="2"/>
-      <c r="F120" s="2"/>
-      <c r="G120" s="2"/>
-      <c r="H120" s="2"/>
-      <c r="I120" s="2"/>
-      <c r="J120" s="2"/>
-      <c r="K120" s="2"/>
-      <c r="L120" s="2"/>
-      <c r="M120" s="2" t="s">
+      <c r="B126" s="1"/>
+      <c r="C126" s="1"/>
+      <c r="D126" s="1"/>
+      <c r="E126" s="2"/>
+      <c r="F126" s="2"/>
+      <c r="G126" s="2"/>
+      <c r="H126" s="2"/>
+      <c r="I126" s="2"/>
+      <c r="J126" s="2"/>
+      <c r="K126" s="2"/>
+      <c r="L126" s="2"/>
+      <c r="M126" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="N120" s="2"/>
-    </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A121" s="79" t="s">
+      <c r="N126" s="2"/>
+    </row>
+    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A127" s="79" t="s">
         <v>496</v>
       </c>
-      <c r="B121" s="80"/>
-      <c r="C121" s="80"/>
-      <c r="D121" s="80"/>
-      <c r="E121" s="81"/>
-      <c r="F121" s="81"/>
-      <c r="G121" s="81"/>
-      <c r="H121" s="81"/>
-      <c r="I121" s="81"/>
-      <c r="J121" s="81"/>
-      <c r="K121" s="81"/>
-      <c r="L121" s="81"/>
-      <c r="M121" s="81"/>
-      <c r="N121" s="81"/>
-    </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F122" t="s">
-        <v>306</v>
-      </c>
-      <c r="J122" t="s">
-        <v>386</v>
-      </c>
-      <c r="K122" s="82">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F122,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="L122" t="s">
-        <v>28</v>
-      </c>
-      <c r="M122" s="26" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F123" t="s">
-        <v>307</v>
-      </c>
-      <c r="J123" t="s">
-        <v>386</v>
-      </c>
-      <c r="K123" s="82">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F123,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="M123" s="3"/>
-    </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F124" t="s">
-        <v>308</v>
-      </c>
-      <c r="J124" t="s">
-        <v>386</v>
-      </c>
-      <c r="K124" s="82">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F124,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="M124" s="3"/>
-    </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F125" t="s">
-        <v>2</v>
-      </c>
-      <c r="J125" t="s">
-        <v>386</v>
-      </c>
-      <c r="K125" s="82">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F125,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="M125" s="3"/>
-    </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F126" t="s">
-        <v>12</v>
-      </c>
-      <c r="J126" t="s">
-        <v>386</v>
-      </c>
-      <c r="K126" s="82">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F126,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="M126" s="3"/>
-    </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F127" t="s">
-        <v>33</v>
-      </c>
-      <c r="J127" t="s">
-        <v>386</v>
-      </c>
-      <c r="K127" s="82">
-        <f>INDEX('feed pars'!C$6:C$43,MATCH(F127,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
-      </c>
-      <c r="M127" s="3"/>
+      <c r="B127" s="80"/>
+      <c r="C127" s="80"/>
+      <c r="D127" s="80"/>
+      <c r="E127" s="81"/>
+      <c r="F127" s="81"/>
+      <c r="G127" s="81"/>
+      <c r="H127" s="81"/>
+      <c r="I127" s="81"/>
+      <c r="J127" s="81"/>
+      <c r="K127" s="81"/>
+      <c r="L127" s="81"/>
+      <c r="M127" s="81"/>
+      <c r="N127" s="81"/>
     </row>
     <row r="128" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F128" t="s">
-        <v>17</v>
+        <v>306</v>
       </c>
       <c r="J128" t="s">
         <v>386</v>
       </c>
       <c r="K128" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F128,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
-      </c>
-      <c r="M128" s="3"/>
+        <v>100</v>
+      </c>
+      <c r="L128" t="s">
+        <v>28</v>
+      </c>
+      <c r="M128" s="26" t="s">
+        <v>389</v>
+      </c>
     </row>
     <row r="129" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F129" t="s">
-        <v>37</v>
+        <v>307</v>
       </c>
       <c r="J129" t="s">
         <v>386</v>
       </c>
       <c r="K129" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F129,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="M129" s="3"/>
     </row>
     <row r="130" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F130" t="s">
-        <v>38</v>
+        <v>308</v>
       </c>
       <c r="J130" t="s">
         <v>386</v>
       </c>
       <c r="K130" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F130,'feed pars'!B$6:B$43,0))</f>
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="M130" s="3"/>
     </row>
     <row r="131" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F131" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="J131" t="s">
         <v>386</v>
       </c>
       <c r="K131" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F131,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="M131" s="3"/>
     </row>
     <row r="132" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F132" t="s">
-        <v>313</v>
+        <v>12</v>
       </c>
       <c r="J132" t="s">
         <v>386</v>
       </c>
       <c r="K132" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F132,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="M132" s="3"/>
     </row>
     <row r="133" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F133" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="J133" t="s">
         <v>386</v>
       </c>
       <c r="K133" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F133,'feed pars'!B$6:B$43,0))</f>
-        <v>67.5</v>
+        <v>100</v>
       </c>
       <c r="M133" s="3"/>
     </row>
     <row r="134" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F134" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="J134" t="s">
         <v>386</v>
@@ -4959,72 +5036,72 @@
     </row>
     <row r="135" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F135" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="J135" t="s">
         <v>386</v>
       </c>
       <c r="K135" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F135,'feed pars'!B$6:B$43,0))</f>
-        <v>86.8</v>
+        <v>87</v>
       </c>
       <c r="M135" s="3"/>
     </row>
     <row r="136" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F136" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J136" t="s">
         <v>386</v>
       </c>
       <c r="K136" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F136,'feed pars'!B$6:B$43,0))</f>
-        <v>92.5</v>
+        <v>86</v>
       </c>
       <c r="M136" s="3"/>
     </row>
     <row r="137" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F137" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="J137" t="s">
         <v>386</v>
       </c>
       <c r="K137" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F137,'feed pars'!B$6:B$43,0))</f>
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="M137" s="3"/>
     </row>
     <row r="138" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F138" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J138" t="s">
         <v>386</v>
       </c>
       <c r="K138" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F138,'feed pars'!B$6:B$43,0))</f>
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="M138" s="3"/>
     </row>
     <row r="139" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F139" t="s">
-        <v>302</v>
+        <v>40</v>
       </c>
       <c r="J139" t="s">
         <v>386</v>
       </c>
       <c r="K139" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F139,'feed pars'!B$6:B$43,0))</f>
-        <v>85</v>
+        <v>67.5</v>
       </c>
       <c r="M139" s="3"/>
     </row>
     <row r="140" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F140" t="s">
-        <v>314</v>
+        <v>41</v>
       </c>
       <c r="J140" t="s">
         <v>386</v>
@@ -5037,877 +5114,863 @@
     </row>
     <row r="141" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F141" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J141" t="s">
         <v>386</v>
       </c>
       <c r="K141" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F141,'feed pars'!B$6:B$43,0))</f>
-        <v>87.5</v>
+        <v>86.8</v>
       </c>
       <c r="M141" s="3"/>
     </row>
     <row r="142" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F142" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="J142" t="s">
         <v>386</v>
       </c>
       <c r="K142" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F142,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>92.5</v>
       </c>
       <c r="M142" s="3"/>
     </row>
     <row r="143" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F143" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="J143" t="s">
         <v>386</v>
       </c>
       <c r="K143" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F143,'feed pars'!B$6:B$43,0))</f>
-        <v>89.5</v>
+        <v>92</v>
       </c>
       <c r="M143" s="3"/>
     </row>
     <row r="144" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F144" t="s">
-        <v>46</v>
+        <v>310</v>
       </c>
       <c r="J144" t="s">
         <v>386</v>
       </c>
       <c r="K144" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F144,'feed pars'!B$6:B$43,0))</f>
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="M144" s="3"/>
     </row>
     <row r="145" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F145" t="s">
-        <v>47</v>
+        <v>302</v>
       </c>
       <c r="J145" t="s">
         <v>386</v>
       </c>
       <c r="K145" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F145,'feed pars'!B$6:B$43,0))</f>
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="M145" s="3"/>
     </row>
     <row r="146" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F146" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J146" t="s">
         <v>386</v>
       </c>
       <c r="K146" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F146,'feed pars'!B$6:B$43,0))</f>
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="M146" s="3"/>
     </row>
     <row r="147" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F147" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="J147" t="s">
         <v>386</v>
       </c>
       <c r="K147" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F147,'feed pars'!B$6:B$43,0))</f>
-        <v>87</v>
+        <v>87.5</v>
       </c>
       <c r="M147" s="3"/>
     </row>
     <row r="148" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F148" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="J148" t="s">
         <v>386</v>
       </c>
       <c r="K148" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F148,'feed pars'!B$6:B$43,0))</f>
-        <v>88.5</v>
+        <v>87</v>
       </c>
       <c r="M148" s="3"/>
     </row>
     <row r="149" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F149" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="J149" t="s">
         <v>386</v>
       </c>
       <c r="K149" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F149,'feed pars'!B$6:B$43,0))</f>
-        <v>90</v>
+        <v>89.5</v>
       </c>
       <c r="M149" s="3"/>
     </row>
     <row r="150" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F150" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="J150" t="s">
         <v>386</v>
       </c>
       <c r="K150" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F150,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
+        <v>91</v>
       </c>
       <c r="M150" s="3"/>
     </row>
     <row r="151" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F151" t="s">
-        <v>309</v>
+        <v>47</v>
       </c>
       <c r="J151" t="s">
         <v>386</v>
       </c>
       <c r="K151" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F151,'feed pars'!B$6:B$43,0))</f>
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="M151" s="3"/>
     </row>
     <row r="152" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F152" t="s">
-        <v>384</v>
+        <v>315</v>
       </c>
       <c r="J152" t="s">
         <v>386</v>
       </c>
       <c r="K152" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F152,'feed pars'!B$6:B$43,0))</f>
-        <v>88.5</v>
+        <v>90</v>
       </c>
       <c r="M152" s="3"/>
     </row>
     <row r="153" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F153" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="J153" t="s">
         <v>386</v>
       </c>
       <c r="K153" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F153,'feed pars'!B$6:B$43,0))</f>
-        <v>75.5</v>
+        <v>87</v>
       </c>
       <c r="M153" s="3"/>
     </row>
     <row r="154" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F154" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="J154" t="s">
         <v>386</v>
       </c>
       <c r="K154" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F154,'feed pars'!B$6:B$43,0))</f>
-        <v>89.5</v>
+        <v>88.5</v>
       </c>
       <c r="M154" s="3"/>
     </row>
     <row r="155" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F155" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="J155" t="s">
         <v>386</v>
       </c>
       <c r="K155" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F155,'feed pars'!B$6:B$43,0))</f>
-        <v>6.25</v>
+        <v>90</v>
       </c>
       <c r="M155" s="3"/>
     </row>
     <row r="156" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F156" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="J156" t="s">
         <v>386</v>
       </c>
       <c r="K156" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F156,'feed pars'!B$6:B$43,0))</f>
-        <v>97</v>
+        <v>11</v>
       </c>
       <c r="M156" s="3"/>
     </row>
     <row r="157" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F157" t="s">
-        <v>56</v>
+        <v>309</v>
       </c>
       <c r="J157" t="s">
         <v>386</v>
       </c>
       <c r="K157" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F157,'feed pars'!B$6:B$43,0))</f>
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M157" s="3"/>
     </row>
     <row r="158" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F158" t="s">
-        <v>57</v>
+        <v>384</v>
       </c>
       <c r="J158" t="s">
         <v>386</v>
       </c>
       <c r="K158" s="82">
         <f>INDEX('feed pars'!C$6:C$43,MATCH(F158,'feed pars'!B$6:B$43,0))</f>
-        <v>92</v>
+        <v>88.5</v>
       </c>
       <c r="M158" s="3"/>
     </row>
     <row r="159" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F159" t="s">
-        <v>320</v>
+        <v>52</v>
       </c>
       <c r="J159" t="s">
         <v>386</v>
       </c>
-      <c r="K159" s="86">
-        <v>100</v>
+      <c r="K159" s="82">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F159,'feed pars'!B$6:B$43,0))</f>
+        <v>75.5</v>
       </c>
       <c r="M159" s="3"/>
     </row>
     <row r="160" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F160" t="s">
-        <v>306</v>
+        <v>53</v>
       </c>
       <c r="J160" t="s">
-        <v>498</v>
-      </c>
-      <c r="K160" s="25">
-        <f>INDEX('feed pars'!D$6:D$43,MATCH(F160,'feed pars'!B$6:B$43,0))</f>
-        <v>17.316948400000001</v>
-      </c>
-      <c r="L160" t="s">
-        <v>497</v>
-      </c>
-      <c r="M160" s="26" t="s">
-        <v>499</v>
-      </c>
+        <v>386</v>
+      </c>
+      <c r="K160" s="82">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F160,'feed pars'!B$6:B$43,0))</f>
+        <v>89.5</v>
+      </c>
+      <c r="M160" s="3"/>
     </row>
     <row r="161" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F161" t="s">
-        <v>307</v>
+        <v>54</v>
       </c>
       <c r="J161" t="s">
-        <v>498</v>
-      </c>
-      <c r="K161" s="25">
-        <f>INDEX('feed pars'!D$6:D$43,MATCH(F161,'feed pars'!B$6:B$43,0))</f>
-        <v>17.150216</v>
+        <v>386</v>
+      </c>
+      <c r="K161" s="82">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F161,'feed pars'!B$6:B$43,0))</f>
+        <v>6.25</v>
       </c>
       <c r="M161" s="3"/>
     </row>
     <row r="162" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F162" t="s">
-        <v>308</v>
+        <v>55</v>
       </c>
       <c r="J162" t="s">
-        <v>498</v>
-      </c>
-      <c r="K162" s="25">
-        <f>INDEX('feed pars'!D$6:D$43,MATCH(F162,'feed pars'!B$6:B$43,0))</f>
-        <v>16.819680000000002</v>
+        <v>386</v>
+      </c>
+      <c r="K162" s="82">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F162,'feed pars'!B$6:B$43,0))</f>
+        <v>97</v>
       </c>
       <c r="M162" s="3"/>
     </row>
     <row r="163" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F163" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="J163" t="s">
-        <v>498</v>
-      </c>
-      <c r="K163" s="25">
-        <f>INDEX('feed pars'!D$6:D$43,MATCH(F163,'feed pars'!B$6:B$43,0))</f>
-        <v>17.160257599999998</v>
+        <v>386</v>
+      </c>
+      <c r="K163" s="82">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F163,'feed pars'!B$6:B$43,0))</f>
+        <v>91</v>
       </c>
       <c r="M163" s="3"/>
     </row>
     <row r="164" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F164" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="J164" t="s">
-        <v>498</v>
-      </c>
-      <c r="K164" s="25">
-        <f>INDEX('feed pars'!D$6:D$43,MATCH(F164,'feed pars'!B$6:B$43,0))</f>
-        <v>17.6573168</v>
+        <v>386</v>
+      </c>
+      <c r="K164" s="82">
+        <f>INDEX('feed pars'!C$6:C$43,MATCH(F164,'feed pars'!B$6:B$43,0))</f>
+        <v>92</v>
       </c>
       <c r="M164" s="3"/>
     </row>
     <row r="165" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F165" t="s">
-        <v>33</v>
+        <v>320</v>
       </c>
       <c r="J165" t="s">
-        <v>498</v>
-      </c>
-      <c r="K165" s="25">
-        <f>INDEX('feed pars'!D$6:D$43,MATCH(F165,'feed pars'!B$6:B$43,0))</f>
-        <v>17.411437066666668</v>
+        <v>386</v>
+      </c>
+      <c r="K165" s="86">
+        <v>100</v>
       </c>
       <c r="M165" s="3"/>
     </row>
     <row r="166" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F166" t="s">
-        <v>17</v>
+        <v>306</v>
       </c>
       <c r="J166" t="s">
         <v>498</v>
       </c>
       <c r="K166" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F166,'feed pars'!B$6:B$43,0))</f>
-        <v>18.210023200000002</v>
-      </c>
-      <c r="M166" s="3"/>
+        <v>17.316948400000001</v>
+      </c>
+      <c r="L166" t="s">
+        <v>497</v>
+      </c>
+      <c r="M166" s="26" t="s">
+        <v>499</v>
+      </c>
     </row>
     <row r="167" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F167" t="s">
-        <v>37</v>
+        <v>307</v>
       </c>
       <c r="J167" t="s">
         <v>498</v>
       </c>
       <c r="K167" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F167,'feed pars'!B$6:B$43,0))</f>
-        <v>18.089524000000001</v>
+        <v>17.150216</v>
       </c>
       <c r="M167" s="3"/>
     </row>
     <row r="168" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F168" t="s">
-        <v>38</v>
+        <v>308</v>
       </c>
       <c r="J168" t="s">
         <v>498</v>
       </c>
       <c r="K168" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F168,'feed pars'!B$6:B$43,0))</f>
-        <v>18.6602216</v>
+        <v>16.819680000000002</v>
       </c>
       <c r="M168" s="3"/>
     </row>
     <row r="169" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F169" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="J169" t="s">
         <v>498</v>
       </c>
       <c r="K169" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F169,'feed pars'!B$6:B$43,0))</f>
-        <v>18.2284328</v>
+        <v>17.160257599999998</v>
       </c>
       <c r="M169" s="3"/>
     </row>
     <row r="170" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F170" t="s">
-        <v>313</v>
+        <v>12</v>
       </c>
       <c r="J170" t="s">
         <v>498</v>
       </c>
       <c r="K170" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F170,'feed pars'!B$6:B$43,0))</f>
-        <v>17.924256</v>
+        <v>17.6573168</v>
       </c>
       <c r="M170" s="3"/>
     </row>
     <row r="171" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F171" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="J171" t="s">
         <v>498</v>
       </c>
       <c r="K171" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F171,'feed pars'!B$6:B$43,0))</f>
-        <v>18.3899352</v>
+        <v>17.411437066666668</v>
       </c>
       <c r="M171" s="3"/>
     </row>
     <row r="172" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F172" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="J172" t="s">
         <v>498</v>
       </c>
       <c r="K172" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F172,'feed pars'!B$6:B$43,0))</f>
-        <v>18.478217600000001</v>
+        <v>18.210023200000002</v>
       </c>
       <c r="M172" s="3"/>
     </row>
     <row r="173" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F173" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="J173" t="s">
         <v>498</v>
       </c>
       <c r="K173" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F173,'feed pars'!B$6:B$43,0))</f>
-        <v>18.737207199999997</v>
+        <v>18.089524000000001</v>
       </c>
       <c r="M173" s="3"/>
     </row>
     <row r="174" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F174" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J174" t="s">
         <v>498</v>
       </c>
       <c r="K174" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F174,'feed pars'!B$6:B$43,0))</f>
-        <v>27.903096000000001</v>
+        <v>18.6602216</v>
       </c>
       <c r="M174" s="3"/>
     </row>
     <row r="175" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F175" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="J175" t="s">
         <v>498</v>
       </c>
       <c r="K175" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F175,'feed pars'!B$6:B$43,0))</f>
-        <v>26.501456000000001</v>
+        <v>18.2284328</v>
       </c>
       <c r="M175" s="3"/>
     </row>
     <row r="176" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F176" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J176" t="s">
         <v>498</v>
       </c>
       <c r="K176" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F176,'feed pars'!B$6:B$43,0))</f>
-        <v>39.329599999999999</v>
+        <v>17.924256</v>
       </c>
       <c r="M176" s="3"/>
     </row>
     <row r="177" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F177" t="s">
-        <v>302</v>
+        <v>40</v>
       </c>
       <c r="J177" t="s">
         <v>498</v>
       </c>
       <c r="K177" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F177,'feed pars'!B$6:B$43,0))</f>
-        <v>16.927627199999996</v>
+        <v>18.3899352</v>
       </c>
       <c r="M177" s="3"/>
     </row>
     <row r="178" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F178" t="s">
-        <v>314</v>
+        <v>41</v>
       </c>
       <c r="J178" t="s">
         <v>498</v>
       </c>
       <c r="K178" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F178,'feed pars'!B$6:B$43,0))</f>
-        <v>22.965976000000001</v>
+        <v>18.478217600000001</v>
       </c>
       <c r="M178" s="3"/>
     </row>
     <row r="179" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F179" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J179" t="s">
         <v>498</v>
       </c>
       <c r="K179" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F179,'feed pars'!B$6:B$43,0))</f>
-        <v>19.589487999999999</v>
+        <v>18.737207199999997</v>
       </c>
       <c r="M179" s="3"/>
     </row>
     <row r="180" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F180" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="J180" t="s">
         <v>498</v>
       </c>
       <c r="K180" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F180,'feed pars'!B$6:B$43,0))</f>
-        <v>20.560594400000003</v>
+        <v>27.903096000000001</v>
       </c>
       <c r="M180" s="3"/>
     </row>
     <row r="181" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F181" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="J181" t="s">
         <v>498</v>
       </c>
       <c r="K181" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F181,'feed pars'!B$6:B$43,0))</f>
-        <v>19.4920008</v>
+        <v>26.501456000000001</v>
       </c>
       <c r="M181" s="3"/>
     </row>
     <row r="182" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F182" t="s">
-        <v>46</v>
+        <v>310</v>
       </c>
       <c r="J182" t="s">
         <v>498</v>
       </c>
       <c r="K182" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F182,'feed pars'!B$6:B$43,0))</f>
-        <v>19.083224000000001</v>
+        <v>39.329599999999999</v>
       </c>
       <c r="M182" s="3"/>
     </row>
     <row r="183" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F183" t="s">
-        <v>47</v>
+        <v>302</v>
       </c>
       <c r="J183" t="s">
         <v>498</v>
       </c>
       <c r="K183" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F183,'feed pars'!B$6:B$43,0))</f>
-        <v>19.581538399999999</v>
+        <v>16.927627199999996</v>
       </c>
       <c r="M183" s="3"/>
     </row>
     <row r="184" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F184" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J184" t="s">
         <v>498</v>
       </c>
       <c r="K184" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F184,'feed pars'!B$6:B$43,0))</f>
-        <v>16.971140800000001</v>
+        <v>22.965976000000001</v>
       </c>
       <c r="M184" s="3"/>
     </row>
     <row r="185" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F185" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="J185" t="s">
         <v>498</v>
       </c>
       <c r="K185" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F185,'feed pars'!B$6:B$43,0))</f>
-        <v>18.194124000000002</v>
+        <v>19.589487999999999</v>
       </c>
       <c r="M185" s="3"/>
     </row>
     <row r="186" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F186" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="J186" t="s">
         <v>498</v>
       </c>
       <c r="K186" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F186,'feed pars'!B$6:B$43,0))</f>
-        <v>17.8828344</v>
+        <v>20.560594400000003</v>
       </c>
       <c r="M186" s="3"/>
     </row>
     <row r="187" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F187" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="J187" t="s">
         <v>498</v>
       </c>
       <c r="K187" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F187,'feed pars'!B$6:B$43,0))</f>
-        <v>19.659779199999999</v>
+        <v>19.4920008</v>
       </c>
       <c r="M187" s="3"/>
     </row>
     <row r="188" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F188" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="J188" t="s">
         <v>498</v>
       </c>
       <c r="K188" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F188,'feed pars'!B$6:B$43,0))</f>
-        <v>18.8602168</v>
+        <v>19.083224000000001</v>
       </c>
       <c r="M188" s="3"/>
     </row>
     <row r="189" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F189" t="s">
-        <v>309</v>
+        <v>47</v>
       </c>
       <c r="J189" t="s">
         <v>498</v>
       </c>
       <c r="K189" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F189,'feed pars'!B$6:B$43,0))</f>
-        <v>19.848896</v>
+        <v>19.581538399999999</v>
       </c>
       <c r="M189" s="3"/>
     </row>
     <row r="190" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F190" t="s">
-        <v>384</v>
+        <v>315</v>
       </c>
       <c r="J190" t="s">
         <v>498</v>
       </c>
       <c r="K190" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F190,'feed pars'!B$6:B$43,0))</f>
-        <v>22.900705599999998</v>
+        <v>16.971140800000001</v>
       </c>
       <c r="M190" s="3"/>
     </row>
     <row r="191" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F191" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="J191" t="s">
         <v>498</v>
       </c>
       <c r="K191" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F191,'feed pars'!B$6:B$43,0))</f>
-        <v>16.1615368</v>
+        <v>18.194124000000002</v>
       </c>
       <c r="M191" s="3"/>
     </row>
     <row r="192" spans="6:13" x14ac:dyDescent="0.25">
       <c r="F192" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="J192" t="s">
         <v>498</v>
       </c>
       <c r="K192" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F192,'feed pars'!B$6:B$43,0))</f>
-        <v>17.334312000000001</v>
+        <v>17.8828344</v>
       </c>
       <c r="M192" s="3"/>
     </row>
     <row r="193" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F193" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="J193" t="s">
         <v>498</v>
       </c>
       <c r="K193" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F193,'feed pars'!B$6:B$43,0))</f>
-        <v>16.464040000000001</v>
+        <v>19.659779199999999</v>
       </c>
       <c r="M193" s="3"/>
     </row>
     <row r="194" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F194" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="J194" t="s">
         <v>498</v>
       </c>
       <c r="K194" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F194,'feed pars'!B$6:B$43,0))</f>
-        <v>16.975324799999999</v>
+        <v>18.8602168</v>
       </c>
       <c r="M194" s="3"/>
     </row>
     <row r="195" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F195" t="s">
-        <v>56</v>
+        <v>309</v>
       </c>
       <c r="J195" t="s">
         <v>498</v>
       </c>
       <c r="K195" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F195,'feed pars'!B$6:B$43,0))</f>
-        <v>23.055932000000002</v>
+        <v>19.848896</v>
       </c>
       <c r="M195" s="3"/>
     </row>
     <row r="196" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F196" t="s">
-        <v>57</v>
+        <v>384</v>
       </c>
       <c r="J196" t="s">
         <v>498</v>
       </c>
       <c r="K196" s="25">
         <f>INDEX('feed pars'!D$6:D$43,MATCH(F196,'feed pars'!B$6:B$43,0))</f>
-        <v>22.254696000000003</v>
+        <v>22.900705599999998</v>
       </c>
       <c r="M196" s="3"/>
     </row>
     <row r="197" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F197" t="s">
-        <v>320</v>
+        <v>52</v>
       </c>
       <c r="J197" t="s">
         <v>498</v>
       </c>
-      <c r="K197" s="85">
-        <v>0</v>
+      <c r="K197" s="25">
+        <f>INDEX('feed pars'!D$6:D$43,MATCH(F197,'feed pars'!B$6:B$43,0))</f>
+        <v>16.1615368</v>
       </c>
       <c r="M197" s="3"/>
     </row>
     <row r="198" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A198" s="7" t="s">
+      <c r="F198" t="s">
+        <v>53</v>
+      </c>
+      <c r="J198" t="s">
+        <v>498</v>
+      </c>
+      <c r="K198" s="25">
+        <f>INDEX('feed pars'!D$6:D$43,MATCH(F198,'feed pars'!B$6:B$43,0))</f>
+        <v>17.334312000000001</v>
+      </c>
+      <c r="M198" s="3"/>
+    </row>
+    <row r="199" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F199" t="s">
+        <v>54</v>
+      </c>
+      <c r="J199" t="s">
+        <v>498</v>
+      </c>
+      <c r="K199" s="25">
+        <f>INDEX('feed pars'!D$6:D$43,MATCH(F199,'feed pars'!B$6:B$43,0))</f>
+        <v>16.464040000000001</v>
+      </c>
+      <c r="M199" s="3"/>
+    </row>
+    <row r="200" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F200" t="s">
+        <v>55</v>
+      </c>
+      <c r="J200" t="s">
+        <v>498</v>
+      </c>
+      <c r="K200" s="25">
+        <f>INDEX('feed pars'!D$6:D$43,MATCH(F200,'feed pars'!B$6:B$43,0))</f>
+        <v>16.975324799999999</v>
+      </c>
+      <c r="M200" s="3"/>
+    </row>
+    <row r="201" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F201" t="s">
+        <v>56</v>
+      </c>
+      <c r="J201" t="s">
+        <v>498</v>
+      </c>
+      <c r="K201" s="25">
+        <f>INDEX('feed pars'!D$6:D$43,MATCH(F201,'feed pars'!B$6:B$43,0))</f>
+        <v>23.055932000000002</v>
+      </c>
+      <c r="M201" s="3"/>
+    </row>
+    <row r="202" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F202" t="s">
+        <v>57</v>
+      </c>
+      <c r="J202" t="s">
+        <v>498</v>
+      </c>
+      <c r="K202" s="25">
+        <f>INDEX('feed pars'!D$6:D$43,MATCH(F202,'feed pars'!B$6:B$43,0))</f>
+        <v>22.254696000000003</v>
+      </c>
+      <c r="M202" s="3"/>
+    </row>
+    <row r="203" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F203" t="s">
+        <v>320</v>
+      </c>
+      <c r="J203" t="s">
+        <v>498</v>
+      </c>
+      <c r="K203" s="85">
+        <v>0</v>
+      </c>
+      <c r="M203" s="3"/>
+    </row>
+    <row r="204" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A204" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B198" s="7"/>
-      <c r="C198" s="6"/>
-      <c r="D198" s="6"/>
-      <c r="E198" s="6"/>
-      <c r="F198" s="6"/>
-      <c r="G198" s="6"/>
-      <c r="H198" s="6"/>
-      <c r="I198" s="6"/>
-      <c r="J198" s="6"/>
-      <c r="K198" s="6"/>
-      <c r="L198" s="6"/>
-      <c r="M198" s="6"/>
-      <c r="N198" s="6"/>
-    </row>
-    <row r="199" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A199" t="s">
-        <v>24</v>
-      </c>
-      <c r="F199" t="s">
-        <v>306</v>
-      </c>
-      <c r="J199" t="s">
-        <v>18</v>
-      </c>
-      <c r="K199" s="25">
-        <f>INDEX('feed pars'!I$6:I$43,MATCH(F199,'feed pars'!B$6:B$43,0))</f>
-        <v>11.3</v>
-      </c>
-      <c r="L199" t="s">
-        <v>19</v>
-      </c>
-      <c r="M199" s="26" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="200" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A200" t="s">
-        <v>24</v>
-      </c>
-      <c r="F200" t="s">
-        <v>307</v>
-      </c>
-      <c r="J200" t="s">
-        <v>18</v>
-      </c>
-      <c r="K200" s="25">
-        <f>INDEX('feed pars'!I$6:I$43,MATCH(F200,'feed pars'!B$6:B$43,0))</f>
-        <v>10.1</v>
-      </c>
-      <c r="M200" s="3"/>
-    </row>
-    <row r="201" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A201" t="s">
-        <v>24</v>
-      </c>
-      <c r="F201" t="s">
-        <v>308</v>
-      </c>
-      <c r="J201" t="s">
-        <v>18</v>
-      </c>
-      <c r="K201" s="25">
-        <f>INDEX('feed pars'!I$6:I$43,MATCH(F201,'feed pars'!B$6:B$43,0))</f>
-        <v>9.25</v>
-      </c>
-      <c r="M201" s="3"/>
-    </row>
-    <row r="202" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A202" t="s">
-        <v>24</v>
-      </c>
-      <c r="F202" t="s">
-        <v>12</v>
-      </c>
-      <c r="J202" t="s">
-        <v>18</v>
-      </c>
-      <c r="K202" s="25">
-        <f>INDEX('feed pars'!I$6:I$43,MATCH(F202,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="203" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A203" t="s">
-        <v>24</v>
-      </c>
-      <c r="F203" t="s">
-        <v>33</v>
-      </c>
-      <c r="J203" t="s">
-        <v>18</v>
-      </c>
-      <c r="K203" s="25">
-        <f>INDEX('feed pars'!I$6:I$43,MATCH(F203,'feed pars'!B$6:B$43,0))</f>
-        <v>9.9416666666666664</v>
-      </c>
-    </row>
-    <row r="204" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A204" t="s">
-        <v>24</v>
-      </c>
-      <c r="F204" t="s">
-        <v>17</v>
-      </c>
-      <c r="J204" t="s">
-        <v>18</v>
-      </c>
-      <c r="K204" s="25">
-        <f>INDEX('feed pars'!I$6:I$43,MATCH(F204,'feed pars'!B$6:B$43,0))</f>
-        <v>14.1</v>
-      </c>
+      <c r="B204" s="7"/>
+      <c r="C204" s="6"/>
+      <c r="D204" s="6"/>
+      <c r="E204" s="6"/>
+      <c r="F204" s="6"/>
+      <c r="G204" s="6"/>
+      <c r="H204" s="6"/>
+      <c r="I204" s="6"/>
+      <c r="J204" s="6"/>
+      <c r="K204" s="6"/>
+      <c r="L204" s="6"/>
+      <c r="M204" s="6"/>
+      <c r="N204" s="6"/>
     </row>
     <row r="205" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>24</v>
       </c>
       <c r="F205" t="s">
-        <v>37</v>
+        <v>306</v>
       </c>
       <c r="J205" t="s">
         <v>18</v>
       </c>
       <c r="K205" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F205,'feed pars'!B$6:B$43,0))</f>
-        <v>13.2</v>
+        <v>11.3</v>
+      </c>
+      <c r="L205" t="s">
+        <v>19</v>
+      </c>
+      <c r="M205" s="26" t="s">
+        <v>502</v>
       </c>
     </row>
     <row r="206" spans="1:14" x14ac:dyDescent="0.25">
@@ -5915,44 +5978,46 @@
         <v>24</v>
       </c>
       <c r="F206" t="s">
-        <v>38</v>
+        <v>307</v>
       </c>
       <c r="J206" t="s">
         <v>18</v>
       </c>
       <c r="K206" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F206,'feed pars'!B$6:B$43,0))</f>
-        <v>11.7</v>
-      </c>
+        <v>10.1</v>
+      </c>
+      <c r="M206" s="3"/>
     </row>
     <row r="207" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>24</v>
       </c>
       <c r="F207" t="s">
-        <v>39</v>
+        <v>308</v>
       </c>
       <c r="J207" t="s">
         <v>18</v>
       </c>
       <c r="K207" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F207,'feed pars'!B$6:B$43,0))</f>
-        <v>14</v>
-      </c>
+        <v>9.25</v>
+      </c>
+      <c r="M207" s="3"/>
     </row>
     <row r="208" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>24</v>
       </c>
       <c r="F208" t="s">
-        <v>313</v>
+        <v>12</v>
       </c>
       <c r="J208" t="s">
         <v>18</v>
       </c>
       <c r="K208" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F208,'feed pars'!B$6:B$43,0))</f>
-        <v>13.9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="209" spans="1:11" x14ac:dyDescent="0.25">
@@ -5960,14 +6025,14 @@
         <v>24</v>
       </c>
       <c r="F209" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="J209" t="s">
         <v>18</v>
       </c>
       <c r="K209" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F209,'feed pars'!B$6:B$43,0))</f>
-        <v>12.8</v>
+        <v>9.9416666666666664</v>
       </c>
     </row>
     <row r="210" spans="1:11" x14ac:dyDescent="0.25">
@@ -5975,14 +6040,14 @@
         <v>24</v>
       </c>
       <c r="F210" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="J210" t="s">
         <v>18</v>
       </c>
       <c r="K210" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F210,'feed pars'!B$6:B$43,0))</f>
-        <v>13.8</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="211" spans="1:11" x14ac:dyDescent="0.25">
@@ -5990,14 +6055,14 @@
         <v>24</v>
       </c>
       <c r="F211" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="J211" t="s">
         <v>18</v>
       </c>
       <c r="K211" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F211,'feed pars'!B$6:B$43,0))</f>
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="212" spans="1:11" x14ac:dyDescent="0.25">
@@ -6005,14 +6070,14 @@
         <v>24</v>
       </c>
       <c r="F212" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J212" t="s">
         <v>18</v>
       </c>
       <c r="K212" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F212,'feed pars'!B$6:B$43,0))</f>
-        <v>22.1</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="213" spans="1:11" x14ac:dyDescent="0.25">
@@ -6020,14 +6085,14 @@
         <v>24</v>
       </c>
       <c r="F213" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="J213" t="s">
         <v>18</v>
       </c>
       <c r="K213" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F213,'feed pars'!B$6:B$43,0))</f>
-        <v>20.100000000000001</v>
+        <v>14</v>
       </c>
     </row>
     <row r="214" spans="1:11" x14ac:dyDescent="0.25">
@@ -6035,14 +6100,14 @@
         <v>24</v>
       </c>
       <c r="F214" t="s">
-        <v>302</v>
+        <v>313</v>
       </c>
       <c r="J214" t="s">
         <v>18</v>
       </c>
       <c r="K214" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F214,'feed pars'!B$6:B$43,0))</f>
-        <v>6.6</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="215" spans="1:11" x14ac:dyDescent="0.25">
@@ -6050,14 +6115,14 @@
         <v>24</v>
       </c>
       <c r="F215" t="s">
-        <v>310</v>
+        <v>40</v>
       </c>
       <c r="J215" t="s">
         <v>18</v>
       </c>
       <c r="K215" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F215,'feed pars'!B$6:B$43,0))</f>
-        <v>36.6</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="216" spans="1:11" x14ac:dyDescent="0.25">
@@ -6065,14 +6130,14 @@
         <v>24</v>
       </c>
       <c r="F216" t="s">
-        <v>314</v>
+        <v>41</v>
       </c>
       <c r="J216" t="s">
         <v>18</v>
       </c>
       <c r="K216" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F216,'feed pars'!B$6:B$43,0))</f>
-        <v>16.399999999999999</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="217" spans="1:11" x14ac:dyDescent="0.25">
@@ -6080,14 +6145,14 @@
         <v>24</v>
       </c>
       <c r="F217" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J217" t="s">
         <v>18</v>
       </c>
       <c r="K217" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F217,'feed pars'!B$6:B$43,0))</f>
-        <v>14.6</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="218" spans="1:11" x14ac:dyDescent="0.25">
@@ -6095,14 +6160,14 @@
         <v>24</v>
       </c>
       <c r="F218" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J218" t="s">
         <v>18</v>
       </c>
       <c r="K218" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F218,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="219" spans="1:11" x14ac:dyDescent="0.25">
@@ -6110,14 +6175,14 @@
         <v>24</v>
       </c>
       <c r="F219" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="J219" t="s">
         <v>18</v>
       </c>
       <c r="K219" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F219,'feed pars'!B$6:B$43,0))</f>
-        <v>11.4</v>
+        <v>20.100000000000001</v>
       </c>
     </row>
     <row r="220" spans="1:11" x14ac:dyDescent="0.25">
@@ -6125,14 +6190,14 @@
         <v>24</v>
       </c>
       <c r="F220" t="s">
-        <v>47</v>
+        <v>302</v>
       </c>
       <c r="J220" t="s">
         <v>18</v>
       </c>
       <c r="K220" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F220,'feed pars'!B$6:B$43,0))</f>
-        <v>13.4</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="221" spans="1:11" x14ac:dyDescent="0.25">
@@ -6140,14 +6205,14 @@
         <v>24</v>
       </c>
       <c r="F221" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="J221" t="s">
         <v>18</v>
       </c>
       <c r="K221" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F221,'feed pars'!B$6:B$43,0))</f>
-        <v>8.5</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="222" spans="1:11" x14ac:dyDescent="0.25">
@@ -6155,14 +6220,14 @@
         <v>24</v>
       </c>
       <c r="F222" t="s">
-        <v>48</v>
+        <v>314</v>
       </c>
       <c r="J222" t="s">
         <v>18</v>
       </c>
       <c r="K222" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F222,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
+        <v>16.399999999999999</v>
       </c>
     </row>
     <row r="223" spans="1:11" x14ac:dyDescent="0.25">
@@ -6170,14 +6235,14 @@
         <v>24</v>
       </c>
       <c r="F223" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J223" t="s">
         <v>18</v>
       </c>
       <c r="K223" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F223,'feed pars'!B$6:B$43,0))</f>
-        <v>13.3</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="224" spans="1:11" x14ac:dyDescent="0.25">
@@ -6185,14 +6250,14 @@
         <v>24</v>
       </c>
       <c r="F224" t="s">
-        <v>309</v>
+        <v>36</v>
       </c>
       <c r="J224" t="s">
         <v>18</v>
       </c>
       <c r="K224" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F224,'feed pars'!B$6:B$43,0))</f>
-        <v>11.6</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="225" spans="1:13" x14ac:dyDescent="0.25">
@@ -6200,14 +6265,14 @@
         <v>24</v>
       </c>
       <c r="F225" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="J225" t="s">
         <v>18</v>
       </c>
       <c r="K225" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F225,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="226" spans="1:13" x14ac:dyDescent="0.25">
@@ -6215,14 +6280,14 @@
         <v>24</v>
       </c>
       <c r="F226" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="J226" t="s">
         <v>18</v>
       </c>
       <c r="K226" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F226,'feed pars'!B$6:B$43,0))</f>
-        <v>12.3</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="227" spans="1:13" x14ac:dyDescent="0.25">
@@ -6230,14 +6295,14 @@
         <v>24</v>
       </c>
       <c r="F227" t="s">
-        <v>54</v>
+        <v>315</v>
       </c>
       <c r="J227" t="s">
         <v>18</v>
       </c>
       <c r="K227" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F227,'feed pars'!B$6:B$43,0))</f>
-        <v>13.6</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="228" spans="1:13" x14ac:dyDescent="0.25">
@@ -6245,14 +6310,14 @@
         <v>24</v>
       </c>
       <c r="F228" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="J228" t="s">
         <v>18</v>
       </c>
       <c r="K228" s="25">
         <f>INDEX('feed pars'!I$6:I$43,MATCH(F228,'feed pars'!B$6:B$43,0))</f>
-        <v>15.5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="229" spans="1:13" x14ac:dyDescent="0.25">
@@ -6260,13 +6325,14 @@
         <v>24</v>
       </c>
       <c r="F229" t="s">
-        <v>320</v>
+        <v>50</v>
       </c>
       <c r="J229" t="s">
         <v>18</v>
       </c>
-      <c r="K229" s="3">
-        <v>0</v>
+      <c r="K229" s="25">
+        <f>INDEX('feed pars'!I$6:I$43,MATCH(F229,'feed pars'!B$6:B$43,0))</f>
+        <v>13.3</v>
       </c>
     </row>
     <row r="230" spans="1:13" x14ac:dyDescent="0.25">
@@ -6274,20 +6340,14 @@
         <v>24</v>
       </c>
       <c r="F230" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="J230" t="s">
-        <v>500</v>
-      </c>
-      <c r="K230" s="82">
-        <f>INDEX('feed pars'!K$6:K$43,MATCH(F230,'feed pars'!B$6:B$43,0))</f>
-        <v>20</v>
-      </c>
-      <c r="L230" t="s">
-        <v>501</v>
-      </c>
-      <c r="M230" s="26" t="s">
-        <v>505</v>
+        <v>18</v>
+      </c>
+      <c r="K230" s="25">
+        <f>INDEX('feed pars'!I$6:I$43,MATCH(F230,'feed pars'!B$6:B$43,0))</f>
+        <v>11.6</v>
       </c>
     </row>
     <row r="231" spans="1:13" x14ac:dyDescent="0.25">
@@ -6295,46 +6355,44 @@
         <v>24</v>
       </c>
       <c r="F231" t="s">
-        <v>307</v>
+        <v>52</v>
       </c>
       <c r="J231" t="s">
-        <v>500</v>
-      </c>
-      <c r="K231" s="82">
-        <f>INDEX('feed pars'!K$6:K$43,MATCH(F231,'feed pars'!B$6:B$43,0))</f>
-        <v>20</v>
-      </c>
-      <c r="M231" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="K231" s="25">
+        <f>INDEX('feed pars'!I$6:I$43,MATCH(F231,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
     </row>
     <row r="232" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>24</v>
       </c>
       <c r="F232" t="s">
-        <v>308</v>
+        <v>53</v>
       </c>
       <c r="J232" t="s">
-        <v>500</v>
-      </c>
-      <c r="K232" s="82">
-        <f>INDEX('feed pars'!K$6:K$43,MATCH(F232,'feed pars'!B$6:B$43,0))</f>
-        <v>36</v>
-      </c>
-      <c r="M232" s="3"/>
+        <v>18</v>
+      </c>
+      <c r="K232" s="25">
+        <f>INDEX('feed pars'!I$6:I$43,MATCH(F232,'feed pars'!B$6:B$43,0))</f>
+        <v>12.3</v>
+      </c>
     </row>
     <row r="233" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>24</v>
       </c>
       <c r="F233" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="J233" t="s">
-        <v>500</v>
-      </c>
-      <c r="K233" s="82">
-        <f>INDEX('feed pars'!K$6:K$43,MATCH(F233,'feed pars'!B$6:B$43,0))</f>
-        <v>30</v>
+        <v>18</v>
+      </c>
+      <c r="K233" s="25">
+        <f>INDEX('feed pars'!I$6:I$43,MATCH(F233,'feed pars'!B$6:B$43,0))</f>
+        <v>13.6</v>
       </c>
     </row>
     <row r="234" spans="1:13" x14ac:dyDescent="0.25">
@@ -6342,14 +6400,14 @@
         <v>24</v>
       </c>
       <c r="F234" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="J234" t="s">
-        <v>500</v>
-      </c>
-      <c r="K234" s="82">
-        <f>INDEX('feed pars'!K$6:K$43,MATCH(F234,'feed pars'!B$6:B$43,0))</f>
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="K234" s="25">
+        <f>INDEX('feed pars'!I$6:I$43,MATCH(F234,'feed pars'!B$6:B$43,0))</f>
+        <v>15.5</v>
       </c>
     </row>
     <row r="235" spans="1:13" x14ac:dyDescent="0.25">
@@ -6357,14 +6415,13 @@
         <v>24</v>
       </c>
       <c r="F235" t="s">
-        <v>17</v>
+        <v>320</v>
       </c>
       <c r="J235" t="s">
-        <v>500</v>
-      </c>
-      <c r="K235" s="82">
-        <f>INDEX('feed pars'!K$6:K$43,MATCH(F235,'feed pars'!B$6:B$43,0))</f>
-        <v>25</v>
+        <v>18</v>
+      </c>
+      <c r="K235" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="236" spans="1:13" x14ac:dyDescent="0.25">
@@ -6372,14 +6429,20 @@
         <v>24</v>
       </c>
       <c r="F236" t="s">
-        <v>37</v>
+        <v>306</v>
       </c>
       <c r="J236" t="s">
         <v>500</v>
       </c>
       <c r="K236" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F236,'feed pars'!B$6:B$43,0))</f>
-        <v>27</v>
+        <v>20</v>
+      </c>
+      <c r="L236" t="s">
+        <v>501</v>
+      </c>
+      <c r="M236" s="26" t="s">
+        <v>505</v>
       </c>
     </row>
     <row r="237" spans="1:13" x14ac:dyDescent="0.25">
@@ -6387,44 +6450,46 @@
         <v>24</v>
       </c>
       <c r="F237" t="s">
-        <v>38</v>
+        <v>307</v>
       </c>
       <c r="J237" t="s">
         <v>500</v>
       </c>
       <c r="K237" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F237,'feed pars'!B$6:B$43,0))</f>
-        <v>61</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="M237" s="3"/>
     </row>
     <row r="238" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>24</v>
       </c>
       <c r="F238" t="s">
-        <v>39</v>
+        <v>308</v>
       </c>
       <c r="J238" t="s">
         <v>500</v>
       </c>
       <c r="K238" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F238,'feed pars'!B$6:B$43,0))</f>
-        <v>26</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="M238" s="3"/>
     </row>
     <row r="239" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>24</v>
       </c>
       <c r="F239" t="s">
-        <v>313</v>
+        <v>12</v>
       </c>
       <c r="J239" t="s">
         <v>500</v>
       </c>
       <c r="K239" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F239,'feed pars'!B$6:B$43,0))</f>
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="240" spans="1:13" x14ac:dyDescent="0.25">
@@ -6432,14 +6497,14 @@
         <v>24</v>
       </c>
       <c r="F240" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="J240" t="s">
         <v>500</v>
       </c>
       <c r="K240" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F240,'feed pars'!B$6:B$43,0))</f>
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="241" spans="1:11" x14ac:dyDescent="0.25">
@@ -6447,14 +6512,14 @@
         <v>24</v>
       </c>
       <c r="F241" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="J241" t="s">
         <v>500</v>
       </c>
       <c r="K241" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F241,'feed pars'!B$6:B$43,0))</f>
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="242" spans="1:11" x14ac:dyDescent="0.25">
@@ -6462,14 +6527,14 @@
         <v>24</v>
       </c>
       <c r="F242" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="J242" t="s">
         <v>500</v>
       </c>
       <c r="K242" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F242,'feed pars'!B$6:B$43,0))</f>
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="243" spans="1:11" x14ac:dyDescent="0.25">
@@ -6477,14 +6542,14 @@
         <v>24</v>
       </c>
       <c r="F243" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J243" t="s">
         <v>500</v>
       </c>
       <c r="K243" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F243,'feed pars'!B$6:B$43,0))</f>
-        <v>460</v>
+        <v>61</v>
       </c>
     </row>
     <row r="244" spans="1:11" x14ac:dyDescent="0.25">
@@ -6492,14 +6557,14 @@
         <v>24</v>
       </c>
       <c r="F244" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="J244" t="s">
         <v>500</v>
       </c>
       <c r="K244" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F244,'feed pars'!B$6:B$43,0))</f>
-        <v>380</v>
+        <v>26</v>
       </c>
     </row>
     <row r="245" spans="1:11" x14ac:dyDescent="0.25">
@@ -6507,7 +6572,7 @@
         <v>24</v>
       </c>
       <c r="F245" t="s">
-        <v>302</v>
+        <v>313</v>
       </c>
       <c r="J245" t="s">
         <v>500</v>
@@ -6522,14 +6587,14 @@
         <v>24</v>
       </c>
       <c r="F246" t="s">
-        <v>310</v>
+        <v>40</v>
       </c>
       <c r="J246" t="s">
         <v>500</v>
       </c>
       <c r="K246" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F246,'feed pars'!B$6:B$43,0))</f>
-        <v>1000</v>
+        <v>40</v>
       </c>
     </row>
     <row r="247" spans="1:11" x14ac:dyDescent="0.25">
@@ -6537,14 +6602,14 @@
         <v>24</v>
       </c>
       <c r="F247" t="s">
-        <v>314</v>
+        <v>41</v>
       </c>
       <c r="J247" t="s">
         <v>500</v>
       </c>
       <c r="K247" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F247,'feed pars'!B$6:B$43,0))</f>
-        <v>180</v>
+        <v>17</v>
       </c>
     </row>
     <row r="248" spans="1:11" x14ac:dyDescent="0.25">
@@ -6552,14 +6617,14 @@
         <v>24</v>
       </c>
       <c r="F248" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J248" t="s">
         <v>500</v>
       </c>
       <c r="K248" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F248,'feed pars'!B$6:B$43,0))</f>
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="249" spans="1:11" x14ac:dyDescent="0.25">
@@ -6567,14 +6632,14 @@
         <v>24</v>
       </c>
       <c r="F249" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J249" t="s">
         <v>500</v>
       </c>
       <c r="K249" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F249,'feed pars'!B$6:B$43,0))</f>
-        <v>46</v>
+        <v>460</v>
       </c>
     </row>
     <row r="250" spans="1:11" x14ac:dyDescent="0.25">
@@ -6582,14 +6647,14 @@
         <v>24</v>
       </c>
       <c r="F250" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="J250" t="s">
         <v>500</v>
       </c>
       <c r="K250" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F250,'feed pars'!B$6:B$43,0))</f>
-        <v>10</v>
+        <v>380</v>
       </c>
     </row>
     <row r="251" spans="1:11" x14ac:dyDescent="0.25">
@@ -6597,14 +6662,14 @@
         <v>24</v>
       </c>
       <c r="F251" t="s">
-        <v>47</v>
+        <v>302</v>
       </c>
       <c r="J251" t="s">
         <v>500</v>
       </c>
       <c r="K251" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F251,'feed pars'!B$6:B$43,0))</f>
-        <v>97</v>
+        <v>20</v>
       </c>
     </row>
     <row r="252" spans="1:11" x14ac:dyDescent="0.25">
@@ -6612,14 +6677,14 @@
         <v>24</v>
       </c>
       <c r="F252" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="J252" t="s">
         <v>500</v>
       </c>
       <c r="K252" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F252,'feed pars'!B$6:B$43,0))</f>
-        <v>27</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="253" spans="1:11" x14ac:dyDescent="0.25">
@@ -6627,14 +6692,14 @@
         <v>24</v>
       </c>
       <c r="F253" t="s">
-        <v>48</v>
+        <v>314</v>
       </c>
       <c r="J253" t="s">
         <v>500</v>
       </c>
       <c r="K253" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F253,'feed pars'!B$6:B$43,0))</f>
-        <v>45</v>
+        <v>180</v>
       </c>
     </row>
     <row r="254" spans="1:11" x14ac:dyDescent="0.25">
@@ -6642,14 +6707,14 @@
         <v>24</v>
       </c>
       <c r="F254" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J254" t="s">
         <v>500</v>
       </c>
       <c r="K254" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F254,'feed pars'!B$6:B$43,0))</f>
-        <v>45</v>
+        <v>10</v>
       </c>
     </row>
     <row r="255" spans="1:11" x14ac:dyDescent="0.25">
@@ -6657,14 +6722,14 @@
         <v>24</v>
       </c>
       <c r="F255" t="s">
-        <v>309</v>
+        <v>36</v>
       </c>
       <c r="J255" t="s">
         <v>500</v>
       </c>
       <c r="K255" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F255,'feed pars'!B$6:B$43,0))</f>
-        <v>80</v>
+        <v>46</v>
       </c>
     </row>
     <row r="256" spans="1:11" x14ac:dyDescent="0.25">
@@ -6672,14 +6737,14 @@
         <v>24</v>
       </c>
       <c r="F256" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="J256" t="s">
         <v>500</v>
       </c>
       <c r="K256" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F256,'feed pars'!B$6:B$43,0))</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="257" spans="1:14" x14ac:dyDescent="0.25">
@@ -6687,14 +6752,14 @@
         <v>24</v>
       </c>
       <c r="F257" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="J257" t="s">
         <v>500</v>
       </c>
       <c r="K257" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F257,'feed pars'!B$6:B$43,0))</f>
-        <v>32</v>
+        <v>97</v>
       </c>
     </row>
     <row r="258" spans="1:14" x14ac:dyDescent="0.25">
@@ -6702,14 +6767,14 @@
         <v>24</v>
       </c>
       <c r="F258" t="s">
-        <v>54</v>
+        <v>315</v>
       </c>
       <c r="J258" t="s">
         <v>500</v>
       </c>
       <c r="K258" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F258,'feed pars'!B$6:B$43,0))</f>
-        <v>10</v>
+        <v>27</v>
       </c>
     </row>
     <row r="259" spans="1:14" x14ac:dyDescent="0.25">
@@ -6717,14 +6782,14 @@
         <v>24</v>
       </c>
       <c r="F259" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="J259" t="s">
         <v>500</v>
       </c>
       <c r="K259" s="82">
         <f>INDEX('feed pars'!K$6:K$43,MATCH(F259,'feed pars'!B$6:B$43,0))</f>
-        <v>33</v>
+        <v>45</v>
       </c>
     </row>
     <row r="260" spans="1:14" x14ac:dyDescent="0.25">
@@ -6732,130 +6797,142 @@
         <v>24</v>
       </c>
       <c r="F260" t="s">
-        <v>320</v>
+        <v>50</v>
       </c>
       <c r="J260" t="s">
         <v>500</v>
       </c>
-      <c r="K260" s="3">
-        <v>0</v>
+      <c r="K260" s="82">
+        <f>INDEX('feed pars'!K$6:K$43,MATCH(F260,'feed pars'!B$6:B$43,0))</f>
+        <v>45</v>
       </c>
     </row>
     <row r="261" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A261" s="7" t="s">
-        <v>405</v>
-      </c>
-      <c r="B261" s="7"/>
-      <c r="C261" s="6"/>
-      <c r="D261" s="6"/>
-      <c r="E261" s="6"/>
-      <c r="F261" s="6"/>
-      <c r="G261" s="6"/>
-      <c r="H261" s="6"/>
-      <c r="I261" s="6"/>
-      <c r="J261" s="6"/>
-      <c r="K261" s="6"/>
-      <c r="L261" s="6"/>
-      <c r="M261" s="6"/>
-      <c r="N261" s="6"/>
+      <c r="A261" t="s">
+        <v>24</v>
+      </c>
+      <c r="F261" t="s">
+        <v>309</v>
+      </c>
+      <c r="J261" t="s">
+        <v>500</v>
+      </c>
+      <c r="K261" s="82">
+        <f>INDEX('feed pars'!K$6:K$43,MATCH(F261,'feed pars'!B$6:B$43,0))</f>
+        <v>80</v>
+      </c>
     </row>
     <row r="262" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>391</v>
+        <v>24</v>
       </c>
       <c r="F262" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="J262" t="s">
-        <v>18</v>
-      </c>
-      <c r="K262" s="25">
-        <f>INDEX('feed pars'!I$6:I$43,MATCH(F262,'feed pars'!B$6:B$43,0))</f>
-        <v>9.1</v>
-      </c>
-      <c r="L262" t="s">
-        <v>19</v>
-      </c>
-      <c r="M262" s="26" t="s">
-        <v>502</v>
+        <v>500</v>
+      </c>
+      <c r="K262" s="82">
+        <f>INDEX('feed pars'!K$6:K$43,MATCH(F262,'feed pars'!B$6:B$43,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="263" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>391</v>
+        <v>24</v>
       </c>
       <c r="F263" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="J263" t="s">
-        <v>18</v>
-      </c>
-      <c r="K263" s="31">
-        <f>K203</f>
-        <v>9.9416666666666664</v>
+        <v>500</v>
+      </c>
+      <c r="K263" s="82">
+        <f>INDEX('feed pars'!K$6:K$43,MATCH(F263,'feed pars'!B$6:B$43,0))</f>
+        <v>32</v>
       </c>
     </row>
     <row r="264" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K264" s="31"/>
+      <c r="A264" t="s">
+        <v>24</v>
+      </c>
+      <c r="F264" t="s">
+        <v>54</v>
+      </c>
+      <c r="J264" t="s">
+        <v>500</v>
+      </c>
+      <c r="K264" s="82">
+        <f>INDEX('feed pars'!K$6:K$43,MATCH(F264,'feed pars'!B$6:B$43,0))</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="265" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>391</v>
+        <v>24</v>
       </c>
       <c r="F265" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="J265" t="s">
-        <v>18</v>
-      </c>
-      <c r="K265" s="31">
-        <f>K206</f>
-        <v>11.7</v>
+        <v>500</v>
+      </c>
+      <c r="K265" s="82">
+        <f>INDEX('feed pars'!K$6:K$43,MATCH(F265,'feed pars'!B$6:B$43,0))</f>
+        <v>33</v>
       </c>
     </row>
     <row r="266" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>391</v>
+        <v>24</v>
       </c>
       <c r="F266" t="s">
-        <v>37</v>
+        <v>320</v>
       </c>
       <c r="J266" t="s">
-        <v>18</v>
-      </c>
-      <c r="K266" s="31">
-        <f>K205</f>
-        <v>13.2</v>
+        <v>500</v>
+      </c>
+      <c r="K266" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="267" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A267" t="s">
-        <v>391</v>
-      </c>
-      <c r="F267" t="s">
-        <v>17</v>
-      </c>
-      <c r="J267" t="s">
-        <v>18</v>
-      </c>
-      <c r="K267" s="31">
-        <f>K204</f>
-        <v>14.1</v>
-      </c>
+      <c r="A267" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="B267" s="7"/>
+      <c r="C267" s="6"/>
+      <c r="D267" s="6"/>
+      <c r="E267" s="6"/>
+      <c r="F267" s="6"/>
+      <c r="G267" s="6"/>
+      <c r="H267" s="6"/>
+      <c r="I267" s="6"/>
+      <c r="J267" s="6"/>
+      <c r="K267" s="6"/>
+      <c r="L267" s="6"/>
+      <c r="M267" s="6"/>
+      <c r="N267" s="6"/>
     </row>
     <row r="268" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>391</v>
       </c>
       <c r="F268" t="s">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="J268" t="s">
         <v>18</v>
       </c>
-      <c r="K268" s="31">
-        <f t="shared" ref="K268:K274" si="14">K205</f>
-        <v>13.2</v>
+      <c r="K268" s="25">
+        <f>INDEX('feed pars'!I$6:I$43,MATCH(F268,'feed pars'!B$6:B$43,0))</f>
+        <v>9.1</v>
+      </c>
+      <c r="L268" t="s">
+        <v>19</v>
+      </c>
+      <c r="M268" s="26" t="s">
+        <v>502</v>
       </c>
     </row>
     <row r="269" spans="1:14" x14ac:dyDescent="0.25">
@@ -6863,44 +6940,32 @@
         <v>391</v>
       </c>
       <c r="F269" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="J269" t="s">
         <v>18</v>
       </c>
       <c r="K269" s="31">
-        <f t="shared" si="14"/>
-        <v>11.7</v>
+        <f>K209</f>
+        <v>9.9416666666666664</v>
       </c>
     </row>
     <row r="270" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A270" t="s">
-        <v>391</v>
-      </c>
-      <c r="F270" t="s">
-        <v>310</v>
-      </c>
-      <c r="J270" t="s">
-        <v>18</v>
-      </c>
-      <c r="K270" s="31">
-        <f t="shared" si="14"/>
-        <v>14</v>
-      </c>
+      <c r="K270" s="31"/>
     </row>
     <row r="271" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>391</v>
       </c>
       <c r="F271" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="J271" t="s">
         <v>18</v>
       </c>
       <c r="K271" s="31">
-        <f t="shared" si="14"/>
-        <v>13.9</v>
+        <f>K212</f>
+        <v>11.7</v>
       </c>
     </row>
     <row r="272" spans="1:14" x14ac:dyDescent="0.25">
@@ -6908,14 +6973,14 @@
         <v>391</v>
       </c>
       <c r="F272" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="J272" t="s">
         <v>18</v>
       </c>
       <c r="K272" s="31">
-        <f t="shared" si="14"/>
-        <v>12.8</v>
+        <f>K211</f>
+        <v>13.2</v>
       </c>
     </row>
     <row r="273" spans="1:14" x14ac:dyDescent="0.25">
@@ -6923,14 +6988,14 @@
         <v>391</v>
       </c>
       <c r="F273" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="J273" t="s">
         <v>18</v>
       </c>
       <c r="K273" s="31">
-        <f t="shared" si="14"/>
-        <v>13.8</v>
+        <f>K210</f>
+        <v>14.1</v>
       </c>
     </row>
     <row r="274" spans="1:14" x14ac:dyDescent="0.25">
@@ -6938,168 +7003,144 @@
         <v>391</v>
       </c>
       <c r="F274" t="s">
-        <v>315</v>
+        <v>49</v>
       </c>
       <c r="J274" t="s">
         <v>18</v>
       </c>
       <c r="K274" s="31">
+        <f t="shared" ref="K274:K280" si="14">K211</f>
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="275" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>391</v>
+      </c>
+      <c r="F275" t="s">
+        <v>48</v>
+      </c>
+      <c r="J275" t="s">
+        <v>18</v>
+      </c>
+      <c r="K275" s="31">
+        <f t="shared" si="14"/>
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="276" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>391</v>
+      </c>
+      <c r="F276" t="s">
+        <v>310</v>
+      </c>
+      <c r="J276" t="s">
+        <v>18</v>
+      </c>
+      <c r="K276" s="31">
+        <f t="shared" si="14"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="277" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A277" t="s">
+        <v>391</v>
+      </c>
+      <c r="F277" t="s">
+        <v>53</v>
+      </c>
+      <c r="J277" t="s">
+        <v>18</v>
+      </c>
+      <c r="K277" s="31">
+        <f t="shared" si="14"/>
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="278" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>391</v>
+      </c>
+      <c r="F278" t="s">
+        <v>52</v>
+      </c>
+      <c r="J278" t="s">
+        <v>18</v>
+      </c>
+      <c r="K278" s="31">
+        <f t="shared" si="14"/>
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="279" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>391</v>
+      </c>
+      <c r="F279" t="s">
+        <v>56</v>
+      </c>
+      <c r="J279" t="s">
+        <v>18</v>
+      </c>
+      <c r="K279" s="31">
+        <f t="shared" si="14"/>
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="280" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
+        <v>391</v>
+      </c>
+      <c r="F280" t="s">
+        <v>315</v>
+      </c>
+      <c r="J280" t="s">
+        <v>18</v>
+      </c>
+      <c r="K280" s="31">
         <f t="shared" si="14"/>
         <v>13.3</v>
       </c>
     </row>
-    <row r="275" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K275" s="3"/>
-    </row>
-    <row r="276" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A276" s="8" t="s">
+    <row r="281" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K281" s="3"/>
+    </row>
+    <row r="282" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A282" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B276" s="8"/>
-      <c r="C276" s="9"/>
-      <c r="D276" s="9"/>
-      <c r="E276" s="9"/>
-      <c r="F276" s="9"/>
-      <c r="G276" s="9"/>
-      <c r="H276" s="9"/>
-      <c r="I276" s="9"/>
-      <c r="J276" s="9"/>
-      <c r="K276" s="9"/>
-      <c r="L276" s="9"/>
-      <c r="M276" s="9"/>
-      <c r="N276" s="9"/>
-    </row>
-    <row r="277" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A277" s="27" t="s">
+      <c r="B282" s="8"/>
+      <c r="C282" s="9"/>
+      <c r="D282" s="9"/>
+      <c r="E282" s="9"/>
+      <c r="F282" s="9"/>
+      <c r="G282" s="9"/>
+      <c r="H282" s="9"/>
+      <c r="I282" s="9"/>
+      <c r="J282" s="9"/>
+      <c r="K282" s="9"/>
+      <c r="L282" s="9"/>
+      <c r="M282" s="9"/>
+      <c r="N282" s="9"/>
+    </row>
+    <row r="283" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A283" s="27" t="s">
         <v>387</v>
       </c>
-      <c r="B277" s="28"/>
-      <c r="C277" s="29"/>
-      <c r="D277" s="29"/>
-      <c r="E277" s="29"/>
-      <c r="F277" s="29"/>
-      <c r="G277" s="29"/>
-      <c r="H277" s="29"/>
-      <c r="I277" s="29"/>
-      <c r="J277" s="29"/>
-      <c r="K277" s="29"/>
-      <c r="L277" s="29"/>
-      <c r="M277" s="29"/>
-      <c r="N277" s="29"/>
-    </row>
-    <row r="278" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A278" t="s">
-        <v>25</v>
-      </c>
-      <c r="E278" t="s">
-        <v>296</v>
-      </c>
-      <c r="F278" t="s">
-        <v>17</v>
-      </c>
-      <c r="J278" t="s">
-        <v>18</v>
-      </c>
-      <c r="K278" s="25">
-        <f>INDEX('feed pars'!U$6:U$43,MATCH(F278,'feed pars'!B$6:B$43,0))</f>
-        <v>12.3</v>
-      </c>
-      <c r="L278" t="s">
-        <v>297</v>
-      </c>
-      <c r="M278" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="279" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A279" t="s">
-        <v>25</v>
-      </c>
-      <c r="E279" t="s">
-        <v>296</v>
-      </c>
-      <c r="F279" t="s">
-        <v>37</v>
-      </c>
-      <c r="J279" t="s">
-        <v>18</v>
-      </c>
-      <c r="K279" s="25">
-        <f>INDEX('feed pars'!U$6:U$43,MATCH(F279,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
-      </c>
-    </row>
-    <row r="280" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A280" t="s">
-        <v>25</v>
-      </c>
-      <c r="E280" t="s">
-        <v>296</v>
-      </c>
-      <c r="F280" t="s">
-        <v>38</v>
-      </c>
-      <c r="J280" t="s">
-        <v>18</v>
-      </c>
-      <c r="K280" s="25">
-        <f>INDEX('feed pars'!U$6:U$43,MATCH(F280,'feed pars'!B$6:B$43,0))</f>
-        <v>9.4</v>
-      </c>
-    </row>
-    <row r="281" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A281" t="s">
-        <v>25</v>
-      </c>
-      <c r="E281" t="s">
-        <v>296</v>
-      </c>
-      <c r="F281" t="s">
-        <v>39</v>
-      </c>
-      <c r="J281" t="s">
-        <v>18</v>
-      </c>
-      <c r="K281" s="25">
-        <f>INDEX('feed pars'!U$6:U$43,MATCH(F281,'feed pars'!B$6:B$43,0))</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="282" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A282" t="s">
-        <v>25</v>
-      </c>
-      <c r="E282" t="s">
-        <v>296</v>
-      </c>
-      <c r="F282" t="s">
-        <v>40</v>
-      </c>
-      <c r="J282" t="s">
-        <v>18</v>
-      </c>
-      <c r="K282" s="25">
-        <f>INDEX('feed pars'!U$6:U$43,MATCH(F282,'feed pars'!B$6:B$43,0))</f>
-        <v>13.2</v>
-      </c>
-    </row>
-    <row r="283" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A283" t="s">
-        <v>25</v>
-      </c>
-      <c r="E283" t="s">
-        <v>296</v>
-      </c>
-      <c r="F283" t="s">
-        <v>41</v>
-      </c>
-      <c r="J283" t="s">
-        <v>18</v>
-      </c>
-      <c r="K283" s="25">
-        <f>INDEX('feed pars'!U$6:U$43,MATCH(F283,'feed pars'!B$6:B$43,0))</f>
-        <v>11.5</v>
-      </c>
+      <c r="B283" s="28"/>
+      <c r="C283" s="29"/>
+      <c r="D283" s="29"/>
+      <c r="E283" s="29"/>
+      <c r="F283" s="29"/>
+      <c r="G283" s="29"/>
+      <c r="H283" s="29"/>
+      <c r="I283" s="29"/>
+      <c r="J283" s="29"/>
+      <c r="K283" s="29"/>
+      <c r="L283" s="29"/>
+      <c r="M283" s="29"/>
+      <c r="N283" s="29"/>
     </row>
     <row r="284" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
@@ -7109,14 +7150,20 @@
         <v>296</v>
       </c>
       <c r="F284" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="J284" t="s">
         <v>18</v>
       </c>
       <c r="K284" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F284,'feed pars'!B$6:B$43,0))</f>
-        <v>10.9</v>
+        <v>12.3</v>
+      </c>
+      <c r="L284" t="s">
+        <v>297</v>
+      </c>
+      <c r="M284" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="285" spans="1:14" x14ac:dyDescent="0.25">
@@ -7127,14 +7174,14 @@
         <v>296</v>
       </c>
       <c r="F285" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J285" t="s">
         <v>18</v>
       </c>
       <c r="K285" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F285,'feed pars'!B$6:B$43,0))</f>
-        <v>18.5</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="286" spans="1:14" x14ac:dyDescent="0.25">
@@ -7145,14 +7192,14 @@
         <v>296</v>
       </c>
       <c r="F286" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="J286" t="s">
         <v>18</v>
       </c>
       <c r="K286" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F286,'feed pars'!B$6:B$43,0))</f>
-        <v>17.5</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="287" spans="1:14" x14ac:dyDescent="0.25">
@@ -7163,14 +7210,14 @@
         <v>296</v>
       </c>
       <c r="F287" t="s">
-        <v>310</v>
+        <v>39</v>
       </c>
       <c r="J287" t="s">
         <v>18</v>
       </c>
       <c r="K287" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F287,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="288" spans="1:14" x14ac:dyDescent="0.25">
@@ -7181,17 +7228,17 @@
         <v>296</v>
       </c>
       <c r="F288" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J288" t="s">
         <v>18</v>
       </c>
       <c r="K288" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F288,'feed pars'!B$6:B$43,0))</f>
-        <v>9.9</v>
-      </c>
-    </row>
-    <row r="289" spans="1:14" x14ac:dyDescent="0.25">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="289" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>25</v>
       </c>
@@ -7199,17 +7246,17 @@
         <v>296</v>
       </c>
       <c r="F289" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="J289" t="s">
         <v>18</v>
       </c>
       <c r="K289" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F289,'feed pars'!B$6:B$43,0))</f>
-        <v>10.3</v>
-      </c>
-    </row>
-    <row r="290" spans="1:14" x14ac:dyDescent="0.25">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="290" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>25</v>
       </c>
@@ -7217,17 +7264,17 @@
         <v>296</v>
       </c>
       <c r="F290" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J290" t="s">
         <v>18</v>
       </c>
       <c r="K290" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F290,'feed pars'!B$6:B$43,0))</f>
-        <v>7.7</v>
-      </c>
-    </row>
-    <row r="291" spans="1:14" x14ac:dyDescent="0.25">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="291" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>25</v>
       </c>
@@ -7235,17 +7282,17 @@
         <v>296</v>
       </c>
       <c r="F291" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="J291" t="s">
         <v>18</v>
       </c>
       <c r="K291" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F291,'feed pars'!B$6:B$43,0))</f>
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="292" spans="1:14" x14ac:dyDescent="0.25">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="292" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>25</v>
       </c>
@@ -7253,17 +7300,17 @@
         <v>296</v>
       </c>
       <c r="F292" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="J292" t="s">
         <v>18</v>
       </c>
       <c r="K292" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F292,'feed pars'!B$6:B$43,0))</f>
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="293" spans="1:14" x14ac:dyDescent="0.25">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="293" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>25</v>
       </c>
@@ -7271,17 +7318,17 @@
         <v>296</v>
       </c>
       <c r="F293" t="s">
-        <v>48</v>
+        <v>310</v>
       </c>
       <c r="J293" t="s">
         <v>18</v>
       </c>
       <c r="K293" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F293,'feed pars'!B$6:B$43,0))</f>
-        <v>7.8</v>
-      </c>
-    </row>
-    <row r="294" spans="1:14" x14ac:dyDescent="0.25">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="294" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>25</v>
       </c>
@@ -7289,17 +7336,17 @@
         <v>296</v>
       </c>
       <c r="F294" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="J294" t="s">
         <v>18</v>
       </c>
       <c r="K294" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F294,'feed pars'!B$6:B$43,0))</f>
-        <v>9.1999999999999993</v>
-      </c>
-    </row>
-    <row r="295" spans="1:14" x14ac:dyDescent="0.25">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="295" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>25</v>
       </c>
@@ -7307,17 +7354,17 @@
         <v>296</v>
       </c>
       <c r="F295" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="J295" t="s">
         <v>18</v>
       </c>
       <c r="K295" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F295,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
-      </c>
-    </row>
-    <row r="296" spans="1:14" x14ac:dyDescent="0.25">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="296" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>25</v>
       </c>
@@ -7325,17 +7372,17 @@
         <v>296</v>
       </c>
       <c r="F296" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J296" t="s">
         <v>18</v>
       </c>
       <c r="K296" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F296,'feed pars'!B$6:B$43,0))</f>
-        <v>8.9</v>
-      </c>
-    </row>
-    <row r="297" spans="1:14" x14ac:dyDescent="0.25">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="297" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>25</v>
       </c>
@@ -7343,17 +7390,17 @@
         <v>296</v>
       </c>
       <c r="F297" t="s">
-        <v>309</v>
+        <v>46</v>
       </c>
       <c r="J297" t="s">
         <v>18</v>
       </c>
       <c r="K297" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F297,'feed pars'!B$6:B$43,0))</f>
-        <v>7.0888888888888877</v>
-      </c>
-    </row>
-    <row r="298" spans="1:14" x14ac:dyDescent="0.25">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="298" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>25</v>
       </c>
@@ -7361,17 +7408,17 @@
         <v>296</v>
       </c>
       <c r="F298" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="J298" t="s">
         <v>18</v>
       </c>
       <c r="K298" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F298,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="299" spans="1:14" x14ac:dyDescent="0.25">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="299" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>25</v>
       </c>
@@ -7379,17 +7426,17 @@
         <v>296</v>
       </c>
       <c r="F299" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="J299" t="s">
         <v>18</v>
       </c>
       <c r="K299" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F299,'feed pars'!B$6:B$43,0))</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="300" spans="1:14" x14ac:dyDescent="0.25">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="300" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>25</v>
       </c>
@@ -7397,17 +7444,17 @@
         <v>296</v>
       </c>
       <c r="F300" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="J300" t="s">
         <v>18</v>
       </c>
       <c r="K300" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F300,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="301" spans="1:14" x14ac:dyDescent="0.25">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="301" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>25</v>
       </c>
@@ -7415,17 +7462,17 @@
         <v>296</v>
       </c>
       <c r="F301" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="J301" t="s">
         <v>18</v>
       </c>
       <c r="K301" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F301,'feed pars'!B$6:B$43,0))</f>
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="302" spans="1:14" x14ac:dyDescent="0.25">
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="302" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>25</v>
       </c>
@@ -7433,17 +7480,17 @@
         <v>296</v>
       </c>
       <c r="F302" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="J302" t="s">
         <v>18</v>
       </c>
       <c r="K302" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F302,'feed pars'!B$6:B$43,0))</f>
-        <v>11.3</v>
-      </c>
-    </row>
-    <row r="303" spans="1:14" x14ac:dyDescent="0.25">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="303" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>25</v>
       </c>
@@ -7451,278 +7498,296 @@
         <v>296</v>
       </c>
       <c r="F303" t="s">
-        <v>57</v>
+        <v>309</v>
       </c>
       <c r="J303" t="s">
         <v>18</v>
       </c>
       <c r="K303" s="25">
         <f>INDEX('feed pars'!U$6:U$43,MATCH(F303,'feed pars'!B$6:B$43,0))</f>
-        <v>10.8</v>
-      </c>
-    </row>
-    <row r="304" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A304" s="27" t="s">
-        <v>388</v>
-      </c>
-      <c r="B304" s="28"/>
-      <c r="C304" s="29"/>
-      <c r="D304" s="29"/>
-      <c r="E304" s="29"/>
-      <c r="F304" s="29"/>
-      <c r="G304" s="29"/>
-      <c r="H304" s="29"/>
-      <c r="I304" s="29"/>
-      <c r="J304" s="29"/>
-      <c r="K304" s="29"/>
-      <c r="L304" s="29"/>
-      <c r="M304" s="29"/>
-      <c r="N304" s="29"/>
-    </row>
-    <row r="305" spans="1:13" x14ac:dyDescent="0.25">
+        <v>7.0888888888888877</v>
+      </c>
+    </row>
+    <row r="304" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A304" t="s">
+        <v>25</v>
+      </c>
+      <c r="E304" t="s">
+        <v>296</v>
+      </c>
+      <c r="F304" t="s">
+        <v>52</v>
+      </c>
+      <c r="J304" t="s">
+        <v>18</v>
+      </c>
+      <c r="K304" s="25">
+        <f>INDEX('feed pars'!U$6:U$43,MATCH(F304,'feed pars'!B$6:B$43,0))</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="305" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>25</v>
       </c>
+      <c r="E305" t="s">
+        <v>296</v>
+      </c>
       <c r="F305" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="J305" t="s">
         <v>18</v>
       </c>
       <c r="K305" s="25">
-        <f>INDEX('feed pars'!T$6:T$43,MATCH(F305,'feed pars'!B$6:B$43,0))</f>
-        <v>12.1</v>
-      </c>
-      <c r="L305" t="s">
-        <v>22</v>
-      </c>
-      <c r="M305" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="306" spans="1:13" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!U$6:U$43,MATCH(F305,'feed pars'!B$6:B$43,0))</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="306" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>25</v>
       </c>
+      <c r="E306" t="s">
+        <v>296</v>
+      </c>
       <c r="F306" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="J306" t="s">
         <v>18</v>
       </c>
       <c r="K306" s="25">
-        <f>INDEX('feed pars'!T$6:T$43,MATCH(F306,'feed pars'!B$6:B$43,0))</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="307" spans="1:13" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!U$6:U$43,MATCH(F306,'feed pars'!B$6:B$43,0))</f>
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="307" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>25</v>
       </c>
+      <c r="E307" t="s">
+        <v>296</v>
+      </c>
       <c r="F307" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="J307" t="s">
         <v>18</v>
       </c>
       <c r="K307" s="25">
-        <f>INDEX('feed pars'!T$6:T$43,MATCH(F307,'feed pars'!B$6:B$43,0))</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="308" spans="1:13" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!U$6:U$43,MATCH(F307,'feed pars'!B$6:B$43,0))</f>
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="308" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>25</v>
       </c>
+      <c r="E308" t="s">
+        <v>296</v>
+      </c>
       <c r="F308" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="J308" t="s">
         <v>18</v>
       </c>
       <c r="K308" s="25">
-        <f>INDEX('feed pars'!T$6:T$43,MATCH(F308,'feed pars'!B$6:B$43,0))</f>
-        <v>11.9</v>
-      </c>
-    </row>
-    <row r="309" spans="1:13" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!U$6:U$43,MATCH(F308,'feed pars'!B$6:B$43,0))</f>
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="309" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>25</v>
       </c>
+      <c r="E309" t="s">
+        <v>296</v>
+      </c>
       <c r="F309" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="J309" t="s">
         <v>18</v>
       </c>
       <c r="K309" s="25">
-        <f>INDEX('feed pars'!T$6:T$43,MATCH(F309,'feed pars'!B$6:B$43,0))</f>
-        <v>12.8</v>
-      </c>
-    </row>
-    <row r="310" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A310" t="s">
-        <v>25</v>
-      </c>
-      <c r="F310" t="s">
-        <v>41</v>
-      </c>
-      <c r="J310" t="s">
-        <v>18</v>
-      </c>
-      <c r="K310" s="25">
-        <f>INDEX('feed pars'!T$6:T$43,MATCH(F310,'feed pars'!B$6:B$43,0))</f>
-        <v>11.2</v>
-      </c>
-    </row>
-    <row r="311" spans="1:13" x14ac:dyDescent="0.25">
+        <f>INDEX('feed pars'!U$6:U$43,MATCH(F309,'feed pars'!B$6:B$43,0))</f>
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="310" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A310" s="27" t="s">
+        <v>388</v>
+      </c>
+      <c r="B310" s="28"/>
+      <c r="C310" s="29"/>
+      <c r="D310" s="29"/>
+      <c r="E310" s="29"/>
+      <c r="F310" s="29"/>
+      <c r="G310" s="29"/>
+      <c r="H310" s="29"/>
+      <c r="I310" s="29"/>
+      <c r="J310" s="29"/>
+      <c r="K310" s="29"/>
+      <c r="L310" s="29"/>
+      <c r="M310" s="29"/>
+      <c r="N310" s="29"/>
+    </row>
+    <row r="311" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>25</v>
       </c>
       <c r="F311" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="J311" t="s">
         <v>18</v>
       </c>
       <c r="K311" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F311,'feed pars'!B$6:B$43,0))</f>
-        <v>10.7</v>
-      </c>
-    </row>
-    <row r="312" spans="1:13" x14ac:dyDescent="0.25">
+        <v>12.1</v>
+      </c>
+      <c r="L311" t="s">
+        <v>22</v>
+      </c>
+      <c r="M311" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="312" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>25</v>
       </c>
       <c r="F312" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J312" t="s">
         <v>18</v>
       </c>
       <c r="K312" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F312,'feed pars'!B$6:B$43,0))</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="313" spans="1:13" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="313" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>25</v>
       </c>
       <c r="F313" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="J313" t="s">
         <v>18</v>
       </c>
       <c r="K313" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F313,'feed pars'!B$6:B$43,0))</f>
-        <v>17.3</v>
-      </c>
-    </row>
-    <row r="314" spans="1:13" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="314" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>25</v>
       </c>
       <c r="F314" t="s">
-        <v>310</v>
+        <v>39</v>
       </c>
       <c r="J314" t="s">
         <v>18</v>
       </c>
       <c r="K314" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F314,'feed pars'!B$6:B$43,0))</f>
-        <v>29.8</v>
-      </c>
-    </row>
-    <row r="315" spans="1:13" x14ac:dyDescent="0.25">
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="315" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>25</v>
       </c>
       <c r="F315" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J315" t="s">
         <v>18</v>
       </c>
       <c r="K315" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F315,'feed pars'!B$6:B$43,0))</f>
-        <v>9.3000000000000007</v>
-      </c>
-    </row>
-    <row r="316" spans="1:13" x14ac:dyDescent="0.25">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="316" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>25</v>
       </c>
       <c r="F316" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="J316" t="s">
         <v>18</v>
       </c>
       <c r="K316" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F316,'feed pars'!B$6:B$43,0))</f>
-        <v>9.6999999999999993</v>
-      </c>
-    </row>
-    <row r="317" spans="1:13" x14ac:dyDescent="0.25">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="317" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>25</v>
       </c>
       <c r="F317" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J317" t="s">
         <v>18</v>
       </c>
       <c r="K317" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F317,'feed pars'!B$6:B$43,0))</f>
-        <v>7.1</v>
-      </c>
-    </row>
-    <row r="318" spans="1:13" x14ac:dyDescent="0.25">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="318" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>25</v>
       </c>
       <c r="F318" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="J318" t="s">
         <v>18</v>
       </c>
       <c r="K318" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F318,'feed pars'!B$6:B$43,0))</f>
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="319" spans="1:13" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="319" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>25</v>
       </c>
       <c r="F319" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="J319" t="s">
         <v>18</v>
       </c>
       <c r="K319" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F319,'feed pars'!B$6:B$43,0))</f>
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="320" spans="1:13" x14ac:dyDescent="0.25">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="320" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>25</v>
       </c>
       <c r="F320" t="s">
-        <v>48</v>
+        <v>310</v>
       </c>
       <c r="J320" t="s">
         <v>18</v>
       </c>
       <c r="K320" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F320,'feed pars'!B$6:B$43,0))</f>
-        <v>7.2</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="321" spans="1:11" x14ac:dyDescent="0.25">
@@ -7730,14 +7795,14 @@
         <v>25</v>
       </c>
       <c r="F321" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="J321" t="s">
         <v>18</v>
       </c>
       <c r="K321" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F321,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
+        <v>9.3000000000000007</v>
       </c>
     </row>
     <row r="322" spans="1:11" x14ac:dyDescent="0.25">
@@ -7745,14 +7810,14 @@
         <v>25</v>
       </c>
       <c r="F322" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="J322" t="s">
         <v>18</v>
       </c>
       <c r="K322" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F322,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1</v>
+        <v>9.6999999999999993</v>
       </c>
     </row>
     <row r="323" spans="1:11" x14ac:dyDescent="0.25">
@@ -7760,14 +7825,14 @@
         <v>25</v>
       </c>
       <c r="F323" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="J323" t="s">
         <v>18</v>
       </c>
       <c r="K323" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F323,'feed pars'!B$6:B$43,0))</f>
-        <v>8.1999999999999993</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="324" spans="1:11" x14ac:dyDescent="0.25">
@@ -7775,14 +7840,14 @@
         <v>25</v>
       </c>
       <c r="F324" t="s">
-        <v>309</v>
+        <v>46</v>
       </c>
       <c r="J324" t="s">
         <v>18</v>
       </c>
       <c r="K324" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F324,'feed pars'!B$6:B$43,0))</f>
-        <v>6.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="325" spans="1:11" x14ac:dyDescent="0.25">
@@ -7790,14 +7855,14 @@
         <v>25</v>
       </c>
       <c r="F325" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="J325" t="s">
         <v>18</v>
       </c>
       <c r="K325" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F325,'feed pars'!B$6:B$43,0))</f>
-        <v>8.6999999999999993</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="326" spans="1:11" x14ac:dyDescent="0.25">
@@ -7805,14 +7870,14 @@
         <v>25</v>
       </c>
       <c r="F326" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="J326" t="s">
         <v>18</v>
       </c>
       <c r="K326" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F326,'feed pars'!B$6:B$43,0))</f>
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="327" spans="1:11" x14ac:dyDescent="0.25">
@@ -7820,14 +7885,14 @@
         <v>25</v>
       </c>
       <c r="F327" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="J327" t="s">
         <v>18</v>
       </c>
       <c r="K327" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F327,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="328" spans="1:11" x14ac:dyDescent="0.25">
@@ -7835,14 +7900,14 @@
         <v>25</v>
       </c>
       <c r="F328" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="J328" t="s">
         <v>18</v>
       </c>
       <c r="K328" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F328,'feed pars'!B$6:B$43,0))</f>
-        <v>12.4</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="329" spans="1:11" x14ac:dyDescent="0.25">
@@ -7850,14 +7915,14 @@
         <v>25</v>
       </c>
       <c r="F329" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="J329" t="s">
         <v>18</v>
       </c>
       <c r="K329" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F329,'feed pars'!B$6:B$43,0))</f>
-        <v>11.1</v>
+        <v>8.1999999999999993</v>
       </c>
     </row>
     <row r="330" spans="1:11" x14ac:dyDescent="0.25">
@@ -7865,13 +7930,103 @@
         <v>25</v>
       </c>
       <c r="F330" t="s">
-        <v>57</v>
+        <v>309</v>
       </c>
       <c r="J330" t="s">
         <v>18</v>
       </c>
       <c r="K330" s="25">
         <f>INDEX('feed pars'!T$6:T$43,MATCH(F330,'feed pars'!B$6:B$43,0))</f>
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="331" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A331" t="s">
+        <v>25</v>
+      </c>
+      <c r="F331" t="s">
+        <v>52</v>
+      </c>
+      <c r="J331" t="s">
+        <v>18</v>
+      </c>
+      <c r="K331" s="25">
+        <f>INDEX('feed pars'!T$6:T$43,MATCH(F331,'feed pars'!B$6:B$43,0))</f>
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="332" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A332" t="s">
+        <v>25</v>
+      </c>
+      <c r="F332" t="s">
+        <v>53</v>
+      </c>
+      <c r="J332" t="s">
+        <v>18</v>
+      </c>
+      <c r="K332" s="25">
+        <f>INDEX('feed pars'!T$6:T$43,MATCH(F332,'feed pars'!B$6:B$43,0))</f>
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="333" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A333" t="s">
+        <v>25</v>
+      </c>
+      <c r="F333" t="s">
+        <v>54</v>
+      </c>
+      <c r="J333" t="s">
+        <v>18</v>
+      </c>
+      <c r="K333" s="25">
+        <f>INDEX('feed pars'!T$6:T$43,MATCH(F333,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="334" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A334" t="s">
+        <v>25</v>
+      </c>
+      <c r="F334" t="s">
+        <v>55</v>
+      </c>
+      <c r="J334" t="s">
+        <v>18</v>
+      </c>
+      <c r="K334" s="25">
+        <f>INDEX('feed pars'!T$6:T$43,MATCH(F334,'feed pars'!B$6:B$43,0))</f>
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="335" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A335" t="s">
+        <v>25</v>
+      </c>
+      <c r="F335" t="s">
+        <v>56</v>
+      </c>
+      <c r="J335" t="s">
+        <v>18</v>
+      </c>
+      <c r="K335" s="25">
+        <f>INDEX('feed pars'!T$6:T$43,MATCH(F335,'feed pars'!B$6:B$43,0))</f>
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="336" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A336" t="s">
+        <v>25</v>
+      </c>
+      <c r="F336" t="s">
+        <v>57</v>
+      </c>
+      <c r="J336" t="s">
+        <v>18</v>
+      </c>
+      <c r="K336" s="25">
+        <f>INDEX('feed pars'!T$6:T$43,MATCH(F336,'feed pars'!B$6:B$43,0))</f>
         <v>10.8</v>
       </c>
     </row>

</xml_diff>